<commit_message>
Log MQTT data 2026-08-08 06:27 UTC
</commit_message>
<xml_diff>
--- a/logs/raiv_tracker_2026-08-08.xlsx
+++ b/logs/raiv_tracker_2026-08-08.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F86"/>
+  <dimension ref="A1:F171"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -469,7 +469,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr"/>
       <c r="F2" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g2</t>
@@ -497,7 +496,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr"/>
       <c r="F3" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g3</t>
@@ -525,7 +523,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr"/>
       <c r="F4" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g4</t>
@@ -553,7 +550,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr"/>
       <c r="F5" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g5</t>
@@ -581,7 +577,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr"/>
       <c r="F6" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g6</t>
@@ -609,7 +604,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr"/>
       <c r="F7" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g7</t>
@@ -637,7 +631,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E8" t="inlineStr"/>
       <c r="F8" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g13</t>
@@ -665,7 +658,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E9" t="inlineStr"/>
       <c r="F9" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g15</t>
@@ -693,7 +685,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E10" t="inlineStr"/>
       <c r="F10" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g17</t>
@@ -721,7 +712,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E11" t="inlineStr"/>
       <c r="F11" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g18</t>
@@ -749,7 +739,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E12" t="inlineStr"/>
       <c r="F12" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g19</t>
@@ -777,7 +766,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E13" t="inlineStr"/>
       <c r="F13" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g22</t>
@@ -805,7 +793,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E14" t="inlineStr"/>
       <c r="F14" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g23</t>
@@ -833,7 +820,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E15" t="inlineStr"/>
       <c r="F15" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g24</t>
@@ -861,7 +847,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E16" t="inlineStr"/>
       <c r="F16" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g1</t>
@@ -889,7 +874,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E17" t="inlineStr"/>
       <c r="F17" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g8</t>
@@ -917,7 +901,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E18" t="inlineStr"/>
       <c r="F18" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g9</t>
@@ -945,7 +928,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E19" t="inlineStr"/>
       <c r="F19" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g10</t>
@@ -973,7 +955,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E20" t="inlineStr"/>
       <c r="F20" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g11</t>
@@ -1001,7 +982,6 @@
           <t>1</t>
         </is>
       </c>
-      <c r="E21" t="inlineStr"/>
       <c r="F21" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g12</t>
@@ -1029,7 +1009,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E22" t="inlineStr"/>
       <c r="F22" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g14</t>
@@ -1057,7 +1036,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E23" t="inlineStr"/>
       <c r="F23" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g16</t>
@@ -1085,7 +1063,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E24" t="inlineStr"/>
       <c r="F24" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g25</t>
@@ -1113,7 +1090,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E25" t="inlineStr"/>
       <c r="F25" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g33</t>
@@ -1141,7 +1117,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E26" t="inlineStr"/>
       <c r="F26" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g34</t>
@@ -1169,7 +1144,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E27" t="inlineStr"/>
       <c r="F27" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g36</t>
@@ -1197,7 +1171,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E28" t="inlineStr"/>
       <c r="F28" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g20</t>
@@ -1225,7 +1198,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E29" t="inlineStr"/>
       <c r="F29" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g21</t>
@@ -1253,7 +1225,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E30" t="inlineStr"/>
       <c r="F30" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g40</t>
@@ -1281,7 +1252,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E31" t="inlineStr"/>
       <c r="F31" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g26</t>
@@ -1309,7 +1279,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E32" t="inlineStr"/>
       <c r="F32" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g27</t>
@@ -1337,7 +1306,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E33" t="inlineStr"/>
       <c r="F33" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g28</t>
@@ -1365,7 +1333,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E34" t="inlineStr"/>
       <c r="F34" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g29</t>
@@ -1393,7 +1360,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E35" t="inlineStr"/>
       <c r="F35" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g30</t>
@@ -1421,7 +1387,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E36" t="inlineStr"/>
       <c r="F36" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g31</t>
@@ -1449,7 +1414,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E37" t="inlineStr"/>
       <c r="F37" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g32</t>
@@ -1477,7 +1441,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E38" t="inlineStr"/>
       <c r="F38" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g35</t>
@@ -1505,7 +1468,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E39" t="inlineStr"/>
       <c r="F39" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g37</t>
@@ -1533,7 +1495,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E40" t="inlineStr"/>
       <c r="F40" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g38</t>
@@ -1561,7 +1522,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E41" t="inlineStr"/>
       <c r="F41" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g39</t>
@@ -2823,6 +2783,2386 @@
         <v>3</v>
       </c>
       <c r="F86" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>2026-08-08T06:26:13</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>CountLaidButton</t>
+        </is>
+      </c>
+      <c r="D87" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E87" t="inlineStr"/>
+      <c r="F87" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g2</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>2026-08-08T06:26:13</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>CountLaidDetector</t>
+        </is>
+      </c>
+      <c r="D88" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E88" t="inlineStr"/>
+      <c r="F88" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g3</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>2026-08-08T06:26:13</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>TotalTiePlatesLaid</t>
+        </is>
+      </c>
+      <c r="D89" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E89" t="inlineStr"/>
+      <c r="F89" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g1</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>2026-08-08T06:26:13</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>usr_TPStime Hours10th</t>
+        </is>
+      </c>
+      <c r="D90" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E90" t="inlineStr"/>
+      <c r="F90" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g8</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>2026-08-08T06:26:13</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>usrTPS_miles xxx</t>
+        </is>
+      </c>
+      <c r="D91" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E91" t="inlineStr"/>
+      <c r="F91" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g9</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>2026-08-08T06:26:13</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>TPS Connected</t>
+        </is>
+      </c>
+      <c r="D92" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E92" t="inlineStr"/>
+      <c r="F92" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g10</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>2026-08-08T06:26:13</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>TPS Enabled</t>
+        </is>
+      </c>
+      <c r="D93" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E93" t="inlineStr"/>
+      <c r="F93" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g11</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>2026-08-08T06:26:13</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>14in Job</t>
+        </is>
+      </c>
+      <c r="D94" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E94" t="inlineStr"/>
+      <c r="F94" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g12</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>2026-08-08T06:26:13</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>CountLaidEncoder</t>
+        </is>
+      </c>
+      <c r="D95" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E95" t="inlineStr"/>
+      <c r="F95" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g4</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>2026-08-08T06:26:13</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>CountLaid14in</t>
+        </is>
+      </c>
+      <c r="D96" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E96" t="inlineStr"/>
+      <c r="F96" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g5</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>2026-08-08T06:26:13</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>CountLaid18in</t>
+        </is>
+      </c>
+      <c r="D97" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E97" t="inlineStr"/>
+      <c r="F97" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g6</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>2026-08-08T06:26:13</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>CountLaidPandral</t>
+        </is>
+      </c>
+      <c r="D98" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E98" t="inlineStr"/>
+      <c r="F98" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g7</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>2026-08-08T06:26:13</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>18in Job</t>
+        </is>
+      </c>
+      <c r="D99" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E99" t="inlineStr"/>
+      <c r="F99" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g13</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>2026-08-08T06:26:13</t>
+        </is>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>CountAcceptedTotal</t>
+        </is>
+      </c>
+      <c r="D100" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E100" t="inlineStr"/>
+      <c r="F100" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g15</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>2026-08-08T06:26:13</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>Servos_Enabled</t>
+        </is>
+      </c>
+      <c r="D101" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E101" t="inlineStr"/>
+      <c r="F101" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g17</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>2026-08-08T06:26:13</t>
+        </is>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>TotalPickPartsCount</t>
+        </is>
+      </c>
+      <c r="D102" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E102" t="inlineStr"/>
+      <c r="F102" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g18</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>2026-08-08T06:26:13</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>AcceptsPartsCount</t>
+        </is>
+      </c>
+      <c r="D103" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E103" t="inlineStr"/>
+      <c r="F103" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g19</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>2026-08-08T06:26:13</t>
+        </is>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>day_Servotime Hours10th</t>
+        </is>
+      </c>
+      <c r="D104" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E104" t="inlineStr"/>
+      <c r="F104" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g22</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>2026-08-08T06:26:13</t>
+        </is>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>tk_Cycle</t>
+        </is>
+      </c>
+      <c r="D105" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E105" t="inlineStr"/>
+      <c r="F105" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g23</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>2026-08-08T06:26:13</t>
+        </is>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>tk_Abort</t>
+        </is>
+      </c>
+      <c r="D106" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E106" t="inlineStr"/>
+      <c r="F106" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g24</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>2026-08-08T06:26:13</t>
+        </is>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>tk_ClearPos</t>
+        </is>
+      </c>
+      <c r="D107" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E107" t="inlineStr"/>
+      <c r="F107" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g25</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>2026-08-08T06:26:13</t>
+        </is>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>temp_J2motor</t>
+        </is>
+      </c>
+      <c r="D108" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E108" t="inlineStr"/>
+      <c r="F108" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g33</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>2026-08-08T06:26:13</t>
+        </is>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C109" t="inlineStr">
+        <is>
+          <t>temp_J3motor</t>
+        </is>
+      </c>
+      <c r="D109" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E109" t="inlineStr"/>
+      <c r="F109" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g34</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>2026-08-08T06:26:13</t>
+        </is>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C110" t="inlineStr">
+        <is>
+          <t>temp_J5motor</t>
+        </is>
+      </c>
+      <c r="D110" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E110" t="inlineStr"/>
+      <c r="F110" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g36</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>2026-08-08T06:26:13</t>
+        </is>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C111" t="inlineStr">
+        <is>
+          <t>Pandral Job</t>
+        </is>
+      </c>
+      <c r="D111" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E111" t="inlineStr"/>
+      <c r="F111" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g14</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>2026-08-08T06:26:13</t>
+        </is>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C112" t="inlineStr">
+        <is>
+          <t>CountRejectedTotal</t>
+        </is>
+      </c>
+      <c r="D112" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E112" t="inlineStr"/>
+      <c r="F112" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g16</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>2026-08-08T06:26:13</t>
+        </is>
+      </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C113" t="inlineStr">
+        <is>
+          <t>RejectPartsCount</t>
+        </is>
+      </c>
+      <c r="D113" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E113" t="inlineStr"/>
+      <c r="F113" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g20</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>2026-08-08T06:26:13</t>
+        </is>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C114" t="inlineStr">
+        <is>
+          <t>tk_Cycle hrs</t>
+        </is>
+      </c>
+      <c r="D114" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E114" t="inlineStr"/>
+      <c r="F114" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g21</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>2026-08-08T06:26:13</t>
+        </is>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C115" t="inlineStr">
+        <is>
+          <t>tk_Warmup</t>
+        </is>
+      </c>
+      <c r="D115" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E115" t="inlineStr"/>
+      <c r="F115" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g26</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>2026-08-08T06:26:13</t>
+        </is>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C116" t="inlineStr">
+        <is>
+          <t>FindingParts min</t>
+        </is>
+      </c>
+      <c r="D116" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E116" t="inlineStr"/>
+      <c r="F116" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g27</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>2026-08-08T06:26:13</t>
+        </is>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C117" t="inlineStr">
+        <is>
+          <t>PickingParts min</t>
+        </is>
+      </c>
+      <c r="D117" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E117" t="inlineStr"/>
+      <c r="F117" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g28</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="inlineStr">
+        <is>
+          <t>2026-08-08T06:26:13</t>
+        </is>
+      </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C118" t="inlineStr">
+        <is>
+          <t>PlacingParts min</t>
+        </is>
+      </c>
+      <c r="D118" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E118" t="inlineStr"/>
+      <c r="F118" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g29</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="inlineStr">
+        <is>
+          <t>2026-08-08T06:26:13</t>
+        </is>
+      </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C119" t="inlineStr">
+        <is>
+          <t>CountPickedReject14in</t>
+        </is>
+      </c>
+      <c r="D119" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E119" t="inlineStr"/>
+      <c r="F119" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g30</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="inlineStr">
+        <is>
+          <t>2026-08-08T06:26:13</t>
+        </is>
+      </c>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C120" t="inlineStr">
+        <is>
+          <t>temp_dsi</t>
+        </is>
+      </c>
+      <c r="D120" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E120" t="inlineStr"/>
+      <c r="F120" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g31</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="inlineStr">
+        <is>
+          <t>2026-08-08T06:26:13</t>
+        </is>
+      </c>
+      <c r="B121" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C121" t="inlineStr">
+        <is>
+          <t>temp_J1motor</t>
+        </is>
+      </c>
+      <c r="D121" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E121" t="inlineStr"/>
+      <c r="F121" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g32</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="inlineStr">
+        <is>
+          <t>2026-08-08T06:26:13</t>
+        </is>
+      </c>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C122" t="inlineStr">
+        <is>
+          <t>temp_J4motor</t>
+        </is>
+      </c>
+      <c r="D122" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E122" t="inlineStr"/>
+      <c r="F122" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g35</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="inlineStr">
+        <is>
+          <t>2026-08-08T06:26:13</t>
+        </is>
+      </c>
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C123" t="inlineStr">
+        <is>
+          <t>temp_J6motor</t>
+        </is>
+      </c>
+      <c r="D123" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E123" t="inlineStr"/>
+      <c r="F123" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g37</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="inlineStr">
+        <is>
+          <t>2026-08-08T06:26:13</t>
+        </is>
+      </c>
+      <c r="B124" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C124" t="inlineStr">
+        <is>
+          <t>CountPickedRejectOTM</t>
+        </is>
+      </c>
+      <c r="D124" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E124" t="inlineStr"/>
+      <c r="F124" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g38</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="inlineStr">
+        <is>
+          <t>2026-08-08T06:26:13</t>
+        </is>
+      </c>
+      <c r="B125" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C125" t="inlineStr">
+        <is>
+          <t>CountPickedRejectPandral</t>
+        </is>
+      </c>
+      <c r="D125" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E125" t="inlineStr"/>
+      <c r="F125" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g39</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="inlineStr">
+        <is>
+          <t>2026-08-08T06:26:13</t>
+        </is>
+      </c>
+      <c r="B126" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C126" t="inlineStr">
+        <is>
+          <t>CountPickedReject18in</t>
+        </is>
+      </c>
+      <c r="D126" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E126" t="inlineStr"/>
+      <c r="F126" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g40</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="inlineStr">
+        <is>
+          <t>2026-08-08T06:27:00</t>
+        </is>
+      </c>
+      <c r="B127" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C127" t="inlineStr">
+        <is>
+          <t>_1st_SCAN</t>
+        </is>
+      </c>
+      <c r="D127" t="b">
+        <v>0</v>
+      </c>
+      <c r="E127" t="n">
+        <v>11</v>
+      </c>
+      <c r="F127" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="inlineStr">
+        <is>
+          <t>2026-08-08T06:27:00</t>
+        </is>
+      </c>
+      <c r="B128" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C128" t="inlineStr">
+        <is>
+          <t>TieDetectOffset_B</t>
+        </is>
+      </c>
+      <c r="D128" t="b">
+        <v>0</v>
+      </c>
+      <c r="E128" t="n">
+        <v>11</v>
+      </c>
+      <c r="F128" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="inlineStr">
+        <is>
+          <t>2026-08-08T06:27:00</t>
+        </is>
+      </c>
+      <c r="B129" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C129" t="inlineStr">
+        <is>
+          <t>Tie Detector</t>
+        </is>
+      </c>
+      <c r="D129" t="b">
+        <v>0</v>
+      </c>
+      <c r="E129" t="n">
+        <v>11</v>
+      </c>
+      <c r="F129" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="inlineStr">
+        <is>
+          <t>2026-08-08T06:27:00</t>
+        </is>
+      </c>
+      <c r="B130" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C130" t="inlineStr">
+        <is>
+          <t>TPS Full</t>
+        </is>
+      </c>
+      <c r="D130" t="b">
+        <v>0</v>
+      </c>
+      <c r="E130" t="n">
+        <v>11</v>
+      </c>
+      <c r="F130" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="inlineStr">
+        <is>
+          <t>2026-08-08T06:27:00</t>
+        </is>
+      </c>
+      <c r="B131" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C131" t="inlineStr">
+        <is>
+          <t>TieDetectOffset_A</t>
+        </is>
+      </c>
+      <c r="D131" t="b">
+        <v>0</v>
+      </c>
+      <c r="E131" t="n">
+        <v>11</v>
+      </c>
+      <c r="F131" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" t="inlineStr">
+        <is>
+          <t>2026-08-08T06:27:00</t>
+        </is>
+      </c>
+      <c r="B132" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C132" t="inlineStr">
+        <is>
+          <t>TPS Connected</t>
+        </is>
+      </c>
+      <c r="D132" t="b">
+        <v>0</v>
+      </c>
+      <c r="E132" t="n">
+        <v>11</v>
+      </c>
+      <c r="F132" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" t="inlineStr">
+        <is>
+          <t>2026-08-08T06:27:00</t>
+        </is>
+      </c>
+      <c r="B133" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C133" t="inlineStr">
+        <is>
+          <t>TPS_Enable_ Button</t>
+        </is>
+      </c>
+      <c r="D133" t="b">
+        <v>0</v>
+      </c>
+      <c r="E133" t="n">
+        <v>11</v>
+      </c>
+      <c r="F133" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" t="inlineStr">
+        <is>
+          <t>2026-08-08T06:27:00</t>
+        </is>
+      </c>
+      <c r="B134" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C134" t="inlineStr">
+        <is>
+          <t>AirEagle Eject Plate</t>
+        </is>
+      </c>
+      <c r="D134" t="b">
+        <v>0</v>
+      </c>
+      <c r="E134" t="n">
+        <v>11</v>
+      </c>
+      <c r="F134" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" t="inlineStr">
+        <is>
+          <t>2026-08-08T06:27:00</t>
+        </is>
+      </c>
+      <c r="B135" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C135" t="inlineStr">
+        <is>
+          <t>tk_Cycle</t>
+        </is>
+      </c>
+      <c r="D135" t="b">
+        <v>0</v>
+      </c>
+      <c r="E135" t="n">
+        <v>11</v>
+      </c>
+      <c r="F135" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" t="inlineStr">
+        <is>
+          <t>2026-08-08T06:27:00</t>
+        </is>
+      </c>
+      <c r="B136" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C136" t="inlineStr">
+        <is>
+          <t>Servos_Enabled</t>
+        </is>
+      </c>
+      <c r="D136" t="b">
+        <v>0</v>
+      </c>
+      <c r="E136" t="n">
+        <v>11</v>
+      </c>
+      <c r="F136" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" t="inlineStr">
+        <is>
+          <t>2026-08-08T06:27:00</t>
+        </is>
+      </c>
+      <c r="B137" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C137" t="inlineStr">
+        <is>
+          <t>TPS Enabled</t>
+        </is>
+      </c>
+      <c r="D137" t="b">
+        <v>0</v>
+      </c>
+      <c r="E137" t="n">
+        <v>11</v>
+      </c>
+      <c r="F137" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" t="inlineStr">
+        <is>
+          <t>2026-08-08T06:27:00</t>
+        </is>
+      </c>
+      <c r="B138" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C138" t="inlineStr">
+        <is>
+          <t>tk_Abort</t>
+        </is>
+      </c>
+      <c r="D138" t="b">
+        <v>0</v>
+      </c>
+      <c r="E138" t="n">
+        <v>11</v>
+      </c>
+      <c r="F138" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" t="inlineStr">
+        <is>
+          <t>2026-08-08T06:27:00</t>
+        </is>
+      </c>
+      <c r="B139" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C139" t="inlineStr">
+        <is>
+          <t>Robot_isMoving</t>
+        </is>
+      </c>
+      <c r="D139" t="b">
+        <v>0</v>
+      </c>
+      <c r="E139" t="n">
+        <v>11</v>
+      </c>
+      <c r="F139" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" t="inlineStr">
+        <is>
+          <t>2026-08-08T06:27:00</t>
+        </is>
+      </c>
+      <c r="B140" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C140" t="inlineStr">
+        <is>
+          <t>Eject Tie Plate</t>
+        </is>
+      </c>
+      <c r="D140" t="b">
+        <v>0</v>
+      </c>
+      <c r="E140" t="n">
+        <v>11</v>
+      </c>
+      <c r="F140" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" t="inlineStr">
+        <is>
+          <t>2026-08-08T06:27:00</t>
+        </is>
+      </c>
+      <c r="B141" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C141" t="inlineStr">
+        <is>
+          <t>TPS BACKUP ALARM</t>
+        </is>
+      </c>
+      <c r="D141" t="b">
+        <v>0</v>
+      </c>
+      <c r="E141" t="n">
+        <v>11</v>
+      </c>
+      <c r="F141" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" t="inlineStr">
+        <is>
+          <t>2026-08-08T06:27:00</t>
+        </is>
+      </c>
+      <c r="B142" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C142" t="inlineStr">
+        <is>
+          <t>14in Job</t>
+        </is>
+      </c>
+      <c r="D142" t="b">
+        <v>1</v>
+      </c>
+      <c r="E142" t="n">
+        <v>11</v>
+      </c>
+      <c r="F142" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" t="inlineStr">
+        <is>
+          <t>2026-08-08T06:27:00</t>
+        </is>
+      </c>
+      <c r="B143" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C143" t="inlineStr">
+        <is>
+          <t>18in Job</t>
+        </is>
+      </c>
+      <c r="D143" t="b">
+        <v>0</v>
+      </c>
+      <c r="E143" t="n">
+        <v>11</v>
+      </c>
+      <c r="F143" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" t="inlineStr">
+        <is>
+          <t>2026-08-08T06:27:00</t>
+        </is>
+      </c>
+      <c r="B144" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C144" t="inlineStr">
+        <is>
+          <t>Pandral Job</t>
+        </is>
+      </c>
+      <c r="D144" t="b">
+        <v>0</v>
+      </c>
+      <c r="E144" t="n">
+        <v>11</v>
+      </c>
+      <c r="F144" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" t="inlineStr">
+        <is>
+          <t>2026-08-08T06:27:00</t>
+        </is>
+      </c>
+      <c r="B145" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C145" t="inlineStr">
+        <is>
+          <t>DoubleLay Job</t>
+        </is>
+      </c>
+      <c r="D145" t="b">
+        <v>0</v>
+      </c>
+      <c r="E145" t="n">
+        <v>11</v>
+      </c>
+      <c r="F145" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" t="inlineStr">
+        <is>
+          <t>2026-08-08T06:27:00</t>
+        </is>
+      </c>
+      <c r="B146" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C146" t="inlineStr">
+        <is>
+          <t>TPSjam_FLAG</t>
+        </is>
+      </c>
+      <c r="D146" t="b">
+        <v>0</v>
+      </c>
+      <c r="E146" t="n">
+        <v>11</v>
+      </c>
+      <c r="F146" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" t="inlineStr">
+        <is>
+          <t>2026-08-08T06:27:00</t>
+        </is>
+      </c>
+      <c r="B147" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C147" t="inlineStr">
+        <is>
+          <t>RoCalRequest</t>
+        </is>
+      </c>
+      <c r="D147" t="b">
+        <v>0</v>
+      </c>
+      <c r="E147" t="n">
+        <v>11</v>
+      </c>
+      <c r="F147" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" t="inlineStr">
+        <is>
+          <t>2026-08-08T06:27:00</t>
+        </is>
+      </c>
+      <c r="B148" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C148" t="inlineStr">
+        <is>
+          <t>tkCycle_TotalSeconds</t>
+        </is>
+      </c>
+      <c r="D148" t="n">
+        <v>0</v>
+      </c>
+      <c r="E148" t="n">
+        <v>9</v>
+      </c>
+      <c r="F148" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" t="inlineStr">
+        <is>
+          <t>2026-08-08T06:27:00</t>
+        </is>
+      </c>
+      <c r="B149" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C149" t="inlineStr">
+        <is>
+          <t>tkCycle_NoMoveSec</t>
+        </is>
+      </c>
+      <c r="D149" t="n">
+        <v>0</v>
+      </c>
+      <c r="E149" t="n">
+        <v>9</v>
+      </c>
+      <c r="F149" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" t="inlineStr">
+        <is>
+          <t>2026-08-08T06:27:00</t>
+        </is>
+      </c>
+      <c r="B150" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C150" t="inlineStr">
+        <is>
+          <t>tkCycle_MoveSeconds</t>
+        </is>
+      </c>
+      <c r="D150" t="n">
+        <v>0</v>
+      </c>
+      <c r="E150" t="n">
+        <v>9</v>
+      </c>
+      <c r="F150" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" t="inlineStr">
+        <is>
+          <t>2026-08-08T06:27:00</t>
+        </is>
+      </c>
+      <c r="B151" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C151" t="inlineStr">
+        <is>
+          <t>Percent time moveing</t>
+        </is>
+      </c>
+      <c r="D151" t="n">
+        <v>0</v>
+      </c>
+      <c r="E151" t="n">
+        <v>9</v>
+      </c>
+      <c r="F151" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" t="inlineStr">
+        <is>
+          <t>2026-08-08T06:27:00</t>
+        </is>
+      </c>
+      <c r="B152" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C152" t="inlineStr">
+        <is>
+          <t>Percent time not moving</t>
+        </is>
+      </c>
+      <c r="D152" t="n">
+        <v>0</v>
+      </c>
+      <c r="E152" t="n">
+        <v>9</v>
+      </c>
+      <c r="F152" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" t="inlineStr">
+        <is>
+          <t>2026-08-08T06:27:00</t>
+        </is>
+      </c>
+      <c r="B153" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C153" t="inlineStr">
+        <is>
+          <t>TotalPickPartsCount</t>
+        </is>
+      </c>
+      <c r="D153" t="n">
+        <v>0</v>
+      </c>
+      <c r="E153" t="n">
+        <v>9</v>
+      </c>
+      <c r="F153" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" t="inlineStr">
+        <is>
+          <t>2026-08-08T06:27:00</t>
+        </is>
+      </c>
+      <c r="B154" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C154" t="inlineStr">
+        <is>
+          <t>RejectPartsCount</t>
+        </is>
+      </c>
+      <c r="D154" t="n">
+        <v>0</v>
+      </c>
+      <c r="E154" t="n">
+        <v>9</v>
+      </c>
+      <c r="F154" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" t="inlineStr">
+        <is>
+          <t>2026-08-08T06:27:00</t>
+        </is>
+      </c>
+      <c r="B155" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C155" t="inlineStr">
+        <is>
+          <t>AcceptsPartsCount</t>
+        </is>
+      </c>
+      <c r="D155" t="n">
+        <v>0</v>
+      </c>
+      <c r="E155" t="n">
+        <v>9</v>
+      </c>
+      <c r="F155" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" t="inlineStr">
+        <is>
+          <t>2026-08-08T06:27:00</t>
+        </is>
+      </c>
+      <c r="B156" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C156" t="inlineStr">
+        <is>
+          <t>percentCount_accept</t>
+        </is>
+      </c>
+      <c r="D156" t="n">
+        <v>0</v>
+      </c>
+      <c r="E156" t="n">
+        <v>9</v>
+      </c>
+      <c r="F156" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" t="inlineStr">
+        <is>
+          <t>2026-08-08T06:27:00</t>
+        </is>
+      </c>
+      <c r="B157" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C157" t="inlineStr">
+        <is>
+          <t>percentCount_reject</t>
+        </is>
+      </c>
+      <c r="D157" t="n">
+        <v>0</v>
+      </c>
+      <c r="E157" t="n">
+        <v>9</v>
+      </c>
+      <c r="F157" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" t="inlineStr">
+        <is>
+          <t>2026-08-08T06:27:00</t>
+        </is>
+      </c>
+      <c r="B158" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C158" t="inlineStr">
+        <is>
+          <t>Avg Parts per min_total</t>
+        </is>
+      </c>
+      <c r="D158" t="n">
+        <v>0</v>
+      </c>
+      <c r="E158" t="n">
+        <v>9</v>
+      </c>
+      <c r="F158" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" t="inlineStr">
+        <is>
+          <t>2026-08-08T06:27:00</t>
+        </is>
+      </c>
+      <c r="B159" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C159" t="inlineStr">
+        <is>
+          <t>TotalPickedParts</t>
+        </is>
+      </c>
+      <c r="D159" t="n">
+        <v>0</v>
+      </c>
+      <c r="E159" t="n">
+        <v>3</v>
+      </c>
+      <c r="F159" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" t="inlineStr">
+        <is>
+          <t>2026-08-08T06:27:00</t>
+        </is>
+      </c>
+      <c r="B160" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C160" t="inlineStr">
+        <is>
+          <t>TotalPickedAcceptParts</t>
+        </is>
+      </c>
+      <c r="D160" t="n">
+        <v>0</v>
+      </c>
+      <c r="E160" t="n">
+        <v>3</v>
+      </c>
+      <c r="F160" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" t="inlineStr">
+        <is>
+          <t>2026-08-08T06:27:00</t>
+        </is>
+      </c>
+      <c r="B161" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C161" t="inlineStr">
+        <is>
+          <t>TotalPickedRejectParts</t>
+        </is>
+      </c>
+      <c r="D161" t="n">
+        <v>0</v>
+      </c>
+      <c r="E161" t="n">
+        <v>3</v>
+      </c>
+      <c r="F161" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" t="inlineStr">
+        <is>
+          <t>2026-08-08T06:27:00</t>
+        </is>
+      </c>
+      <c r="B162" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C162" t="inlineStr">
+        <is>
+          <t>TotalTiePlatesLaid</t>
+        </is>
+      </c>
+      <c r="D162" t="n">
+        <v>0</v>
+      </c>
+      <c r="E162" t="n">
+        <v>3</v>
+      </c>
+      <c r="F162" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" t="inlineStr">
+        <is>
+          <t>2026-08-08T06:27:00</t>
+        </is>
+      </c>
+      <c r="B163" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C163" t="inlineStr">
+        <is>
+          <t>Daily_TotalLaidPlates</t>
+        </is>
+      </c>
+      <c r="D163" t="n">
+        <v>0</v>
+      </c>
+      <c r="E163" t="n">
+        <v>3</v>
+      </c>
+      <c r="F163" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" t="inlineStr">
+        <is>
+          <t>2026-08-08T06:27:00</t>
+        </is>
+      </c>
+      <c r="B164" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C164" t="inlineStr">
+        <is>
+          <t>CountPicked14in</t>
+        </is>
+      </c>
+      <c r="D164" t="n">
+        <v>0</v>
+      </c>
+      <c r="E164" t="n">
+        <v>3</v>
+      </c>
+      <c r="F164" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" t="inlineStr">
+        <is>
+          <t>2026-08-08T06:27:00</t>
+        </is>
+      </c>
+      <c r="B165" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C165" t="inlineStr">
+        <is>
+          <t>CountPicked18in</t>
+        </is>
+      </c>
+      <c r="D165" t="n">
+        <v>0</v>
+      </c>
+      <c r="E165" t="n">
+        <v>3</v>
+      </c>
+      <c r="F165" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" t="inlineStr">
+        <is>
+          <t>2026-08-08T06:27:00</t>
+        </is>
+      </c>
+      <c r="B166" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C166" t="inlineStr">
+        <is>
+          <t>CountPickedPandral</t>
+        </is>
+      </c>
+      <c r="D166" t="n">
+        <v>0</v>
+      </c>
+      <c r="E166" t="n">
+        <v>3</v>
+      </c>
+      <c r="F166" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" t="inlineStr">
+        <is>
+          <t>2026-08-08T06:27:00</t>
+        </is>
+      </c>
+      <c r="B167" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C167" t="inlineStr">
+        <is>
+          <t>CountPickedOTM</t>
+        </is>
+      </c>
+      <c r="D167" t="n">
+        <v>0</v>
+      </c>
+      <c r="E167" t="n">
+        <v>3</v>
+      </c>
+      <c r="F167" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" t="inlineStr">
+        <is>
+          <t>2026-08-08T06:27:00</t>
+        </is>
+      </c>
+      <c r="B168" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C168" t="inlineStr">
+        <is>
+          <t>RoCals</t>
+        </is>
+      </c>
+      <c r="D168" t="n">
+        <v>0</v>
+      </c>
+      <c r="E168" t="n">
+        <v>3</v>
+      </c>
+      <c r="F168" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" t="inlineStr">
+        <is>
+          <t>2026-08-08T06:27:00</t>
+        </is>
+      </c>
+      <c r="B169" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C169" t="inlineStr">
+        <is>
+          <t>TPS_JamsUsr</t>
+        </is>
+      </c>
+      <c r="D169" t="n">
+        <v>0</v>
+      </c>
+      <c r="E169" t="n">
+        <v>3</v>
+      </c>
+      <c r="F169" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" t="inlineStr">
+        <is>
+          <t>2026-08-08T06:27:00</t>
+        </is>
+      </c>
+      <c r="B170" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C170" t="inlineStr">
+        <is>
+          <t>TPS_JamsMASTER</t>
+        </is>
+      </c>
+      <c r="D170" t="n">
+        <v>0</v>
+      </c>
+      <c r="E170" t="n">
+        <v>3</v>
+      </c>
+      <c r="F170" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" t="inlineStr">
+        <is>
+          <t>2026-08-08T06:27:00</t>
+        </is>
+      </c>
+      <c r="B171" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C171" t="inlineStr">
+        <is>
+          <t>ABORT_Master</t>
+        </is>
+      </c>
+      <c r="D171" t="n">
+        <v>0</v>
+      </c>
+      <c r="E171" t="n">
+        <v>3</v>
+      </c>
+      <c r="F171" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/plc</t>
         </is>

</xml_diff>

<commit_message>
Log MQTT data 2026-08-08 08:24 UTC
</commit_message>
<xml_diff>
--- a/logs/raiv_tracker_2026-08-08.xlsx
+++ b/logs/raiv_tracker_2026-08-08.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F171"/>
+  <dimension ref="A1:F301"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2809,7 +2809,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E87" t="inlineStr"/>
       <c r="F87" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g2</t>
@@ -2837,7 +2836,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E88" t="inlineStr"/>
       <c r="F88" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g3</t>
@@ -2865,7 +2863,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E89" t="inlineStr"/>
       <c r="F89" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g1</t>
@@ -2893,7 +2890,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E90" t="inlineStr"/>
       <c r="F90" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g8</t>
@@ -2921,7 +2917,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E91" t="inlineStr"/>
       <c r="F91" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g9</t>
@@ -2949,7 +2944,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E92" t="inlineStr"/>
       <c r="F92" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g10</t>
@@ -2977,7 +2971,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E93" t="inlineStr"/>
       <c r="F93" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g11</t>
@@ -3005,7 +2998,6 @@
           <t>1</t>
         </is>
       </c>
-      <c r="E94" t="inlineStr"/>
       <c r="F94" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g12</t>
@@ -3033,7 +3025,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E95" t="inlineStr"/>
       <c r="F95" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g4</t>
@@ -3061,7 +3052,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E96" t="inlineStr"/>
       <c r="F96" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g5</t>
@@ -3089,7 +3079,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E97" t="inlineStr"/>
       <c r="F97" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g6</t>
@@ -3117,7 +3106,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E98" t="inlineStr"/>
       <c r="F98" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g7</t>
@@ -3145,7 +3133,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E99" t="inlineStr"/>
       <c r="F99" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g13</t>
@@ -3173,7 +3160,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E100" t="inlineStr"/>
       <c r="F100" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g15</t>
@@ -3201,7 +3187,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E101" t="inlineStr"/>
       <c r="F101" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g17</t>
@@ -3229,7 +3214,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E102" t="inlineStr"/>
       <c r="F102" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g18</t>
@@ -3257,7 +3241,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E103" t="inlineStr"/>
       <c r="F103" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g19</t>
@@ -3285,7 +3268,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E104" t="inlineStr"/>
       <c r="F104" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g22</t>
@@ -3313,7 +3295,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E105" t="inlineStr"/>
       <c r="F105" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g23</t>
@@ -3341,7 +3322,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E106" t="inlineStr"/>
       <c r="F106" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g24</t>
@@ -3369,7 +3349,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E107" t="inlineStr"/>
       <c r="F107" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g25</t>
@@ -3397,7 +3376,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E108" t="inlineStr"/>
       <c r="F108" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g33</t>
@@ -3425,7 +3403,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E109" t="inlineStr"/>
       <c r="F109" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g34</t>
@@ -3453,7 +3430,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E110" t="inlineStr"/>
       <c r="F110" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g36</t>
@@ -3481,7 +3457,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E111" t="inlineStr"/>
       <c r="F111" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g14</t>
@@ -3509,7 +3484,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E112" t="inlineStr"/>
       <c r="F112" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g16</t>
@@ -3537,7 +3511,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E113" t="inlineStr"/>
       <c r="F113" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g20</t>
@@ -3565,7 +3538,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E114" t="inlineStr"/>
       <c r="F114" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g21</t>
@@ -3593,7 +3565,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E115" t="inlineStr"/>
       <c r="F115" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g26</t>
@@ -3621,7 +3592,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E116" t="inlineStr"/>
       <c r="F116" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g27</t>
@@ -3649,7 +3619,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E117" t="inlineStr"/>
       <c r="F117" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g28</t>
@@ -3677,7 +3646,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E118" t="inlineStr"/>
       <c r="F118" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g29</t>
@@ -3705,7 +3673,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E119" t="inlineStr"/>
       <c r="F119" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g30</t>
@@ -3733,7 +3700,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E120" t="inlineStr"/>
       <c r="F120" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g31</t>
@@ -3761,7 +3727,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E121" t="inlineStr"/>
       <c r="F121" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g32</t>
@@ -3789,7 +3754,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E122" t="inlineStr"/>
       <c r="F122" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g35</t>
@@ -3817,7 +3781,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E123" t="inlineStr"/>
       <c r="F123" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g37</t>
@@ -3845,7 +3808,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E124" t="inlineStr"/>
       <c r="F124" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g38</t>
@@ -3873,7 +3835,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E125" t="inlineStr"/>
       <c r="F125" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g39</t>
@@ -3901,7 +3862,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E126" t="inlineStr"/>
       <c r="F126" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g40</t>
@@ -5163,6 +5123,3646 @@
         <v>3</v>
       </c>
       <c r="F171" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" t="inlineStr">
+        <is>
+          <t>2026-08-08T08:23:00</t>
+        </is>
+      </c>
+      <c r="B172" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C172" t="inlineStr">
+        <is>
+          <t>_1st_SCAN</t>
+        </is>
+      </c>
+      <c r="D172" t="b">
+        <v>0</v>
+      </c>
+      <c r="E172" t="n">
+        <v>11</v>
+      </c>
+      <c r="F172" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" t="inlineStr">
+        <is>
+          <t>2026-08-08T08:23:00</t>
+        </is>
+      </c>
+      <c r="B173" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C173" t="inlineStr">
+        <is>
+          <t>TieDetectOffset_B</t>
+        </is>
+      </c>
+      <c r="D173" t="b">
+        <v>0</v>
+      </c>
+      <c r="E173" t="n">
+        <v>11</v>
+      </c>
+      <c r="F173" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" t="inlineStr">
+        <is>
+          <t>2026-08-08T08:23:00</t>
+        </is>
+      </c>
+      <c r="B174" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C174" t="inlineStr">
+        <is>
+          <t>Tie Detector</t>
+        </is>
+      </c>
+      <c r="D174" t="b">
+        <v>0</v>
+      </c>
+      <c r="E174" t="n">
+        <v>11</v>
+      </c>
+      <c r="F174" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" t="inlineStr">
+        <is>
+          <t>2026-08-08T08:23:00</t>
+        </is>
+      </c>
+      <c r="B175" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C175" t="inlineStr">
+        <is>
+          <t>TPS Full</t>
+        </is>
+      </c>
+      <c r="D175" t="b">
+        <v>0</v>
+      </c>
+      <c r="E175" t="n">
+        <v>11</v>
+      </c>
+      <c r="F175" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" t="inlineStr">
+        <is>
+          <t>2026-08-08T08:23:00</t>
+        </is>
+      </c>
+      <c r="B176" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C176" t="inlineStr">
+        <is>
+          <t>TieDetectOffset_A</t>
+        </is>
+      </c>
+      <c r="D176" t="b">
+        <v>0</v>
+      </c>
+      <c r="E176" t="n">
+        <v>11</v>
+      </c>
+      <c r="F176" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" t="inlineStr">
+        <is>
+          <t>2026-08-08T08:23:00</t>
+        </is>
+      </c>
+      <c r="B177" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C177" t="inlineStr">
+        <is>
+          <t>TPS Connected</t>
+        </is>
+      </c>
+      <c r="D177" t="b">
+        <v>0</v>
+      </c>
+      <c r="E177" t="n">
+        <v>11</v>
+      </c>
+      <c r="F177" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" t="inlineStr">
+        <is>
+          <t>2026-08-08T08:23:00</t>
+        </is>
+      </c>
+      <c r="B178" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C178" t="inlineStr">
+        <is>
+          <t>TPS_Enable_ Button</t>
+        </is>
+      </c>
+      <c r="D178" t="b">
+        <v>0</v>
+      </c>
+      <c r="E178" t="n">
+        <v>11</v>
+      </c>
+      <c r="F178" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" t="inlineStr">
+        <is>
+          <t>2026-08-08T08:23:00</t>
+        </is>
+      </c>
+      <c r="B179" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C179" t="inlineStr">
+        <is>
+          <t>AirEagle Eject Plate</t>
+        </is>
+      </c>
+      <c r="D179" t="b">
+        <v>0</v>
+      </c>
+      <c r="E179" t="n">
+        <v>11</v>
+      </c>
+      <c r="F179" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" t="inlineStr">
+        <is>
+          <t>2026-08-08T08:23:00</t>
+        </is>
+      </c>
+      <c r="B180" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C180" t="inlineStr">
+        <is>
+          <t>tk_Cycle</t>
+        </is>
+      </c>
+      <c r="D180" t="b">
+        <v>0</v>
+      </c>
+      <c r="E180" t="n">
+        <v>11</v>
+      </c>
+      <c r="F180" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" t="inlineStr">
+        <is>
+          <t>2026-08-08T08:23:00</t>
+        </is>
+      </c>
+      <c r="B181" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C181" t="inlineStr">
+        <is>
+          <t>Servos_Enabled</t>
+        </is>
+      </c>
+      <c r="D181" t="b">
+        <v>0</v>
+      </c>
+      <c r="E181" t="n">
+        <v>11</v>
+      </c>
+      <c r="F181" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" t="inlineStr">
+        <is>
+          <t>2026-08-08T08:23:00</t>
+        </is>
+      </c>
+      <c r="B182" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C182" t="inlineStr">
+        <is>
+          <t>TPS Enabled</t>
+        </is>
+      </c>
+      <c r="D182" t="b">
+        <v>0</v>
+      </c>
+      <c r="E182" t="n">
+        <v>11</v>
+      </c>
+      <c r="F182" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" t="inlineStr">
+        <is>
+          <t>2026-08-08T08:23:00</t>
+        </is>
+      </c>
+      <c r="B183" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C183" t="inlineStr">
+        <is>
+          <t>tk_Abort</t>
+        </is>
+      </c>
+      <c r="D183" t="b">
+        <v>0</v>
+      </c>
+      <c r="E183" t="n">
+        <v>11</v>
+      </c>
+      <c r="F183" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" t="inlineStr">
+        <is>
+          <t>2026-08-08T08:23:00</t>
+        </is>
+      </c>
+      <c r="B184" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C184" t="inlineStr">
+        <is>
+          <t>Robot_isMoving</t>
+        </is>
+      </c>
+      <c r="D184" t="b">
+        <v>0</v>
+      </c>
+      <c r="E184" t="n">
+        <v>11</v>
+      </c>
+      <c r="F184" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" t="inlineStr">
+        <is>
+          <t>2026-08-08T08:23:00</t>
+        </is>
+      </c>
+      <c r="B185" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C185" t="inlineStr">
+        <is>
+          <t>Eject Tie Plate</t>
+        </is>
+      </c>
+      <c r="D185" t="b">
+        <v>0</v>
+      </c>
+      <c r="E185" t="n">
+        <v>11</v>
+      </c>
+      <c r="F185" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" t="inlineStr">
+        <is>
+          <t>2026-08-08T08:23:00</t>
+        </is>
+      </c>
+      <c r="B186" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C186" t="inlineStr">
+        <is>
+          <t>TPS BACKUP ALARM</t>
+        </is>
+      </c>
+      <c r="D186" t="b">
+        <v>0</v>
+      </c>
+      <c r="E186" t="n">
+        <v>11</v>
+      </c>
+      <c r="F186" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" t="inlineStr">
+        <is>
+          <t>2026-08-08T08:23:00</t>
+        </is>
+      </c>
+      <c r="B187" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C187" t="inlineStr">
+        <is>
+          <t>14in Job</t>
+        </is>
+      </c>
+      <c r="D187" t="b">
+        <v>1</v>
+      </c>
+      <c r="E187" t="n">
+        <v>11</v>
+      </c>
+      <c r="F187" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188" t="inlineStr">
+        <is>
+          <t>2026-08-08T08:23:00</t>
+        </is>
+      </c>
+      <c r="B188" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C188" t="inlineStr">
+        <is>
+          <t>18in Job</t>
+        </is>
+      </c>
+      <c r="D188" t="b">
+        <v>0</v>
+      </c>
+      <c r="E188" t="n">
+        <v>11</v>
+      </c>
+      <c r="F188" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="189">
+      <c r="A189" t="inlineStr">
+        <is>
+          <t>2026-08-08T08:23:00</t>
+        </is>
+      </c>
+      <c r="B189" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C189" t="inlineStr">
+        <is>
+          <t>Pandral Job</t>
+        </is>
+      </c>
+      <c r="D189" t="b">
+        <v>0</v>
+      </c>
+      <c r="E189" t="n">
+        <v>11</v>
+      </c>
+      <c r="F189" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190" t="inlineStr">
+        <is>
+          <t>2026-08-08T08:23:00</t>
+        </is>
+      </c>
+      <c r="B190" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C190" t="inlineStr">
+        <is>
+          <t>DoubleLay Job</t>
+        </is>
+      </c>
+      <c r="D190" t="b">
+        <v>0</v>
+      </c>
+      <c r="E190" t="n">
+        <v>11</v>
+      </c>
+      <c r="F190" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191" t="inlineStr">
+        <is>
+          <t>2026-08-08T08:23:00</t>
+        </is>
+      </c>
+      <c r="B191" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C191" t="inlineStr">
+        <is>
+          <t>TPSjam_FLAG</t>
+        </is>
+      </c>
+      <c r="D191" t="b">
+        <v>0</v>
+      </c>
+      <c r="E191" t="n">
+        <v>11</v>
+      </c>
+      <c r="F191" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="192">
+      <c r="A192" t="inlineStr">
+        <is>
+          <t>2026-08-08T08:23:00</t>
+        </is>
+      </c>
+      <c r="B192" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C192" t="inlineStr">
+        <is>
+          <t>RoCalRequest</t>
+        </is>
+      </c>
+      <c r="D192" t="b">
+        <v>0</v>
+      </c>
+      <c r="E192" t="n">
+        <v>11</v>
+      </c>
+      <c r="F192" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="193">
+      <c r="A193" t="inlineStr">
+        <is>
+          <t>2026-08-08T08:23:00</t>
+        </is>
+      </c>
+      <c r="B193" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C193" t="inlineStr">
+        <is>
+          <t>tkCycle_TotalSeconds</t>
+        </is>
+      </c>
+      <c r="D193" t="n">
+        <v>0</v>
+      </c>
+      <c r="E193" t="n">
+        <v>9</v>
+      </c>
+      <c r="F193" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="194">
+      <c r="A194" t="inlineStr">
+        <is>
+          <t>2026-08-08T08:23:00</t>
+        </is>
+      </c>
+      <c r="B194" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C194" t="inlineStr">
+        <is>
+          <t>tkCycle_NoMoveSec</t>
+        </is>
+      </c>
+      <c r="D194" t="n">
+        <v>0</v>
+      </c>
+      <c r="E194" t="n">
+        <v>9</v>
+      </c>
+      <c r="F194" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="195">
+      <c r="A195" t="inlineStr">
+        <is>
+          <t>2026-08-08T08:23:00</t>
+        </is>
+      </c>
+      <c r="B195" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C195" t="inlineStr">
+        <is>
+          <t>tkCycle_MoveSeconds</t>
+        </is>
+      </c>
+      <c r="D195" t="n">
+        <v>0</v>
+      </c>
+      <c r="E195" t="n">
+        <v>9</v>
+      </c>
+      <c r="F195" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="196">
+      <c r="A196" t="inlineStr">
+        <is>
+          <t>2026-08-08T08:23:00</t>
+        </is>
+      </c>
+      <c r="B196" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C196" t="inlineStr">
+        <is>
+          <t>Percent time moveing</t>
+        </is>
+      </c>
+      <c r="D196" t="n">
+        <v>0</v>
+      </c>
+      <c r="E196" t="n">
+        <v>9</v>
+      </c>
+      <c r="F196" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="197">
+      <c r="A197" t="inlineStr">
+        <is>
+          <t>2026-08-08T08:23:00</t>
+        </is>
+      </c>
+      <c r="B197" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C197" t="inlineStr">
+        <is>
+          <t>Percent time not moving</t>
+        </is>
+      </c>
+      <c r="D197" t="n">
+        <v>0</v>
+      </c>
+      <c r="E197" t="n">
+        <v>9</v>
+      </c>
+      <c r="F197" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="198">
+      <c r="A198" t="inlineStr">
+        <is>
+          <t>2026-08-08T08:23:00</t>
+        </is>
+      </c>
+      <c r="B198" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C198" t="inlineStr">
+        <is>
+          <t>TotalPickPartsCount</t>
+        </is>
+      </c>
+      <c r="D198" t="n">
+        <v>0</v>
+      </c>
+      <c r="E198" t="n">
+        <v>9</v>
+      </c>
+      <c r="F198" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="199">
+      <c r="A199" t="inlineStr">
+        <is>
+          <t>2026-08-08T08:23:00</t>
+        </is>
+      </c>
+      <c r="B199" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C199" t="inlineStr">
+        <is>
+          <t>RejectPartsCount</t>
+        </is>
+      </c>
+      <c r="D199" t="n">
+        <v>0</v>
+      </c>
+      <c r="E199" t="n">
+        <v>9</v>
+      </c>
+      <c r="F199" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="200">
+      <c r="A200" t="inlineStr">
+        <is>
+          <t>2026-08-08T08:23:00</t>
+        </is>
+      </c>
+      <c r="B200" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C200" t="inlineStr">
+        <is>
+          <t>AcceptsPartsCount</t>
+        </is>
+      </c>
+      <c r="D200" t="n">
+        <v>0</v>
+      </c>
+      <c r="E200" t="n">
+        <v>9</v>
+      </c>
+      <c r="F200" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="201">
+      <c r="A201" t="inlineStr">
+        <is>
+          <t>2026-08-08T08:23:00</t>
+        </is>
+      </c>
+      <c r="B201" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C201" t="inlineStr">
+        <is>
+          <t>percentCount_accept</t>
+        </is>
+      </c>
+      <c r="D201" t="n">
+        <v>0</v>
+      </c>
+      <c r="E201" t="n">
+        <v>9</v>
+      </c>
+      <c r="F201" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="202">
+      <c r="A202" t="inlineStr">
+        <is>
+          <t>2026-08-08T08:23:00</t>
+        </is>
+      </c>
+      <c r="B202" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C202" t="inlineStr">
+        <is>
+          <t>percentCount_reject</t>
+        </is>
+      </c>
+      <c r="D202" t="n">
+        <v>0</v>
+      </c>
+      <c r="E202" t="n">
+        <v>9</v>
+      </c>
+      <c r="F202" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="203">
+      <c r="A203" t="inlineStr">
+        <is>
+          <t>2026-08-08T08:23:00</t>
+        </is>
+      </c>
+      <c r="B203" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C203" t="inlineStr">
+        <is>
+          <t>Avg Parts per min_total</t>
+        </is>
+      </c>
+      <c r="D203" t="n">
+        <v>0</v>
+      </c>
+      <c r="E203" t="n">
+        <v>9</v>
+      </c>
+      <c r="F203" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="204">
+      <c r="A204" t="inlineStr">
+        <is>
+          <t>2026-08-08T08:23:00</t>
+        </is>
+      </c>
+      <c r="B204" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C204" t="inlineStr">
+        <is>
+          <t>TotalPickedParts</t>
+        </is>
+      </c>
+      <c r="D204" t="n">
+        <v>0</v>
+      </c>
+      <c r="E204" t="n">
+        <v>3</v>
+      </c>
+      <c r="F204" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="205">
+      <c r="A205" t="inlineStr">
+        <is>
+          <t>2026-08-08T08:23:00</t>
+        </is>
+      </c>
+      <c r="B205" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C205" t="inlineStr">
+        <is>
+          <t>TotalPickedAcceptParts</t>
+        </is>
+      </c>
+      <c r="D205" t="n">
+        <v>0</v>
+      </c>
+      <c r="E205" t="n">
+        <v>3</v>
+      </c>
+      <c r="F205" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="206">
+      <c r="A206" t="inlineStr">
+        <is>
+          <t>2026-08-08T08:23:00</t>
+        </is>
+      </c>
+      <c r="B206" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C206" t="inlineStr">
+        <is>
+          <t>TotalPickedRejectParts</t>
+        </is>
+      </c>
+      <c r="D206" t="n">
+        <v>0</v>
+      </c>
+      <c r="E206" t="n">
+        <v>3</v>
+      </c>
+      <c r="F206" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="207">
+      <c r="A207" t="inlineStr">
+        <is>
+          <t>2026-08-08T08:23:00</t>
+        </is>
+      </c>
+      <c r="B207" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C207" t="inlineStr">
+        <is>
+          <t>TotalTiePlatesLaid</t>
+        </is>
+      </c>
+      <c r="D207" t="n">
+        <v>0</v>
+      </c>
+      <c r="E207" t="n">
+        <v>3</v>
+      </c>
+      <c r="F207" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="208">
+      <c r="A208" t="inlineStr">
+        <is>
+          <t>2026-08-08T08:23:00</t>
+        </is>
+      </c>
+      <c r="B208" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C208" t="inlineStr">
+        <is>
+          <t>Daily_TotalLaidPlates</t>
+        </is>
+      </c>
+      <c r="D208" t="n">
+        <v>0</v>
+      </c>
+      <c r="E208" t="n">
+        <v>3</v>
+      </c>
+      <c r="F208" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="209">
+      <c r="A209" t="inlineStr">
+        <is>
+          <t>2026-08-08T08:23:00</t>
+        </is>
+      </c>
+      <c r="B209" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C209" t="inlineStr">
+        <is>
+          <t>CountPicked14in</t>
+        </is>
+      </c>
+      <c r="D209" t="n">
+        <v>0</v>
+      </c>
+      <c r="E209" t="n">
+        <v>3</v>
+      </c>
+      <c r="F209" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="210">
+      <c r="A210" t="inlineStr">
+        <is>
+          <t>2026-08-08T08:23:00</t>
+        </is>
+      </c>
+      <c r="B210" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C210" t="inlineStr">
+        <is>
+          <t>CountPicked18in</t>
+        </is>
+      </c>
+      <c r="D210" t="n">
+        <v>0</v>
+      </c>
+      <c r="E210" t="n">
+        <v>3</v>
+      </c>
+      <c r="F210" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="211">
+      <c r="A211" t="inlineStr">
+        <is>
+          <t>2026-08-08T08:23:00</t>
+        </is>
+      </c>
+      <c r="B211" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C211" t="inlineStr">
+        <is>
+          <t>CountPickedPandral</t>
+        </is>
+      </c>
+      <c r="D211" t="n">
+        <v>0</v>
+      </c>
+      <c r="E211" t="n">
+        <v>3</v>
+      </c>
+      <c r="F211" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="212">
+      <c r="A212" t="inlineStr">
+        <is>
+          <t>2026-08-08T08:23:00</t>
+        </is>
+      </c>
+      <c r="B212" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C212" t="inlineStr">
+        <is>
+          <t>CountPickedOTM</t>
+        </is>
+      </c>
+      <c r="D212" t="n">
+        <v>0</v>
+      </c>
+      <c r="E212" t="n">
+        <v>3</v>
+      </c>
+      <c r="F212" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="213">
+      <c r="A213" t="inlineStr">
+        <is>
+          <t>2026-08-08T08:23:00</t>
+        </is>
+      </c>
+      <c r="B213" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C213" t="inlineStr">
+        <is>
+          <t>RoCals</t>
+        </is>
+      </c>
+      <c r="D213" t="n">
+        <v>0</v>
+      </c>
+      <c r="E213" t="n">
+        <v>3</v>
+      </c>
+      <c r="F213" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="214">
+      <c r="A214" t="inlineStr">
+        <is>
+          <t>2026-08-08T08:23:00</t>
+        </is>
+      </c>
+      <c r="B214" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C214" t="inlineStr">
+        <is>
+          <t>TPS_JamsUsr</t>
+        </is>
+      </c>
+      <c r="D214" t="n">
+        <v>0</v>
+      </c>
+      <c r="E214" t="n">
+        <v>3</v>
+      </c>
+      <c r="F214" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="215">
+      <c r="A215" t="inlineStr">
+        <is>
+          <t>2026-08-08T08:23:00</t>
+        </is>
+      </c>
+      <c r="B215" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C215" t="inlineStr">
+        <is>
+          <t>TPS_JamsMASTER</t>
+        </is>
+      </c>
+      <c r="D215" t="n">
+        <v>0</v>
+      </c>
+      <c r="E215" t="n">
+        <v>3</v>
+      </c>
+      <c r="F215" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="216">
+      <c r="A216" t="inlineStr">
+        <is>
+          <t>2026-08-08T08:23:00</t>
+        </is>
+      </c>
+      <c r="B216" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C216" t="inlineStr">
+        <is>
+          <t>ABORT_Master</t>
+        </is>
+      </c>
+      <c r="D216" t="n">
+        <v>0</v>
+      </c>
+      <c r="E216" t="n">
+        <v>3</v>
+      </c>
+      <c r="F216" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="217">
+      <c r="A217" t="inlineStr">
+        <is>
+          <t>2026-08-08T08:23:13</t>
+        </is>
+      </c>
+      <c r="B217" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C217" t="inlineStr">
+        <is>
+          <t>CountLaidButton</t>
+        </is>
+      </c>
+      <c r="D217" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E217" t="inlineStr"/>
+      <c r="F217" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g2</t>
+        </is>
+      </c>
+    </row>
+    <row r="218">
+      <c r="A218" t="inlineStr">
+        <is>
+          <t>2026-08-08T08:23:13</t>
+        </is>
+      </c>
+      <c r="B218" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C218" t="inlineStr">
+        <is>
+          <t>CountLaidDetector</t>
+        </is>
+      </c>
+      <c r="D218" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E218" t="inlineStr"/>
+      <c r="F218" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g3</t>
+        </is>
+      </c>
+    </row>
+    <row r="219">
+      <c r="A219" t="inlineStr">
+        <is>
+          <t>2026-08-08T08:23:13</t>
+        </is>
+      </c>
+      <c r="B219" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C219" t="inlineStr">
+        <is>
+          <t>CountLaidEncoder</t>
+        </is>
+      </c>
+      <c r="D219" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E219" t="inlineStr"/>
+      <c r="F219" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g4</t>
+        </is>
+      </c>
+    </row>
+    <row r="220">
+      <c r="A220" t="inlineStr">
+        <is>
+          <t>2026-08-08T08:23:13</t>
+        </is>
+      </c>
+      <c r="B220" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C220" t="inlineStr">
+        <is>
+          <t>CountLaid14in</t>
+        </is>
+      </c>
+      <c r="D220" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E220" t="inlineStr"/>
+      <c r="F220" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g5</t>
+        </is>
+      </c>
+    </row>
+    <row r="221">
+      <c r="A221" t="inlineStr">
+        <is>
+          <t>2026-08-08T08:23:13</t>
+        </is>
+      </c>
+      <c r="B221" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C221" t="inlineStr">
+        <is>
+          <t>CountLaid18in</t>
+        </is>
+      </c>
+      <c r="D221" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E221" t="inlineStr"/>
+      <c r="F221" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g6</t>
+        </is>
+      </c>
+    </row>
+    <row r="222">
+      <c r="A222" t="inlineStr">
+        <is>
+          <t>2026-08-08T08:23:13</t>
+        </is>
+      </c>
+      <c r="B222" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C222" t="inlineStr">
+        <is>
+          <t>CountLaidPandral</t>
+        </is>
+      </c>
+      <c r="D222" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E222" t="inlineStr"/>
+      <c r="F222" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g7</t>
+        </is>
+      </c>
+    </row>
+    <row r="223">
+      <c r="A223" t="inlineStr">
+        <is>
+          <t>2026-08-08T08:23:13</t>
+        </is>
+      </c>
+      <c r="B223" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C223" t="inlineStr">
+        <is>
+          <t>18in Job</t>
+        </is>
+      </c>
+      <c r="D223" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E223" t="inlineStr"/>
+      <c r="F223" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g13</t>
+        </is>
+      </c>
+    </row>
+    <row r="224">
+      <c r="A224" t="inlineStr">
+        <is>
+          <t>2026-08-08T08:23:13</t>
+        </is>
+      </c>
+      <c r="B224" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C224" t="inlineStr">
+        <is>
+          <t>CountAcceptedTotal</t>
+        </is>
+      </c>
+      <c r="D224" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E224" t="inlineStr"/>
+      <c r="F224" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g15</t>
+        </is>
+      </c>
+    </row>
+    <row r="225">
+      <c r="A225" t="inlineStr">
+        <is>
+          <t>2026-08-08T08:23:13</t>
+        </is>
+      </c>
+      <c r="B225" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C225" t="inlineStr">
+        <is>
+          <t>Servos_Enabled</t>
+        </is>
+      </c>
+      <c r="D225" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E225" t="inlineStr"/>
+      <c r="F225" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g17</t>
+        </is>
+      </c>
+    </row>
+    <row r="226">
+      <c r="A226" t="inlineStr">
+        <is>
+          <t>2026-08-08T08:23:13</t>
+        </is>
+      </c>
+      <c r="B226" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C226" t="inlineStr">
+        <is>
+          <t>TotalPickPartsCount</t>
+        </is>
+      </c>
+      <c r="D226" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E226" t="inlineStr"/>
+      <c r="F226" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g18</t>
+        </is>
+      </c>
+    </row>
+    <row r="227">
+      <c r="A227" t="inlineStr">
+        <is>
+          <t>2026-08-08T08:23:13</t>
+        </is>
+      </c>
+      <c r="B227" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C227" t="inlineStr">
+        <is>
+          <t>AcceptsPartsCount</t>
+        </is>
+      </c>
+      <c r="D227" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E227" t="inlineStr"/>
+      <c r="F227" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g19</t>
+        </is>
+      </c>
+    </row>
+    <row r="228">
+      <c r="A228" t="inlineStr">
+        <is>
+          <t>2026-08-08T08:23:13</t>
+        </is>
+      </c>
+      <c r="B228" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C228" t="inlineStr">
+        <is>
+          <t>day_Servotime Hours10th</t>
+        </is>
+      </c>
+      <c r="D228" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E228" t="inlineStr"/>
+      <c r="F228" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g22</t>
+        </is>
+      </c>
+    </row>
+    <row r="229">
+      <c r="A229" t="inlineStr">
+        <is>
+          <t>2026-08-08T08:23:13</t>
+        </is>
+      </c>
+      <c r="B229" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C229" t="inlineStr">
+        <is>
+          <t>tk_Cycle</t>
+        </is>
+      </c>
+      <c r="D229" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E229" t="inlineStr"/>
+      <c r="F229" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g23</t>
+        </is>
+      </c>
+    </row>
+    <row r="230">
+      <c r="A230" t="inlineStr">
+        <is>
+          <t>2026-08-08T08:23:13</t>
+        </is>
+      </c>
+      <c r="B230" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C230" t="inlineStr">
+        <is>
+          <t>tk_Abort</t>
+        </is>
+      </c>
+      <c r="D230" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E230" t="inlineStr"/>
+      <c r="F230" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g24</t>
+        </is>
+      </c>
+    </row>
+    <row r="231">
+      <c r="A231" t="inlineStr">
+        <is>
+          <t>2026-08-08T08:23:13</t>
+        </is>
+      </c>
+      <c r="B231" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C231" t="inlineStr">
+        <is>
+          <t>tk_ClearPos</t>
+        </is>
+      </c>
+      <c r="D231" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E231" t="inlineStr"/>
+      <c r="F231" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g25</t>
+        </is>
+      </c>
+    </row>
+    <row r="232">
+      <c r="A232" t="inlineStr">
+        <is>
+          <t>2026-08-08T08:23:13</t>
+        </is>
+      </c>
+      <c r="B232" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C232" t="inlineStr">
+        <is>
+          <t>TotalTiePlatesLaid</t>
+        </is>
+      </c>
+      <c r="D232" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E232" t="inlineStr"/>
+      <c r="F232" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g1</t>
+        </is>
+      </c>
+    </row>
+    <row r="233">
+      <c r="A233" t="inlineStr">
+        <is>
+          <t>2026-08-08T08:23:13</t>
+        </is>
+      </c>
+      <c r="B233" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C233" t="inlineStr">
+        <is>
+          <t>usr_TPStime Hours10th</t>
+        </is>
+      </c>
+      <c r="D233" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E233" t="inlineStr"/>
+      <c r="F233" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g8</t>
+        </is>
+      </c>
+    </row>
+    <row r="234">
+      <c r="A234" t="inlineStr">
+        <is>
+          <t>2026-08-08T08:23:13</t>
+        </is>
+      </c>
+      <c r="B234" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C234" t="inlineStr">
+        <is>
+          <t>usrTPS_miles xxx</t>
+        </is>
+      </c>
+      <c r="D234" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E234" t="inlineStr"/>
+      <c r="F234" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g9</t>
+        </is>
+      </c>
+    </row>
+    <row r="235">
+      <c r="A235" t="inlineStr">
+        <is>
+          <t>2026-08-08T08:23:13</t>
+        </is>
+      </c>
+      <c r="B235" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C235" t="inlineStr">
+        <is>
+          <t>TPS Connected</t>
+        </is>
+      </c>
+      <c r="D235" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E235" t="inlineStr"/>
+      <c r="F235" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g10</t>
+        </is>
+      </c>
+    </row>
+    <row r="236">
+      <c r="A236" t="inlineStr">
+        <is>
+          <t>2026-08-08T08:23:13</t>
+        </is>
+      </c>
+      <c r="B236" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C236" t="inlineStr">
+        <is>
+          <t>TPS Enabled</t>
+        </is>
+      </c>
+      <c r="D236" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E236" t="inlineStr"/>
+      <c r="F236" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g11</t>
+        </is>
+      </c>
+    </row>
+    <row r="237">
+      <c r="A237" t="inlineStr">
+        <is>
+          <t>2026-08-08T08:23:13</t>
+        </is>
+      </c>
+      <c r="B237" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C237" t="inlineStr">
+        <is>
+          <t>14in Job</t>
+        </is>
+      </c>
+      <c r="D237" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E237" t="inlineStr"/>
+      <c r="F237" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g12</t>
+        </is>
+      </c>
+    </row>
+    <row r="238">
+      <c r="A238" t="inlineStr">
+        <is>
+          <t>2026-08-08T08:23:13</t>
+        </is>
+      </c>
+      <c r="B238" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C238" t="inlineStr">
+        <is>
+          <t>Pandral Job</t>
+        </is>
+      </c>
+      <c r="D238" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E238" t="inlineStr"/>
+      <c r="F238" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g14</t>
+        </is>
+      </c>
+    </row>
+    <row r="239">
+      <c r="A239" t="inlineStr">
+        <is>
+          <t>2026-08-08T08:23:13</t>
+        </is>
+      </c>
+      <c r="B239" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C239" t="inlineStr">
+        <is>
+          <t>temp_J2motor</t>
+        </is>
+      </c>
+      <c r="D239" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E239" t="inlineStr"/>
+      <c r="F239" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g33</t>
+        </is>
+      </c>
+    </row>
+    <row r="240">
+      <c r="A240" t="inlineStr">
+        <is>
+          <t>2026-08-08T08:23:13</t>
+        </is>
+      </c>
+      <c r="B240" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C240" t="inlineStr">
+        <is>
+          <t>CountRejectedTotal</t>
+        </is>
+      </c>
+      <c r="D240" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E240" t="inlineStr"/>
+      <c r="F240" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g16</t>
+        </is>
+      </c>
+    </row>
+    <row r="241">
+      <c r="A241" t="inlineStr">
+        <is>
+          <t>2026-08-08T08:23:13</t>
+        </is>
+      </c>
+      <c r="B241" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C241" t="inlineStr">
+        <is>
+          <t>temp_J3motor</t>
+        </is>
+      </c>
+      <c r="D241" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E241" t="inlineStr"/>
+      <c r="F241" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g34</t>
+        </is>
+      </c>
+    </row>
+    <row r="242">
+      <c r="A242" t="inlineStr">
+        <is>
+          <t>2026-08-08T08:23:13</t>
+        </is>
+      </c>
+      <c r="B242" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C242" t="inlineStr">
+        <is>
+          <t>temp_J5motor</t>
+        </is>
+      </c>
+      <c r="D242" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E242" t="inlineStr"/>
+      <c r="F242" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g36</t>
+        </is>
+      </c>
+    </row>
+    <row r="243">
+      <c r="A243" t="inlineStr">
+        <is>
+          <t>2026-08-08T08:23:13</t>
+        </is>
+      </c>
+      <c r="B243" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C243" t="inlineStr">
+        <is>
+          <t>CountPickedReject18in</t>
+        </is>
+      </c>
+      <c r="D243" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E243" t="inlineStr"/>
+      <c r="F243" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g40</t>
+        </is>
+      </c>
+    </row>
+    <row r="244">
+      <c r="A244" t="inlineStr">
+        <is>
+          <t>2026-08-08T08:23:13</t>
+        </is>
+      </c>
+      <c r="B244" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C244" t="inlineStr">
+        <is>
+          <t>RejectPartsCount</t>
+        </is>
+      </c>
+      <c r="D244" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E244" t="inlineStr"/>
+      <c r="F244" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g20</t>
+        </is>
+      </c>
+    </row>
+    <row r="245">
+      <c r="A245" t="inlineStr">
+        <is>
+          <t>2026-08-08T08:23:13</t>
+        </is>
+      </c>
+      <c r="B245" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C245" t="inlineStr">
+        <is>
+          <t>tk_Cycle hrs</t>
+        </is>
+      </c>
+      <c r="D245" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E245" t="inlineStr"/>
+      <c r="F245" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g21</t>
+        </is>
+      </c>
+    </row>
+    <row r="246">
+      <c r="A246" t="inlineStr">
+        <is>
+          <t>2026-08-08T08:23:13</t>
+        </is>
+      </c>
+      <c r="B246" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C246" t="inlineStr">
+        <is>
+          <t>tk_Warmup</t>
+        </is>
+      </c>
+      <c r="D246" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E246" t="inlineStr"/>
+      <c r="F246" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g26</t>
+        </is>
+      </c>
+    </row>
+    <row r="247">
+      <c r="A247" t="inlineStr">
+        <is>
+          <t>2026-08-08T08:23:13</t>
+        </is>
+      </c>
+      <c r="B247" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C247" t="inlineStr">
+        <is>
+          <t>FindingParts min</t>
+        </is>
+      </c>
+      <c r="D247" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E247" t="inlineStr"/>
+      <c r="F247" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g27</t>
+        </is>
+      </c>
+    </row>
+    <row r="248">
+      <c r="A248" t="inlineStr">
+        <is>
+          <t>2026-08-08T08:23:13</t>
+        </is>
+      </c>
+      <c r="B248" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C248" t="inlineStr">
+        <is>
+          <t>PickingParts min</t>
+        </is>
+      </c>
+      <c r="D248" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E248" t="inlineStr"/>
+      <c r="F248" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g28</t>
+        </is>
+      </c>
+    </row>
+    <row r="249">
+      <c r="A249" t="inlineStr">
+        <is>
+          <t>2026-08-08T08:23:13</t>
+        </is>
+      </c>
+      <c r="B249" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C249" t="inlineStr">
+        <is>
+          <t>PlacingParts min</t>
+        </is>
+      </c>
+      <c r="D249" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E249" t="inlineStr"/>
+      <c r="F249" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g29</t>
+        </is>
+      </c>
+    </row>
+    <row r="250">
+      <c r="A250" t="inlineStr">
+        <is>
+          <t>2026-08-08T08:23:13</t>
+        </is>
+      </c>
+      <c r="B250" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C250" t="inlineStr">
+        <is>
+          <t>CountPickedReject14in</t>
+        </is>
+      </c>
+      <c r="D250" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E250" t="inlineStr"/>
+      <c r="F250" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g30</t>
+        </is>
+      </c>
+    </row>
+    <row r="251">
+      <c r="A251" t="inlineStr">
+        <is>
+          <t>2026-08-08T08:23:13</t>
+        </is>
+      </c>
+      <c r="B251" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C251" t="inlineStr">
+        <is>
+          <t>temp_dsi</t>
+        </is>
+      </c>
+      <c r="D251" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E251" t="inlineStr"/>
+      <c r="F251" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g31</t>
+        </is>
+      </c>
+    </row>
+    <row r="252">
+      <c r="A252" t="inlineStr">
+        <is>
+          <t>2026-08-08T08:23:13</t>
+        </is>
+      </c>
+      <c r="B252" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C252" t="inlineStr">
+        <is>
+          <t>temp_J1motor</t>
+        </is>
+      </c>
+      <c r="D252" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E252" t="inlineStr"/>
+      <c r="F252" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g32</t>
+        </is>
+      </c>
+    </row>
+    <row r="253">
+      <c r="A253" t="inlineStr">
+        <is>
+          <t>2026-08-08T08:23:13</t>
+        </is>
+      </c>
+      <c r="B253" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C253" t="inlineStr">
+        <is>
+          <t>temp_J4motor</t>
+        </is>
+      </c>
+      <c r="D253" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E253" t="inlineStr"/>
+      <c r="F253" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g35</t>
+        </is>
+      </c>
+    </row>
+    <row r="254">
+      <c r="A254" t="inlineStr">
+        <is>
+          <t>2026-08-08T08:23:13</t>
+        </is>
+      </c>
+      <c r="B254" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C254" t="inlineStr">
+        <is>
+          <t>temp_J6motor</t>
+        </is>
+      </c>
+      <c r="D254" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E254" t="inlineStr"/>
+      <c r="F254" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g37</t>
+        </is>
+      </c>
+    </row>
+    <row r="255">
+      <c r="A255" t="inlineStr">
+        <is>
+          <t>2026-08-08T08:23:13</t>
+        </is>
+      </c>
+      <c r="B255" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C255" t="inlineStr">
+        <is>
+          <t>CountPickedRejectOTM</t>
+        </is>
+      </c>
+      <c r="D255" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E255" t="inlineStr"/>
+      <c r="F255" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g38</t>
+        </is>
+      </c>
+    </row>
+    <row r="256">
+      <c r="A256" t="inlineStr">
+        <is>
+          <t>2026-08-08T08:23:13</t>
+        </is>
+      </c>
+      <c r="B256" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C256" t="inlineStr">
+        <is>
+          <t>CountPickedRejectPandral</t>
+        </is>
+      </c>
+      <c r="D256" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E256" t="inlineStr"/>
+      <c r="F256" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g39</t>
+        </is>
+      </c>
+    </row>
+    <row r="257">
+      <c r="A257" t="inlineStr">
+        <is>
+          <t>2026-08-08T08:24:00</t>
+        </is>
+      </c>
+      <c r="B257" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C257" t="inlineStr">
+        <is>
+          <t>_1st_SCAN</t>
+        </is>
+      </c>
+      <c r="D257" t="b">
+        <v>0</v>
+      </c>
+      <c r="E257" t="n">
+        <v>11</v>
+      </c>
+      <c r="F257" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="258">
+      <c r="A258" t="inlineStr">
+        <is>
+          <t>2026-08-08T08:24:00</t>
+        </is>
+      </c>
+      <c r="B258" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C258" t="inlineStr">
+        <is>
+          <t>TieDetectOffset_B</t>
+        </is>
+      </c>
+      <c r="D258" t="b">
+        <v>0</v>
+      </c>
+      <c r="E258" t="n">
+        <v>11</v>
+      </c>
+      <c r="F258" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="259">
+      <c r="A259" t="inlineStr">
+        <is>
+          <t>2026-08-08T08:24:00</t>
+        </is>
+      </c>
+      <c r="B259" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C259" t="inlineStr">
+        <is>
+          <t>Tie Detector</t>
+        </is>
+      </c>
+      <c r="D259" t="b">
+        <v>0</v>
+      </c>
+      <c r="E259" t="n">
+        <v>11</v>
+      </c>
+      <c r="F259" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="260">
+      <c r="A260" t="inlineStr">
+        <is>
+          <t>2026-08-08T08:24:00</t>
+        </is>
+      </c>
+      <c r="B260" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C260" t="inlineStr">
+        <is>
+          <t>TPS Full</t>
+        </is>
+      </c>
+      <c r="D260" t="b">
+        <v>0</v>
+      </c>
+      <c r="E260" t="n">
+        <v>11</v>
+      </c>
+      <c r="F260" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="261">
+      <c r="A261" t="inlineStr">
+        <is>
+          <t>2026-08-08T08:24:00</t>
+        </is>
+      </c>
+      <c r="B261" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C261" t="inlineStr">
+        <is>
+          <t>TieDetectOffset_A</t>
+        </is>
+      </c>
+      <c r="D261" t="b">
+        <v>0</v>
+      </c>
+      <c r="E261" t="n">
+        <v>11</v>
+      </c>
+      <c r="F261" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="262">
+      <c r="A262" t="inlineStr">
+        <is>
+          <t>2026-08-08T08:24:00</t>
+        </is>
+      </c>
+      <c r="B262" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C262" t="inlineStr">
+        <is>
+          <t>TPS Connected</t>
+        </is>
+      </c>
+      <c r="D262" t="b">
+        <v>0</v>
+      </c>
+      <c r="E262" t="n">
+        <v>11</v>
+      </c>
+      <c r="F262" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="263">
+      <c r="A263" t="inlineStr">
+        <is>
+          <t>2026-08-08T08:24:00</t>
+        </is>
+      </c>
+      <c r="B263" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C263" t="inlineStr">
+        <is>
+          <t>TPS_Enable_ Button</t>
+        </is>
+      </c>
+      <c r="D263" t="b">
+        <v>0</v>
+      </c>
+      <c r="E263" t="n">
+        <v>11</v>
+      </c>
+      <c r="F263" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="264">
+      <c r="A264" t="inlineStr">
+        <is>
+          <t>2026-08-08T08:24:00</t>
+        </is>
+      </c>
+      <c r="B264" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C264" t="inlineStr">
+        <is>
+          <t>AirEagle Eject Plate</t>
+        </is>
+      </c>
+      <c r="D264" t="b">
+        <v>0</v>
+      </c>
+      <c r="E264" t="n">
+        <v>11</v>
+      </c>
+      <c r="F264" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="265">
+      <c r="A265" t="inlineStr">
+        <is>
+          <t>2026-08-08T08:24:00</t>
+        </is>
+      </c>
+      <c r="B265" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C265" t="inlineStr">
+        <is>
+          <t>tk_Cycle</t>
+        </is>
+      </c>
+      <c r="D265" t="b">
+        <v>0</v>
+      </c>
+      <c r="E265" t="n">
+        <v>11</v>
+      </c>
+      <c r="F265" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="266">
+      <c r="A266" t="inlineStr">
+        <is>
+          <t>2026-08-08T08:24:00</t>
+        </is>
+      </c>
+      <c r="B266" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C266" t="inlineStr">
+        <is>
+          <t>Servos_Enabled</t>
+        </is>
+      </c>
+      <c r="D266" t="b">
+        <v>0</v>
+      </c>
+      <c r="E266" t="n">
+        <v>11</v>
+      </c>
+      <c r="F266" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="267">
+      <c r="A267" t="inlineStr">
+        <is>
+          <t>2026-08-08T08:24:00</t>
+        </is>
+      </c>
+      <c r="B267" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C267" t="inlineStr">
+        <is>
+          <t>TPS Enabled</t>
+        </is>
+      </c>
+      <c r="D267" t="b">
+        <v>0</v>
+      </c>
+      <c r="E267" t="n">
+        <v>11</v>
+      </c>
+      <c r="F267" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="268">
+      <c r="A268" t="inlineStr">
+        <is>
+          <t>2026-08-08T08:24:00</t>
+        </is>
+      </c>
+      <c r="B268" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C268" t="inlineStr">
+        <is>
+          <t>tk_Abort</t>
+        </is>
+      </c>
+      <c r="D268" t="b">
+        <v>0</v>
+      </c>
+      <c r="E268" t="n">
+        <v>11</v>
+      </c>
+      <c r="F268" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="269">
+      <c r="A269" t="inlineStr">
+        <is>
+          <t>2026-08-08T08:24:00</t>
+        </is>
+      </c>
+      <c r="B269" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C269" t="inlineStr">
+        <is>
+          <t>Robot_isMoving</t>
+        </is>
+      </c>
+      <c r="D269" t="b">
+        <v>0</v>
+      </c>
+      <c r="E269" t="n">
+        <v>11</v>
+      </c>
+      <c r="F269" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="270">
+      <c r="A270" t="inlineStr">
+        <is>
+          <t>2026-08-08T08:24:00</t>
+        </is>
+      </c>
+      <c r="B270" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C270" t="inlineStr">
+        <is>
+          <t>Eject Tie Plate</t>
+        </is>
+      </c>
+      <c r="D270" t="b">
+        <v>0</v>
+      </c>
+      <c r="E270" t="n">
+        <v>11</v>
+      </c>
+      <c r="F270" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="271">
+      <c r="A271" t="inlineStr">
+        <is>
+          <t>2026-08-08T08:24:00</t>
+        </is>
+      </c>
+      <c r="B271" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C271" t="inlineStr">
+        <is>
+          <t>TPS BACKUP ALARM</t>
+        </is>
+      </c>
+      <c r="D271" t="b">
+        <v>0</v>
+      </c>
+      <c r="E271" t="n">
+        <v>11</v>
+      </c>
+      <c r="F271" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="272">
+      <c r="A272" t="inlineStr">
+        <is>
+          <t>2026-08-08T08:24:00</t>
+        </is>
+      </c>
+      <c r="B272" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C272" t="inlineStr">
+        <is>
+          <t>14in Job</t>
+        </is>
+      </c>
+      <c r="D272" t="b">
+        <v>1</v>
+      </c>
+      <c r="E272" t="n">
+        <v>11</v>
+      </c>
+      <c r="F272" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="273">
+      <c r="A273" t="inlineStr">
+        <is>
+          <t>2026-08-08T08:24:00</t>
+        </is>
+      </c>
+      <c r="B273" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C273" t="inlineStr">
+        <is>
+          <t>18in Job</t>
+        </is>
+      </c>
+      <c r="D273" t="b">
+        <v>0</v>
+      </c>
+      <c r="E273" t="n">
+        <v>11</v>
+      </c>
+      <c r="F273" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="274">
+      <c r="A274" t="inlineStr">
+        <is>
+          <t>2026-08-08T08:24:00</t>
+        </is>
+      </c>
+      <c r="B274" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C274" t="inlineStr">
+        <is>
+          <t>Pandral Job</t>
+        </is>
+      </c>
+      <c r="D274" t="b">
+        <v>0</v>
+      </c>
+      <c r="E274" t="n">
+        <v>11</v>
+      </c>
+      <c r="F274" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="275">
+      <c r="A275" t="inlineStr">
+        <is>
+          <t>2026-08-08T08:24:00</t>
+        </is>
+      </c>
+      <c r="B275" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C275" t="inlineStr">
+        <is>
+          <t>DoubleLay Job</t>
+        </is>
+      </c>
+      <c r="D275" t="b">
+        <v>0</v>
+      </c>
+      <c r="E275" t="n">
+        <v>11</v>
+      </c>
+      <c r="F275" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="276">
+      <c r="A276" t="inlineStr">
+        <is>
+          <t>2026-08-08T08:24:00</t>
+        </is>
+      </c>
+      <c r="B276" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C276" t="inlineStr">
+        <is>
+          <t>TPSjam_FLAG</t>
+        </is>
+      </c>
+      <c r="D276" t="b">
+        <v>0</v>
+      </c>
+      <c r="E276" t="n">
+        <v>11</v>
+      </c>
+      <c r="F276" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="277">
+      <c r="A277" t="inlineStr">
+        <is>
+          <t>2026-08-08T08:24:00</t>
+        </is>
+      </c>
+      <c r="B277" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C277" t="inlineStr">
+        <is>
+          <t>RoCalRequest</t>
+        </is>
+      </c>
+      <c r="D277" t="b">
+        <v>0</v>
+      </c>
+      <c r="E277" t="n">
+        <v>11</v>
+      </c>
+      <c r="F277" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="278">
+      <c r="A278" t="inlineStr">
+        <is>
+          <t>2026-08-08T08:24:00</t>
+        </is>
+      </c>
+      <c r="B278" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C278" t="inlineStr">
+        <is>
+          <t>tkCycle_TotalSeconds</t>
+        </is>
+      </c>
+      <c r="D278" t="n">
+        <v>0</v>
+      </c>
+      <c r="E278" t="n">
+        <v>9</v>
+      </c>
+      <c r="F278" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="279">
+      <c r="A279" t="inlineStr">
+        <is>
+          <t>2026-08-08T08:24:00</t>
+        </is>
+      </c>
+      <c r="B279" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C279" t="inlineStr">
+        <is>
+          <t>tkCycle_NoMoveSec</t>
+        </is>
+      </c>
+      <c r="D279" t="n">
+        <v>0</v>
+      </c>
+      <c r="E279" t="n">
+        <v>9</v>
+      </c>
+      <c r="F279" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="280">
+      <c r="A280" t="inlineStr">
+        <is>
+          <t>2026-08-08T08:24:00</t>
+        </is>
+      </c>
+      <c r="B280" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C280" t="inlineStr">
+        <is>
+          <t>tkCycle_MoveSeconds</t>
+        </is>
+      </c>
+      <c r="D280" t="n">
+        <v>0</v>
+      </c>
+      <c r="E280" t="n">
+        <v>9</v>
+      </c>
+      <c r="F280" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="281">
+      <c r="A281" t="inlineStr">
+        <is>
+          <t>2026-08-08T08:24:00</t>
+        </is>
+      </c>
+      <c r="B281" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C281" t="inlineStr">
+        <is>
+          <t>Percent time moveing</t>
+        </is>
+      </c>
+      <c r="D281" t="n">
+        <v>0</v>
+      </c>
+      <c r="E281" t="n">
+        <v>9</v>
+      </c>
+      <c r="F281" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="282">
+      <c r="A282" t="inlineStr">
+        <is>
+          <t>2026-08-08T08:24:00</t>
+        </is>
+      </c>
+      <c r="B282" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C282" t="inlineStr">
+        <is>
+          <t>Percent time not moving</t>
+        </is>
+      </c>
+      <c r="D282" t="n">
+        <v>0</v>
+      </c>
+      <c r="E282" t="n">
+        <v>9</v>
+      </c>
+      <c r="F282" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="283">
+      <c r="A283" t="inlineStr">
+        <is>
+          <t>2026-08-08T08:24:00</t>
+        </is>
+      </c>
+      <c r="B283" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C283" t="inlineStr">
+        <is>
+          <t>TotalPickPartsCount</t>
+        </is>
+      </c>
+      <c r="D283" t="n">
+        <v>0</v>
+      </c>
+      <c r="E283" t="n">
+        <v>9</v>
+      </c>
+      <c r="F283" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="284">
+      <c r="A284" t="inlineStr">
+        <is>
+          <t>2026-08-08T08:24:00</t>
+        </is>
+      </c>
+      <c r="B284" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C284" t="inlineStr">
+        <is>
+          <t>RejectPartsCount</t>
+        </is>
+      </c>
+      <c r="D284" t="n">
+        <v>0</v>
+      </c>
+      <c r="E284" t="n">
+        <v>9</v>
+      </c>
+      <c r="F284" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="285">
+      <c r="A285" t="inlineStr">
+        <is>
+          <t>2026-08-08T08:24:00</t>
+        </is>
+      </c>
+      <c r="B285" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C285" t="inlineStr">
+        <is>
+          <t>AcceptsPartsCount</t>
+        </is>
+      </c>
+      <c r="D285" t="n">
+        <v>0</v>
+      </c>
+      <c r="E285" t="n">
+        <v>9</v>
+      </c>
+      <c r="F285" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="286">
+      <c r="A286" t="inlineStr">
+        <is>
+          <t>2026-08-08T08:24:00</t>
+        </is>
+      </c>
+      <c r="B286" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C286" t="inlineStr">
+        <is>
+          <t>percentCount_accept</t>
+        </is>
+      </c>
+      <c r="D286" t="n">
+        <v>0</v>
+      </c>
+      <c r="E286" t="n">
+        <v>9</v>
+      </c>
+      <c r="F286" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="287">
+      <c r="A287" t="inlineStr">
+        <is>
+          <t>2026-08-08T08:24:00</t>
+        </is>
+      </c>
+      <c r="B287" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C287" t="inlineStr">
+        <is>
+          <t>percentCount_reject</t>
+        </is>
+      </c>
+      <c r="D287" t="n">
+        <v>0</v>
+      </c>
+      <c r="E287" t="n">
+        <v>9</v>
+      </c>
+      <c r="F287" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="288">
+      <c r="A288" t="inlineStr">
+        <is>
+          <t>2026-08-08T08:24:00</t>
+        </is>
+      </c>
+      <c r="B288" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C288" t="inlineStr">
+        <is>
+          <t>Avg Parts per min_total</t>
+        </is>
+      </c>
+      <c r="D288" t="n">
+        <v>0</v>
+      </c>
+      <c r="E288" t="n">
+        <v>9</v>
+      </c>
+      <c r="F288" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="289">
+      <c r="A289" t="inlineStr">
+        <is>
+          <t>2026-08-08T08:24:00</t>
+        </is>
+      </c>
+      <c r="B289" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C289" t="inlineStr">
+        <is>
+          <t>TotalPickedParts</t>
+        </is>
+      </c>
+      <c r="D289" t="n">
+        <v>0</v>
+      </c>
+      <c r="E289" t="n">
+        <v>3</v>
+      </c>
+      <c r="F289" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="290">
+      <c r="A290" t="inlineStr">
+        <is>
+          <t>2026-08-08T08:24:00</t>
+        </is>
+      </c>
+      <c r="B290" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C290" t="inlineStr">
+        <is>
+          <t>TotalPickedAcceptParts</t>
+        </is>
+      </c>
+      <c r="D290" t="n">
+        <v>0</v>
+      </c>
+      <c r="E290" t="n">
+        <v>3</v>
+      </c>
+      <c r="F290" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="291">
+      <c r="A291" t="inlineStr">
+        <is>
+          <t>2026-08-08T08:24:00</t>
+        </is>
+      </c>
+      <c r="B291" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C291" t="inlineStr">
+        <is>
+          <t>TotalPickedRejectParts</t>
+        </is>
+      </c>
+      <c r="D291" t="n">
+        <v>0</v>
+      </c>
+      <c r="E291" t="n">
+        <v>3</v>
+      </c>
+      <c r="F291" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="292">
+      <c r="A292" t="inlineStr">
+        <is>
+          <t>2026-08-08T08:24:00</t>
+        </is>
+      </c>
+      <c r="B292" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C292" t="inlineStr">
+        <is>
+          <t>TotalTiePlatesLaid</t>
+        </is>
+      </c>
+      <c r="D292" t="n">
+        <v>0</v>
+      </c>
+      <c r="E292" t="n">
+        <v>3</v>
+      </c>
+      <c r="F292" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="293">
+      <c r="A293" t="inlineStr">
+        <is>
+          <t>2026-08-08T08:24:00</t>
+        </is>
+      </c>
+      <c r="B293" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C293" t="inlineStr">
+        <is>
+          <t>Daily_TotalLaidPlates</t>
+        </is>
+      </c>
+      <c r="D293" t="n">
+        <v>0</v>
+      </c>
+      <c r="E293" t="n">
+        <v>3</v>
+      </c>
+      <c r="F293" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="294">
+      <c r="A294" t="inlineStr">
+        <is>
+          <t>2026-08-08T08:24:00</t>
+        </is>
+      </c>
+      <c r="B294" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C294" t="inlineStr">
+        <is>
+          <t>CountPicked14in</t>
+        </is>
+      </c>
+      <c r="D294" t="n">
+        <v>0</v>
+      </c>
+      <c r="E294" t="n">
+        <v>3</v>
+      </c>
+      <c r="F294" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="295">
+      <c r="A295" t="inlineStr">
+        <is>
+          <t>2026-08-08T08:24:00</t>
+        </is>
+      </c>
+      <c r="B295" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C295" t="inlineStr">
+        <is>
+          <t>CountPicked18in</t>
+        </is>
+      </c>
+      <c r="D295" t="n">
+        <v>0</v>
+      </c>
+      <c r="E295" t="n">
+        <v>3</v>
+      </c>
+      <c r="F295" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="296">
+      <c r="A296" t="inlineStr">
+        <is>
+          <t>2026-08-08T08:24:00</t>
+        </is>
+      </c>
+      <c r="B296" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C296" t="inlineStr">
+        <is>
+          <t>CountPickedPandral</t>
+        </is>
+      </c>
+      <c r="D296" t="n">
+        <v>0</v>
+      </c>
+      <c r="E296" t="n">
+        <v>3</v>
+      </c>
+      <c r="F296" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="297">
+      <c r="A297" t="inlineStr">
+        <is>
+          <t>2026-08-08T08:24:00</t>
+        </is>
+      </c>
+      <c r="B297" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C297" t="inlineStr">
+        <is>
+          <t>CountPickedOTM</t>
+        </is>
+      </c>
+      <c r="D297" t="n">
+        <v>0</v>
+      </c>
+      <c r="E297" t="n">
+        <v>3</v>
+      </c>
+      <c r="F297" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="298">
+      <c r="A298" t="inlineStr">
+        <is>
+          <t>2026-08-08T08:24:00</t>
+        </is>
+      </c>
+      <c r="B298" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C298" t="inlineStr">
+        <is>
+          <t>RoCals</t>
+        </is>
+      </c>
+      <c r="D298" t="n">
+        <v>0</v>
+      </c>
+      <c r="E298" t="n">
+        <v>3</v>
+      </c>
+      <c r="F298" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="299">
+      <c r="A299" t="inlineStr">
+        <is>
+          <t>2026-08-08T08:24:00</t>
+        </is>
+      </c>
+      <c r="B299" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C299" t="inlineStr">
+        <is>
+          <t>TPS_JamsUsr</t>
+        </is>
+      </c>
+      <c r="D299" t="n">
+        <v>0</v>
+      </c>
+      <c r="E299" t="n">
+        <v>3</v>
+      </c>
+      <c r="F299" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="300">
+      <c r="A300" t="inlineStr">
+        <is>
+          <t>2026-08-08T08:24:00</t>
+        </is>
+      </c>
+      <c r="B300" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C300" t="inlineStr">
+        <is>
+          <t>TPS_JamsMASTER</t>
+        </is>
+      </c>
+      <c r="D300" t="n">
+        <v>0</v>
+      </c>
+      <c r="E300" t="n">
+        <v>3</v>
+      </c>
+      <c r="F300" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="301">
+      <c r="A301" t="inlineStr">
+        <is>
+          <t>2026-08-08T08:24:00</t>
+        </is>
+      </c>
+      <c r="B301" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C301" t="inlineStr">
+        <is>
+          <t>ABORT_Master</t>
+        </is>
+      </c>
+      <c r="D301" t="n">
+        <v>0</v>
+      </c>
+      <c r="E301" t="n">
+        <v>3</v>
+      </c>
+      <c r="F301" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/plc</t>
         </is>

</xml_diff>

<commit_message>
Log MQTT data 2026-08-08 10:06 UTC
</commit_message>
<xml_diff>
--- a/logs/raiv_tracker_2026-08-08.xlsx
+++ b/logs/raiv_tracker_2026-08-08.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F301"/>
+  <dimension ref="A1:F386"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6409,7 +6409,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E217" t="inlineStr"/>
       <c r="F217" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g2</t>
@@ -6437,7 +6436,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E218" t="inlineStr"/>
       <c r="F218" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g3</t>
@@ -6465,7 +6463,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E219" t="inlineStr"/>
       <c r="F219" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g4</t>
@@ -6493,7 +6490,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E220" t="inlineStr"/>
       <c r="F220" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g5</t>
@@ -6521,7 +6517,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E221" t="inlineStr"/>
       <c r="F221" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g6</t>
@@ -6549,7 +6544,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E222" t="inlineStr"/>
       <c r="F222" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g7</t>
@@ -6577,7 +6571,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E223" t="inlineStr"/>
       <c r="F223" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g13</t>
@@ -6605,7 +6598,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E224" t="inlineStr"/>
       <c r="F224" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g15</t>
@@ -6633,7 +6625,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E225" t="inlineStr"/>
       <c r="F225" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g17</t>
@@ -6661,7 +6652,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E226" t="inlineStr"/>
       <c r="F226" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g18</t>
@@ -6689,7 +6679,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E227" t="inlineStr"/>
       <c r="F227" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g19</t>
@@ -6717,7 +6706,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E228" t="inlineStr"/>
       <c r="F228" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g22</t>
@@ -6745,7 +6733,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E229" t="inlineStr"/>
       <c r="F229" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g23</t>
@@ -6773,7 +6760,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E230" t="inlineStr"/>
       <c r="F230" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g24</t>
@@ -6801,7 +6787,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E231" t="inlineStr"/>
       <c r="F231" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g25</t>
@@ -6829,7 +6814,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E232" t="inlineStr"/>
       <c r="F232" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g1</t>
@@ -6857,7 +6841,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E233" t="inlineStr"/>
       <c r="F233" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g8</t>
@@ -6885,7 +6868,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E234" t="inlineStr"/>
       <c r="F234" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g9</t>
@@ -6913,7 +6895,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E235" t="inlineStr"/>
       <c r="F235" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g10</t>
@@ -6941,7 +6922,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E236" t="inlineStr"/>
       <c r="F236" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g11</t>
@@ -6969,7 +6949,6 @@
           <t>1</t>
         </is>
       </c>
-      <c r="E237" t="inlineStr"/>
       <c r="F237" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g12</t>
@@ -6997,7 +6976,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E238" t="inlineStr"/>
       <c r="F238" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g14</t>
@@ -7025,7 +7003,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E239" t="inlineStr"/>
       <c r="F239" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g33</t>
@@ -7053,7 +7030,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E240" t="inlineStr"/>
       <c r="F240" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g16</t>
@@ -7081,7 +7057,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E241" t="inlineStr"/>
       <c r="F241" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g34</t>
@@ -7109,7 +7084,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E242" t="inlineStr"/>
       <c r="F242" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g36</t>
@@ -7137,7 +7111,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E243" t="inlineStr"/>
       <c r="F243" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g40</t>
@@ -7165,7 +7138,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E244" t="inlineStr"/>
       <c r="F244" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g20</t>
@@ -7193,7 +7165,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E245" t="inlineStr"/>
       <c r="F245" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g21</t>
@@ -7221,7 +7192,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E246" t="inlineStr"/>
       <c r="F246" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g26</t>
@@ -7249,7 +7219,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E247" t="inlineStr"/>
       <c r="F247" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g27</t>
@@ -7277,7 +7246,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E248" t="inlineStr"/>
       <c r="F248" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g28</t>
@@ -7305,7 +7273,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E249" t="inlineStr"/>
       <c r="F249" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g29</t>
@@ -7333,7 +7300,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E250" t="inlineStr"/>
       <c r="F250" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g30</t>
@@ -7361,7 +7327,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E251" t="inlineStr"/>
       <c r="F251" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g31</t>
@@ -7389,7 +7354,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E252" t="inlineStr"/>
       <c r="F252" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g32</t>
@@ -7417,7 +7381,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E253" t="inlineStr"/>
       <c r="F253" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g35</t>
@@ -7445,7 +7408,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E254" t="inlineStr"/>
       <c r="F254" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g37</t>
@@ -7473,7 +7435,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E255" t="inlineStr"/>
       <c r="F255" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g38</t>
@@ -7501,7 +7462,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E256" t="inlineStr"/>
       <c r="F256" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g39</t>
@@ -8765,6 +8725,2386 @@
       <c r="F301" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="302">
+      <c r="A302" t="inlineStr">
+        <is>
+          <t>2026-08-08T10:06:00</t>
+        </is>
+      </c>
+      <c r="B302" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C302" t="inlineStr">
+        <is>
+          <t>_1st_SCAN</t>
+        </is>
+      </c>
+      <c r="D302" t="b">
+        <v>0</v>
+      </c>
+      <c r="E302" t="n">
+        <v>11</v>
+      </c>
+      <c r="F302" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="303">
+      <c r="A303" t="inlineStr">
+        <is>
+          <t>2026-08-08T10:06:00</t>
+        </is>
+      </c>
+      <c r="B303" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C303" t="inlineStr">
+        <is>
+          <t>TieDetectOffset_B</t>
+        </is>
+      </c>
+      <c r="D303" t="b">
+        <v>0</v>
+      </c>
+      <c r="E303" t="n">
+        <v>11</v>
+      </c>
+      <c r="F303" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="304">
+      <c r="A304" t="inlineStr">
+        <is>
+          <t>2026-08-08T10:06:00</t>
+        </is>
+      </c>
+      <c r="B304" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C304" t="inlineStr">
+        <is>
+          <t>Tie Detector</t>
+        </is>
+      </c>
+      <c r="D304" t="b">
+        <v>0</v>
+      </c>
+      <c r="E304" t="n">
+        <v>11</v>
+      </c>
+      <c r="F304" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="305">
+      <c r="A305" t="inlineStr">
+        <is>
+          <t>2026-08-08T10:06:00</t>
+        </is>
+      </c>
+      <c r="B305" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C305" t="inlineStr">
+        <is>
+          <t>TPS Full</t>
+        </is>
+      </c>
+      <c r="D305" t="b">
+        <v>0</v>
+      </c>
+      <c r="E305" t="n">
+        <v>11</v>
+      </c>
+      <c r="F305" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="306">
+      <c r="A306" t="inlineStr">
+        <is>
+          <t>2026-08-08T10:06:00</t>
+        </is>
+      </c>
+      <c r="B306" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C306" t="inlineStr">
+        <is>
+          <t>TieDetectOffset_A</t>
+        </is>
+      </c>
+      <c r="D306" t="b">
+        <v>0</v>
+      </c>
+      <c r="E306" t="n">
+        <v>11</v>
+      </c>
+      <c r="F306" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="307">
+      <c r="A307" t="inlineStr">
+        <is>
+          <t>2026-08-08T10:06:00</t>
+        </is>
+      </c>
+      <c r="B307" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C307" t="inlineStr">
+        <is>
+          <t>TPS Connected</t>
+        </is>
+      </c>
+      <c r="D307" t="b">
+        <v>0</v>
+      </c>
+      <c r="E307" t="n">
+        <v>11</v>
+      </c>
+      <c r="F307" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="308">
+      <c r="A308" t="inlineStr">
+        <is>
+          <t>2026-08-08T10:06:00</t>
+        </is>
+      </c>
+      <c r="B308" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C308" t="inlineStr">
+        <is>
+          <t>TPS_Enable_ Button</t>
+        </is>
+      </c>
+      <c r="D308" t="b">
+        <v>0</v>
+      </c>
+      <c r="E308" t="n">
+        <v>11</v>
+      </c>
+      <c r="F308" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="309">
+      <c r="A309" t="inlineStr">
+        <is>
+          <t>2026-08-08T10:06:00</t>
+        </is>
+      </c>
+      <c r="B309" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C309" t="inlineStr">
+        <is>
+          <t>AirEagle Eject Plate</t>
+        </is>
+      </c>
+      <c r="D309" t="b">
+        <v>0</v>
+      </c>
+      <c r="E309" t="n">
+        <v>11</v>
+      </c>
+      <c r="F309" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="310">
+      <c r="A310" t="inlineStr">
+        <is>
+          <t>2026-08-08T10:06:00</t>
+        </is>
+      </c>
+      <c r="B310" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C310" t="inlineStr">
+        <is>
+          <t>tk_Cycle</t>
+        </is>
+      </c>
+      <c r="D310" t="b">
+        <v>0</v>
+      </c>
+      <c r="E310" t="n">
+        <v>11</v>
+      </c>
+      <c r="F310" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="311">
+      <c r="A311" t="inlineStr">
+        <is>
+          <t>2026-08-08T10:06:00</t>
+        </is>
+      </c>
+      <c r="B311" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C311" t="inlineStr">
+        <is>
+          <t>Servos_Enabled</t>
+        </is>
+      </c>
+      <c r="D311" t="b">
+        <v>0</v>
+      </c>
+      <c r="E311" t="n">
+        <v>11</v>
+      </c>
+      <c r="F311" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="312">
+      <c r="A312" t="inlineStr">
+        <is>
+          <t>2026-08-08T10:06:00</t>
+        </is>
+      </c>
+      <c r="B312" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C312" t="inlineStr">
+        <is>
+          <t>TPS Enabled</t>
+        </is>
+      </c>
+      <c r="D312" t="b">
+        <v>0</v>
+      </c>
+      <c r="E312" t="n">
+        <v>11</v>
+      </c>
+      <c r="F312" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="313">
+      <c r="A313" t="inlineStr">
+        <is>
+          <t>2026-08-08T10:06:00</t>
+        </is>
+      </c>
+      <c r="B313" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C313" t="inlineStr">
+        <is>
+          <t>tk_Abort</t>
+        </is>
+      </c>
+      <c r="D313" t="b">
+        <v>0</v>
+      </c>
+      <c r="E313" t="n">
+        <v>11</v>
+      </c>
+      <c r="F313" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="314">
+      <c r="A314" t="inlineStr">
+        <is>
+          <t>2026-08-08T10:06:00</t>
+        </is>
+      </c>
+      <c r="B314" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C314" t="inlineStr">
+        <is>
+          <t>Robot_isMoving</t>
+        </is>
+      </c>
+      <c r="D314" t="b">
+        <v>0</v>
+      </c>
+      <c r="E314" t="n">
+        <v>11</v>
+      </c>
+      <c r="F314" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="315">
+      <c r="A315" t="inlineStr">
+        <is>
+          <t>2026-08-08T10:06:00</t>
+        </is>
+      </c>
+      <c r="B315" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C315" t="inlineStr">
+        <is>
+          <t>Eject Tie Plate</t>
+        </is>
+      </c>
+      <c r="D315" t="b">
+        <v>0</v>
+      </c>
+      <c r="E315" t="n">
+        <v>11</v>
+      </c>
+      <c r="F315" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="316">
+      <c r="A316" t="inlineStr">
+        <is>
+          <t>2026-08-08T10:06:00</t>
+        </is>
+      </c>
+      <c r="B316" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C316" t="inlineStr">
+        <is>
+          <t>TPS BACKUP ALARM</t>
+        </is>
+      </c>
+      <c r="D316" t="b">
+        <v>0</v>
+      </c>
+      <c r="E316" t="n">
+        <v>11</v>
+      </c>
+      <c r="F316" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="317">
+      <c r="A317" t="inlineStr">
+        <is>
+          <t>2026-08-08T10:06:00</t>
+        </is>
+      </c>
+      <c r="B317" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C317" t="inlineStr">
+        <is>
+          <t>14in Job</t>
+        </is>
+      </c>
+      <c r="D317" t="b">
+        <v>1</v>
+      </c>
+      <c r="E317" t="n">
+        <v>11</v>
+      </c>
+      <c r="F317" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="318">
+      <c r="A318" t="inlineStr">
+        <is>
+          <t>2026-08-08T10:06:00</t>
+        </is>
+      </c>
+      <c r="B318" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C318" t="inlineStr">
+        <is>
+          <t>18in Job</t>
+        </is>
+      </c>
+      <c r="D318" t="b">
+        <v>0</v>
+      </c>
+      <c r="E318" t="n">
+        <v>11</v>
+      </c>
+      <c r="F318" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="319">
+      <c r="A319" t="inlineStr">
+        <is>
+          <t>2026-08-08T10:06:00</t>
+        </is>
+      </c>
+      <c r="B319" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C319" t="inlineStr">
+        <is>
+          <t>Pandral Job</t>
+        </is>
+      </c>
+      <c r="D319" t="b">
+        <v>0</v>
+      </c>
+      <c r="E319" t="n">
+        <v>11</v>
+      </c>
+      <c r="F319" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="320">
+      <c r="A320" t="inlineStr">
+        <is>
+          <t>2026-08-08T10:06:00</t>
+        </is>
+      </c>
+      <c r="B320" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C320" t="inlineStr">
+        <is>
+          <t>DoubleLay Job</t>
+        </is>
+      </c>
+      <c r="D320" t="b">
+        <v>0</v>
+      </c>
+      <c r="E320" t="n">
+        <v>11</v>
+      </c>
+      <c r="F320" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="321">
+      <c r="A321" t="inlineStr">
+        <is>
+          <t>2026-08-08T10:06:00</t>
+        </is>
+      </c>
+      <c r="B321" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C321" t="inlineStr">
+        <is>
+          <t>TPSjam_FLAG</t>
+        </is>
+      </c>
+      <c r="D321" t="b">
+        <v>0</v>
+      </c>
+      <c r="E321" t="n">
+        <v>11</v>
+      </c>
+      <c r="F321" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="322">
+      <c r="A322" t="inlineStr">
+        <is>
+          <t>2026-08-08T10:06:00</t>
+        </is>
+      </c>
+      <c r="B322" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C322" t="inlineStr">
+        <is>
+          <t>RoCalRequest</t>
+        </is>
+      </c>
+      <c r="D322" t="b">
+        <v>0</v>
+      </c>
+      <c r="E322" t="n">
+        <v>11</v>
+      </c>
+      <c r="F322" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="323">
+      <c r="A323" t="inlineStr">
+        <is>
+          <t>2026-08-08T10:06:00</t>
+        </is>
+      </c>
+      <c r="B323" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C323" t="inlineStr">
+        <is>
+          <t>tkCycle_TotalSeconds</t>
+        </is>
+      </c>
+      <c r="D323" t="n">
+        <v>0</v>
+      </c>
+      <c r="E323" t="n">
+        <v>9</v>
+      </c>
+      <c r="F323" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="324">
+      <c r="A324" t="inlineStr">
+        <is>
+          <t>2026-08-08T10:06:00</t>
+        </is>
+      </c>
+      <c r="B324" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C324" t="inlineStr">
+        <is>
+          <t>tkCycle_NoMoveSec</t>
+        </is>
+      </c>
+      <c r="D324" t="n">
+        <v>0</v>
+      </c>
+      <c r="E324" t="n">
+        <v>9</v>
+      </c>
+      <c r="F324" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="325">
+      <c r="A325" t="inlineStr">
+        <is>
+          <t>2026-08-08T10:06:00</t>
+        </is>
+      </c>
+      <c r="B325" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C325" t="inlineStr">
+        <is>
+          <t>tkCycle_MoveSeconds</t>
+        </is>
+      </c>
+      <c r="D325" t="n">
+        <v>0</v>
+      </c>
+      <c r="E325" t="n">
+        <v>9</v>
+      </c>
+      <c r="F325" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="326">
+      <c r="A326" t="inlineStr">
+        <is>
+          <t>2026-08-08T10:06:00</t>
+        </is>
+      </c>
+      <c r="B326" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C326" t="inlineStr">
+        <is>
+          <t>Percent time moveing</t>
+        </is>
+      </c>
+      <c r="D326" t="n">
+        <v>0</v>
+      </c>
+      <c r="E326" t="n">
+        <v>9</v>
+      </c>
+      <c r="F326" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="327">
+      <c r="A327" t="inlineStr">
+        <is>
+          <t>2026-08-08T10:06:00</t>
+        </is>
+      </c>
+      <c r="B327" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C327" t="inlineStr">
+        <is>
+          <t>Percent time not moving</t>
+        </is>
+      </c>
+      <c r="D327" t="n">
+        <v>0</v>
+      </c>
+      <c r="E327" t="n">
+        <v>9</v>
+      </c>
+      <c r="F327" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="328">
+      <c r="A328" t="inlineStr">
+        <is>
+          <t>2026-08-08T10:06:00</t>
+        </is>
+      </c>
+      <c r="B328" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C328" t="inlineStr">
+        <is>
+          <t>TotalPickPartsCount</t>
+        </is>
+      </c>
+      <c r="D328" t="n">
+        <v>0</v>
+      </c>
+      <c r="E328" t="n">
+        <v>9</v>
+      </c>
+      <c r="F328" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="329">
+      <c r="A329" t="inlineStr">
+        <is>
+          <t>2026-08-08T10:06:00</t>
+        </is>
+      </c>
+      <c r="B329" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C329" t="inlineStr">
+        <is>
+          <t>RejectPartsCount</t>
+        </is>
+      </c>
+      <c r="D329" t="n">
+        <v>0</v>
+      </c>
+      <c r="E329" t="n">
+        <v>9</v>
+      </c>
+      <c r="F329" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="330">
+      <c r="A330" t="inlineStr">
+        <is>
+          <t>2026-08-08T10:06:00</t>
+        </is>
+      </c>
+      <c r="B330" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C330" t="inlineStr">
+        <is>
+          <t>AcceptsPartsCount</t>
+        </is>
+      </c>
+      <c r="D330" t="n">
+        <v>0</v>
+      </c>
+      <c r="E330" t="n">
+        <v>9</v>
+      </c>
+      <c r="F330" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="331">
+      <c r="A331" t="inlineStr">
+        <is>
+          <t>2026-08-08T10:06:00</t>
+        </is>
+      </c>
+      <c r="B331" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C331" t="inlineStr">
+        <is>
+          <t>percentCount_accept</t>
+        </is>
+      </c>
+      <c r="D331" t="n">
+        <v>0</v>
+      </c>
+      <c r="E331" t="n">
+        <v>9</v>
+      </c>
+      <c r="F331" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="332">
+      <c r="A332" t="inlineStr">
+        <is>
+          <t>2026-08-08T10:06:00</t>
+        </is>
+      </c>
+      <c r="B332" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C332" t="inlineStr">
+        <is>
+          <t>percentCount_reject</t>
+        </is>
+      </c>
+      <c r="D332" t="n">
+        <v>0</v>
+      </c>
+      <c r="E332" t="n">
+        <v>9</v>
+      </c>
+      <c r="F332" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="333">
+      <c r="A333" t="inlineStr">
+        <is>
+          <t>2026-08-08T10:06:00</t>
+        </is>
+      </c>
+      <c r="B333" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C333" t="inlineStr">
+        <is>
+          <t>Avg Parts per min_total</t>
+        </is>
+      </c>
+      <c r="D333" t="n">
+        <v>0</v>
+      </c>
+      <c r="E333" t="n">
+        <v>9</v>
+      </c>
+      <c r="F333" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="334">
+      <c r="A334" t="inlineStr">
+        <is>
+          <t>2026-08-08T10:06:00</t>
+        </is>
+      </c>
+      <c r="B334" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C334" t="inlineStr">
+        <is>
+          <t>TotalPickedParts</t>
+        </is>
+      </c>
+      <c r="D334" t="n">
+        <v>0</v>
+      </c>
+      <c r="E334" t="n">
+        <v>3</v>
+      </c>
+      <c r="F334" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="335">
+      <c r="A335" t="inlineStr">
+        <is>
+          <t>2026-08-08T10:06:00</t>
+        </is>
+      </c>
+      <c r="B335" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C335" t="inlineStr">
+        <is>
+          <t>TotalPickedAcceptParts</t>
+        </is>
+      </c>
+      <c r="D335" t="n">
+        <v>0</v>
+      </c>
+      <c r="E335" t="n">
+        <v>3</v>
+      </c>
+      <c r="F335" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="336">
+      <c r="A336" t="inlineStr">
+        <is>
+          <t>2026-08-08T10:06:00</t>
+        </is>
+      </c>
+      <c r="B336" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C336" t="inlineStr">
+        <is>
+          <t>TotalPickedRejectParts</t>
+        </is>
+      </c>
+      <c r="D336" t="n">
+        <v>0</v>
+      </c>
+      <c r="E336" t="n">
+        <v>3</v>
+      </c>
+      <c r="F336" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="337">
+      <c r="A337" t="inlineStr">
+        <is>
+          <t>2026-08-08T10:06:00</t>
+        </is>
+      </c>
+      <c r="B337" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C337" t="inlineStr">
+        <is>
+          <t>TotalTiePlatesLaid</t>
+        </is>
+      </c>
+      <c r="D337" t="n">
+        <v>0</v>
+      </c>
+      <c r="E337" t="n">
+        <v>3</v>
+      </c>
+      <c r="F337" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="338">
+      <c r="A338" t="inlineStr">
+        <is>
+          <t>2026-08-08T10:06:00</t>
+        </is>
+      </c>
+      <c r="B338" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C338" t="inlineStr">
+        <is>
+          <t>Daily_TotalLaidPlates</t>
+        </is>
+      </c>
+      <c r="D338" t="n">
+        <v>0</v>
+      </c>
+      <c r="E338" t="n">
+        <v>3</v>
+      </c>
+      <c r="F338" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="339">
+      <c r="A339" t="inlineStr">
+        <is>
+          <t>2026-08-08T10:06:00</t>
+        </is>
+      </c>
+      <c r="B339" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C339" t="inlineStr">
+        <is>
+          <t>CountPicked14in</t>
+        </is>
+      </c>
+      <c r="D339" t="n">
+        <v>0</v>
+      </c>
+      <c r="E339" t="n">
+        <v>3</v>
+      </c>
+      <c r="F339" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="340">
+      <c r="A340" t="inlineStr">
+        <is>
+          <t>2026-08-08T10:06:00</t>
+        </is>
+      </c>
+      <c r="B340" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C340" t="inlineStr">
+        <is>
+          <t>CountPicked18in</t>
+        </is>
+      </c>
+      <c r="D340" t="n">
+        <v>0</v>
+      </c>
+      <c r="E340" t="n">
+        <v>3</v>
+      </c>
+      <c r="F340" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="341">
+      <c r="A341" t="inlineStr">
+        <is>
+          <t>2026-08-08T10:06:00</t>
+        </is>
+      </c>
+      <c r="B341" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C341" t="inlineStr">
+        <is>
+          <t>CountPickedPandral</t>
+        </is>
+      </c>
+      <c r="D341" t="n">
+        <v>0</v>
+      </c>
+      <c r="E341" t="n">
+        <v>3</v>
+      </c>
+      <c r="F341" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="342">
+      <c r="A342" t="inlineStr">
+        <is>
+          <t>2026-08-08T10:06:00</t>
+        </is>
+      </c>
+      <c r="B342" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C342" t="inlineStr">
+        <is>
+          <t>CountPickedOTM</t>
+        </is>
+      </c>
+      <c r="D342" t="n">
+        <v>0</v>
+      </c>
+      <c r="E342" t="n">
+        <v>3</v>
+      </c>
+      <c r="F342" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="343">
+      <c r="A343" t="inlineStr">
+        <is>
+          <t>2026-08-08T10:06:00</t>
+        </is>
+      </c>
+      <c r="B343" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C343" t="inlineStr">
+        <is>
+          <t>RoCals</t>
+        </is>
+      </c>
+      <c r="D343" t="n">
+        <v>0</v>
+      </c>
+      <c r="E343" t="n">
+        <v>3</v>
+      </c>
+      <c r="F343" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="344">
+      <c r="A344" t="inlineStr">
+        <is>
+          <t>2026-08-08T10:06:00</t>
+        </is>
+      </c>
+      <c r="B344" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C344" t="inlineStr">
+        <is>
+          <t>TPS_JamsUsr</t>
+        </is>
+      </c>
+      <c r="D344" t="n">
+        <v>0</v>
+      </c>
+      <c r="E344" t="n">
+        <v>3</v>
+      </c>
+      <c r="F344" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="345">
+      <c r="A345" t="inlineStr">
+        <is>
+          <t>2026-08-08T10:06:00</t>
+        </is>
+      </c>
+      <c r="B345" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C345" t="inlineStr">
+        <is>
+          <t>TPS_JamsMASTER</t>
+        </is>
+      </c>
+      <c r="D345" t="n">
+        <v>0</v>
+      </c>
+      <c r="E345" t="n">
+        <v>3</v>
+      </c>
+      <c r="F345" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="346">
+      <c r="A346" t="inlineStr">
+        <is>
+          <t>2026-08-08T10:06:00</t>
+        </is>
+      </c>
+      <c r="B346" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C346" t="inlineStr">
+        <is>
+          <t>ABORT_Master</t>
+        </is>
+      </c>
+      <c r="D346" t="n">
+        <v>0</v>
+      </c>
+      <c r="E346" t="n">
+        <v>3</v>
+      </c>
+      <c r="F346" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="347">
+      <c r="A347" t="inlineStr">
+        <is>
+          <t>2026-08-08T10:06:13</t>
+        </is>
+      </c>
+      <c r="B347" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C347" t="inlineStr">
+        <is>
+          <t>TotalTiePlatesLaid</t>
+        </is>
+      </c>
+      <c r="D347" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E347" t="inlineStr"/>
+      <c r="F347" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g1</t>
+        </is>
+      </c>
+    </row>
+    <row r="348">
+      <c r="A348" t="inlineStr">
+        <is>
+          <t>2026-08-08T10:06:13</t>
+        </is>
+      </c>
+      <c r="B348" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C348" t="inlineStr">
+        <is>
+          <t>CountLaidButton</t>
+        </is>
+      </c>
+      <c r="D348" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E348" t="inlineStr"/>
+      <c r="F348" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g2</t>
+        </is>
+      </c>
+    </row>
+    <row r="349">
+      <c r="A349" t="inlineStr">
+        <is>
+          <t>2026-08-08T10:06:13</t>
+        </is>
+      </c>
+      <c r="B349" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C349" t="inlineStr">
+        <is>
+          <t>CountLaidDetector</t>
+        </is>
+      </c>
+      <c r="D349" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E349" t="inlineStr"/>
+      <c r="F349" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g3</t>
+        </is>
+      </c>
+    </row>
+    <row r="350">
+      <c r="A350" t="inlineStr">
+        <is>
+          <t>2026-08-08T10:06:13</t>
+        </is>
+      </c>
+      <c r="B350" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C350" t="inlineStr">
+        <is>
+          <t>CountLaidEncoder</t>
+        </is>
+      </c>
+      <c r="D350" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E350" t="inlineStr"/>
+      <c r="F350" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g4</t>
+        </is>
+      </c>
+    </row>
+    <row r="351">
+      <c r="A351" t="inlineStr">
+        <is>
+          <t>2026-08-08T10:06:13</t>
+        </is>
+      </c>
+      <c r="B351" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C351" t="inlineStr">
+        <is>
+          <t>CountLaid14in</t>
+        </is>
+      </c>
+      <c r="D351" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E351" t="inlineStr"/>
+      <c r="F351" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g5</t>
+        </is>
+      </c>
+    </row>
+    <row r="352">
+      <c r="A352" t="inlineStr">
+        <is>
+          <t>2026-08-08T10:06:13</t>
+        </is>
+      </c>
+      <c r="B352" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C352" t="inlineStr">
+        <is>
+          <t>CountLaid18in</t>
+        </is>
+      </c>
+      <c r="D352" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E352" t="inlineStr"/>
+      <c r="F352" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g6</t>
+        </is>
+      </c>
+    </row>
+    <row r="353">
+      <c r="A353" t="inlineStr">
+        <is>
+          <t>2026-08-08T10:06:13</t>
+        </is>
+      </c>
+      <c r="B353" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C353" t="inlineStr">
+        <is>
+          <t>CountLaidPandral</t>
+        </is>
+      </c>
+      <c r="D353" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E353" t="inlineStr"/>
+      <c r="F353" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g7</t>
+        </is>
+      </c>
+    </row>
+    <row r="354">
+      <c r="A354" t="inlineStr">
+        <is>
+          <t>2026-08-08T10:06:13</t>
+        </is>
+      </c>
+      <c r="B354" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C354" t="inlineStr">
+        <is>
+          <t>usr_TPStime Hours10th</t>
+        </is>
+      </c>
+      <c r="D354" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E354" t="inlineStr"/>
+      <c r="F354" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g8</t>
+        </is>
+      </c>
+    </row>
+    <row r="355">
+      <c r="A355" t="inlineStr">
+        <is>
+          <t>2026-08-08T10:06:13</t>
+        </is>
+      </c>
+      <c r="B355" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C355" t="inlineStr">
+        <is>
+          <t>usrTPS_miles xxx</t>
+        </is>
+      </c>
+      <c r="D355" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E355" t="inlineStr"/>
+      <c r="F355" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g9</t>
+        </is>
+      </c>
+    </row>
+    <row r="356">
+      <c r="A356" t="inlineStr">
+        <is>
+          <t>2026-08-08T10:06:13</t>
+        </is>
+      </c>
+      <c r="B356" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C356" t="inlineStr">
+        <is>
+          <t>18in Job</t>
+        </is>
+      </c>
+      <c r="D356" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E356" t="inlineStr"/>
+      <c r="F356" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g13</t>
+        </is>
+      </c>
+    </row>
+    <row r="357">
+      <c r="A357" t="inlineStr">
+        <is>
+          <t>2026-08-08T10:06:13</t>
+        </is>
+      </c>
+      <c r="B357" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C357" t="inlineStr">
+        <is>
+          <t>CountAcceptedTotal</t>
+        </is>
+      </c>
+      <c r="D357" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E357" t="inlineStr"/>
+      <c r="F357" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g15</t>
+        </is>
+      </c>
+    </row>
+    <row r="358">
+      <c r="A358" t="inlineStr">
+        <is>
+          <t>2026-08-08T10:06:13</t>
+        </is>
+      </c>
+      <c r="B358" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C358" t="inlineStr">
+        <is>
+          <t>Servos_Enabled</t>
+        </is>
+      </c>
+      <c r="D358" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E358" t="inlineStr"/>
+      <c r="F358" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g17</t>
+        </is>
+      </c>
+    </row>
+    <row r="359">
+      <c r="A359" t="inlineStr">
+        <is>
+          <t>2026-08-08T10:06:13</t>
+        </is>
+      </c>
+      <c r="B359" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C359" t="inlineStr">
+        <is>
+          <t>TotalPickPartsCount</t>
+        </is>
+      </c>
+      <c r="D359" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E359" t="inlineStr"/>
+      <c r="F359" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g18</t>
+        </is>
+      </c>
+    </row>
+    <row r="360">
+      <c r="A360" t="inlineStr">
+        <is>
+          <t>2026-08-08T10:06:13</t>
+        </is>
+      </c>
+      <c r="B360" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C360" t="inlineStr">
+        <is>
+          <t>AcceptsPartsCount</t>
+        </is>
+      </c>
+      <c r="D360" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E360" t="inlineStr"/>
+      <c r="F360" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g19</t>
+        </is>
+      </c>
+    </row>
+    <row r="361">
+      <c r="A361" t="inlineStr">
+        <is>
+          <t>2026-08-08T10:06:13</t>
+        </is>
+      </c>
+      <c r="B361" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C361" t="inlineStr">
+        <is>
+          <t>day_Servotime Hours10th</t>
+        </is>
+      </c>
+      <c r="D361" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E361" t="inlineStr"/>
+      <c r="F361" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g22</t>
+        </is>
+      </c>
+    </row>
+    <row r="362">
+      <c r="A362" t="inlineStr">
+        <is>
+          <t>2026-08-08T10:06:13</t>
+        </is>
+      </c>
+      <c r="B362" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C362" t="inlineStr">
+        <is>
+          <t>tk_Cycle</t>
+        </is>
+      </c>
+      <c r="D362" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E362" t="inlineStr"/>
+      <c r="F362" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g23</t>
+        </is>
+      </c>
+    </row>
+    <row r="363">
+      <c r="A363" t="inlineStr">
+        <is>
+          <t>2026-08-08T10:06:13</t>
+        </is>
+      </c>
+      <c r="B363" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C363" t="inlineStr">
+        <is>
+          <t>tk_Abort</t>
+        </is>
+      </c>
+      <c r="D363" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E363" t="inlineStr"/>
+      <c r="F363" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g24</t>
+        </is>
+      </c>
+    </row>
+    <row r="364">
+      <c r="A364" t="inlineStr">
+        <is>
+          <t>2026-08-08T10:06:13</t>
+        </is>
+      </c>
+      <c r="B364" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C364" t="inlineStr">
+        <is>
+          <t>tk_ClearPos</t>
+        </is>
+      </c>
+      <c r="D364" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E364" t="inlineStr"/>
+      <c r="F364" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g25</t>
+        </is>
+      </c>
+    </row>
+    <row r="365">
+      <c r="A365" t="inlineStr">
+        <is>
+          <t>2026-08-08T10:06:13</t>
+        </is>
+      </c>
+      <c r="B365" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C365" t="inlineStr">
+        <is>
+          <t>TPS Connected</t>
+        </is>
+      </c>
+      <c r="D365" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E365" t="inlineStr"/>
+      <c r="F365" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g10</t>
+        </is>
+      </c>
+    </row>
+    <row r="366">
+      <c r="A366" t="inlineStr">
+        <is>
+          <t>2026-08-08T10:06:13</t>
+        </is>
+      </c>
+      <c r="B366" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C366" t="inlineStr">
+        <is>
+          <t>TPS Enabled</t>
+        </is>
+      </c>
+      <c r="D366" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E366" t="inlineStr"/>
+      <c r="F366" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g11</t>
+        </is>
+      </c>
+    </row>
+    <row r="367">
+      <c r="A367" t="inlineStr">
+        <is>
+          <t>2026-08-08T10:06:13</t>
+        </is>
+      </c>
+      <c r="B367" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C367" t="inlineStr">
+        <is>
+          <t>14in Job</t>
+        </is>
+      </c>
+      <c r="D367" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E367" t="inlineStr"/>
+      <c r="F367" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g12</t>
+        </is>
+      </c>
+    </row>
+    <row r="368">
+      <c r="A368" t="inlineStr">
+        <is>
+          <t>2026-08-08T10:06:13</t>
+        </is>
+      </c>
+      <c r="B368" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C368" t="inlineStr">
+        <is>
+          <t>Pandral Job</t>
+        </is>
+      </c>
+      <c r="D368" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E368" t="inlineStr"/>
+      <c r="F368" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g14</t>
+        </is>
+      </c>
+    </row>
+    <row r="369">
+      <c r="A369" t="inlineStr">
+        <is>
+          <t>2026-08-08T10:06:13</t>
+        </is>
+      </c>
+      <c r="B369" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C369" t="inlineStr">
+        <is>
+          <t>CountRejectedTotal</t>
+        </is>
+      </c>
+      <c r="D369" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E369" t="inlineStr"/>
+      <c r="F369" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g16</t>
+        </is>
+      </c>
+    </row>
+    <row r="370">
+      <c r="A370" t="inlineStr">
+        <is>
+          <t>2026-08-08T10:06:13</t>
+        </is>
+      </c>
+      <c r="B370" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C370" t="inlineStr">
+        <is>
+          <t>RejectPartsCount</t>
+        </is>
+      </c>
+      <c r="D370" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E370" t="inlineStr"/>
+      <c r="F370" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g20</t>
+        </is>
+      </c>
+    </row>
+    <row r="371">
+      <c r="A371" t="inlineStr">
+        <is>
+          <t>2026-08-08T10:06:13</t>
+        </is>
+      </c>
+      <c r="B371" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C371" t="inlineStr">
+        <is>
+          <t>tk_Cycle hrs</t>
+        </is>
+      </c>
+      <c r="D371" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E371" t="inlineStr"/>
+      <c r="F371" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g21</t>
+        </is>
+      </c>
+    </row>
+    <row r="372">
+      <c r="A372" t="inlineStr">
+        <is>
+          <t>2026-08-08T10:06:13</t>
+        </is>
+      </c>
+      <c r="B372" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C372" t="inlineStr">
+        <is>
+          <t>tk_Warmup</t>
+        </is>
+      </c>
+      <c r="D372" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E372" t="inlineStr"/>
+      <c r="F372" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g26</t>
+        </is>
+      </c>
+    </row>
+    <row r="373">
+      <c r="A373" t="inlineStr">
+        <is>
+          <t>2026-08-08T10:06:13</t>
+        </is>
+      </c>
+      <c r="B373" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C373" t="inlineStr">
+        <is>
+          <t>FindingParts min</t>
+        </is>
+      </c>
+      <c r="D373" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E373" t="inlineStr"/>
+      <c r="F373" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g27</t>
+        </is>
+      </c>
+    </row>
+    <row r="374">
+      <c r="A374" t="inlineStr">
+        <is>
+          <t>2026-08-08T10:06:13</t>
+        </is>
+      </c>
+      <c r="B374" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C374" t="inlineStr">
+        <is>
+          <t>PickingParts min</t>
+        </is>
+      </c>
+      <c r="D374" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E374" t="inlineStr"/>
+      <c r="F374" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g28</t>
+        </is>
+      </c>
+    </row>
+    <row r="375">
+      <c r="A375" t="inlineStr">
+        <is>
+          <t>2026-08-08T10:06:13</t>
+        </is>
+      </c>
+      <c r="B375" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C375" t="inlineStr">
+        <is>
+          <t>PlacingParts min</t>
+        </is>
+      </c>
+      <c r="D375" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E375" t="inlineStr"/>
+      <c r="F375" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g29</t>
+        </is>
+      </c>
+    </row>
+    <row r="376">
+      <c r="A376" t="inlineStr">
+        <is>
+          <t>2026-08-08T10:06:13</t>
+        </is>
+      </c>
+      <c r="B376" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C376" t="inlineStr">
+        <is>
+          <t>CountPickedReject14in</t>
+        </is>
+      </c>
+      <c r="D376" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E376" t="inlineStr"/>
+      <c r="F376" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g30</t>
+        </is>
+      </c>
+    </row>
+    <row r="377">
+      <c r="A377" t="inlineStr">
+        <is>
+          <t>2026-08-08T10:06:13</t>
+        </is>
+      </c>
+      <c r="B377" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C377" t="inlineStr">
+        <is>
+          <t>temp_dsi</t>
+        </is>
+      </c>
+      <c r="D377" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E377" t="inlineStr"/>
+      <c r="F377" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g31</t>
+        </is>
+      </c>
+    </row>
+    <row r="378">
+      <c r="A378" t="inlineStr">
+        <is>
+          <t>2026-08-08T10:06:13</t>
+        </is>
+      </c>
+      <c r="B378" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C378" t="inlineStr">
+        <is>
+          <t>temp_J1motor</t>
+        </is>
+      </c>
+      <c r="D378" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E378" t="inlineStr"/>
+      <c r="F378" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g32</t>
+        </is>
+      </c>
+    </row>
+    <row r="379">
+      <c r="A379" t="inlineStr">
+        <is>
+          <t>2026-08-08T10:06:13</t>
+        </is>
+      </c>
+      <c r="B379" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C379" t="inlineStr">
+        <is>
+          <t>temp_J4motor</t>
+        </is>
+      </c>
+      <c r="D379" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E379" t="inlineStr"/>
+      <c r="F379" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g35</t>
+        </is>
+      </c>
+    </row>
+    <row r="380">
+      <c r="A380" t="inlineStr">
+        <is>
+          <t>2026-08-08T10:06:13</t>
+        </is>
+      </c>
+      <c r="B380" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C380" t="inlineStr">
+        <is>
+          <t>temp_J6motor</t>
+        </is>
+      </c>
+      <c r="D380" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E380" t="inlineStr"/>
+      <c r="F380" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g37</t>
+        </is>
+      </c>
+    </row>
+    <row r="381">
+      <c r="A381" t="inlineStr">
+        <is>
+          <t>2026-08-08T10:06:13</t>
+        </is>
+      </c>
+      <c r="B381" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C381" t="inlineStr">
+        <is>
+          <t>CountPickedRejectOTM</t>
+        </is>
+      </c>
+      <c r="D381" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E381" t="inlineStr"/>
+      <c r="F381" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g38</t>
+        </is>
+      </c>
+    </row>
+    <row r="382">
+      <c r="A382" t="inlineStr">
+        <is>
+          <t>2026-08-08T10:06:13</t>
+        </is>
+      </c>
+      <c r="B382" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C382" t="inlineStr">
+        <is>
+          <t>CountPickedRejectPandral</t>
+        </is>
+      </c>
+      <c r="D382" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E382" t="inlineStr"/>
+      <c r="F382" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g39</t>
+        </is>
+      </c>
+    </row>
+    <row r="383">
+      <c r="A383" t="inlineStr">
+        <is>
+          <t>2026-08-08T10:06:13</t>
+        </is>
+      </c>
+      <c r="B383" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C383" t="inlineStr">
+        <is>
+          <t>temp_J2motor</t>
+        </is>
+      </c>
+      <c r="D383" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E383" t="inlineStr"/>
+      <c r="F383" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g33</t>
+        </is>
+      </c>
+    </row>
+    <row r="384">
+      <c r="A384" t="inlineStr">
+        <is>
+          <t>2026-08-08T10:06:13</t>
+        </is>
+      </c>
+      <c r="B384" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C384" t="inlineStr">
+        <is>
+          <t>temp_J3motor</t>
+        </is>
+      </c>
+      <c r="D384" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E384" t="inlineStr"/>
+      <c r="F384" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g34</t>
+        </is>
+      </c>
+    </row>
+    <row r="385">
+      <c r="A385" t="inlineStr">
+        <is>
+          <t>2026-08-08T10:06:13</t>
+        </is>
+      </c>
+      <c r="B385" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C385" t="inlineStr">
+        <is>
+          <t>temp_J5motor</t>
+        </is>
+      </c>
+      <c r="D385" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E385" t="inlineStr"/>
+      <c r="F385" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g36</t>
+        </is>
+      </c>
+    </row>
+    <row r="386">
+      <c r="A386" t="inlineStr">
+        <is>
+          <t>2026-08-08T10:06:13</t>
+        </is>
+      </c>
+      <c r="B386" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C386" t="inlineStr">
+        <is>
+          <t>CountPickedReject18in</t>
+        </is>
+      </c>
+      <c r="D386" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E386" t="inlineStr"/>
+      <c r="F386" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g40</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Log MQTT data 2026-08-08 11:45 UTC
</commit_message>
<xml_diff>
--- a/logs/raiv_tracker_2026-08-08.xlsx
+++ b/logs/raiv_tracker_2026-08-08.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F386"/>
+  <dimension ref="A1:F516"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -10009,7 +10009,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E347" t="inlineStr"/>
       <c r="F347" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g1</t>
@@ -10037,7 +10036,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E348" t="inlineStr"/>
       <c r="F348" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g2</t>
@@ -10065,7 +10063,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E349" t="inlineStr"/>
       <c r="F349" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g3</t>
@@ -10093,7 +10090,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E350" t="inlineStr"/>
       <c r="F350" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g4</t>
@@ -10121,7 +10117,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E351" t="inlineStr"/>
       <c r="F351" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g5</t>
@@ -10149,7 +10144,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E352" t="inlineStr"/>
       <c r="F352" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g6</t>
@@ -10177,7 +10171,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E353" t="inlineStr"/>
       <c r="F353" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g7</t>
@@ -10205,7 +10198,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E354" t="inlineStr"/>
       <c r="F354" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g8</t>
@@ -10233,7 +10225,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E355" t="inlineStr"/>
       <c r="F355" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g9</t>
@@ -10261,7 +10252,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E356" t="inlineStr"/>
       <c r="F356" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g13</t>
@@ -10289,7 +10279,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E357" t="inlineStr"/>
       <c r="F357" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g15</t>
@@ -10317,7 +10306,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E358" t="inlineStr"/>
       <c r="F358" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g17</t>
@@ -10345,7 +10333,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E359" t="inlineStr"/>
       <c r="F359" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g18</t>
@@ -10373,7 +10360,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E360" t="inlineStr"/>
       <c r="F360" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g19</t>
@@ -10401,7 +10387,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E361" t="inlineStr"/>
       <c r="F361" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g22</t>
@@ -10429,7 +10414,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E362" t="inlineStr"/>
       <c r="F362" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g23</t>
@@ -10457,7 +10441,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E363" t="inlineStr"/>
       <c r="F363" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g24</t>
@@ -10485,7 +10468,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E364" t="inlineStr"/>
       <c r="F364" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g25</t>
@@ -10513,7 +10495,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E365" t="inlineStr"/>
       <c r="F365" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g10</t>
@@ -10541,7 +10522,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E366" t="inlineStr"/>
       <c r="F366" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g11</t>
@@ -10569,7 +10549,6 @@
           <t>1</t>
         </is>
       </c>
-      <c r="E367" t="inlineStr"/>
       <c r="F367" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g12</t>
@@ -10597,7 +10576,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E368" t="inlineStr"/>
       <c r="F368" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g14</t>
@@ -10625,7 +10603,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E369" t="inlineStr"/>
       <c r="F369" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g16</t>
@@ -10653,7 +10630,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E370" t="inlineStr"/>
       <c r="F370" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g20</t>
@@ -10681,7 +10657,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E371" t="inlineStr"/>
       <c r="F371" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g21</t>
@@ -10709,7 +10684,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E372" t="inlineStr"/>
       <c r="F372" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g26</t>
@@ -10737,7 +10711,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E373" t="inlineStr"/>
       <c r="F373" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g27</t>
@@ -10765,7 +10738,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E374" t="inlineStr"/>
       <c r="F374" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g28</t>
@@ -10793,7 +10765,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E375" t="inlineStr"/>
       <c r="F375" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g29</t>
@@ -10821,7 +10792,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E376" t="inlineStr"/>
       <c r="F376" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g30</t>
@@ -10849,7 +10819,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E377" t="inlineStr"/>
       <c r="F377" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g31</t>
@@ -10877,7 +10846,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E378" t="inlineStr"/>
       <c r="F378" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g32</t>
@@ -10905,7 +10873,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E379" t="inlineStr"/>
       <c r="F379" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g35</t>
@@ -10933,7 +10900,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E380" t="inlineStr"/>
       <c r="F380" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g37</t>
@@ -10961,7 +10927,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E381" t="inlineStr"/>
       <c r="F381" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g38</t>
@@ -10989,7 +10954,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E382" t="inlineStr"/>
       <c r="F382" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g39</t>
@@ -11017,7 +10981,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E383" t="inlineStr"/>
       <c r="F383" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g33</t>
@@ -11045,7 +11008,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E384" t="inlineStr"/>
       <c r="F384" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g34</t>
@@ -11073,7 +11035,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E385" t="inlineStr"/>
       <c r="F385" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g36</t>
@@ -11101,10 +11062,3649 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E386" t="inlineStr"/>
       <c r="F386" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g40</t>
+        </is>
+      </c>
+    </row>
+    <row r="387">
+      <c r="A387" t="inlineStr">
+        <is>
+          <t>2026-08-08T11:44:00</t>
+        </is>
+      </c>
+      <c r="B387" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C387" t="inlineStr">
+        <is>
+          <t>_1st_SCAN</t>
+        </is>
+      </c>
+      <c r="D387" t="b">
+        <v>0</v>
+      </c>
+      <c r="E387" t="n">
+        <v>11</v>
+      </c>
+      <c r="F387" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="388">
+      <c r="A388" t="inlineStr">
+        <is>
+          <t>2026-08-08T11:44:00</t>
+        </is>
+      </c>
+      <c r="B388" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C388" t="inlineStr">
+        <is>
+          <t>TieDetectOffset_B</t>
+        </is>
+      </c>
+      <c r="D388" t="b">
+        <v>0</v>
+      </c>
+      <c r="E388" t="n">
+        <v>11</v>
+      </c>
+      <c r="F388" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="389">
+      <c r="A389" t="inlineStr">
+        <is>
+          <t>2026-08-08T11:44:00</t>
+        </is>
+      </c>
+      <c r="B389" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C389" t="inlineStr">
+        <is>
+          <t>Tie Detector</t>
+        </is>
+      </c>
+      <c r="D389" t="b">
+        <v>0</v>
+      </c>
+      <c r="E389" t="n">
+        <v>11</v>
+      </c>
+      <c r="F389" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="390">
+      <c r="A390" t="inlineStr">
+        <is>
+          <t>2026-08-08T11:44:00</t>
+        </is>
+      </c>
+      <c r="B390" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C390" t="inlineStr">
+        <is>
+          <t>TPS Full</t>
+        </is>
+      </c>
+      <c r="D390" t="b">
+        <v>0</v>
+      </c>
+      <c r="E390" t="n">
+        <v>11</v>
+      </c>
+      <c r="F390" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="391">
+      <c r="A391" t="inlineStr">
+        <is>
+          <t>2026-08-08T11:44:00</t>
+        </is>
+      </c>
+      <c r="B391" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C391" t="inlineStr">
+        <is>
+          <t>TieDetectOffset_A</t>
+        </is>
+      </c>
+      <c r="D391" t="b">
+        <v>0</v>
+      </c>
+      <c r="E391" t="n">
+        <v>11</v>
+      </c>
+      <c r="F391" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="392">
+      <c r="A392" t="inlineStr">
+        <is>
+          <t>2026-08-08T11:44:00</t>
+        </is>
+      </c>
+      <c r="B392" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C392" t="inlineStr">
+        <is>
+          <t>TPS Connected</t>
+        </is>
+      </c>
+      <c r="D392" t="b">
+        <v>0</v>
+      </c>
+      <c r="E392" t="n">
+        <v>11</v>
+      </c>
+      <c r="F392" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="393">
+      <c r="A393" t="inlineStr">
+        <is>
+          <t>2026-08-08T11:44:00</t>
+        </is>
+      </c>
+      <c r="B393" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C393" t="inlineStr">
+        <is>
+          <t>TPS_Enable_ Button</t>
+        </is>
+      </c>
+      <c r="D393" t="b">
+        <v>0</v>
+      </c>
+      <c r="E393" t="n">
+        <v>11</v>
+      </c>
+      <c r="F393" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="394">
+      <c r="A394" t="inlineStr">
+        <is>
+          <t>2026-08-08T11:44:00</t>
+        </is>
+      </c>
+      <c r="B394" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C394" t="inlineStr">
+        <is>
+          <t>AirEagle Eject Plate</t>
+        </is>
+      </c>
+      <c r="D394" t="b">
+        <v>0</v>
+      </c>
+      <c r="E394" t="n">
+        <v>11</v>
+      </c>
+      <c r="F394" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="395">
+      <c r="A395" t="inlineStr">
+        <is>
+          <t>2026-08-08T11:44:00</t>
+        </is>
+      </c>
+      <c r="B395" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C395" t="inlineStr">
+        <is>
+          <t>tk_Cycle</t>
+        </is>
+      </c>
+      <c r="D395" t="b">
+        <v>0</v>
+      </c>
+      <c r="E395" t="n">
+        <v>11</v>
+      </c>
+      <c r="F395" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="396">
+      <c r="A396" t="inlineStr">
+        <is>
+          <t>2026-08-08T11:44:00</t>
+        </is>
+      </c>
+      <c r="B396" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C396" t="inlineStr">
+        <is>
+          <t>Servos_Enabled</t>
+        </is>
+      </c>
+      <c r="D396" t="b">
+        <v>0</v>
+      </c>
+      <c r="E396" t="n">
+        <v>11</v>
+      </c>
+      <c r="F396" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="397">
+      <c r="A397" t="inlineStr">
+        <is>
+          <t>2026-08-08T11:44:00</t>
+        </is>
+      </c>
+      <c r="B397" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C397" t="inlineStr">
+        <is>
+          <t>TPS Enabled</t>
+        </is>
+      </c>
+      <c r="D397" t="b">
+        <v>0</v>
+      </c>
+      <c r="E397" t="n">
+        <v>11</v>
+      </c>
+      <c r="F397" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="398">
+      <c r="A398" t="inlineStr">
+        <is>
+          <t>2026-08-08T11:44:00</t>
+        </is>
+      </c>
+      <c r="B398" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C398" t="inlineStr">
+        <is>
+          <t>tk_Abort</t>
+        </is>
+      </c>
+      <c r="D398" t="b">
+        <v>0</v>
+      </c>
+      <c r="E398" t="n">
+        <v>11</v>
+      </c>
+      <c r="F398" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="399">
+      <c r="A399" t="inlineStr">
+        <is>
+          <t>2026-08-08T11:44:00</t>
+        </is>
+      </c>
+      <c r="B399" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C399" t="inlineStr">
+        <is>
+          <t>Robot_isMoving</t>
+        </is>
+      </c>
+      <c r="D399" t="b">
+        <v>0</v>
+      </c>
+      <c r="E399" t="n">
+        <v>11</v>
+      </c>
+      <c r="F399" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="400">
+      <c r="A400" t="inlineStr">
+        <is>
+          <t>2026-08-08T11:44:00</t>
+        </is>
+      </c>
+      <c r="B400" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C400" t="inlineStr">
+        <is>
+          <t>Eject Tie Plate</t>
+        </is>
+      </c>
+      <c r="D400" t="b">
+        <v>0</v>
+      </c>
+      <c r="E400" t="n">
+        <v>11</v>
+      </c>
+      <c r="F400" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="401">
+      <c r="A401" t="inlineStr">
+        <is>
+          <t>2026-08-08T11:44:00</t>
+        </is>
+      </c>
+      <c r="B401" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C401" t="inlineStr">
+        <is>
+          <t>TPS BACKUP ALARM</t>
+        </is>
+      </c>
+      <c r="D401" t="b">
+        <v>0</v>
+      </c>
+      <c r="E401" t="n">
+        <v>11</v>
+      </c>
+      <c r="F401" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="402">
+      <c r="A402" t="inlineStr">
+        <is>
+          <t>2026-08-08T11:44:00</t>
+        </is>
+      </c>
+      <c r="B402" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C402" t="inlineStr">
+        <is>
+          <t>14in Job</t>
+        </is>
+      </c>
+      <c r="D402" t="b">
+        <v>1</v>
+      </c>
+      <c r="E402" t="n">
+        <v>11</v>
+      </c>
+      <c r="F402" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="403">
+      <c r="A403" t="inlineStr">
+        <is>
+          <t>2026-08-08T11:44:00</t>
+        </is>
+      </c>
+      <c r="B403" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C403" t="inlineStr">
+        <is>
+          <t>18in Job</t>
+        </is>
+      </c>
+      <c r="D403" t="b">
+        <v>0</v>
+      </c>
+      <c r="E403" t="n">
+        <v>11</v>
+      </c>
+      <c r="F403" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="404">
+      <c r="A404" t="inlineStr">
+        <is>
+          <t>2026-08-08T11:44:00</t>
+        </is>
+      </c>
+      <c r="B404" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C404" t="inlineStr">
+        <is>
+          <t>Pandral Job</t>
+        </is>
+      </c>
+      <c r="D404" t="b">
+        <v>0</v>
+      </c>
+      <c r="E404" t="n">
+        <v>11</v>
+      </c>
+      <c r="F404" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="405">
+      <c r="A405" t="inlineStr">
+        <is>
+          <t>2026-08-08T11:44:00</t>
+        </is>
+      </c>
+      <c r="B405" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C405" t="inlineStr">
+        <is>
+          <t>DoubleLay Job</t>
+        </is>
+      </c>
+      <c r="D405" t="b">
+        <v>0</v>
+      </c>
+      <c r="E405" t="n">
+        <v>11</v>
+      </c>
+      <c r="F405" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="406">
+      <c r="A406" t="inlineStr">
+        <is>
+          <t>2026-08-08T11:44:00</t>
+        </is>
+      </c>
+      <c r="B406" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C406" t="inlineStr">
+        <is>
+          <t>TPSjam_FLAG</t>
+        </is>
+      </c>
+      <c r="D406" t="b">
+        <v>0</v>
+      </c>
+      <c r="E406" t="n">
+        <v>11</v>
+      </c>
+      <c r="F406" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="407">
+      <c r="A407" t="inlineStr">
+        <is>
+          <t>2026-08-08T11:44:00</t>
+        </is>
+      </c>
+      <c r="B407" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C407" t="inlineStr">
+        <is>
+          <t>RoCalRequest</t>
+        </is>
+      </c>
+      <c r="D407" t="b">
+        <v>0</v>
+      </c>
+      <c r="E407" t="n">
+        <v>11</v>
+      </c>
+      <c r="F407" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="408">
+      <c r="A408" t="inlineStr">
+        <is>
+          <t>2026-08-08T11:44:00</t>
+        </is>
+      </c>
+      <c r="B408" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C408" t="inlineStr">
+        <is>
+          <t>tkCycle_TotalSeconds</t>
+        </is>
+      </c>
+      <c r="D408" t="n">
+        <v>0</v>
+      </c>
+      <c r="E408" t="n">
+        <v>9</v>
+      </c>
+      <c r="F408" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="409">
+      <c r="A409" t="inlineStr">
+        <is>
+          <t>2026-08-08T11:44:00</t>
+        </is>
+      </c>
+      <c r="B409" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C409" t="inlineStr">
+        <is>
+          <t>tkCycle_NoMoveSec</t>
+        </is>
+      </c>
+      <c r="D409" t="n">
+        <v>0</v>
+      </c>
+      <c r="E409" t="n">
+        <v>9</v>
+      </c>
+      <c r="F409" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="410">
+      <c r="A410" t="inlineStr">
+        <is>
+          <t>2026-08-08T11:44:00</t>
+        </is>
+      </c>
+      <c r="B410" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C410" t="inlineStr">
+        <is>
+          <t>tkCycle_MoveSeconds</t>
+        </is>
+      </c>
+      <c r="D410" t="n">
+        <v>0</v>
+      </c>
+      <c r="E410" t="n">
+        <v>9</v>
+      </c>
+      <c r="F410" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="411">
+      <c r="A411" t="inlineStr">
+        <is>
+          <t>2026-08-08T11:44:00</t>
+        </is>
+      </c>
+      <c r="B411" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C411" t="inlineStr">
+        <is>
+          <t>Percent time moveing</t>
+        </is>
+      </c>
+      <c r="D411" t="n">
+        <v>0</v>
+      </c>
+      <c r="E411" t="n">
+        <v>9</v>
+      </c>
+      <c r="F411" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="412">
+      <c r="A412" t="inlineStr">
+        <is>
+          <t>2026-08-08T11:44:00</t>
+        </is>
+      </c>
+      <c r="B412" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C412" t="inlineStr">
+        <is>
+          <t>Percent time not moving</t>
+        </is>
+      </c>
+      <c r="D412" t="n">
+        <v>0</v>
+      </c>
+      <c r="E412" t="n">
+        <v>9</v>
+      </c>
+      <c r="F412" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="413">
+      <c r="A413" t="inlineStr">
+        <is>
+          <t>2026-08-08T11:44:00</t>
+        </is>
+      </c>
+      <c r="B413" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C413" t="inlineStr">
+        <is>
+          <t>TotalPickPartsCount</t>
+        </is>
+      </c>
+      <c r="D413" t="n">
+        <v>0</v>
+      </c>
+      <c r="E413" t="n">
+        <v>9</v>
+      </c>
+      <c r="F413" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="414">
+      <c r="A414" t="inlineStr">
+        <is>
+          <t>2026-08-08T11:44:00</t>
+        </is>
+      </c>
+      <c r="B414" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C414" t="inlineStr">
+        <is>
+          <t>RejectPartsCount</t>
+        </is>
+      </c>
+      <c r="D414" t="n">
+        <v>0</v>
+      </c>
+      <c r="E414" t="n">
+        <v>9</v>
+      </c>
+      <c r="F414" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="415">
+      <c r="A415" t="inlineStr">
+        <is>
+          <t>2026-08-08T11:44:00</t>
+        </is>
+      </c>
+      <c r="B415" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C415" t="inlineStr">
+        <is>
+          <t>AcceptsPartsCount</t>
+        </is>
+      </c>
+      <c r="D415" t="n">
+        <v>0</v>
+      </c>
+      <c r="E415" t="n">
+        <v>9</v>
+      </c>
+      <c r="F415" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="416">
+      <c r="A416" t="inlineStr">
+        <is>
+          <t>2026-08-08T11:44:00</t>
+        </is>
+      </c>
+      <c r="B416" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C416" t="inlineStr">
+        <is>
+          <t>percentCount_accept</t>
+        </is>
+      </c>
+      <c r="D416" t="n">
+        <v>0</v>
+      </c>
+      <c r="E416" t="n">
+        <v>9</v>
+      </c>
+      <c r="F416" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="417">
+      <c r="A417" t="inlineStr">
+        <is>
+          <t>2026-08-08T11:44:00</t>
+        </is>
+      </c>
+      <c r="B417" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C417" t="inlineStr">
+        <is>
+          <t>percentCount_reject</t>
+        </is>
+      </c>
+      <c r="D417" t="n">
+        <v>0</v>
+      </c>
+      <c r="E417" t="n">
+        <v>9</v>
+      </c>
+      <c r="F417" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="418">
+      <c r="A418" t="inlineStr">
+        <is>
+          <t>2026-08-08T11:44:00</t>
+        </is>
+      </c>
+      <c r="B418" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C418" t="inlineStr">
+        <is>
+          <t>Avg Parts per min_total</t>
+        </is>
+      </c>
+      <c r="D418" t="n">
+        <v>0</v>
+      </c>
+      <c r="E418" t="n">
+        <v>9</v>
+      </c>
+      <c r="F418" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="419">
+      <c r="A419" t="inlineStr">
+        <is>
+          <t>2026-08-08T11:44:00</t>
+        </is>
+      </c>
+      <c r="B419" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C419" t="inlineStr">
+        <is>
+          <t>TotalPickedParts</t>
+        </is>
+      </c>
+      <c r="D419" t="n">
+        <v>0</v>
+      </c>
+      <c r="E419" t="n">
+        <v>3</v>
+      </c>
+      <c r="F419" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="420">
+      <c r="A420" t="inlineStr">
+        <is>
+          <t>2026-08-08T11:44:00</t>
+        </is>
+      </c>
+      <c r="B420" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C420" t="inlineStr">
+        <is>
+          <t>TotalPickedAcceptParts</t>
+        </is>
+      </c>
+      <c r="D420" t="n">
+        <v>0</v>
+      </c>
+      <c r="E420" t="n">
+        <v>3</v>
+      </c>
+      <c r="F420" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="421">
+      <c r="A421" t="inlineStr">
+        <is>
+          <t>2026-08-08T11:44:00</t>
+        </is>
+      </c>
+      <c r="B421" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C421" t="inlineStr">
+        <is>
+          <t>TotalPickedRejectParts</t>
+        </is>
+      </c>
+      <c r="D421" t="n">
+        <v>0</v>
+      </c>
+      <c r="E421" t="n">
+        <v>3</v>
+      </c>
+      <c r="F421" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="422">
+      <c r="A422" t="inlineStr">
+        <is>
+          <t>2026-08-08T11:44:00</t>
+        </is>
+      </c>
+      <c r="B422" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C422" t="inlineStr">
+        <is>
+          <t>TotalTiePlatesLaid</t>
+        </is>
+      </c>
+      <c r="D422" t="n">
+        <v>0</v>
+      </c>
+      <c r="E422" t="n">
+        <v>3</v>
+      </c>
+      <c r="F422" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="423">
+      <c r="A423" t="inlineStr">
+        <is>
+          <t>2026-08-08T11:44:00</t>
+        </is>
+      </c>
+      <c r="B423" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C423" t="inlineStr">
+        <is>
+          <t>Daily_TotalLaidPlates</t>
+        </is>
+      </c>
+      <c r="D423" t="n">
+        <v>0</v>
+      </c>
+      <c r="E423" t="n">
+        <v>3</v>
+      </c>
+      <c r="F423" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="424">
+      <c r="A424" t="inlineStr">
+        <is>
+          <t>2026-08-08T11:44:00</t>
+        </is>
+      </c>
+      <c r="B424" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C424" t="inlineStr">
+        <is>
+          <t>CountPicked14in</t>
+        </is>
+      </c>
+      <c r="D424" t="n">
+        <v>0</v>
+      </c>
+      <c r="E424" t="n">
+        <v>3</v>
+      </c>
+      <c r="F424" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="425">
+      <c r="A425" t="inlineStr">
+        <is>
+          <t>2026-08-08T11:44:00</t>
+        </is>
+      </c>
+      <c r="B425" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C425" t="inlineStr">
+        <is>
+          <t>CountPicked18in</t>
+        </is>
+      </c>
+      <c r="D425" t="n">
+        <v>0</v>
+      </c>
+      <c r="E425" t="n">
+        <v>3</v>
+      </c>
+      <c r="F425" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="426">
+      <c r="A426" t="inlineStr">
+        <is>
+          <t>2026-08-08T11:44:00</t>
+        </is>
+      </c>
+      <c r="B426" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C426" t="inlineStr">
+        <is>
+          <t>CountPickedPandral</t>
+        </is>
+      </c>
+      <c r="D426" t="n">
+        <v>0</v>
+      </c>
+      <c r="E426" t="n">
+        <v>3</v>
+      </c>
+      <c r="F426" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="427">
+      <c r="A427" t="inlineStr">
+        <is>
+          <t>2026-08-08T11:44:00</t>
+        </is>
+      </c>
+      <c r="B427" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C427" t="inlineStr">
+        <is>
+          <t>CountPickedOTM</t>
+        </is>
+      </c>
+      <c r="D427" t="n">
+        <v>0</v>
+      </c>
+      <c r="E427" t="n">
+        <v>3</v>
+      </c>
+      <c r="F427" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="428">
+      <c r="A428" t="inlineStr">
+        <is>
+          <t>2026-08-08T11:44:00</t>
+        </is>
+      </c>
+      <c r="B428" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C428" t="inlineStr">
+        <is>
+          <t>RoCals</t>
+        </is>
+      </c>
+      <c r="D428" t="n">
+        <v>0</v>
+      </c>
+      <c r="E428" t="n">
+        <v>3</v>
+      </c>
+      <c r="F428" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="429">
+      <c r="A429" t="inlineStr">
+        <is>
+          <t>2026-08-08T11:44:00</t>
+        </is>
+      </c>
+      <c r="B429" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C429" t="inlineStr">
+        <is>
+          <t>TPS_JamsUsr</t>
+        </is>
+      </c>
+      <c r="D429" t="n">
+        <v>0</v>
+      </c>
+      <c r="E429" t="n">
+        <v>3</v>
+      </c>
+      <c r="F429" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="430">
+      <c r="A430" t="inlineStr">
+        <is>
+          <t>2026-08-08T11:44:00</t>
+        </is>
+      </c>
+      <c r="B430" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C430" t="inlineStr">
+        <is>
+          <t>TPS_JamsMASTER</t>
+        </is>
+      </c>
+      <c r="D430" t="n">
+        <v>0</v>
+      </c>
+      <c r="E430" t="n">
+        <v>3</v>
+      </c>
+      <c r="F430" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="431">
+      <c r="A431" t="inlineStr">
+        <is>
+          <t>2026-08-08T11:44:00</t>
+        </is>
+      </c>
+      <c r="B431" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C431" t="inlineStr">
+        <is>
+          <t>ABORT_Master</t>
+        </is>
+      </c>
+      <c r="D431" t="n">
+        <v>0</v>
+      </c>
+      <c r="E431" t="n">
+        <v>3</v>
+      </c>
+      <c r="F431" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="432">
+      <c r="A432" t="inlineStr">
+        <is>
+          <t>2026-08-08T11:44:13</t>
+        </is>
+      </c>
+      <c r="B432" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C432" t="inlineStr">
+        <is>
+          <t>TotalTiePlatesLaid</t>
+        </is>
+      </c>
+      <c r="D432" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E432" t="inlineStr"/>
+      <c r="F432" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g1</t>
+        </is>
+      </c>
+    </row>
+    <row r="433">
+      <c r="A433" t="inlineStr">
+        <is>
+          <t>2026-08-08T11:44:13</t>
+        </is>
+      </c>
+      <c r="B433" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C433" t="inlineStr">
+        <is>
+          <t>CountLaidButton</t>
+        </is>
+      </c>
+      <c r="D433" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E433" t="inlineStr"/>
+      <c r="F433" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g2</t>
+        </is>
+      </c>
+    </row>
+    <row r="434">
+      <c r="A434" t="inlineStr">
+        <is>
+          <t>2026-08-08T11:44:13</t>
+        </is>
+      </c>
+      <c r="B434" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C434" t="inlineStr">
+        <is>
+          <t>CountLaidDetector</t>
+        </is>
+      </c>
+      <c r="D434" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E434" t="inlineStr"/>
+      <c r="F434" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g3</t>
+        </is>
+      </c>
+    </row>
+    <row r="435">
+      <c r="A435" t="inlineStr">
+        <is>
+          <t>2026-08-08T11:44:13</t>
+        </is>
+      </c>
+      <c r="B435" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C435" t="inlineStr">
+        <is>
+          <t>CountLaidEncoder</t>
+        </is>
+      </c>
+      <c r="D435" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E435" t="inlineStr"/>
+      <c r="F435" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g4</t>
+        </is>
+      </c>
+    </row>
+    <row r="436">
+      <c r="A436" t="inlineStr">
+        <is>
+          <t>2026-08-08T11:44:13</t>
+        </is>
+      </c>
+      <c r="B436" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C436" t="inlineStr">
+        <is>
+          <t>CountLaid14in</t>
+        </is>
+      </c>
+      <c r="D436" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E436" t="inlineStr"/>
+      <c r="F436" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g5</t>
+        </is>
+      </c>
+    </row>
+    <row r="437">
+      <c r="A437" t="inlineStr">
+        <is>
+          <t>2026-08-08T11:44:13</t>
+        </is>
+      </c>
+      <c r="B437" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C437" t="inlineStr">
+        <is>
+          <t>CountLaid18in</t>
+        </is>
+      </c>
+      <c r="D437" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E437" t="inlineStr"/>
+      <c r="F437" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g6</t>
+        </is>
+      </c>
+    </row>
+    <row r="438">
+      <c r="A438" t="inlineStr">
+        <is>
+          <t>2026-08-08T11:44:13</t>
+        </is>
+      </c>
+      <c r="B438" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C438" t="inlineStr">
+        <is>
+          <t>CountLaidPandral</t>
+        </is>
+      </c>
+      <c r="D438" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E438" t="inlineStr"/>
+      <c r="F438" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g7</t>
+        </is>
+      </c>
+    </row>
+    <row r="439">
+      <c r="A439" t="inlineStr">
+        <is>
+          <t>2026-08-08T11:44:13</t>
+        </is>
+      </c>
+      <c r="B439" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C439" t="inlineStr">
+        <is>
+          <t>18in Job</t>
+        </is>
+      </c>
+      <c r="D439" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E439" t="inlineStr"/>
+      <c r="F439" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g13</t>
+        </is>
+      </c>
+    </row>
+    <row r="440">
+      <c r="A440" t="inlineStr">
+        <is>
+          <t>2026-08-08T11:44:13</t>
+        </is>
+      </c>
+      <c r="B440" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C440" t="inlineStr">
+        <is>
+          <t>CountAcceptedTotal</t>
+        </is>
+      </c>
+      <c r="D440" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E440" t="inlineStr"/>
+      <c r="F440" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g15</t>
+        </is>
+      </c>
+    </row>
+    <row r="441">
+      <c r="A441" t="inlineStr">
+        <is>
+          <t>2026-08-08T11:44:13</t>
+        </is>
+      </c>
+      <c r="B441" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C441" t="inlineStr">
+        <is>
+          <t>Servos_Enabled</t>
+        </is>
+      </c>
+      <c r="D441" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E441" t="inlineStr"/>
+      <c r="F441" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g17</t>
+        </is>
+      </c>
+    </row>
+    <row r="442">
+      <c r="A442" t="inlineStr">
+        <is>
+          <t>2026-08-08T11:44:13</t>
+        </is>
+      </c>
+      <c r="B442" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C442" t="inlineStr">
+        <is>
+          <t>TotalPickPartsCount</t>
+        </is>
+      </c>
+      <c r="D442" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E442" t="inlineStr"/>
+      <c r="F442" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g18</t>
+        </is>
+      </c>
+    </row>
+    <row r="443">
+      <c r="A443" t="inlineStr">
+        <is>
+          <t>2026-08-08T11:44:13</t>
+        </is>
+      </c>
+      <c r="B443" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C443" t="inlineStr">
+        <is>
+          <t>AcceptsPartsCount</t>
+        </is>
+      </c>
+      <c r="D443" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E443" t="inlineStr"/>
+      <c r="F443" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g19</t>
+        </is>
+      </c>
+    </row>
+    <row r="444">
+      <c r="A444" t="inlineStr">
+        <is>
+          <t>2026-08-08T11:44:13</t>
+        </is>
+      </c>
+      <c r="B444" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C444" t="inlineStr">
+        <is>
+          <t>day_Servotime Hours10th</t>
+        </is>
+      </c>
+      <c r="D444" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E444" t="inlineStr"/>
+      <c r="F444" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g22</t>
+        </is>
+      </c>
+    </row>
+    <row r="445">
+      <c r="A445" t="inlineStr">
+        <is>
+          <t>2026-08-08T11:44:13</t>
+        </is>
+      </c>
+      <c r="B445" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C445" t="inlineStr">
+        <is>
+          <t>tk_Cycle</t>
+        </is>
+      </c>
+      <c r="D445" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E445" t="inlineStr"/>
+      <c r="F445" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g23</t>
+        </is>
+      </c>
+    </row>
+    <row r="446">
+      <c r="A446" t="inlineStr">
+        <is>
+          <t>2026-08-08T11:44:13</t>
+        </is>
+      </c>
+      <c r="B446" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C446" t="inlineStr">
+        <is>
+          <t>tk_Abort</t>
+        </is>
+      </c>
+      <c r="D446" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E446" t="inlineStr"/>
+      <c r="F446" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g24</t>
+        </is>
+      </c>
+    </row>
+    <row r="447">
+      <c r="A447" t="inlineStr">
+        <is>
+          <t>2026-08-08T11:44:13</t>
+        </is>
+      </c>
+      <c r="B447" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C447" t="inlineStr">
+        <is>
+          <t>tk_ClearPos</t>
+        </is>
+      </c>
+      <c r="D447" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E447" t="inlineStr"/>
+      <c r="F447" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g25</t>
+        </is>
+      </c>
+    </row>
+    <row r="448">
+      <c r="A448" t="inlineStr">
+        <is>
+          <t>2026-08-08T11:44:13</t>
+        </is>
+      </c>
+      <c r="B448" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C448" t="inlineStr">
+        <is>
+          <t>temp_J2motor</t>
+        </is>
+      </c>
+      <c r="D448" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E448" t="inlineStr"/>
+      <c r="F448" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g33</t>
+        </is>
+      </c>
+    </row>
+    <row r="449">
+      <c r="A449" t="inlineStr">
+        <is>
+          <t>2026-08-08T11:44:13</t>
+        </is>
+      </c>
+      <c r="B449" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C449" t="inlineStr">
+        <is>
+          <t>usr_TPStime Hours10th</t>
+        </is>
+      </c>
+      <c r="D449" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E449" t="inlineStr"/>
+      <c r="F449" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g8</t>
+        </is>
+      </c>
+    </row>
+    <row r="450">
+      <c r="A450" t="inlineStr">
+        <is>
+          <t>2026-08-08T11:44:13</t>
+        </is>
+      </c>
+      <c r="B450" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C450" t="inlineStr">
+        <is>
+          <t>usrTPS_miles xxx</t>
+        </is>
+      </c>
+      <c r="D450" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E450" t="inlineStr"/>
+      <c r="F450" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g9</t>
+        </is>
+      </c>
+    </row>
+    <row r="451">
+      <c r="A451" t="inlineStr">
+        <is>
+          <t>2026-08-08T11:44:13</t>
+        </is>
+      </c>
+      <c r="B451" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C451" t="inlineStr">
+        <is>
+          <t>TPS Connected</t>
+        </is>
+      </c>
+      <c r="D451" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E451" t="inlineStr"/>
+      <c r="F451" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g10</t>
+        </is>
+      </c>
+    </row>
+    <row r="452">
+      <c r="A452" t="inlineStr">
+        <is>
+          <t>2026-08-08T11:44:13</t>
+        </is>
+      </c>
+      <c r="B452" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C452" t="inlineStr">
+        <is>
+          <t>TPS Enabled</t>
+        </is>
+      </c>
+      <c r="D452" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E452" t="inlineStr"/>
+      <c r="F452" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g11</t>
+        </is>
+      </c>
+    </row>
+    <row r="453">
+      <c r="A453" t="inlineStr">
+        <is>
+          <t>2026-08-08T11:44:13</t>
+        </is>
+      </c>
+      <c r="B453" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C453" t="inlineStr">
+        <is>
+          <t>14in Job</t>
+        </is>
+      </c>
+      <c r="D453" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E453" t="inlineStr"/>
+      <c r="F453" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g12</t>
+        </is>
+      </c>
+    </row>
+    <row r="454">
+      <c r="A454" t="inlineStr">
+        <is>
+          <t>2026-08-08T11:44:13</t>
+        </is>
+      </c>
+      <c r="B454" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C454" t="inlineStr">
+        <is>
+          <t>Pandral Job</t>
+        </is>
+      </c>
+      <c r="D454" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E454" t="inlineStr"/>
+      <c r="F454" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g14</t>
+        </is>
+      </c>
+    </row>
+    <row r="455">
+      <c r="A455" t="inlineStr">
+        <is>
+          <t>2026-08-08T11:44:13</t>
+        </is>
+      </c>
+      <c r="B455" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C455" t="inlineStr">
+        <is>
+          <t>CountRejectedTotal</t>
+        </is>
+      </c>
+      <c r="D455" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E455" t="inlineStr"/>
+      <c r="F455" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g16</t>
+        </is>
+      </c>
+    </row>
+    <row r="456">
+      <c r="A456" t="inlineStr">
+        <is>
+          <t>2026-08-08T11:44:13</t>
+        </is>
+      </c>
+      <c r="B456" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C456" t="inlineStr">
+        <is>
+          <t>RejectPartsCount</t>
+        </is>
+      </c>
+      <c r="D456" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E456" t="inlineStr"/>
+      <c r="F456" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g20</t>
+        </is>
+      </c>
+    </row>
+    <row r="457">
+      <c r="A457" t="inlineStr">
+        <is>
+          <t>2026-08-08T11:44:13</t>
+        </is>
+      </c>
+      <c r="B457" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C457" t="inlineStr">
+        <is>
+          <t>tk_Cycle hrs</t>
+        </is>
+      </c>
+      <c r="D457" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E457" t="inlineStr"/>
+      <c r="F457" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g21</t>
+        </is>
+      </c>
+    </row>
+    <row r="458">
+      <c r="A458" t="inlineStr">
+        <is>
+          <t>2026-08-08T11:44:13</t>
+        </is>
+      </c>
+      <c r="B458" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C458" t="inlineStr">
+        <is>
+          <t>temp_J3motor</t>
+        </is>
+      </c>
+      <c r="D458" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E458" t="inlineStr"/>
+      <c r="F458" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g34</t>
+        </is>
+      </c>
+    </row>
+    <row r="459">
+      <c r="A459" t="inlineStr">
+        <is>
+          <t>2026-08-08T11:44:13</t>
+        </is>
+      </c>
+      <c r="B459" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C459" t="inlineStr">
+        <is>
+          <t>tk_Warmup</t>
+        </is>
+      </c>
+      <c r="D459" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E459" t="inlineStr"/>
+      <c r="F459" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g26</t>
+        </is>
+      </c>
+    </row>
+    <row r="460">
+      <c r="A460" t="inlineStr">
+        <is>
+          <t>2026-08-08T11:44:13</t>
+        </is>
+      </c>
+      <c r="B460" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C460" t="inlineStr">
+        <is>
+          <t>FindingParts min</t>
+        </is>
+      </c>
+      <c r="D460" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E460" t="inlineStr"/>
+      <c r="F460" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g27</t>
+        </is>
+      </c>
+    </row>
+    <row r="461">
+      <c r="A461" t="inlineStr">
+        <is>
+          <t>2026-08-08T11:44:13</t>
+        </is>
+      </c>
+      <c r="B461" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C461" t="inlineStr">
+        <is>
+          <t>temp_J5motor</t>
+        </is>
+      </c>
+      <c r="D461" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E461" t="inlineStr"/>
+      <c r="F461" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g36</t>
+        </is>
+      </c>
+    </row>
+    <row r="462">
+      <c r="A462" t="inlineStr">
+        <is>
+          <t>2026-08-08T11:44:13</t>
+        </is>
+      </c>
+      <c r="B462" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C462" t="inlineStr">
+        <is>
+          <t>CountPickedReject18in</t>
+        </is>
+      </c>
+      <c r="D462" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E462" t="inlineStr"/>
+      <c r="F462" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g40</t>
+        </is>
+      </c>
+    </row>
+    <row r="463">
+      <c r="A463" t="inlineStr">
+        <is>
+          <t>2026-08-08T11:44:13</t>
+        </is>
+      </c>
+      <c r="B463" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C463" t="inlineStr">
+        <is>
+          <t>PickingParts min</t>
+        </is>
+      </c>
+      <c r="D463" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E463" t="inlineStr"/>
+      <c r="F463" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g28</t>
+        </is>
+      </c>
+    </row>
+    <row r="464">
+      <c r="A464" t="inlineStr">
+        <is>
+          <t>2026-08-08T11:44:13</t>
+        </is>
+      </c>
+      <c r="B464" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C464" t="inlineStr">
+        <is>
+          <t>PlacingParts min</t>
+        </is>
+      </c>
+      <c r="D464" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E464" t="inlineStr"/>
+      <c r="F464" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g29</t>
+        </is>
+      </c>
+    </row>
+    <row r="465">
+      <c r="A465" t="inlineStr">
+        <is>
+          <t>2026-08-08T11:44:13</t>
+        </is>
+      </c>
+      <c r="B465" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C465" t="inlineStr">
+        <is>
+          <t>CountPickedReject14in</t>
+        </is>
+      </c>
+      <c r="D465" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E465" t="inlineStr"/>
+      <c r="F465" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g30</t>
+        </is>
+      </c>
+    </row>
+    <row r="466">
+      <c r="A466" t="inlineStr">
+        <is>
+          <t>2026-08-08T11:44:13</t>
+        </is>
+      </c>
+      <c r="B466" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C466" t="inlineStr">
+        <is>
+          <t>temp_dsi</t>
+        </is>
+      </c>
+      <c r="D466" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E466" t="inlineStr"/>
+      <c r="F466" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g31</t>
+        </is>
+      </c>
+    </row>
+    <row r="467">
+      <c r="A467" t="inlineStr">
+        <is>
+          <t>2026-08-08T11:44:13</t>
+        </is>
+      </c>
+      <c r="B467" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C467" t="inlineStr">
+        <is>
+          <t>temp_J1motor</t>
+        </is>
+      </c>
+      <c r="D467" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E467" t="inlineStr"/>
+      <c r="F467" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g32</t>
+        </is>
+      </c>
+    </row>
+    <row r="468">
+      <c r="A468" t="inlineStr">
+        <is>
+          <t>2026-08-08T11:44:13</t>
+        </is>
+      </c>
+      <c r="B468" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C468" t="inlineStr">
+        <is>
+          <t>temp_J4motor</t>
+        </is>
+      </c>
+      <c r="D468" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E468" t="inlineStr"/>
+      <c r="F468" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g35</t>
+        </is>
+      </c>
+    </row>
+    <row r="469">
+      <c r="A469" t="inlineStr">
+        <is>
+          <t>2026-08-08T11:44:13</t>
+        </is>
+      </c>
+      <c r="B469" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C469" t="inlineStr">
+        <is>
+          <t>temp_J6motor</t>
+        </is>
+      </c>
+      <c r="D469" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E469" t="inlineStr"/>
+      <c r="F469" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g37</t>
+        </is>
+      </c>
+    </row>
+    <row r="470">
+      <c r="A470" t="inlineStr">
+        <is>
+          <t>2026-08-08T11:44:13</t>
+        </is>
+      </c>
+      <c r="B470" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C470" t="inlineStr">
+        <is>
+          <t>CountPickedRejectOTM</t>
+        </is>
+      </c>
+      <c r="D470" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E470" t="inlineStr"/>
+      <c r="F470" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g38</t>
+        </is>
+      </c>
+    </row>
+    <row r="471">
+      <c r="A471" t="inlineStr">
+        <is>
+          <t>2026-08-08T11:44:13</t>
+        </is>
+      </c>
+      <c r="B471" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C471" t="inlineStr">
+        <is>
+          <t>CountPickedRejectPandral</t>
+        </is>
+      </c>
+      <c r="D471" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E471" t="inlineStr"/>
+      <c r="F471" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g39</t>
+        </is>
+      </c>
+    </row>
+    <row r="472">
+      <c r="A472" t="inlineStr">
+        <is>
+          <t>2026-08-08T11:45:00</t>
+        </is>
+      </c>
+      <c r="B472" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C472" t="inlineStr">
+        <is>
+          <t>_1st_SCAN</t>
+        </is>
+      </c>
+      <c r="D472" t="b">
+        <v>0</v>
+      </c>
+      <c r="E472" t="n">
+        <v>11</v>
+      </c>
+      <c r="F472" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="473">
+      <c r="A473" t="inlineStr">
+        <is>
+          <t>2026-08-08T11:45:00</t>
+        </is>
+      </c>
+      <c r="B473" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C473" t="inlineStr">
+        <is>
+          <t>TieDetectOffset_B</t>
+        </is>
+      </c>
+      <c r="D473" t="b">
+        <v>0</v>
+      </c>
+      <c r="E473" t="n">
+        <v>11</v>
+      </c>
+      <c r="F473" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="474">
+      <c r="A474" t="inlineStr">
+        <is>
+          <t>2026-08-08T11:45:00</t>
+        </is>
+      </c>
+      <c r="B474" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C474" t="inlineStr">
+        <is>
+          <t>Tie Detector</t>
+        </is>
+      </c>
+      <c r="D474" t="b">
+        <v>0</v>
+      </c>
+      <c r="E474" t="n">
+        <v>11</v>
+      </c>
+      <c r="F474" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="475">
+      <c r="A475" t="inlineStr">
+        <is>
+          <t>2026-08-08T11:45:00</t>
+        </is>
+      </c>
+      <c r="B475" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C475" t="inlineStr">
+        <is>
+          <t>TPS Full</t>
+        </is>
+      </c>
+      <c r="D475" t="b">
+        <v>0</v>
+      </c>
+      <c r="E475" t="n">
+        <v>11</v>
+      </c>
+      <c r="F475" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="476">
+      <c r="A476" t="inlineStr">
+        <is>
+          <t>2026-08-08T11:45:00</t>
+        </is>
+      </c>
+      <c r="B476" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C476" t="inlineStr">
+        <is>
+          <t>TieDetectOffset_A</t>
+        </is>
+      </c>
+      <c r="D476" t="b">
+        <v>0</v>
+      </c>
+      <c r="E476" t="n">
+        <v>11</v>
+      </c>
+      <c r="F476" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="477">
+      <c r="A477" t="inlineStr">
+        <is>
+          <t>2026-08-08T11:45:00</t>
+        </is>
+      </c>
+      <c r="B477" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C477" t="inlineStr">
+        <is>
+          <t>TPS Connected</t>
+        </is>
+      </c>
+      <c r="D477" t="b">
+        <v>0</v>
+      </c>
+      <c r="E477" t="n">
+        <v>11</v>
+      </c>
+      <c r="F477" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="478">
+      <c r="A478" t="inlineStr">
+        <is>
+          <t>2026-08-08T11:45:00</t>
+        </is>
+      </c>
+      <c r="B478" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C478" t="inlineStr">
+        <is>
+          <t>TPS_Enable_ Button</t>
+        </is>
+      </c>
+      <c r="D478" t="b">
+        <v>0</v>
+      </c>
+      <c r="E478" t="n">
+        <v>11</v>
+      </c>
+      <c r="F478" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="479">
+      <c r="A479" t="inlineStr">
+        <is>
+          <t>2026-08-08T11:45:00</t>
+        </is>
+      </c>
+      <c r="B479" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C479" t="inlineStr">
+        <is>
+          <t>AirEagle Eject Plate</t>
+        </is>
+      </c>
+      <c r="D479" t="b">
+        <v>0</v>
+      </c>
+      <c r="E479" t="n">
+        <v>11</v>
+      </c>
+      <c r="F479" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="480">
+      <c r="A480" t="inlineStr">
+        <is>
+          <t>2026-08-08T11:45:00</t>
+        </is>
+      </c>
+      <c r="B480" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C480" t="inlineStr">
+        <is>
+          <t>tk_Cycle</t>
+        </is>
+      </c>
+      <c r="D480" t="b">
+        <v>0</v>
+      </c>
+      <c r="E480" t="n">
+        <v>11</v>
+      </c>
+      <c r="F480" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="481">
+      <c r="A481" t="inlineStr">
+        <is>
+          <t>2026-08-08T11:45:00</t>
+        </is>
+      </c>
+      <c r="B481" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C481" t="inlineStr">
+        <is>
+          <t>Servos_Enabled</t>
+        </is>
+      </c>
+      <c r="D481" t="b">
+        <v>0</v>
+      </c>
+      <c r="E481" t="n">
+        <v>11</v>
+      </c>
+      <c r="F481" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="482">
+      <c r="A482" t="inlineStr">
+        <is>
+          <t>2026-08-08T11:45:00</t>
+        </is>
+      </c>
+      <c r="B482" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C482" t="inlineStr">
+        <is>
+          <t>TPS Enabled</t>
+        </is>
+      </c>
+      <c r="D482" t="b">
+        <v>0</v>
+      </c>
+      <c r="E482" t="n">
+        <v>11</v>
+      </c>
+      <c r="F482" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="483">
+      <c r="A483" t="inlineStr">
+        <is>
+          <t>2026-08-08T11:45:00</t>
+        </is>
+      </c>
+      <c r="B483" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C483" t="inlineStr">
+        <is>
+          <t>tk_Abort</t>
+        </is>
+      </c>
+      <c r="D483" t="b">
+        <v>0</v>
+      </c>
+      <c r="E483" t="n">
+        <v>11</v>
+      </c>
+      <c r="F483" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="484">
+      <c r="A484" t="inlineStr">
+        <is>
+          <t>2026-08-08T11:45:00</t>
+        </is>
+      </c>
+      <c r="B484" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C484" t="inlineStr">
+        <is>
+          <t>Robot_isMoving</t>
+        </is>
+      </c>
+      <c r="D484" t="b">
+        <v>0</v>
+      </c>
+      <c r="E484" t="n">
+        <v>11</v>
+      </c>
+      <c r="F484" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="485">
+      <c r="A485" t="inlineStr">
+        <is>
+          <t>2026-08-08T11:45:00</t>
+        </is>
+      </c>
+      <c r="B485" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C485" t="inlineStr">
+        <is>
+          <t>Eject Tie Plate</t>
+        </is>
+      </c>
+      <c r="D485" t="b">
+        <v>0</v>
+      </c>
+      <c r="E485" t="n">
+        <v>11</v>
+      </c>
+      <c r="F485" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="486">
+      <c r="A486" t="inlineStr">
+        <is>
+          <t>2026-08-08T11:45:00</t>
+        </is>
+      </c>
+      <c r="B486" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C486" t="inlineStr">
+        <is>
+          <t>TPS BACKUP ALARM</t>
+        </is>
+      </c>
+      <c r="D486" t="b">
+        <v>0</v>
+      </c>
+      <c r="E486" t="n">
+        <v>11</v>
+      </c>
+      <c r="F486" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="487">
+      <c r="A487" t="inlineStr">
+        <is>
+          <t>2026-08-08T11:45:00</t>
+        </is>
+      </c>
+      <c r="B487" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C487" t="inlineStr">
+        <is>
+          <t>14in Job</t>
+        </is>
+      </c>
+      <c r="D487" t="b">
+        <v>1</v>
+      </c>
+      <c r="E487" t="n">
+        <v>11</v>
+      </c>
+      <c r="F487" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="488">
+      <c r="A488" t="inlineStr">
+        <is>
+          <t>2026-08-08T11:45:00</t>
+        </is>
+      </c>
+      <c r="B488" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C488" t="inlineStr">
+        <is>
+          <t>18in Job</t>
+        </is>
+      </c>
+      <c r="D488" t="b">
+        <v>0</v>
+      </c>
+      <c r="E488" t="n">
+        <v>11</v>
+      </c>
+      <c r="F488" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="489">
+      <c r="A489" t="inlineStr">
+        <is>
+          <t>2026-08-08T11:45:00</t>
+        </is>
+      </c>
+      <c r="B489" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C489" t="inlineStr">
+        <is>
+          <t>Pandral Job</t>
+        </is>
+      </c>
+      <c r="D489" t="b">
+        <v>0</v>
+      </c>
+      <c r="E489" t="n">
+        <v>11</v>
+      </c>
+      <c r="F489" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="490">
+      <c r="A490" t="inlineStr">
+        <is>
+          <t>2026-08-08T11:45:00</t>
+        </is>
+      </c>
+      <c r="B490" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C490" t="inlineStr">
+        <is>
+          <t>DoubleLay Job</t>
+        </is>
+      </c>
+      <c r="D490" t="b">
+        <v>0</v>
+      </c>
+      <c r="E490" t="n">
+        <v>11</v>
+      </c>
+      <c r="F490" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="491">
+      <c r="A491" t="inlineStr">
+        <is>
+          <t>2026-08-08T11:45:00</t>
+        </is>
+      </c>
+      <c r="B491" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C491" t="inlineStr">
+        <is>
+          <t>TPSjam_FLAG</t>
+        </is>
+      </c>
+      <c r="D491" t="b">
+        <v>0</v>
+      </c>
+      <c r="E491" t="n">
+        <v>11</v>
+      </c>
+      <c r="F491" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="492">
+      <c r="A492" t="inlineStr">
+        <is>
+          <t>2026-08-08T11:45:00</t>
+        </is>
+      </c>
+      <c r="B492" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C492" t="inlineStr">
+        <is>
+          <t>RoCalRequest</t>
+        </is>
+      </c>
+      <c r="D492" t="b">
+        <v>0</v>
+      </c>
+      <c r="E492" t="n">
+        <v>11</v>
+      </c>
+      <c r="F492" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="493">
+      <c r="A493" t="inlineStr">
+        <is>
+          <t>2026-08-08T11:45:00</t>
+        </is>
+      </c>
+      <c r="B493" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C493" t="inlineStr">
+        <is>
+          <t>tkCycle_TotalSeconds</t>
+        </is>
+      </c>
+      <c r="D493" t="n">
+        <v>0</v>
+      </c>
+      <c r="E493" t="n">
+        <v>9</v>
+      </c>
+      <c r="F493" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="494">
+      <c r="A494" t="inlineStr">
+        <is>
+          <t>2026-08-08T11:45:00</t>
+        </is>
+      </c>
+      <c r="B494" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C494" t="inlineStr">
+        <is>
+          <t>tkCycle_NoMoveSec</t>
+        </is>
+      </c>
+      <c r="D494" t="n">
+        <v>0</v>
+      </c>
+      <c r="E494" t="n">
+        <v>9</v>
+      </c>
+      <c r="F494" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="495">
+      <c r="A495" t="inlineStr">
+        <is>
+          <t>2026-08-08T11:45:00</t>
+        </is>
+      </c>
+      <c r="B495" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C495" t="inlineStr">
+        <is>
+          <t>tkCycle_MoveSeconds</t>
+        </is>
+      </c>
+      <c r="D495" t="n">
+        <v>0</v>
+      </c>
+      <c r="E495" t="n">
+        <v>9</v>
+      </c>
+      <c r="F495" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="496">
+      <c r="A496" t="inlineStr">
+        <is>
+          <t>2026-08-08T11:45:00</t>
+        </is>
+      </c>
+      <c r="B496" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C496" t="inlineStr">
+        <is>
+          <t>Percent time moveing</t>
+        </is>
+      </c>
+      <c r="D496" t="n">
+        <v>0</v>
+      </c>
+      <c r="E496" t="n">
+        <v>9</v>
+      </c>
+      <c r="F496" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="497">
+      <c r="A497" t="inlineStr">
+        <is>
+          <t>2026-08-08T11:45:00</t>
+        </is>
+      </c>
+      <c r="B497" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C497" t="inlineStr">
+        <is>
+          <t>Percent time not moving</t>
+        </is>
+      </c>
+      <c r="D497" t="n">
+        <v>0</v>
+      </c>
+      <c r="E497" t="n">
+        <v>9</v>
+      </c>
+      <c r="F497" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="498">
+      <c r="A498" t="inlineStr">
+        <is>
+          <t>2026-08-08T11:45:00</t>
+        </is>
+      </c>
+      <c r="B498" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C498" t="inlineStr">
+        <is>
+          <t>TotalPickPartsCount</t>
+        </is>
+      </c>
+      <c r="D498" t="n">
+        <v>0</v>
+      </c>
+      <c r="E498" t="n">
+        <v>9</v>
+      </c>
+      <c r="F498" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="499">
+      <c r="A499" t="inlineStr">
+        <is>
+          <t>2026-08-08T11:45:00</t>
+        </is>
+      </c>
+      <c r="B499" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C499" t="inlineStr">
+        <is>
+          <t>RejectPartsCount</t>
+        </is>
+      </c>
+      <c r="D499" t="n">
+        <v>0</v>
+      </c>
+      <c r="E499" t="n">
+        <v>9</v>
+      </c>
+      <c r="F499" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="500">
+      <c r="A500" t="inlineStr">
+        <is>
+          <t>2026-08-08T11:45:00</t>
+        </is>
+      </c>
+      <c r="B500" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C500" t="inlineStr">
+        <is>
+          <t>AcceptsPartsCount</t>
+        </is>
+      </c>
+      <c r="D500" t="n">
+        <v>0</v>
+      </c>
+      <c r="E500" t="n">
+        <v>9</v>
+      </c>
+      <c r="F500" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="501">
+      <c r="A501" t="inlineStr">
+        <is>
+          <t>2026-08-08T11:45:00</t>
+        </is>
+      </c>
+      <c r="B501" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C501" t="inlineStr">
+        <is>
+          <t>percentCount_accept</t>
+        </is>
+      </c>
+      <c r="D501" t="n">
+        <v>0</v>
+      </c>
+      <c r="E501" t="n">
+        <v>9</v>
+      </c>
+      <c r="F501" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="502">
+      <c r="A502" t="inlineStr">
+        <is>
+          <t>2026-08-08T11:45:00</t>
+        </is>
+      </c>
+      <c r="B502" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C502" t="inlineStr">
+        <is>
+          <t>percentCount_reject</t>
+        </is>
+      </c>
+      <c r="D502" t="n">
+        <v>0</v>
+      </c>
+      <c r="E502" t="n">
+        <v>9</v>
+      </c>
+      <c r="F502" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="503">
+      <c r="A503" t="inlineStr">
+        <is>
+          <t>2026-08-08T11:45:00</t>
+        </is>
+      </c>
+      <c r="B503" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C503" t="inlineStr">
+        <is>
+          <t>Avg Parts per min_total</t>
+        </is>
+      </c>
+      <c r="D503" t="n">
+        <v>0</v>
+      </c>
+      <c r="E503" t="n">
+        <v>9</v>
+      </c>
+      <c r="F503" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="504">
+      <c r="A504" t="inlineStr">
+        <is>
+          <t>2026-08-08T11:45:00</t>
+        </is>
+      </c>
+      <c r="B504" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C504" t="inlineStr">
+        <is>
+          <t>TotalPickedParts</t>
+        </is>
+      </c>
+      <c r="D504" t="n">
+        <v>0</v>
+      </c>
+      <c r="E504" t="n">
+        <v>3</v>
+      </c>
+      <c r="F504" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="505">
+      <c r="A505" t="inlineStr">
+        <is>
+          <t>2026-08-08T11:45:00</t>
+        </is>
+      </c>
+      <c r="B505" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C505" t="inlineStr">
+        <is>
+          <t>TotalPickedAcceptParts</t>
+        </is>
+      </c>
+      <c r="D505" t="n">
+        <v>0</v>
+      </c>
+      <c r="E505" t="n">
+        <v>3</v>
+      </c>
+      <c r="F505" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="506">
+      <c r="A506" t="inlineStr">
+        <is>
+          <t>2026-08-08T11:45:00</t>
+        </is>
+      </c>
+      <c r="B506" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C506" t="inlineStr">
+        <is>
+          <t>TotalPickedRejectParts</t>
+        </is>
+      </c>
+      <c r="D506" t="n">
+        <v>0</v>
+      </c>
+      <c r="E506" t="n">
+        <v>3</v>
+      </c>
+      <c r="F506" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="507">
+      <c r="A507" t="inlineStr">
+        <is>
+          <t>2026-08-08T11:45:00</t>
+        </is>
+      </c>
+      <c r="B507" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C507" t="inlineStr">
+        <is>
+          <t>TotalTiePlatesLaid</t>
+        </is>
+      </c>
+      <c r="D507" t="n">
+        <v>0</v>
+      </c>
+      <c r="E507" t="n">
+        <v>3</v>
+      </c>
+      <c r="F507" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="508">
+      <c r="A508" t="inlineStr">
+        <is>
+          <t>2026-08-08T11:45:00</t>
+        </is>
+      </c>
+      <c r="B508" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C508" t="inlineStr">
+        <is>
+          <t>Daily_TotalLaidPlates</t>
+        </is>
+      </c>
+      <c r="D508" t="n">
+        <v>0</v>
+      </c>
+      <c r="E508" t="n">
+        <v>3</v>
+      </c>
+      <c r="F508" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="509">
+      <c r="A509" t="inlineStr">
+        <is>
+          <t>2026-08-08T11:45:00</t>
+        </is>
+      </c>
+      <c r="B509" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C509" t="inlineStr">
+        <is>
+          <t>CountPicked14in</t>
+        </is>
+      </c>
+      <c r="D509" t="n">
+        <v>0</v>
+      </c>
+      <c r="E509" t="n">
+        <v>3</v>
+      </c>
+      <c r="F509" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="510">
+      <c r="A510" t="inlineStr">
+        <is>
+          <t>2026-08-08T11:45:00</t>
+        </is>
+      </c>
+      <c r="B510" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C510" t="inlineStr">
+        <is>
+          <t>CountPicked18in</t>
+        </is>
+      </c>
+      <c r="D510" t="n">
+        <v>0</v>
+      </c>
+      <c r="E510" t="n">
+        <v>3</v>
+      </c>
+      <c r="F510" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="511">
+      <c r="A511" t="inlineStr">
+        <is>
+          <t>2026-08-08T11:45:00</t>
+        </is>
+      </c>
+      <c r="B511" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C511" t="inlineStr">
+        <is>
+          <t>CountPickedPandral</t>
+        </is>
+      </c>
+      <c r="D511" t="n">
+        <v>0</v>
+      </c>
+      <c r="E511" t="n">
+        <v>3</v>
+      </c>
+      <c r="F511" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="512">
+      <c r="A512" t="inlineStr">
+        <is>
+          <t>2026-08-08T11:45:00</t>
+        </is>
+      </c>
+      <c r="B512" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C512" t="inlineStr">
+        <is>
+          <t>CountPickedOTM</t>
+        </is>
+      </c>
+      <c r="D512" t="n">
+        <v>0</v>
+      </c>
+      <c r="E512" t="n">
+        <v>3</v>
+      </c>
+      <c r="F512" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="513">
+      <c r="A513" t="inlineStr">
+        <is>
+          <t>2026-08-08T11:45:00</t>
+        </is>
+      </c>
+      <c r="B513" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C513" t="inlineStr">
+        <is>
+          <t>RoCals</t>
+        </is>
+      </c>
+      <c r="D513" t="n">
+        <v>0</v>
+      </c>
+      <c r="E513" t="n">
+        <v>3</v>
+      </c>
+      <c r="F513" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="514">
+      <c r="A514" t="inlineStr">
+        <is>
+          <t>2026-08-08T11:45:00</t>
+        </is>
+      </c>
+      <c r="B514" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C514" t="inlineStr">
+        <is>
+          <t>TPS_JamsUsr</t>
+        </is>
+      </c>
+      <c r="D514" t="n">
+        <v>0</v>
+      </c>
+      <c r="E514" t="n">
+        <v>3</v>
+      </c>
+      <c r="F514" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="515">
+      <c r="A515" t="inlineStr">
+        <is>
+          <t>2026-08-08T11:45:00</t>
+        </is>
+      </c>
+      <c r="B515" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C515" t="inlineStr">
+        <is>
+          <t>TPS_JamsMASTER</t>
+        </is>
+      </c>
+      <c r="D515" t="n">
+        <v>0</v>
+      </c>
+      <c r="E515" t="n">
+        <v>3</v>
+      </c>
+      <c r="F515" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="516">
+      <c r="A516" t="inlineStr">
+        <is>
+          <t>2026-08-08T11:45:00</t>
+        </is>
+      </c>
+      <c r="B516" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C516" t="inlineStr">
+        <is>
+          <t>ABORT_Master</t>
+        </is>
+      </c>
+      <c r="D516" t="n">
+        <v>0</v>
+      </c>
+      <c r="E516" t="n">
+        <v>3</v>
+      </c>
+      <c r="F516" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Log MQTT data 2026-08-08 14:03 UTC
</commit_message>
<xml_diff>
--- a/logs/raiv_tracker_2026-08-08.xlsx
+++ b/logs/raiv_tracker_2026-08-08.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F516"/>
+  <dimension ref="A1:F601"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -12349,7 +12349,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E432" t="inlineStr"/>
       <c r="F432" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g1</t>
@@ -12377,7 +12376,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E433" t="inlineStr"/>
       <c r="F433" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g2</t>
@@ -12405,7 +12403,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E434" t="inlineStr"/>
       <c r="F434" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g3</t>
@@ -12433,7 +12430,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E435" t="inlineStr"/>
       <c r="F435" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g4</t>
@@ -12461,7 +12457,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E436" t="inlineStr"/>
       <c r="F436" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g5</t>
@@ -12489,7 +12484,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E437" t="inlineStr"/>
       <c r="F437" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g6</t>
@@ -12517,7 +12511,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E438" t="inlineStr"/>
       <c r="F438" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g7</t>
@@ -12545,7 +12538,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E439" t="inlineStr"/>
       <c r="F439" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g13</t>
@@ -12573,7 +12565,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E440" t="inlineStr"/>
       <c r="F440" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g15</t>
@@ -12601,7 +12592,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E441" t="inlineStr"/>
       <c r="F441" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g17</t>
@@ -12629,7 +12619,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E442" t="inlineStr"/>
       <c r="F442" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g18</t>
@@ -12657,7 +12646,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E443" t="inlineStr"/>
       <c r="F443" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g19</t>
@@ -12685,7 +12673,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E444" t="inlineStr"/>
       <c r="F444" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g22</t>
@@ -12713,7 +12700,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E445" t="inlineStr"/>
       <c r="F445" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g23</t>
@@ -12741,7 +12727,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E446" t="inlineStr"/>
       <c r="F446" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g24</t>
@@ -12769,7 +12754,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E447" t="inlineStr"/>
       <c r="F447" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g25</t>
@@ -12797,7 +12781,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E448" t="inlineStr"/>
       <c r="F448" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g33</t>
@@ -12825,7 +12808,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E449" t="inlineStr"/>
       <c r="F449" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g8</t>
@@ -12853,7 +12835,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E450" t="inlineStr"/>
       <c r="F450" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g9</t>
@@ -12881,7 +12862,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E451" t="inlineStr"/>
       <c r="F451" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g10</t>
@@ -12909,7 +12889,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E452" t="inlineStr"/>
       <c r="F452" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g11</t>
@@ -12937,7 +12916,6 @@
           <t>1</t>
         </is>
       </c>
-      <c r="E453" t="inlineStr"/>
       <c r="F453" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g12</t>
@@ -12965,7 +12943,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E454" t="inlineStr"/>
       <c r="F454" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g14</t>
@@ -12993,7 +12970,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E455" t="inlineStr"/>
       <c r="F455" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g16</t>
@@ -13021,7 +12997,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E456" t="inlineStr"/>
       <c r="F456" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g20</t>
@@ -13049,7 +13024,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E457" t="inlineStr"/>
       <c r="F457" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g21</t>
@@ -13077,7 +13051,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E458" t="inlineStr"/>
       <c r="F458" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g34</t>
@@ -13105,7 +13078,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E459" t="inlineStr"/>
       <c r="F459" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g26</t>
@@ -13133,7 +13105,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E460" t="inlineStr"/>
       <c r="F460" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g27</t>
@@ -13161,7 +13132,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E461" t="inlineStr"/>
       <c r="F461" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g36</t>
@@ -13189,7 +13159,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E462" t="inlineStr"/>
       <c r="F462" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g40</t>
@@ -13217,7 +13186,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E463" t="inlineStr"/>
       <c r="F463" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g28</t>
@@ -13245,7 +13213,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E464" t="inlineStr"/>
       <c r="F464" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g29</t>
@@ -13273,7 +13240,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E465" t="inlineStr"/>
       <c r="F465" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g30</t>
@@ -13301,7 +13267,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E466" t="inlineStr"/>
       <c r="F466" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g31</t>
@@ -13329,7 +13294,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E467" t="inlineStr"/>
       <c r="F467" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g32</t>
@@ -13357,7 +13321,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E468" t="inlineStr"/>
       <c r="F468" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g35</t>
@@ -13385,7 +13348,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E469" t="inlineStr"/>
       <c r="F469" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g37</t>
@@ -13413,7 +13375,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E470" t="inlineStr"/>
       <c r="F470" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g38</t>
@@ -13441,7 +13402,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E471" t="inlineStr"/>
       <c r="F471" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g39</t>
@@ -14703,6 +14663,2386 @@
         <v>3</v>
       </c>
       <c r="F516" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="517">
+      <c r="A517" t="inlineStr">
+        <is>
+          <t>2026-08-08T14:02:13</t>
+        </is>
+      </c>
+      <c r="B517" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C517" t="inlineStr">
+        <is>
+          <t>TotalTiePlatesLaid</t>
+        </is>
+      </c>
+      <c r="D517" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E517" t="inlineStr"/>
+      <c r="F517" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g1</t>
+        </is>
+      </c>
+    </row>
+    <row r="518">
+      <c r="A518" t="inlineStr">
+        <is>
+          <t>2026-08-08T14:02:13</t>
+        </is>
+      </c>
+      <c r="B518" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C518" t="inlineStr">
+        <is>
+          <t>CountLaidButton</t>
+        </is>
+      </c>
+      <c r="D518" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E518" t="inlineStr"/>
+      <c r="F518" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g2</t>
+        </is>
+      </c>
+    </row>
+    <row r="519">
+      <c r="A519" t="inlineStr">
+        <is>
+          <t>2026-08-08T14:02:13</t>
+        </is>
+      </c>
+      <c r="B519" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C519" t="inlineStr">
+        <is>
+          <t>CountLaidDetector</t>
+        </is>
+      </c>
+      <c r="D519" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E519" t="inlineStr"/>
+      <c r="F519" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g3</t>
+        </is>
+      </c>
+    </row>
+    <row r="520">
+      <c r="A520" t="inlineStr">
+        <is>
+          <t>2026-08-08T14:02:13</t>
+        </is>
+      </c>
+      <c r="B520" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C520" t="inlineStr">
+        <is>
+          <t>CountLaidEncoder</t>
+        </is>
+      </c>
+      <c r="D520" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E520" t="inlineStr"/>
+      <c r="F520" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g4</t>
+        </is>
+      </c>
+    </row>
+    <row r="521">
+      <c r="A521" t="inlineStr">
+        <is>
+          <t>2026-08-08T14:02:13</t>
+        </is>
+      </c>
+      <c r="B521" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C521" t="inlineStr">
+        <is>
+          <t>CountLaid14in</t>
+        </is>
+      </c>
+      <c r="D521" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E521" t="inlineStr"/>
+      <c r="F521" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g5</t>
+        </is>
+      </c>
+    </row>
+    <row r="522">
+      <c r="A522" t="inlineStr">
+        <is>
+          <t>2026-08-08T14:02:13</t>
+        </is>
+      </c>
+      <c r="B522" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C522" t="inlineStr">
+        <is>
+          <t>CountLaid18in</t>
+        </is>
+      </c>
+      <c r="D522" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E522" t="inlineStr"/>
+      <c r="F522" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g6</t>
+        </is>
+      </c>
+    </row>
+    <row r="523">
+      <c r="A523" t="inlineStr">
+        <is>
+          <t>2026-08-08T14:02:13</t>
+        </is>
+      </c>
+      <c r="B523" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C523" t="inlineStr">
+        <is>
+          <t>CountLaidPandral</t>
+        </is>
+      </c>
+      <c r="D523" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E523" t="inlineStr"/>
+      <c r="F523" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g7</t>
+        </is>
+      </c>
+    </row>
+    <row r="524">
+      <c r="A524" t="inlineStr">
+        <is>
+          <t>2026-08-08T14:02:13</t>
+        </is>
+      </c>
+      <c r="B524" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C524" t="inlineStr">
+        <is>
+          <t>usr_TPStime Hours10th</t>
+        </is>
+      </c>
+      <c r="D524" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E524" t="inlineStr"/>
+      <c r="F524" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g8</t>
+        </is>
+      </c>
+    </row>
+    <row r="525">
+      <c r="A525" t="inlineStr">
+        <is>
+          <t>2026-08-08T14:02:13</t>
+        </is>
+      </c>
+      <c r="B525" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C525" t="inlineStr">
+        <is>
+          <t>18in Job</t>
+        </is>
+      </c>
+      <c r="D525" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E525" t="inlineStr"/>
+      <c r="F525" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g13</t>
+        </is>
+      </c>
+    </row>
+    <row r="526">
+      <c r="A526" t="inlineStr">
+        <is>
+          <t>2026-08-08T14:02:13</t>
+        </is>
+      </c>
+      <c r="B526" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C526" t="inlineStr">
+        <is>
+          <t>CountAcceptedTotal</t>
+        </is>
+      </c>
+      <c r="D526" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E526" t="inlineStr"/>
+      <c r="F526" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g15</t>
+        </is>
+      </c>
+    </row>
+    <row r="527">
+      <c r="A527" t="inlineStr">
+        <is>
+          <t>2026-08-08T14:02:13</t>
+        </is>
+      </c>
+      <c r="B527" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C527" t="inlineStr">
+        <is>
+          <t>Servos_Enabled</t>
+        </is>
+      </c>
+      <c r="D527" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E527" t="inlineStr"/>
+      <c r="F527" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g17</t>
+        </is>
+      </c>
+    </row>
+    <row r="528">
+      <c r="A528" t="inlineStr">
+        <is>
+          <t>2026-08-08T14:02:13</t>
+        </is>
+      </c>
+      <c r="B528" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C528" t="inlineStr">
+        <is>
+          <t>TotalPickPartsCount</t>
+        </is>
+      </c>
+      <c r="D528" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E528" t="inlineStr"/>
+      <c r="F528" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g18</t>
+        </is>
+      </c>
+    </row>
+    <row r="529">
+      <c r="A529" t="inlineStr">
+        <is>
+          <t>2026-08-08T14:02:13</t>
+        </is>
+      </c>
+      <c r="B529" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C529" t="inlineStr">
+        <is>
+          <t>AcceptsPartsCount</t>
+        </is>
+      </c>
+      <c r="D529" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E529" t="inlineStr"/>
+      <c r="F529" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g19</t>
+        </is>
+      </c>
+    </row>
+    <row r="530">
+      <c r="A530" t="inlineStr">
+        <is>
+          <t>2026-08-08T14:02:13</t>
+        </is>
+      </c>
+      <c r="B530" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C530" t="inlineStr">
+        <is>
+          <t>day_Servotime Hours10th</t>
+        </is>
+      </c>
+      <c r="D530" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E530" t="inlineStr"/>
+      <c r="F530" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g22</t>
+        </is>
+      </c>
+    </row>
+    <row r="531">
+      <c r="A531" t="inlineStr">
+        <is>
+          <t>2026-08-08T14:02:13</t>
+        </is>
+      </c>
+      <c r="B531" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C531" t="inlineStr">
+        <is>
+          <t>tk_Cycle</t>
+        </is>
+      </c>
+      <c r="D531" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E531" t="inlineStr"/>
+      <c r="F531" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g23</t>
+        </is>
+      </c>
+    </row>
+    <row r="532">
+      <c r="A532" t="inlineStr">
+        <is>
+          <t>2026-08-08T14:02:13</t>
+        </is>
+      </c>
+      <c r="B532" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C532" t="inlineStr">
+        <is>
+          <t>tk_Abort</t>
+        </is>
+      </c>
+      <c r="D532" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E532" t="inlineStr"/>
+      <c r="F532" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g24</t>
+        </is>
+      </c>
+    </row>
+    <row r="533">
+      <c r="A533" t="inlineStr">
+        <is>
+          <t>2026-08-08T14:02:13</t>
+        </is>
+      </c>
+      <c r="B533" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C533" t="inlineStr">
+        <is>
+          <t>tk_ClearPos</t>
+        </is>
+      </c>
+      <c r="D533" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E533" t="inlineStr"/>
+      <c r="F533" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g25</t>
+        </is>
+      </c>
+    </row>
+    <row r="534">
+      <c r="A534" t="inlineStr">
+        <is>
+          <t>2026-08-08T14:02:13</t>
+        </is>
+      </c>
+      <c r="B534" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C534" t="inlineStr">
+        <is>
+          <t>temp_J2motor</t>
+        </is>
+      </c>
+      <c r="D534" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E534" t="inlineStr"/>
+      <c r="F534" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g33</t>
+        </is>
+      </c>
+    </row>
+    <row r="535">
+      <c r="A535" t="inlineStr">
+        <is>
+          <t>2026-08-08T14:02:13</t>
+        </is>
+      </c>
+      <c r="B535" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C535" t="inlineStr">
+        <is>
+          <t>temp_J3motor</t>
+        </is>
+      </c>
+      <c r="D535" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E535" t="inlineStr"/>
+      <c r="F535" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g34</t>
+        </is>
+      </c>
+    </row>
+    <row r="536">
+      <c r="A536" t="inlineStr">
+        <is>
+          <t>2026-08-08T14:02:13</t>
+        </is>
+      </c>
+      <c r="B536" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C536" t="inlineStr">
+        <is>
+          <t>temp_J5motor</t>
+        </is>
+      </c>
+      <c r="D536" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E536" t="inlineStr"/>
+      <c r="F536" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g36</t>
+        </is>
+      </c>
+    </row>
+    <row r="537">
+      <c r="A537" t="inlineStr">
+        <is>
+          <t>2026-08-08T14:02:13</t>
+        </is>
+      </c>
+      <c r="B537" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C537" t="inlineStr">
+        <is>
+          <t>CountPickedReject18in</t>
+        </is>
+      </c>
+      <c r="D537" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E537" t="inlineStr"/>
+      <c r="F537" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g40</t>
+        </is>
+      </c>
+    </row>
+    <row r="538">
+      <c r="A538" t="inlineStr">
+        <is>
+          <t>2026-08-08T14:02:13</t>
+        </is>
+      </c>
+      <c r="B538" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C538" t="inlineStr">
+        <is>
+          <t>usrTPS_miles xxx</t>
+        </is>
+      </c>
+      <c r="D538" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E538" t="inlineStr"/>
+      <c r="F538" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g9</t>
+        </is>
+      </c>
+    </row>
+    <row r="539">
+      <c r="A539" t="inlineStr">
+        <is>
+          <t>2026-08-08T14:02:13</t>
+        </is>
+      </c>
+      <c r="B539" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C539" t="inlineStr">
+        <is>
+          <t>TPS Connected</t>
+        </is>
+      </c>
+      <c r="D539" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E539" t="inlineStr"/>
+      <c r="F539" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g10</t>
+        </is>
+      </c>
+    </row>
+    <row r="540">
+      <c r="A540" t="inlineStr">
+        <is>
+          <t>2026-08-08T14:02:13</t>
+        </is>
+      </c>
+      <c r="B540" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C540" t="inlineStr">
+        <is>
+          <t>TPS Enabled</t>
+        </is>
+      </c>
+      <c r="D540" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E540" t="inlineStr"/>
+      <c r="F540" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g11</t>
+        </is>
+      </c>
+    </row>
+    <row r="541">
+      <c r="A541" t="inlineStr">
+        <is>
+          <t>2026-08-08T14:02:13</t>
+        </is>
+      </c>
+      <c r="B541" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C541" t="inlineStr">
+        <is>
+          <t>14in Job</t>
+        </is>
+      </c>
+      <c r="D541" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E541" t="inlineStr"/>
+      <c r="F541" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g12</t>
+        </is>
+      </c>
+    </row>
+    <row r="542">
+      <c r="A542" t="inlineStr">
+        <is>
+          <t>2026-08-08T14:02:13</t>
+        </is>
+      </c>
+      <c r="B542" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C542" t="inlineStr">
+        <is>
+          <t>Pandral Job</t>
+        </is>
+      </c>
+      <c r="D542" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E542" t="inlineStr"/>
+      <c r="F542" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g14</t>
+        </is>
+      </c>
+    </row>
+    <row r="543">
+      <c r="A543" t="inlineStr">
+        <is>
+          <t>2026-08-08T14:02:13</t>
+        </is>
+      </c>
+      <c r="B543" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C543" t="inlineStr">
+        <is>
+          <t>CountRejectedTotal</t>
+        </is>
+      </c>
+      <c r="D543" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E543" t="inlineStr"/>
+      <c r="F543" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g16</t>
+        </is>
+      </c>
+    </row>
+    <row r="544">
+      <c r="A544" t="inlineStr">
+        <is>
+          <t>2026-08-08T14:02:13</t>
+        </is>
+      </c>
+      <c r="B544" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C544" t="inlineStr">
+        <is>
+          <t>RejectPartsCount</t>
+        </is>
+      </c>
+      <c r="D544" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E544" t="inlineStr"/>
+      <c r="F544" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g20</t>
+        </is>
+      </c>
+    </row>
+    <row r="545">
+      <c r="A545" t="inlineStr">
+        <is>
+          <t>2026-08-08T14:02:13</t>
+        </is>
+      </c>
+      <c r="B545" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C545" t="inlineStr">
+        <is>
+          <t>tk_Cycle hrs</t>
+        </is>
+      </c>
+      <c r="D545" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E545" t="inlineStr"/>
+      <c r="F545" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g21</t>
+        </is>
+      </c>
+    </row>
+    <row r="546">
+      <c r="A546" t="inlineStr">
+        <is>
+          <t>2026-08-08T14:02:13</t>
+        </is>
+      </c>
+      <c r="B546" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C546" t="inlineStr">
+        <is>
+          <t>tk_Warmup</t>
+        </is>
+      </c>
+      <c r="D546" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E546" t="inlineStr"/>
+      <c r="F546" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g26</t>
+        </is>
+      </c>
+    </row>
+    <row r="547">
+      <c r="A547" t="inlineStr">
+        <is>
+          <t>2026-08-08T14:02:13</t>
+        </is>
+      </c>
+      <c r="B547" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C547" t="inlineStr">
+        <is>
+          <t>FindingParts min</t>
+        </is>
+      </c>
+      <c r="D547" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E547" t="inlineStr"/>
+      <c r="F547" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g27</t>
+        </is>
+      </c>
+    </row>
+    <row r="548">
+      <c r="A548" t="inlineStr">
+        <is>
+          <t>2026-08-08T14:02:13</t>
+        </is>
+      </c>
+      <c r="B548" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C548" t="inlineStr">
+        <is>
+          <t>PickingParts min</t>
+        </is>
+      </c>
+      <c r="D548" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E548" t="inlineStr"/>
+      <c r="F548" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g28</t>
+        </is>
+      </c>
+    </row>
+    <row r="549">
+      <c r="A549" t="inlineStr">
+        <is>
+          <t>2026-08-08T14:02:13</t>
+        </is>
+      </c>
+      <c r="B549" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C549" t="inlineStr">
+        <is>
+          <t>PlacingParts min</t>
+        </is>
+      </c>
+      <c r="D549" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E549" t="inlineStr"/>
+      <c r="F549" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g29</t>
+        </is>
+      </c>
+    </row>
+    <row r="550">
+      <c r="A550" t="inlineStr">
+        <is>
+          <t>2026-08-08T14:02:13</t>
+        </is>
+      </c>
+      <c r="B550" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C550" t="inlineStr">
+        <is>
+          <t>CountPickedReject14in</t>
+        </is>
+      </c>
+      <c r="D550" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E550" t="inlineStr"/>
+      <c r="F550" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g30</t>
+        </is>
+      </c>
+    </row>
+    <row r="551">
+      <c r="A551" t="inlineStr">
+        <is>
+          <t>2026-08-08T14:02:13</t>
+        </is>
+      </c>
+      <c r="B551" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C551" t="inlineStr">
+        <is>
+          <t>temp_dsi</t>
+        </is>
+      </c>
+      <c r="D551" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E551" t="inlineStr"/>
+      <c r="F551" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g31</t>
+        </is>
+      </c>
+    </row>
+    <row r="552">
+      <c r="A552" t="inlineStr">
+        <is>
+          <t>2026-08-08T14:02:13</t>
+        </is>
+      </c>
+      <c r="B552" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C552" t="inlineStr">
+        <is>
+          <t>temp_J1motor</t>
+        </is>
+      </c>
+      <c r="D552" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E552" t="inlineStr"/>
+      <c r="F552" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g32</t>
+        </is>
+      </c>
+    </row>
+    <row r="553">
+      <c r="A553" t="inlineStr">
+        <is>
+          <t>2026-08-08T14:02:13</t>
+        </is>
+      </c>
+      <c r="B553" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C553" t="inlineStr">
+        <is>
+          <t>temp_J4motor</t>
+        </is>
+      </c>
+      <c r="D553" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E553" t="inlineStr"/>
+      <c r="F553" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g35</t>
+        </is>
+      </c>
+    </row>
+    <row r="554">
+      <c r="A554" t="inlineStr">
+        <is>
+          <t>2026-08-08T14:02:13</t>
+        </is>
+      </c>
+      <c r="B554" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C554" t="inlineStr">
+        <is>
+          <t>temp_J6motor</t>
+        </is>
+      </c>
+      <c r="D554" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E554" t="inlineStr"/>
+      <c r="F554" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g37</t>
+        </is>
+      </c>
+    </row>
+    <row r="555">
+      <c r="A555" t="inlineStr">
+        <is>
+          <t>2026-08-08T14:02:13</t>
+        </is>
+      </c>
+      <c r="B555" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C555" t="inlineStr">
+        <is>
+          <t>CountPickedRejectOTM</t>
+        </is>
+      </c>
+      <c r="D555" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E555" t="inlineStr"/>
+      <c r="F555" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g38</t>
+        </is>
+      </c>
+    </row>
+    <row r="556">
+      <c r="A556" t="inlineStr">
+        <is>
+          <t>2026-08-08T14:02:13</t>
+        </is>
+      </c>
+      <c r="B556" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C556" t="inlineStr">
+        <is>
+          <t>CountPickedRejectPandral</t>
+        </is>
+      </c>
+      <c r="D556" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E556" t="inlineStr"/>
+      <c r="F556" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g39</t>
+        </is>
+      </c>
+    </row>
+    <row r="557">
+      <c r="A557" t="inlineStr">
+        <is>
+          <t>2026-08-08T14:03:00</t>
+        </is>
+      </c>
+      <c r="B557" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C557" t="inlineStr">
+        <is>
+          <t>_1st_SCAN</t>
+        </is>
+      </c>
+      <c r="D557" t="b">
+        <v>0</v>
+      </c>
+      <c r="E557" t="n">
+        <v>11</v>
+      </c>
+      <c r="F557" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="558">
+      <c r="A558" t="inlineStr">
+        <is>
+          <t>2026-08-08T14:03:00</t>
+        </is>
+      </c>
+      <c r="B558" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C558" t="inlineStr">
+        <is>
+          <t>TieDetectOffset_B</t>
+        </is>
+      </c>
+      <c r="D558" t="b">
+        <v>0</v>
+      </c>
+      <c r="E558" t="n">
+        <v>11</v>
+      </c>
+      <c r="F558" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="559">
+      <c r="A559" t="inlineStr">
+        <is>
+          <t>2026-08-08T14:03:00</t>
+        </is>
+      </c>
+      <c r="B559" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C559" t="inlineStr">
+        <is>
+          <t>Tie Detector</t>
+        </is>
+      </c>
+      <c r="D559" t="b">
+        <v>0</v>
+      </c>
+      <c r="E559" t="n">
+        <v>11</v>
+      </c>
+      <c r="F559" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="560">
+      <c r="A560" t="inlineStr">
+        <is>
+          <t>2026-08-08T14:03:00</t>
+        </is>
+      </c>
+      <c r="B560" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C560" t="inlineStr">
+        <is>
+          <t>TPS Full</t>
+        </is>
+      </c>
+      <c r="D560" t="b">
+        <v>0</v>
+      </c>
+      <c r="E560" t="n">
+        <v>11</v>
+      </c>
+      <c r="F560" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="561">
+      <c r="A561" t="inlineStr">
+        <is>
+          <t>2026-08-08T14:03:00</t>
+        </is>
+      </c>
+      <c r="B561" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C561" t="inlineStr">
+        <is>
+          <t>TieDetectOffset_A</t>
+        </is>
+      </c>
+      <c r="D561" t="b">
+        <v>0</v>
+      </c>
+      <c r="E561" t="n">
+        <v>11</v>
+      </c>
+      <c r="F561" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="562">
+      <c r="A562" t="inlineStr">
+        <is>
+          <t>2026-08-08T14:03:00</t>
+        </is>
+      </c>
+      <c r="B562" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C562" t="inlineStr">
+        <is>
+          <t>TPS Connected</t>
+        </is>
+      </c>
+      <c r="D562" t="b">
+        <v>0</v>
+      </c>
+      <c r="E562" t="n">
+        <v>11</v>
+      </c>
+      <c r="F562" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="563">
+      <c r="A563" t="inlineStr">
+        <is>
+          <t>2026-08-08T14:03:00</t>
+        </is>
+      </c>
+      <c r="B563" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C563" t="inlineStr">
+        <is>
+          <t>TPS_Enable_ Button</t>
+        </is>
+      </c>
+      <c r="D563" t="b">
+        <v>0</v>
+      </c>
+      <c r="E563" t="n">
+        <v>11</v>
+      </c>
+      <c r="F563" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="564">
+      <c r="A564" t="inlineStr">
+        <is>
+          <t>2026-08-08T14:03:00</t>
+        </is>
+      </c>
+      <c r="B564" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C564" t="inlineStr">
+        <is>
+          <t>AirEagle Eject Plate</t>
+        </is>
+      </c>
+      <c r="D564" t="b">
+        <v>0</v>
+      </c>
+      <c r="E564" t="n">
+        <v>11</v>
+      </c>
+      <c r="F564" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="565">
+      <c r="A565" t="inlineStr">
+        <is>
+          <t>2026-08-08T14:03:00</t>
+        </is>
+      </c>
+      <c r="B565" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C565" t="inlineStr">
+        <is>
+          <t>tk_Cycle</t>
+        </is>
+      </c>
+      <c r="D565" t="b">
+        <v>0</v>
+      </c>
+      <c r="E565" t="n">
+        <v>11</v>
+      </c>
+      <c r="F565" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="566">
+      <c r="A566" t="inlineStr">
+        <is>
+          <t>2026-08-08T14:03:00</t>
+        </is>
+      </c>
+      <c r="B566" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C566" t="inlineStr">
+        <is>
+          <t>Servos_Enabled</t>
+        </is>
+      </c>
+      <c r="D566" t="b">
+        <v>0</v>
+      </c>
+      <c r="E566" t="n">
+        <v>11</v>
+      </c>
+      <c r="F566" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="567">
+      <c r="A567" t="inlineStr">
+        <is>
+          <t>2026-08-08T14:03:00</t>
+        </is>
+      </c>
+      <c r="B567" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C567" t="inlineStr">
+        <is>
+          <t>TPS Enabled</t>
+        </is>
+      </c>
+      <c r="D567" t="b">
+        <v>0</v>
+      </c>
+      <c r="E567" t="n">
+        <v>11</v>
+      </c>
+      <c r="F567" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="568">
+      <c r="A568" t="inlineStr">
+        <is>
+          <t>2026-08-08T14:03:00</t>
+        </is>
+      </c>
+      <c r="B568" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C568" t="inlineStr">
+        <is>
+          <t>tk_Abort</t>
+        </is>
+      </c>
+      <c r="D568" t="b">
+        <v>0</v>
+      </c>
+      <c r="E568" t="n">
+        <v>11</v>
+      </c>
+      <c r="F568" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="569">
+      <c r="A569" t="inlineStr">
+        <is>
+          <t>2026-08-08T14:03:00</t>
+        </is>
+      </c>
+      <c r="B569" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C569" t="inlineStr">
+        <is>
+          <t>Robot_isMoving</t>
+        </is>
+      </c>
+      <c r="D569" t="b">
+        <v>0</v>
+      </c>
+      <c r="E569" t="n">
+        <v>11</v>
+      </c>
+      <c r="F569" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="570">
+      <c r="A570" t="inlineStr">
+        <is>
+          <t>2026-08-08T14:03:00</t>
+        </is>
+      </c>
+      <c r="B570" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C570" t="inlineStr">
+        <is>
+          <t>Eject Tie Plate</t>
+        </is>
+      </c>
+      <c r="D570" t="b">
+        <v>0</v>
+      </c>
+      <c r="E570" t="n">
+        <v>11</v>
+      </c>
+      <c r="F570" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="571">
+      <c r="A571" t="inlineStr">
+        <is>
+          <t>2026-08-08T14:03:00</t>
+        </is>
+      </c>
+      <c r="B571" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C571" t="inlineStr">
+        <is>
+          <t>TPS BACKUP ALARM</t>
+        </is>
+      </c>
+      <c r="D571" t="b">
+        <v>0</v>
+      </c>
+      <c r="E571" t="n">
+        <v>11</v>
+      </c>
+      <c r="F571" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="572">
+      <c r="A572" t="inlineStr">
+        <is>
+          <t>2026-08-08T14:03:00</t>
+        </is>
+      </c>
+      <c r="B572" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C572" t="inlineStr">
+        <is>
+          <t>14in Job</t>
+        </is>
+      </c>
+      <c r="D572" t="b">
+        <v>1</v>
+      </c>
+      <c r="E572" t="n">
+        <v>11</v>
+      </c>
+      <c r="F572" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="573">
+      <c r="A573" t="inlineStr">
+        <is>
+          <t>2026-08-08T14:03:00</t>
+        </is>
+      </c>
+      <c r="B573" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C573" t="inlineStr">
+        <is>
+          <t>18in Job</t>
+        </is>
+      </c>
+      <c r="D573" t="b">
+        <v>0</v>
+      </c>
+      <c r="E573" t="n">
+        <v>11</v>
+      </c>
+      <c r="F573" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="574">
+      <c r="A574" t="inlineStr">
+        <is>
+          <t>2026-08-08T14:03:00</t>
+        </is>
+      </c>
+      <c r="B574" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C574" t="inlineStr">
+        <is>
+          <t>Pandral Job</t>
+        </is>
+      </c>
+      <c r="D574" t="b">
+        <v>0</v>
+      </c>
+      <c r="E574" t="n">
+        <v>11</v>
+      </c>
+      <c r="F574" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="575">
+      <c r="A575" t="inlineStr">
+        <is>
+          <t>2026-08-08T14:03:00</t>
+        </is>
+      </c>
+      <c r="B575" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C575" t="inlineStr">
+        <is>
+          <t>DoubleLay Job</t>
+        </is>
+      </c>
+      <c r="D575" t="b">
+        <v>0</v>
+      </c>
+      <c r="E575" t="n">
+        <v>11</v>
+      </c>
+      <c r="F575" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="576">
+      <c r="A576" t="inlineStr">
+        <is>
+          <t>2026-08-08T14:03:00</t>
+        </is>
+      </c>
+      <c r="B576" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C576" t="inlineStr">
+        <is>
+          <t>TPSjam_FLAG</t>
+        </is>
+      </c>
+      <c r="D576" t="b">
+        <v>0</v>
+      </c>
+      <c r="E576" t="n">
+        <v>11</v>
+      </c>
+      <c r="F576" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="577">
+      <c r="A577" t="inlineStr">
+        <is>
+          <t>2026-08-08T14:03:00</t>
+        </is>
+      </c>
+      <c r="B577" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C577" t="inlineStr">
+        <is>
+          <t>RoCalRequest</t>
+        </is>
+      </c>
+      <c r="D577" t="b">
+        <v>0</v>
+      </c>
+      <c r="E577" t="n">
+        <v>11</v>
+      </c>
+      <c r="F577" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="578">
+      <c r="A578" t="inlineStr">
+        <is>
+          <t>2026-08-08T14:03:00</t>
+        </is>
+      </c>
+      <c r="B578" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C578" t="inlineStr">
+        <is>
+          <t>tkCycle_TotalSeconds</t>
+        </is>
+      </c>
+      <c r="D578" t="n">
+        <v>0</v>
+      </c>
+      <c r="E578" t="n">
+        <v>9</v>
+      </c>
+      <c r="F578" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="579">
+      <c r="A579" t="inlineStr">
+        <is>
+          <t>2026-08-08T14:03:00</t>
+        </is>
+      </c>
+      <c r="B579" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C579" t="inlineStr">
+        <is>
+          <t>tkCycle_NoMoveSec</t>
+        </is>
+      </c>
+      <c r="D579" t="n">
+        <v>0</v>
+      </c>
+      <c r="E579" t="n">
+        <v>9</v>
+      </c>
+      <c r="F579" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="580">
+      <c r="A580" t="inlineStr">
+        <is>
+          <t>2026-08-08T14:03:00</t>
+        </is>
+      </c>
+      <c r="B580" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C580" t="inlineStr">
+        <is>
+          <t>tkCycle_MoveSeconds</t>
+        </is>
+      </c>
+      <c r="D580" t="n">
+        <v>0</v>
+      </c>
+      <c r="E580" t="n">
+        <v>9</v>
+      </c>
+      <c r="F580" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="581">
+      <c r="A581" t="inlineStr">
+        <is>
+          <t>2026-08-08T14:03:00</t>
+        </is>
+      </c>
+      <c r="B581" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C581" t="inlineStr">
+        <is>
+          <t>Percent time moveing</t>
+        </is>
+      </c>
+      <c r="D581" t="n">
+        <v>0</v>
+      </c>
+      <c r="E581" t="n">
+        <v>9</v>
+      </c>
+      <c r="F581" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="582">
+      <c r="A582" t="inlineStr">
+        <is>
+          <t>2026-08-08T14:03:00</t>
+        </is>
+      </c>
+      <c r="B582" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C582" t="inlineStr">
+        <is>
+          <t>Percent time not moving</t>
+        </is>
+      </c>
+      <c r="D582" t="n">
+        <v>0</v>
+      </c>
+      <c r="E582" t="n">
+        <v>9</v>
+      </c>
+      <c r="F582" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="583">
+      <c r="A583" t="inlineStr">
+        <is>
+          <t>2026-08-08T14:03:00</t>
+        </is>
+      </c>
+      <c r="B583" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C583" t="inlineStr">
+        <is>
+          <t>TotalPickPartsCount</t>
+        </is>
+      </c>
+      <c r="D583" t="n">
+        <v>0</v>
+      </c>
+      <c r="E583" t="n">
+        <v>9</v>
+      </c>
+      <c r="F583" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="584">
+      <c r="A584" t="inlineStr">
+        <is>
+          <t>2026-08-08T14:03:00</t>
+        </is>
+      </c>
+      <c r="B584" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C584" t="inlineStr">
+        <is>
+          <t>RejectPartsCount</t>
+        </is>
+      </c>
+      <c r="D584" t="n">
+        <v>0</v>
+      </c>
+      <c r="E584" t="n">
+        <v>9</v>
+      </c>
+      <c r="F584" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="585">
+      <c r="A585" t="inlineStr">
+        <is>
+          <t>2026-08-08T14:03:00</t>
+        </is>
+      </c>
+      <c r="B585" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C585" t="inlineStr">
+        <is>
+          <t>AcceptsPartsCount</t>
+        </is>
+      </c>
+      <c r="D585" t="n">
+        <v>0</v>
+      </c>
+      <c r="E585" t="n">
+        <v>9</v>
+      </c>
+      <c r="F585" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="586">
+      <c r="A586" t="inlineStr">
+        <is>
+          <t>2026-08-08T14:03:00</t>
+        </is>
+      </c>
+      <c r="B586" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C586" t="inlineStr">
+        <is>
+          <t>percentCount_accept</t>
+        </is>
+      </c>
+      <c r="D586" t="n">
+        <v>0</v>
+      </c>
+      <c r="E586" t="n">
+        <v>9</v>
+      </c>
+      <c r="F586" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="587">
+      <c r="A587" t="inlineStr">
+        <is>
+          <t>2026-08-08T14:03:00</t>
+        </is>
+      </c>
+      <c r="B587" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C587" t="inlineStr">
+        <is>
+          <t>percentCount_reject</t>
+        </is>
+      </c>
+      <c r="D587" t="n">
+        <v>0</v>
+      </c>
+      <c r="E587" t="n">
+        <v>9</v>
+      </c>
+      <c r="F587" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="588">
+      <c r="A588" t="inlineStr">
+        <is>
+          <t>2026-08-08T14:03:00</t>
+        </is>
+      </c>
+      <c r="B588" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C588" t="inlineStr">
+        <is>
+          <t>Avg Parts per min_total</t>
+        </is>
+      </c>
+      <c r="D588" t="n">
+        <v>0</v>
+      </c>
+      <c r="E588" t="n">
+        <v>9</v>
+      </c>
+      <c r="F588" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="589">
+      <c r="A589" t="inlineStr">
+        <is>
+          <t>2026-08-08T14:03:00</t>
+        </is>
+      </c>
+      <c r="B589" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C589" t="inlineStr">
+        <is>
+          <t>TotalPickedParts</t>
+        </is>
+      </c>
+      <c r="D589" t="n">
+        <v>0</v>
+      </c>
+      <c r="E589" t="n">
+        <v>3</v>
+      </c>
+      <c r="F589" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="590">
+      <c r="A590" t="inlineStr">
+        <is>
+          <t>2026-08-08T14:03:00</t>
+        </is>
+      </c>
+      <c r="B590" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C590" t="inlineStr">
+        <is>
+          <t>TotalPickedAcceptParts</t>
+        </is>
+      </c>
+      <c r="D590" t="n">
+        <v>0</v>
+      </c>
+      <c r="E590" t="n">
+        <v>3</v>
+      </c>
+      <c r="F590" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="591">
+      <c r="A591" t="inlineStr">
+        <is>
+          <t>2026-08-08T14:03:00</t>
+        </is>
+      </c>
+      <c r="B591" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C591" t="inlineStr">
+        <is>
+          <t>TotalPickedRejectParts</t>
+        </is>
+      </c>
+      <c r="D591" t="n">
+        <v>0</v>
+      </c>
+      <c r="E591" t="n">
+        <v>3</v>
+      </c>
+      <c r="F591" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="592">
+      <c r="A592" t="inlineStr">
+        <is>
+          <t>2026-08-08T14:03:00</t>
+        </is>
+      </c>
+      <c r="B592" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C592" t="inlineStr">
+        <is>
+          <t>TotalTiePlatesLaid</t>
+        </is>
+      </c>
+      <c r="D592" t="n">
+        <v>0</v>
+      </c>
+      <c r="E592" t="n">
+        <v>3</v>
+      </c>
+      <c r="F592" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="593">
+      <c r="A593" t="inlineStr">
+        <is>
+          <t>2026-08-08T14:03:00</t>
+        </is>
+      </c>
+      <c r="B593" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C593" t="inlineStr">
+        <is>
+          <t>Daily_TotalLaidPlates</t>
+        </is>
+      </c>
+      <c r="D593" t="n">
+        <v>0</v>
+      </c>
+      <c r="E593" t="n">
+        <v>3</v>
+      </c>
+      <c r="F593" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="594">
+      <c r="A594" t="inlineStr">
+        <is>
+          <t>2026-08-08T14:03:00</t>
+        </is>
+      </c>
+      <c r="B594" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C594" t="inlineStr">
+        <is>
+          <t>CountPicked14in</t>
+        </is>
+      </c>
+      <c r="D594" t="n">
+        <v>0</v>
+      </c>
+      <c r="E594" t="n">
+        <v>3</v>
+      </c>
+      <c r="F594" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="595">
+      <c r="A595" t="inlineStr">
+        <is>
+          <t>2026-08-08T14:03:00</t>
+        </is>
+      </c>
+      <c r="B595" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C595" t="inlineStr">
+        <is>
+          <t>CountPicked18in</t>
+        </is>
+      </c>
+      <c r="D595" t="n">
+        <v>0</v>
+      </c>
+      <c r="E595" t="n">
+        <v>3</v>
+      </c>
+      <c r="F595" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="596">
+      <c r="A596" t="inlineStr">
+        <is>
+          <t>2026-08-08T14:03:00</t>
+        </is>
+      </c>
+      <c r="B596" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C596" t="inlineStr">
+        <is>
+          <t>CountPickedPandral</t>
+        </is>
+      </c>
+      <c r="D596" t="n">
+        <v>0</v>
+      </c>
+      <c r="E596" t="n">
+        <v>3</v>
+      </c>
+      <c r="F596" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="597">
+      <c r="A597" t="inlineStr">
+        <is>
+          <t>2026-08-08T14:03:00</t>
+        </is>
+      </c>
+      <c r="B597" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C597" t="inlineStr">
+        <is>
+          <t>CountPickedOTM</t>
+        </is>
+      </c>
+      <c r="D597" t="n">
+        <v>0</v>
+      </c>
+      <c r="E597" t="n">
+        <v>3</v>
+      </c>
+      <c r="F597" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="598">
+      <c r="A598" t="inlineStr">
+        <is>
+          <t>2026-08-08T14:03:00</t>
+        </is>
+      </c>
+      <c r="B598" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C598" t="inlineStr">
+        <is>
+          <t>RoCals</t>
+        </is>
+      </c>
+      <c r="D598" t="n">
+        <v>0</v>
+      </c>
+      <c r="E598" t="n">
+        <v>3</v>
+      </c>
+      <c r="F598" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="599">
+      <c r="A599" t="inlineStr">
+        <is>
+          <t>2026-08-08T14:03:00</t>
+        </is>
+      </c>
+      <c r="B599" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C599" t="inlineStr">
+        <is>
+          <t>TPS_JamsUsr</t>
+        </is>
+      </c>
+      <c r="D599" t="n">
+        <v>0</v>
+      </c>
+      <c r="E599" t="n">
+        <v>3</v>
+      </c>
+      <c r="F599" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="600">
+      <c r="A600" t="inlineStr">
+        <is>
+          <t>2026-08-08T14:03:00</t>
+        </is>
+      </c>
+      <c r="B600" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C600" t="inlineStr">
+        <is>
+          <t>TPS_JamsMASTER</t>
+        </is>
+      </c>
+      <c r="D600" t="n">
+        <v>0</v>
+      </c>
+      <c r="E600" t="n">
+        <v>3</v>
+      </c>
+      <c r="F600" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="601">
+      <c r="A601" t="inlineStr">
+        <is>
+          <t>2026-08-08T14:03:00</t>
+        </is>
+      </c>
+      <c r="B601" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C601" t="inlineStr">
+        <is>
+          <t>ABORT_Master</t>
+        </is>
+      </c>
+      <c r="D601" t="n">
+        <v>0</v>
+      </c>
+      <c r="E601" t="n">
+        <v>3</v>
+      </c>
+      <c r="F601" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/plc</t>
         </is>

</xml_diff>

<commit_message>
Log MQTT data 2026-08-08 15:16 UTC
</commit_message>
<xml_diff>
--- a/logs/raiv_tracker_2026-08-08.xlsx
+++ b/logs/raiv_tracker_2026-08-08.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F601"/>
+  <dimension ref="A1:F686"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -14689,7 +14689,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E517" t="inlineStr"/>
       <c r="F517" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g1</t>
@@ -14717,7 +14716,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E518" t="inlineStr"/>
       <c r="F518" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g2</t>
@@ -14745,7 +14743,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E519" t="inlineStr"/>
       <c r="F519" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g3</t>
@@ -14773,7 +14770,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E520" t="inlineStr"/>
       <c r="F520" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g4</t>
@@ -14801,7 +14797,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E521" t="inlineStr"/>
       <c r="F521" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g5</t>
@@ -14829,7 +14824,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E522" t="inlineStr"/>
       <c r="F522" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g6</t>
@@ -14857,7 +14851,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E523" t="inlineStr"/>
       <c r="F523" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g7</t>
@@ -14885,7 +14878,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E524" t="inlineStr"/>
       <c r="F524" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g8</t>
@@ -14913,7 +14905,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E525" t="inlineStr"/>
       <c r="F525" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g13</t>
@@ -14941,7 +14932,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E526" t="inlineStr"/>
       <c r="F526" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g15</t>
@@ -14969,7 +14959,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E527" t="inlineStr"/>
       <c r="F527" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g17</t>
@@ -14997,7 +14986,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E528" t="inlineStr"/>
       <c r="F528" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g18</t>
@@ -15025,7 +15013,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E529" t="inlineStr"/>
       <c r="F529" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g19</t>
@@ -15053,7 +15040,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E530" t="inlineStr"/>
       <c r="F530" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g22</t>
@@ -15081,7 +15067,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E531" t="inlineStr"/>
       <c r="F531" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g23</t>
@@ -15109,7 +15094,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E532" t="inlineStr"/>
       <c r="F532" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g24</t>
@@ -15137,7 +15121,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E533" t="inlineStr"/>
       <c r="F533" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g25</t>
@@ -15165,7 +15148,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E534" t="inlineStr"/>
       <c r="F534" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g33</t>
@@ -15193,7 +15175,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E535" t="inlineStr"/>
       <c r="F535" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g34</t>
@@ -15221,7 +15202,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E536" t="inlineStr"/>
       <c r="F536" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g36</t>
@@ -15249,7 +15229,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E537" t="inlineStr"/>
       <c r="F537" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g40</t>
@@ -15277,7 +15256,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E538" t="inlineStr"/>
       <c r="F538" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g9</t>
@@ -15305,7 +15283,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E539" t="inlineStr"/>
       <c r="F539" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g10</t>
@@ -15333,7 +15310,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E540" t="inlineStr"/>
       <c r="F540" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g11</t>
@@ -15361,7 +15337,6 @@
           <t>1</t>
         </is>
       </c>
-      <c r="E541" t="inlineStr"/>
       <c r="F541" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g12</t>
@@ -15389,7 +15364,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E542" t="inlineStr"/>
       <c r="F542" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g14</t>
@@ -15417,7 +15391,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E543" t="inlineStr"/>
       <c r="F543" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g16</t>
@@ -15445,7 +15418,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E544" t="inlineStr"/>
       <c r="F544" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g20</t>
@@ -15473,7 +15445,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E545" t="inlineStr"/>
       <c r="F545" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g21</t>
@@ -15501,7 +15472,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E546" t="inlineStr"/>
       <c r="F546" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g26</t>
@@ -15529,7 +15499,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E547" t="inlineStr"/>
       <c r="F547" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g27</t>
@@ -15557,7 +15526,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E548" t="inlineStr"/>
       <c r="F548" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g28</t>
@@ -15585,7 +15553,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E549" t="inlineStr"/>
       <c r="F549" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g29</t>
@@ -15613,7 +15580,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E550" t="inlineStr"/>
       <c r="F550" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g30</t>
@@ -15641,7 +15607,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E551" t="inlineStr"/>
       <c r="F551" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g31</t>
@@ -15669,7 +15634,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E552" t="inlineStr"/>
       <c r="F552" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g32</t>
@@ -15697,7 +15661,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E553" t="inlineStr"/>
       <c r="F553" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g35</t>
@@ -15725,7 +15688,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E554" t="inlineStr"/>
       <c r="F554" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g37</t>
@@ -15753,7 +15715,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E555" t="inlineStr"/>
       <c r="F555" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g38</t>
@@ -15781,7 +15742,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E556" t="inlineStr"/>
       <c r="F556" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g39</t>
@@ -17045,6 +17005,2386 @@
       <c r="F601" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="602">
+      <c r="A602" t="inlineStr">
+        <is>
+          <t>2026-08-08T15:16:00</t>
+        </is>
+      </c>
+      <c r="B602" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C602" t="inlineStr">
+        <is>
+          <t>_1st_SCAN</t>
+        </is>
+      </c>
+      <c r="D602" t="b">
+        <v>0</v>
+      </c>
+      <c r="E602" t="n">
+        <v>11</v>
+      </c>
+      <c r="F602" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="603">
+      <c r="A603" t="inlineStr">
+        <is>
+          <t>2026-08-08T15:16:00</t>
+        </is>
+      </c>
+      <c r="B603" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C603" t="inlineStr">
+        <is>
+          <t>TieDetectOffset_B</t>
+        </is>
+      </c>
+      <c r="D603" t="b">
+        <v>0</v>
+      </c>
+      <c r="E603" t="n">
+        <v>11</v>
+      </c>
+      <c r="F603" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="604">
+      <c r="A604" t="inlineStr">
+        <is>
+          <t>2026-08-08T15:16:00</t>
+        </is>
+      </c>
+      <c r="B604" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C604" t="inlineStr">
+        <is>
+          <t>Tie Detector</t>
+        </is>
+      </c>
+      <c r="D604" t="b">
+        <v>0</v>
+      </c>
+      <c r="E604" t="n">
+        <v>11</v>
+      </c>
+      <c r="F604" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="605">
+      <c r="A605" t="inlineStr">
+        <is>
+          <t>2026-08-08T15:16:00</t>
+        </is>
+      </c>
+      <c r="B605" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C605" t="inlineStr">
+        <is>
+          <t>TPS Full</t>
+        </is>
+      </c>
+      <c r="D605" t="b">
+        <v>0</v>
+      </c>
+      <c r="E605" t="n">
+        <v>11</v>
+      </c>
+      <c r="F605" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="606">
+      <c r="A606" t="inlineStr">
+        <is>
+          <t>2026-08-08T15:16:00</t>
+        </is>
+      </c>
+      <c r="B606" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C606" t="inlineStr">
+        <is>
+          <t>TieDetectOffset_A</t>
+        </is>
+      </c>
+      <c r="D606" t="b">
+        <v>0</v>
+      </c>
+      <c r="E606" t="n">
+        <v>11</v>
+      </c>
+      <c r="F606" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="607">
+      <c r="A607" t="inlineStr">
+        <is>
+          <t>2026-08-08T15:16:00</t>
+        </is>
+      </c>
+      <c r="B607" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C607" t="inlineStr">
+        <is>
+          <t>TPS Connected</t>
+        </is>
+      </c>
+      <c r="D607" t="b">
+        <v>0</v>
+      </c>
+      <c r="E607" t="n">
+        <v>11</v>
+      </c>
+      <c r="F607" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="608">
+      <c r="A608" t="inlineStr">
+        <is>
+          <t>2026-08-08T15:16:00</t>
+        </is>
+      </c>
+      <c r="B608" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C608" t="inlineStr">
+        <is>
+          <t>TPS_Enable_ Button</t>
+        </is>
+      </c>
+      <c r="D608" t="b">
+        <v>0</v>
+      </c>
+      <c r="E608" t="n">
+        <v>11</v>
+      </c>
+      <c r="F608" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="609">
+      <c r="A609" t="inlineStr">
+        <is>
+          <t>2026-08-08T15:16:00</t>
+        </is>
+      </c>
+      <c r="B609" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C609" t="inlineStr">
+        <is>
+          <t>AirEagle Eject Plate</t>
+        </is>
+      </c>
+      <c r="D609" t="b">
+        <v>0</v>
+      </c>
+      <c r="E609" t="n">
+        <v>11</v>
+      </c>
+      <c r="F609" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="610">
+      <c r="A610" t="inlineStr">
+        <is>
+          <t>2026-08-08T15:16:00</t>
+        </is>
+      </c>
+      <c r="B610" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C610" t="inlineStr">
+        <is>
+          <t>tk_Cycle</t>
+        </is>
+      </c>
+      <c r="D610" t="b">
+        <v>0</v>
+      </c>
+      <c r="E610" t="n">
+        <v>11</v>
+      </c>
+      <c r="F610" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="611">
+      <c r="A611" t="inlineStr">
+        <is>
+          <t>2026-08-08T15:16:00</t>
+        </is>
+      </c>
+      <c r="B611" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C611" t="inlineStr">
+        <is>
+          <t>Servos_Enabled</t>
+        </is>
+      </c>
+      <c r="D611" t="b">
+        <v>0</v>
+      </c>
+      <c r="E611" t="n">
+        <v>11</v>
+      </c>
+      <c r="F611" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="612">
+      <c r="A612" t="inlineStr">
+        <is>
+          <t>2026-08-08T15:16:00</t>
+        </is>
+      </c>
+      <c r="B612" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C612" t="inlineStr">
+        <is>
+          <t>TPS Enabled</t>
+        </is>
+      </c>
+      <c r="D612" t="b">
+        <v>0</v>
+      </c>
+      <c r="E612" t="n">
+        <v>11</v>
+      </c>
+      <c r="F612" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="613">
+      <c r="A613" t="inlineStr">
+        <is>
+          <t>2026-08-08T15:16:00</t>
+        </is>
+      </c>
+      <c r="B613" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C613" t="inlineStr">
+        <is>
+          <t>tk_Abort</t>
+        </is>
+      </c>
+      <c r="D613" t="b">
+        <v>0</v>
+      </c>
+      <c r="E613" t="n">
+        <v>11</v>
+      </c>
+      <c r="F613" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="614">
+      <c r="A614" t="inlineStr">
+        <is>
+          <t>2026-08-08T15:16:00</t>
+        </is>
+      </c>
+      <c r="B614" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C614" t="inlineStr">
+        <is>
+          <t>Robot_isMoving</t>
+        </is>
+      </c>
+      <c r="D614" t="b">
+        <v>0</v>
+      </c>
+      <c r="E614" t="n">
+        <v>11</v>
+      </c>
+      <c r="F614" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="615">
+      <c r="A615" t="inlineStr">
+        <is>
+          <t>2026-08-08T15:16:00</t>
+        </is>
+      </c>
+      <c r="B615" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C615" t="inlineStr">
+        <is>
+          <t>Eject Tie Plate</t>
+        </is>
+      </c>
+      <c r="D615" t="b">
+        <v>0</v>
+      </c>
+      <c r="E615" t="n">
+        <v>11</v>
+      </c>
+      <c r="F615" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="616">
+      <c r="A616" t="inlineStr">
+        <is>
+          <t>2026-08-08T15:16:00</t>
+        </is>
+      </c>
+      <c r="B616" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C616" t="inlineStr">
+        <is>
+          <t>TPS BACKUP ALARM</t>
+        </is>
+      </c>
+      <c r="D616" t="b">
+        <v>0</v>
+      </c>
+      <c r="E616" t="n">
+        <v>11</v>
+      </c>
+      <c r="F616" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="617">
+      <c r="A617" t="inlineStr">
+        <is>
+          <t>2026-08-08T15:16:00</t>
+        </is>
+      </c>
+      <c r="B617" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C617" t="inlineStr">
+        <is>
+          <t>14in Job</t>
+        </is>
+      </c>
+      <c r="D617" t="b">
+        <v>1</v>
+      </c>
+      <c r="E617" t="n">
+        <v>11</v>
+      </c>
+      <c r="F617" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="618">
+      <c r="A618" t="inlineStr">
+        <is>
+          <t>2026-08-08T15:16:00</t>
+        </is>
+      </c>
+      <c r="B618" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C618" t="inlineStr">
+        <is>
+          <t>18in Job</t>
+        </is>
+      </c>
+      <c r="D618" t="b">
+        <v>0</v>
+      </c>
+      <c r="E618" t="n">
+        <v>11</v>
+      </c>
+      <c r="F618" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="619">
+      <c r="A619" t="inlineStr">
+        <is>
+          <t>2026-08-08T15:16:00</t>
+        </is>
+      </c>
+      <c r="B619" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C619" t="inlineStr">
+        <is>
+          <t>Pandral Job</t>
+        </is>
+      </c>
+      <c r="D619" t="b">
+        <v>0</v>
+      </c>
+      <c r="E619" t="n">
+        <v>11</v>
+      </c>
+      <c r="F619" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="620">
+      <c r="A620" t="inlineStr">
+        <is>
+          <t>2026-08-08T15:16:00</t>
+        </is>
+      </c>
+      <c r="B620" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C620" t="inlineStr">
+        <is>
+          <t>DoubleLay Job</t>
+        </is>
+      </c>
+      <c r="D620" t="b">
+        <v>0</v>
+      </c>
+      <c r="E620" t="n">
+        <v>11</v>
+      </c>
+      <c r="F620" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="621">
+      <c r="A621" t="inlineStr">
+        <is>
+          <t>2026-08-08T15:16:00</t>
+        </is>
+      </c>
+      <c r="B621" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C621" t="inlineStr">
+        <is>
+          <t>TPSjam_FLAG</t>
+        </is>
+      </c>
+      <c r="D621" t="b">
+        <v>0</v>
+      </c>
+      <c r="E621" t="n">
+        <v>11</v>
+      </c>
+      <c r="F621" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="622">
+      <c r="A622" t="inlineStr">
+        <is>
+          <t>2026-08-08T15:16:00</t>
+        </is>
+      </c>
+      <c r="B622" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C622" t="inlineStr">
+        <is>
+          <t>RoCalRequest</t>
+        </is>
+      </c>
+      <c r="D622" t="b">
+        <v>0</v>
+      </c>
+      <c r="E622" t="n">
+        <v>11</v>
+      </c>
+      <c r="F622" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="623">
+      <c r="A623" t="inlineStr">
+        <is>
+          <t>2026-08-08T15:16:00</t>
+        </is>
+      </c>
+      <c r="B623" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C623" t="inlineStr">
+        <is>
+          <t>tkCycle_TotalSeconds</t>
+        </is>
+      </c>
+      <c r="D623" t="n">
+        <v>0</v>
+      </c>
+      <c r="E623" t="n">
+        <v>9</v>
+      </c>
+      <c r="F623" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="624">
+      <c r="A624" t="inlineStr">
+        <is>
+          <t>2026-08-08T15:16:00</t>
+        </is>
+      </c>
+      <c r="B624" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C624" t="inlineStr">
+        <is>
+          <t>tkCycle_NoMoveSec</t>
+        </is>
+      </c>
+      <c r="D624" t="n">
+        <v>0</v>
+      </c>
+      <c r="E624" t="n">
+        <v>9</v>
+      </c>
+      <c r="F624" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="625">
+      <c r="A625" t="inlineStr">
+        <is>
+          <t>2026-08-08T15:16:00</t>
+        </is>
+      </c>
+      <c r="B625" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C625" t="inlineStr">
+        <is>
+          <t>tkCycle_MoveSeconds</t>
+        </is>
+      </c>
+      <c r="D625" t="n">
+        <v>0</v>
+      </c>
+      <c r="E625" t="n">
+        <v>9</v>
+      </c>
+      <c r="F625" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="626">
+      <c r="A626" t="inlineStr">
+        <is>
+          <t>2026-08-08T15:16:00</t>
+        </is>
+      </c>
+      <c r="B626" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C626" t="inlineStr">
+        <is>
+          <t>Percent time moveing</t>
+        </is>
+      </c>
+      <c r="D626" t="n">
+        <v>0</v>
+      </c>
+      <c r="E626" t="n">
+        <v>9</v>
+      </c>
+      <c r="F626" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="627">
+      <c r="A627" t="inlineStr">
+        <is>
+          <t>2026-08-08T15:16:00</t>
+        </is>
+      </c>
+      <c r="B627" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C627" t="inlineStr">
+        <is>
+          <t>Percent time not moving</t>
+        </is>
+      </c>
+      <c r="D627" t="n">
+        <v>0</v>
+      </c>
+      <c r="E627" t="n">
+        <v>9</v>
+      </c>
+      <c r="F627" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="628">
+      <c r="A628" t="inlineStr">
+        <is>
+          <t>2026-08-08T15:16:00</t>
+        </is>
+      </c>
+      <c r="B628" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C628" t="inlineStr">
+        <is>
+          <t>TotalPickPartsCount</t>
+        </is>
+      </c>
+      <c r="D628" t="n">
+        <v>0</v>
+      </c>
+      <c r="E628" t="n">
+        <v>9</v>
+      </c>
+      <c r="F628" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="629">
+      <c r="A629" t="inlineStr">
+        <is>
+          <t>2026-08-08T15:16:00</t>
+        </is>
+      </c>
+      <c r="B629" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C629" t="inlineStr">
+        <is>
+          <t>RejectPartsCount</t>
+        </is>
+      </c>
+      <c r="D629" t="n">
+        <v>0</v>
+      </c>
+      <c r="E629" t="n">
+        <v>9</v>
+      </c>
+      <c r="F629" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="630">
+      <c r="A630" t="inlineStr">
+        <is>
+          <t>2026-08-08T15:16:00</t>
+        </is>
+      </c>
+      <c r="B630" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C630" t="inlineStr">
+        <is>
+          <t>AcceptsPartsCount</t>
+        </is>
+      </c>
+      <c r="D630" t="n">
+        <v>0</v>
+      </c>
+      <c r="E630" t="n">
+        <v>9</v>
+      </c>
+      <c r="F630" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="631">
+      <c r="A631" t="inlineStr">
+        <is>
+          <t>2026-08-08T15:16:00</t>
+        </is>
+      </c>
+      <c r="B631" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C631" t="inlineStr">
+        <is>
+          <t>percentCount_accept</t>
+        </is>
+      </c>
+      <c r="D631" t="n">
+        <v>0</v>
+      </c>
+      <c r="E631" t="n">
+        <v>9</v>
+      </c>
+      <c r="F631" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="632">
+      <c r="A632" t="inlineStr">
+        <is>
+          <t>2026-08-08T15:16:00</t>
+        </is>
+      </c>
+      <c r="B632" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C632" t="inlineStr">
+        <is>
+          <t>percentCount_reject</t>
+        </is>
+      </c>
+      <c r="D632" t="n">
+        <v>0</v>
+      </c>
+      <c r="E632" t="n">
+        <v>9</v>
+      </c>
+      <c r="F632" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="633">
+      <c r="A633" t="inlineStr">
+        <is>
+          <t>2026-08-08T15:16:00</t>
+        </is>
+      </c>
+      <c r="B633" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C633" t="inlineStr">
+        <is>
+          <t>Avg Parts per min_total</t>
+        </is>
+      </c>
+      <c r="D633" t="n">
+        <v>0</v>
+      </c>
+      <c r="E633" t="n">
+        <v>9</v>
+      </c>
+      <c r="F633" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="634">
+      <c r="A634" t="inlineStr">
+        <is>
+          <t>2026-08-08T15:16:00</t>
+        </is>
+      </c>
+      <c r="B634" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C634" t="inlineStr">
+        <is>
+          <t>TotalPickedParts</t>
+        </is>
+      </c>
+      <c r="D634" t="n">
+        <v>0</v>
+      </c>
+      <c r="E634" t="n">
+        <v>3</v>
+      </c>
+      <c r="F634" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="635">
+      <c r="A635" t="inlineStr">
+        <is>
+          <t>2026-08-08T15:16:00</t>
+        </is>
+      </c>
+      <c r="B635" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C635" t="inlineStr">
+        <is>
+          <t>TotalPickedAcceptParts</t>
+        </is>
+      </c>
+      <c r="D635" t="n">
+        <v>0</v>
+      </c>
+      <c r="E635" t="n">
+        <v>3</v>
+      </c>
+      <c r="F635" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="636">
+      <c r="A636" t="inlineStr">
+        <is>
+          <t>2026-08-08T15:16:00</t>
+        </is>
+      </c>
+      <c r="B636" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C636" t="inlineStr">
+        <is>
+          <t>TotalPickedRejectParts</t>
+        </is>
+      </c>
+      <c r="D636" t="n">
+        <v>0</v>
+      </c>
+      <c r="E636" t="n">
+        <v>3</v>
+      </c>
+      <c r="F636" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="637">
+      <c r="A637" t="inlineStr">
+        <is>
+          <t>2026-08-08T15:16:00</t>
+        </is>
+      </c>
+      <c r="B637" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C637" t="inlineStr">
+        <is>
+          <t>TotalTiePlatesLaid</t>
+        </is>
+      </c>
+      <c r="D637" t="n">
+        <v>0</v>
+      </c>
+      <c r="E637" t="n">
+        <v>3</v>
+      </c>
+      <c r="F637" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="638">
+      <c r="A638" t="inlineStr">
+        <is>
+          <t>2026-08-08T15:16:00</t>
+        </is>
+      </c>
+      <c r="B638" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C638" t="inlineStr">
+        <is>
+          <t>Daily_TotalLaidPlates</t>
+        </is>
+      </c>
+      <c r="D638" t="n">
+        <v>0</v>
+      </c>
+      <c r="E638" t="n">
+        <v>3</v>
+      </c>
+      <c r="F638" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="639">
+      <c r="A639" t="inlineStr">
+        <is>
+          <t>2026-08-08T15:16:00</t>
+        </is>
+      </c>
+      <c r="B639" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C639" t="inlineStr">
+        <is>
+          <t>CountPicked14in</t>
+        </is>
+      </c>
+      <c r="D639" t="n">
+        <v>0</v>
+      </c>
+      <c r="E639" t="n">
+        <v>3</v>
+      </c>
+      <c r="F639" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="640">
+      <c r="A640" t="inlineStr">
+        <is>
+          <t>2026-08-08T15:16:00</t>
+        </is>
+      </c>
+      <c r="B640" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C640" t="inlineStr">
+        <is>
+          <t>CountPicked18in</t>
+        </is>
+      </c>
+      <c r="D640" t="n">
+        <v>0</v>
+      </c>
+      <c r="E640" t="n">
+        <v>3</v>
+      </c>
+      <c r="F640" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="641">
+      <c r="A641" t="inlineStr">
+        <is>
+          <t>2026-08-08T15:16:00</t>
+        </is>
+      </c>
+      <c r="B641" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C641" t="inlineStr">
+        <is>
+          <t>CountPickedPandral</t>
+        </is>
+      </c>
+      <c r="D641" t="n">
+        <v>0</v>
+      </c>
+      <c r="E641" t="n">
+        <v>3</v>
+      </c>
+      <c r="F641" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="642">
+      <c r="A642" t="inlineStr">
+        <is>
+          <t>2026-08-08T15:16:00</t>
+        </is>
+      </c>
+      <c r="B642" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C642" t="inlineStr">
+        <is>
+          <t>CountPickedOTM</t>
+        </is>
+      </c>
+      <c r="D642" t="n">
+        <v>0</v>
+      </c>
+      <c r="E642" t="n">
+        <v>3</v>
+      </c>
+      <c r="F642" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="643">
+      <c r="A643" t="inlineStr">
+        <is>
+          <t>2026-08-08T15:16:00</t>
+        </is>
+      </c>
+      <c r="B643" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C643" t="inlineStr">
+        <is>
+          <t>RoCals</t>
+        </is>
+      </c>
+      <c r="D643" t="n">
+        <v>0</v>
+      </c>
+      <c r="E643" t="n">
+        <v>3</v>
+      </c>
+      <c r="F643" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="644">
+      <c r="A644" t="inlineStr">
+        <is>
+          <t>2026-08-08T15:16:00</t>
+        </is>
+      </c>
+      <c r="B644" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C644" t="inlineStr">
+        <is>
+          <t>TPS_JamsUsr</t>
+        </is>
+      </c>
+      <c r="D644" t="n">
+        <v>0</v>
+      </c>
+      <c r="E644" t="n">
+        <v>3</v>
+      </c>
+      <c r="F644" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="645">
+      <c r="A645" t="inlineStr">
+        <is>
+          <t>2026-08-08T15:16:00</t>
+        </is>
+      </c>
+      <c r="B645" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C645" t="inlineStr">
+        <is>
+          <t>TPS_JamsMASTER</t>
+        </is>
+      </c>
+      <c r="D645" t="n">
+        <v>0</v>
+      </c>
+      <c r="E645" t="n">
+        <v>3</v>
+      </c>
+      <c r="F645" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="646">
+      <c r="A646" t="inlineStr">
+        <is>
+          <t>2026-08-08T15:16:00</t>
+        </is>
+      </c>
+      <c r="B646" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C646" t="inlineStr">
+        <is>
+          <t>ABORT_Master</t>
+        </is>
+      </c>
+      <c r="D646" t="n">
+        <v>0</v>
+      </c>
+      <c r="E646" t="n">
+        <v>3</v>
+      </c>
+      <c r="F646" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="647">
+      <c r="A647" t="inlineStr">
+        <is>
+          <t>2026-08-08T15:16:13</t>
+        </is>
+      </c>
+      <c r="B647" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C647" t="inlineStr">
+        <is>
+          <t>CountLaidButton</t>
+        </is>
+      </c>
+      <c r="D647" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E647" t="inlineStr"/>
+      <c r="F647" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g2</t>
+        </is>
+      </c>
+    </row>
+    <row r="648">
+      <c r="A648" t="inlineStr">
+        <is>
+          <t>2026-08-08T15:16:13</t>
+        </is>
+      </c>
+      <c r="B648" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C648" t="inlineStr">
+        <is>
+          <t>CountLaidDetector</t>
+        </is>
+      </c>
+      <c r="D648" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E648" t="inlineStr"/>
+      <c r="F648" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g3</t>
+        </is>
+      </c>
+    </row>
+    <row r="649">
+      <c r="A649" t="inlineStr">
+        <is>
+          <t>2026-08-08T15:16:13</t>
+        </is>
+      </c>
+      <c r="B649" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C649" t="inlineStr">
+        <is>
+          <t>CountLaidEncoder</t>
+        </is>
+      </c>
+      <c r="D649" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E649" t="inlineStr"/>
+      <c r="F649" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g4</t>
+        </is>
+      </c>
+    </row>
+    <row r="650">
+      <c r="A650" t="inlineStr">
+        <is>
+          <t>2026-08-08T15:16:13</t>
+        </is>
+      </c>
+      <c r="B650" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C650" t="inlineStr">
+        <is>
+          <t>CountLaid14in</t>
+        </is>
+      </c>
+      <c r="D650" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E650" t="inlineStr"/>
+      <c r="F650" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g5</t>
+        </is>
+      </c>
+    </row>
+    <row r="651">
+      <c r="A651" t="inlineStr">
+        <is>
+          <t>2026-08-08T15:16:13</t>
+        </is>
+      </c>
+      <c r="B651" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C651" t="inlineStr">
+        <is>
+          <t>CountLaid18in</t>
+        </is>
+      </c>
+      <c r="D651" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E651" t="inlineStr"/>
+      <c r="F651" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g6</t>
+        </is>
+      </c>
+    </row>
+    <row r="652">
+      <c r="A652" t="inlineStr">
+        <is>
+          <t>2026-08-08T15:16:13</t>
+        </is>
+      </c>
+      <c r="B652" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C652" t="inlineStr">
+        <is>
+          <t>CountLaidPandral</t>
+        </is>
+      </c>
+      <c r="D652" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E652" t="inlineStr"/>
+      <c r="F652" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g7</t>
+        </is>
+      </c>
+    </row>
+    <row r="653">
+      <c r="A653" t="inlineStr">
+        <is>
+          <t>2026-08-08T15:16:13</t>
+        </is>
+      </c>
+      <c r="B653" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C653" t="inlineStr">
+        <is>
+          <t>18in Job</t>
+        </is>
+      </c>
+      <c r="D653" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E653" t="inlineStr"/>
+      <c r="F653" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g13</t>
+        </is>
+      </c>
+    </row>
+    <row r="654">
+      <c r="A654" t="inlineStr">
+        <is>
+          <t>2026-08-08T15:16:13</t>
+        </is>
+      </c>
+      <c r="B654" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C654" t="inlineStr">
+        <is>
+          <t>CountAcceptedTotal</t>
+        </is>
+      </c>
+      <c r="D654" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E654" t="inlineStr"/>
+      <c r="F654" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g15</t>
+        </is>
+      </c>
+    </row>
+    <row r="655">
+      <c r="A655" t="inlineStr">
+        <is>
+          <t>2026-08-08T15:16:13</t>
+        </is>
+      </c>
+      <c r="B655" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C655" t="inlineStr">
+        <is>
+          <t>Servos_Enabled</t>
+        </is>
+      </c>
+      <c r="D655" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E655" t="inlineStr"/>
+      <c r="F655" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g17</t>
+        </is>
+      </c>
+    </row>
+    <row r="656">
+      <c r="A656" t="inlineStr">
+        <is>
+          <t>2026-08-08T15:16:13</t>
+        </is>
+      </c>
+      <c r="B656" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C656" t="inlineStr">
+        <is>
+          <t>TotalPickPartsCount</t>
+        </is>
+      </c>
+      <c r="D656" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E656" t="inlineStr"/>
+      <c r="F656" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g18</t>
+        </is>
+      </c>
+    </row>
+    <row r="657">
+      <c r="A657" t="inlineStr">
+        <is>
+          <t>2026-08-08T15:16:13</t>
+        </is>
+      </c>
+      <c r="B657" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C657" t="inlineStr">
+        <is>
+          <t>AcceptsPartsCount</t>
+        </is>
+      </c>
+      <c r="D657" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E657" t="inlineStr"/>
+      <c r="F657" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g19</t>
+        </is>
+      </c>
+    </row>
+    <row r="658">
+      <c r="A658" t="inlineStr">
+        <is>
+          <t>2026-08-08T15:16:13</t>
+        </is>
+      </c>
+      <c r="B658" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C658" t="inlineStr">
+        <is>
+          <t>day_Servotime Hours10th</t>
+        </is>
+      </c>
+      <c r="D658" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E658" t="inlineStr"/>
+      <c r="F658" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g22</t>
+        </is>
+      </c>
+    </row>
+    <row r="659">
+      <c r="A659" t="inlineStr">
+        <is>
+          <t>2026-08-08T15:16:13</t>
+        </is>
+      </c>
+      <c r="B659" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C659" t="inlineStr">
+        <is>
+          <t>tk_Cycle</t>
+        </is>
+      </c>
+      <c r="D659" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E659" t="inlineStr"/>
+      <c r="F659" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g23</t>
+        </is>
+      </c>
+    </row>
+    <row r="660">
+      <c r="A660" t="inlineStr">
+        <is>
+          <t>2026-08-08T15:16:13</t>
+        </is>
+      </c>
+      <c r="B660" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C660" t="inlineStr">
+        <is>
+          <t>tk_Abort</t>
+        </is>
+      </c>
+      <c r="D660" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E660" t="inlineStr"/>
+      <c r="F660" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g24</t>
+        </is>
+      </c>
+    </row>
+    <row r="661">
+      <c r="A661" t="inlineStr">
+        <is>
+          <t>2026-08-08T15:16:13</t>
+        </is>
+      </c>
+      <c r="B661" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C661" t="inlineStr">
+        <is>
+          <t>tk_ClearPos</t>
+        </is>
+      </c>
+      <c r="D661" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E661" t="inlineStr"/>
+      <c r="F661" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g25</t>
+        </is>
+      </c>
+    </row>
+    <row r="662">
+      <c r="A662" t="inlineStr">
+        <is>
+          <t>2026-08-08T15:16:13</t>
+        </is>
+      </c>
+      <c r="B662" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C662" t="inlineStr">
+        <is>
+          <t>temp_J2motor</t>
+        </is>
+      </c>
+      <c r="D662" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E662" t="inlineStr"/>
+      <c r="F662" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g33</t>
+        </is>
+      </c>
+    </row>
+    <row r="663">
+      <c r="A663" t="inlineStr">
+        <is>
+          <t>2026-08-08T15:16:13</t>
+        </is>
+      </c>
+      <c r="B663" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C663" t="inlineStr">
+        <is>
+          <t>temp_J3motor</t>
+        </is>
+      </c>
+      <c r="D663" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E663" t="inlineStr"/>
+      <c r="F663" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g34</t>
+        </is>
+      </c>
+    </row>
+    <row r="664">
+      <c r="A664" t="inlineStr">
+        <is>
+          <t>2026-08-08T15:16:13</t>
+        </is>
+      </c>
+      <c r="B664" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C664" t="inlineStr">
+        <is>
+          <t>temp_J5motor</t>
+        </is>
+      </c>
+      <c r="D664" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E664" t="inlineStr"/>
+      <c r="F664" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g36</t>
+        </is>
+      </c>
+    </row>
+    <row r="665">
+      <c r="A665" t="inlineStr">
+        <is>
+          <t>2026-08-08T15:16:13</t>
+        </is>
+      </c>
+      <c r="B665" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C665" t="inlineStr">
+        <is>
+          <t>CountPickedReject18in</t>
+        </is>
+      </c>
+      <c r="D665" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E665" t="inlineStr"/>
+      <c r="F665" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g40</t>
+        </is>
+      </c>
+    </row>
+    <row r="666">
+      <c r="A666" t="inlineStr">
+        <is>
+          <t>2026-08-08T15:16:13</t>
+        </is>
+      </c>
+      <c r="B666" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C666" t="inlineStr">
+        <is>
+          <t>TotalTiePlatesLaid</t>
+        </is>
+      </c>
+      <c r="D666" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E666" t="inlineStr"/>
+      <c r="F666" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g1</t>
+        </is>
+      </c>
+    </row>
+    <row r="667">
+      <c r="A667" t="inlineStr">
+        <is>
+          <t>2026-08-08T15:16:13</t>
+        </is>
+      </c>
+      <c r="B667" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C667" t="inlineStr">
+        <is>
+          <t>usr_TPStime Hours10th</t>
+        </is>
+      </c>
+      <c r="D667" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E667" t="inlineStr"/>
+      <c r="F667" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g8</t>
+        </is>
+      </c>
+    </row>
+    <row r="668">
+      <c r="A668" t="inlineStr">
+        <is>
+          <t>2026-08-08T15:16:13</t>
+        </is>
+      </c>
+      <c r="B668" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C668" t="inlineStr">
+        <is>
+          <t>usrTPS_miles xxx</t>
+        </is>
+      </c>
+      <c r="D668" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E668" t="inlineStr"/>
+      <c r="F668" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g9</t>
+        </is>
+      </c>
+    </row>
+    <row r="669">
+      <c r="A669" t="inlineStr">
+        <is>
+          <t>2026-08-08T15:16:13</t>
+        </is>
+      </c>
+      <c r="B669" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C669" t="inlineStr">
+        <is>
+          <t>TPS Connected</t>
+        </is>
+      </c>
+      <c r="D669" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E669" t="inlineStr"/>
+      <c r="F669" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g10</t>
+        </is>
+      </c>
+    </row>
+    <row r="670">
+      <c r="A670" t="inlineStr">
+        <is>
+          <t>2026-08-08T15:16:13</t>
+        </is>
+      </c>
+      <c r="B670" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C670" t="inlineStr">
+        <is>
+          <t>TPS Enabled</t>
+        </is>
+      </c>
+      <c r="D670" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E670" t="inlineStr"/>
+      <c r="F670" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g11</t>
+        </is>
+      </c>
+    </row>
+    <row r="671">
+      <c r="A671" t="inlineStr">
+        <is>
+          <t>2026-08-08T15:16:13</t>
+        </is>
+      </c>
+      <c r="B671" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C671" t="inlineStr">
+        <is>
+          <t>14in Job</t>
+        </is>
+      </c>
+      <c r="D671" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E671" t="inlineStr"/>
+      <c r="F671" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g12</t>
+        </is>
+      </c>
+    </row>
+    <row r="672">
+      <c r="A672" t="inlineStr">
+        <is>
+          <t>2026-08-08T15:16:13</t>
+        </is>
+      </c>
+      <c r="B672" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C672" t="inlineStr">
+        <is>
+          <t>Pandral Job</t>
+        </is>
+      </c>
+      <c r="D672" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E672" t="inlineStr"/>
+      <c r="F672" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g14</t>
+        </is>
+      </c>
+    </row>
+    <row r="673">
+      <c r="A673" t="inlineStr">
+        <is>
+          <t>2026-08-08T15:16:13</t>
+        </is>
+      </c>
+      <c r="B673" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C673" t="inlineStr">
+        <is>
+          <t>CountRejectedTotal</t>
+        </is>
+      </c>
+      <c r="D673" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E673" t="inlineStr"/>
+      <c r="F673" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g16</t>
+        </is>
+      </c>
+    </row>
+    <row r="674">
+      <c r="A674" t="inlineStr">
+        <is>
+          <t>2026-08-08T15:16:13</t>
+        </is>
+      </c>
+      <c r="B674" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C674" t="inlineStr">
+        <is>
+          <t>RejectPartsCount</t>
+        </is>
+      </c>
+      <c r="D674" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E674" t="inlineStr"/>
+      <c r="F674" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g20</t>
+        </is>
+      </c>
+    </row>
+    <row r="675">
+      <c r="A675" t="inlineStr">
+        <is>
+          <t>2026-08-08T15:16:13</t>
+        </is>
+      </c>
+      <c r="B675" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C675" t="inlineStr">
+        <is>
+          <t>tk_Cycle hrs</t>
+        </is>
+      </c>
+      <c r="D675" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E675" t="inlineStr"/>
+      <c r="F675" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g21</t>
+        </is>
+      </c>
+    </row>
+    <row r="676">
+      <c r="A676" t="inlineStr">
+        <is>
+          <t>2026-08-08T15:16:13</t>
+        </is>
+      </c>
+      <c r="B676" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C676" t="inlineStr">
+        <is>
+          <t>tk_Warmup</t>
+        </is>
+      </c>
+      <c r="D676" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E676" t="inlineStr"/>
+      <c r="F676" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g26</t>
+        </is>
+      </c>
+    </row>
+    <row r="677">
+      <c r="A677" t="inlineStr">
+        <is>
+          <t>2026-08-08T15:16:13</t>
+        </is>
+      </c>
+      <c r="B677" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C677" t="inlineStr">
+        <is>
+          <t>FindingParts min</t>
+        </is>
+      </c>
+      <c r="D677" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E677" t="inlineStr"/>
+      <c r="F677" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g27</t>
+        </is>
+      </c>
+    </row>
+    <row r="678">
+      <c r="A678" t="inlineStr">
+        <is>
+          <t>2026-08-08T15:16:13</t>
+        </is>
+      </c>
+      <c r="B678" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C678" t="inlineStr">
+        <is>
+          <t>PickingParts min</t>
+        </is>
+      </c>
+      <c r="D678" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E678" t="inlineStr"/>
+      <c r="F678" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g28</t>
+        </is>
+      </c>
+    </row>
+    <row r="679">
+      <c r="A679" t="inlineStr">
+        <is>
+          <t>2026-08-08T15:16:13</t>
+        </is>
+      </c>
+      <c r="B679" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C679" t="inlineStr">
+        <is>
+          <t>PlacingParts min</t>
+        </is>
+      </c>
+      <c r="D679" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E679" t="inlineStr"/>
+      <c r="F679" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g29</t>
+        </is>
+      </c>
+    </row>
+    <row r="680">
+      <c r="A680" t="inlineStr">
+        <is>
+          <t>2026-08-08T15:16:13</t>
+        </is>
+      </c>
+      <c r="B680" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C680" t="inlineStr">
+        <is>
+          <t>CountPickedReject14in</t>
+        </is>
+      </c>
+      <c r="D680" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E680" t="inlineStr"/>
+      <c r="F680" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g30</t>
+        </is>
+      </c>
+    </row>
+    <row r="681">
+      <c r="A681" t="inlineStr">
+        <is>
+          <t>2026-08-08T15:16:13</t>
+        </is>
+      </c>
+      <c r="B681" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C681" t="inlineStr">
+        <is>
+          <t>temp_dsi</t>
+        </is>
+      </c>
+      <c r="D681" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E681" t="inlineStr"/>
+      <c r="F681" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g31</t>
+        </is>
+      </c>
+    </row>
+    <row r="682">
+      <c r="A682" t="inlineStr">
+        <is>
+          <t>2026-08-08T15:16:13</t>
+        </is>
+      </c>
+      <c r="B682" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C682" t="inlineStr">
+        <is>
+          <t>temp_J1motor</t>
+        </is>
+      </c>
+      <c r="D682" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E682" t="inlineStr"/>
+      <c r="F682" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g32</t>
+        </is>
+      </c>
+    </row>
+    <row r="683">
+      <c r="A683" t="inlineStr">
+        <is>
+          <t>2026-08-08T15:16:13</t>
+        </is>
+      </c>
+      <c r="B683" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C683" t="inlineStr">
+        <is>
+          <t>temp_J4motor</t>
+        </is>
+      </c>
+      <c r="D683" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E683" t="inlineStr"/>
+      <c r="F683" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g35</t>
+        </is>
+      </c>
+    </row>
+    <row r="684">
+      <c r="A684" t="inlineStr">
+        <is>
+          <t>2026-08-08T15:16:13</t>
+        </is>
+      </c>
+      <c r="B684" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C684" t="inlineStr">
+        <is>
+          <t>temp_J6motor</t>
+        </is>
+      </c>
+      <c r="D684" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E684" t="inlineStr"/>
+      <c r="F684" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g37</t>
+        </is>
+      </c>
+    </row>
+    <row r="685">
+      <c r="A685" t="inlineStr">
+        <is>
+          <t>2026-08-08T15:16:13</t>
+        </is>
+      </c>
+      <c r="B685" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C685" t="inlineStr">
+        <is>
+          <t>CountPickedRejectOTM</t>
+        </is>
+      </c>
+      <c r="D685" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E685" t="inlineStr"/>
+      <c r="F685" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g38</t>
+        </is>
+      </c>
+    </row>
+    <row r="686">
+      <c r="A686" t="inlineStr">
+        <is>
+          <t>2026-08-08T15:16:13</t>
+        </is>
+      </c>
+      <c r="B686" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C686" t="inlineStr">
+        <is>
+          <t>CountPickedRejectPandral</t>
+        </is>
+      </c>
+      <c r="D686" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E686" t="inlineStr"/>
+      <c r="F686" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g39</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Log MQTT data 2026-08-08 17:06 UTC
</commit_message>
<xml_diff>
--- a/logs/raiv_tracker_2026-08-08.xlsx
+++ b/logs/raiv_tracker_2026-08-08.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F686"/>
+  <dimension ref="A1:F816"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -18289,7 +18289,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E647" t="inlineStr"/>
       <c r="F647" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g2</t>
@@ -18317,7 +18316,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E648" t="inlineStr"/>
       <c r="F648" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g3</t>
@@ -18345,7 +18343,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E649" t="inlineStr"/>
       <c r="F649" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g4</t>
@@ -18373,7 +18370,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E650" t="inlineStr"/>
       <c r="F650" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g5</t>
@@ -18401,7 +18397,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E651" t="inlineStr"/>
       <c r="F651" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g6</t>
@@ -18429,7 +18424,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E652" t="inlineStr"/>
       <c r="F652" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g7</t>
@@ -18457,7 +18451,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E653" t="inlineStr"/>
       <c r="F653" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g13</t>
@@ -18485,7 +18478,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E654" t="inlineStr"/>
       <c r="F654" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g15</t>
@@ -18513,7 +18505,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E655" t="inlineStr"/>
       <c r="F655" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g17</t>
@@ -18541,7 +18532,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E656" t="inlineStr"/>
       <c r="F656" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g18</t>
@@ -18569,7 +18559,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E657" t="inlineStr"/>
       <c r="F657" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g19</t>
@@ -18597,7 +18586,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E658" t="inlineStr"/>
       <c r="F658" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g22</t>
@@ -18625,7 +18613,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E659" t="inlineStr"/>
       <c r="F659" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g23</t>
@@ -18653,7 +18640,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E660" t="inlineStr"/>
       <c r="F660" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g24</t>
@@ -18681,7 +18667,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E661" t="inlineStr"/>
       <c r="F661" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g25</t>
@@ -18709,7 +18694,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E662" t="inlineStr"/>
       <c r="F662" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g33</t>
@@ -18737,7 +18721,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E663" t="inlineStr"/>
       <c r="F663" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g34</t>
@@ -18765,7 +18748,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E664" t="inlineStr"/>
       <c r="F664" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g36</t>
@@ -18793,7 +18775,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E665" t="inlineStr"/>
       <c r="F665" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g40</t>
@@ -18821,7 +18802,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E666" t="inlineStr"/>
       <c r="F666" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g1</t>
@@ -18849,7 +18829,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E667" t="inlineStr"/>
       <c r="F667" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g8</t>
@@ -18877,7 +18856,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E668" t="inlineStr"/>
       <c r="F668" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g9</t>
@@ -18905,7 +18883,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E669" t="inlineStr"/>
       <c r="F669" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g10</t>
@@ -18933,7 +18910,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E670" t="inlineStr"/>
       <c r="F670" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g11</t>
@@ -18961,7 +18937,6 @@
           <t>1</t>
         </is>
       </c>
-      <c r="E671" t="inlineStr"/>
       <c r="F671" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g12</t>
@@ -18989,7 +18964,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E672" t="inlineStr"/>
       <c r="F672" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g14</t>
@@ -19017,7 +18991,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E673" t="inlineStr"/>
       <c r="F673" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g16</t>
@@ -19045,7 +19018,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E674" t="inlineStr"/>
       <c r="F674" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g20</t>
@@ -19073,7 +19045,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E675" t="inlineStr"/>
       <c r="F675" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g21</t>
@@ -19101,7 +19072,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E676" t="inlineStr"/>
       <c r="F676" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g26</t>
@@ -19129,7 +19099,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E677" t="inlineStr"/>
       <c r="F677" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g27</t>
@@ -19157,7 +19126,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E678" t="inlineStr"/>
       <c r="F678" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g28</t>
@@ -19185,7 +19153,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E679" t="inlineStr"/>
       <c r="F679" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g29</t>
@@ -19213,7 +19180,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E680" t="inlineStr"/>
       <c r="F680" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g30</t>
@@ -19241,7 +19207,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E681" t="inlineStr"/>
       <c r="F681" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g31</t>
@@ -19269,7 +19234,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E682" t="inlineStr"/>
       <c r="F682" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g32</t>
@@ -19297,7 +19261,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E683" t="inlineStr"/>
       <c r="F683" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g35</t>
@@ -19325,7 +19288,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E684" t="inlineStr"/>
       <c r="F684" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g37</t>
@@ -19353,7 +19315,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E685" t="inlineStr"/>
       <c r="F685" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g38</t>
@@ -19381,10 +19342,3649 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E686" t="inlineStr"/>
       <c r="F686" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g39</t>
+        </is>
+      </c>
+    </row>
+    <row r="687">
+      <c r="A687" t="inlineStr">
+        <is>
+          <t>2026-08-08T17:05:00</t>
+        </is>
+      </c>
+      <c r="B687" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C687" t="inlineStr">
+        <is>
+          <t>_1st_SCAN</t>
+        </is>
+      </c>
+      <c r="D687" t="b">
+        <v>0</v>
+      </c>
+      <c r="E687" t="n">
+        <v>11</v>
+      </c>
+      <c r="F687" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="688">
+      <c r="A688" t="inlineStr">
+        <is>
+          <t>2026-08-08T17:05:00</t>
+        </is>
+      </c>
+      <c r="B688" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C688" t="inlineStr">
+        <is>
+          <t>TieDetectOffset_B</t>
+        </is>
+      </c>
+      <c r="D688" t="b">
+        <v>0</v>
+      </c>
+      <c r="E688" t="n">
+        <v>11</v>
+      </c>
+      <c r="F688" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="689">
+      <c r="A689" t="inlineStr">
+        <is>
+          <t>2026-08-08T17:05:00</t>
+        </is>
+      </c>
+      <c r="B689" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C689" t="inlineStr">
+        <is>
+          <t>Tie Detector</t>
+        </is>
+      </c>
+      <c r="D689" t="b">
+        <v>0</v>
+      </c>
+      <c r="E689" t="n">
+        <v>11</v>
+      </c>
+      <c r="F689" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="690">
+      <c r="A690" t="inlineStr">
+        <is>
+          <t>2026-08-08T17:05:00</t>
+        </is>
+      </c>
+      <c r="B690" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C690" t="inlineStr">
+        <is>
+          <t>TPS Full</t>
+        </is>
+      </c>
+      <c r="D690" t="b">
+        <v>0</v>
+      </c>
+      <c r="E690" t="n">
+        <v>11</v>
+      </c>
+      <c r="F690" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="691">
+      <c r="A691" t="inlineStr">
+        <is>
+          <t>2026-08-08T17:05:00</t>
+        </is>
+      </c>
+      <c r="B691" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C691" t="inlineStr">
+        <is>
+          <t>TieDetectOffset_A</t>
+        </is>
+      </c>
+      <c r="D691" t="b">
+        <v>0</v>
+      </c>
+      <c r="E691" t="n">
+        <v>11</v>
+      </c>
+      <c r="F691" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="692">
+      <c r="A692" t="inlineStr">
+        <is>
+          <t>2026-08-08T17:05:00</t>
+        </is>
+      </c>
+      <c r="B692" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C692" t="inlineStr">
+        <is>
+          <t>TPS Connected</t>
+        </is>
+      </c>
+      <c r="D692" t="b">
+        <v>0</v>
+      </c>
+      <c r="E692" t="n">
+        <v>11</v>
+      </c>
+      <c r="F692" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="693">
+      <c r="A693" t="inlineStr">
+        <is>
+          <t>2026-08-08T17:05:00</t>
+        </is>
+      </c>
+      <c r="B693" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C693" t="inlineStr">
+        <is>
+          <t>TPS_Enable_ Button</t>
+        </is>
+      </c>
+      <c r="D693" t="b">
+        <v>0</v>
+      </c>
+      <c r="E693" t="n">
+        <v>11</v>
+      </c>
+      <c r="F693" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="694">
+      <c r="A694" t="inlineStr">
+        <is>
+          <t>2026-08-08T17:05:00</t>
+        </is>
+      </c>
+      <c r="B694" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C694" t="inlineStr">
+        <is>
+          <t>AirEagle Eject Plate</t>
+        </is>
+      </c>
+      <c r="D694" t="b">
+        <v>0</v>
+      </c>
+      <c r="E694" t="n">
+        <v>11</v>
+      </c>
+      <c r="F694" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="695">
+      <c r="A695" t="inlineStr">
+        <is>
+          <t>2026-08-08T17:05:00</t>
+        </is>
+      </c>
+      <c r="B695" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C695" t="inlineStr">
+        <is>
+          <t>tk_Cycle</t>
+        </is>
+      </c>
+      <c r="D695" t="b">
+        <v>0</v>
+      </c>
+      <c r="E695" t="n">
+        <v>11</v>
+      </c>
+      <c r="F695" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="696">
+      <c r="A696" t="inlineStr">
+        <is>
+          <t>2026-08-08T17:05:00</t>
+        </is>
+      </c>
+      <c r="B696" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C696" t="inlineStr">
+        <is>
+          <t>Servos_Enabled</t>
+        </is>
+      </c>
+      <c r="D696" t="b">
+        <v>0</v>
+      </c>
+      <c r="E696" t="n">
+        <v>11</v>
+      </c>
+      <c r="F696" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="697">
+      <c r="A697" t="inlineStr">
+        <is>
+          <t>2026-08-08T17:05:00</t>
+        </is>
+      </c>
+      <c r="B697" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C697" t="inlineStr">
+        <is>
+          <t>TPS Enabled</t>
+        </is>
+      </c>
+      <c r="D697" t="b">
+        <v>0</v>
+      </c>
+      <c r="E697" t="n">
+        <v>11</v>
+      </c>
+      <c r="F697" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="698">
+      <c r="A698" t="inlineStr">
+        <is>
+          <t>2026-08-08T17:05:00</t>
+        </is>
+      </c>
+      <c r="B698" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C698" t="inlineStr">
+        <is>
+          <t>tk_Abort</t>
+        </is>
+      </c>
+      <c r="D698" t="b">
+        <v>0</v>
+      </c>
+      <c r="E698" t="n">
+        <v>11</v>
+      </c>
+      <c r="F698" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="699">
+      <c r="A699" t="inlineStr">
+        <is>
+          <t>2026-08-08T17:05:00</t>
+        </is>
+      </c>
+      <c r="B699" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C699" t="inlineStr">
+        <is>
+          <t>Robot_isMoving</t>
+        </is>
+      </c>
+      <c r="D699" t="b">
+        <v>0</v>
+      </c>
+      <c r="E699" t="n">
+        <v>11</v>
+      </c>
+      <c r="F699" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="700">
+      <c r="A700" t="inlineStr">
+        <is>
+          <t>2026-08-08T17:05:00</t>
+        </is>
+      </c>
+      <c r="B700" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C700" t="inlineStr">
+        <is>
+          <t>Eject Tie Plate</t>
+        </is>
+      </c>
+      <c r="D700" t="b">
+        <v>0</v>
+      </c>
+      <c r="E700" t="n">
+        <v>11</v>
+      </c>
+      <c r="F700" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="701">
+      <c r="A701" t="inlineStr">
+        <is>
+          <t>2026-08-08T17:05:00</t>
+        </is>
+      </c>
+      <c r="B701" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C701" t="inlineStr">
+        <is>
+          <t>TPS BACKUP ALARM</t>
+        </is>
+      </c>
+      <c r="D701" t="b">
+        <v>0</v>
+      </c>
+      <c r="E701" t="n">
+        <v>11</v>
+      </c>
+      <c r="F701" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="702">
+      <c r="A702" t="inlineStr">
+        <is>
+          <t>2026-08-08T17:05:00</t>
+        </is>
+      </c>
+      <c r="B702" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C702" t="inlineStr">
+        <is>
+          <t>14in Job</t>
+        </is>
+      </c>
+      <c r="D702" t="b">
+        <v>1</v>
+      </c>
+      <c r="E702" t="n">
+        <v>11</v>
+      </c>
+      <c r="F702" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="703">
+      <c r="A703" t="inlineStr">
+        <is>
+          <t>2026-08-08T17:05:00</t>
+        </is>
+      </c>
+      <c r="B703" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C703" t="inlineStr">
+        <is>
+          <t>18in Job</t>
+        </is>
+      </c>
+      <c r="D703" t="b">
+        <v>0</v>
+      </c>
+      <c r="E703" t="n">
+        <v>11</v>
+      </c>
+      <c r="F703" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="704">
+      <c r="A704" t="inlineStr">
+        <is>
+          <t>2026-08-08T17:05:00</t>
+        </is>
+      </c>
+      <c r="B704" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C704" t="inlineStr">
+        <is>
+          <t>Pandral Job</t>
+        </is>
+      </c>
+      <c r="D704" t="b">
+        <v>0</v>
+      </c>
+      <c r="E704" t="n">
+        <v>11</v>
+      </c>
+      <c r="F704" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="705">
+      <c r="A705" t="inlineStr">
+        <is>
+          <t>2026-08-08T17:05:00</t>
+        </is>
+      </c>
+      <c r="B705" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C705" t="inlineStr">
+        <is>
+          <t>DoubleLay Job</t>
+        </is>
+      </c>
+      <c r="D705" t="b">
+        <v>0</v>
+      </c>
+      <c r="E705" t="n">
+        <v>11</v>
+      </c>
+      <c r="F705" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="706">
+      <c r="A706" t="inlineStr">
+        <is>
+          <t>2026-08-08T17:05:00</t>
+        </is>
+      </c>
+      <c r="B706" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C706" t="inlineStr">
+        <is>
+          <t>TPSjam_FLAG</t>
+        </is>
+      </c>
+      <c r="D706" t="b">
+        <v>0</v>
+      </c>
+      <c r="E706" t="n">
+        <v>11</v>
+      </c>
+      <c r="F706" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="707">
+      <c r="A707" t="inlineStr">
+        <is>
+          <t>2026-08-08T17:05:00</t>
+        </is>
+      </c>
+      <c r="B707" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C707" t="inlineStr">
+        <is>
+          <t>RoCalRequest</t>
+        </is>
+      </c>
+      <c r="D707" t="b">
+        <v>0</v>
+      </c>
+      <c r="E707" t="n">
+        <v>11</v>
+      </c>
+      <c r="F707" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="708">
+      <c r="A708" t="inlineStr">
+        <is>
+          <t>2026-08-08T17:05:00</t>
+        </is>
+      </c>
+      <c r="B708" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C708" t="inlineStr">
+        <is>
+          <t>tkCycle_TotalSeconds</t>
+        </is>
+      </c>
+      <c r="D708" t="n">
+        <v>0</v>
+      </c>
+      <c r="E708" t="n">
+        <v>9</v>
+      </c>
+      <c r="F708" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="709">
+      <c r="A709" t="inlineStr">
+        <is>
+          <t>2026-08-08T17:05:00</t>
+        </is>
+      </c>
+      <c r="B709" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C709" t="inlineStr">
+        <is>
+          <t>tkCycle_NoMoveSec</t>
+        </is>
+      </c>
+      <c r="D709" t="n">
+        <v>0</v>
+      </c>
+      <c r="E709" t="n">
+        <v>9</v>
+      </c>
+      <c r="F709" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="710">
+      <c r="A710" t="inlineStr">
+        <is>
+          <t>2026-08-08T17:05:00</t>
+        </is>
+      </c>
+      <c r="B710" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C710" t="inlineStr">
+        <is>
+          <t>tkCycle_MoveSeconds</t>
+        </is>
+      </c>
+      <c r="D710" t="n">
+        <v>0</v>
+      </c>
+      <c r="E710" t="n">
+        <v>9</v>
+      </c>
+      <c r="F710" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="711">
+      <c r="A711" t="inlineStr">
+        <is>
+          <t>2026-08-08T17:05:00</t>
+        </is>
+      </c>
+      <c r="B711" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C711" t="inlineStr">
+        <is>
+          <t>Percent time moveing</t>
+        </is>
+      </c>
+      <c r="D711" t="n">
+        <v>0</v>
+      </c>
+      <c r="E711" t="n">
+        <v>9</v>
+      </c>
+      <c r="F711" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="712">
+      <c r="A712" t="inlineStr">
+        <is>
+          <t>2026-08-08T17:05:00</t>
+        </is>
+      </c>
+      <c r="B712" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C712" t="inlineStr">
+        <is>
+          <t>Percent time not moving</t>
+        </is>
+      </c>
+      <c r="D712" t="n">
+        <v>0</v>
+      </c>
+      <c r="E712" t="n">
+        <v>9</v>
+      </c>
+      <c r="F712" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="713">
+      <c r="A713" t="inlineStr">
+        <is>
+          <t>2026-08-08T17:05:00</t>
+        </is>
+      </c>
+      <c r="B713" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C713" t="inlineStr">
+        <is>
+          <t>TotalPickPartsCount</t>
+        </is>
+      </c>
+      <c r="D713" t="n">
+        <v>0</v>
+      </c>
+      <c r="E713" t="n">
+        <v>9</v>
+      </c>
+      <c r="F713" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="714">
+      <c r="A714" t="inlineStr">
+        <is>
+          <t>2026-08-08T17:05:00</t>
+        </is>
+      </c>
+      <c r="B714" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C714" t="inlineStr">
+        <is>
+          <t>RejectPartsCount</t>
+        </is>
+      </c>
+      <c r="D714" t="n">
+        <v>0</v>
+      </c>
+      <c r="E714" t="n">
+        <v>9</v>
+      </c>
+      <c r="F714" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="715">
+      <c r="A715" t="inlineStr">
+        <is>
+          <t>2026-08-08T17:05:00</t>
+        </is>
+      </c>
+      <c r="B715" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C715" t="inlineStr">
+        <is>
+          <t>AcceptsPartsCount</t>
+        </is>
+      </c>
+      <c r="D715" t="n">
+        <v>0</v>
+      </c>
+      <c r="E715" t="n">
+        <v>9</v>
+      </c>
+      <c r="F715" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="716">
+      <c r="A716" t="inlineStr">
+        <is>
+          <t>2026-08-08T17:05:00</t>
+        </is>
+      </c>
+      <c r="B716" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C716" t="inlineStr">
+        <is>
+          <t>percentCount_accept</t>
+        </is>
+      </c>
+      <c r="D716" t="n">
+        <v>0</v>
+      </c>
+      <c r="E716" t="n">
+        <v>9</v>
+      </c>
+      <c r="F716" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="717">
+      <c r="A717" t="inlineStr">
+        <is>
+          <t>2026-08-08T17:05:00</t>
+        </is>
+      </c>
+      <c r="B717" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C717" t="inlineStr">
+        <is>
+          <t>percentCount_reject</t>
+        </is>
+      </c>
+      <c r="D717" t="n">
+        <v>0</v>
+      </c>
+      <c r="E717" t="n">
+        <v>9</v>
+      </c>
+      <c r="F717" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="718">
+      <c r="A718" t="inlineStr">
+        <is>
+          <t>2026-08-08T17:05:00</t>
+        </is>
+      </c>
+      <c r="B718" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C718" t="inlineStr">
+        <is>
+          <t>Avg Parts per min_total</t>
+        </is>
+      </c>
+      <c r="D718" t="n">
+        <v>0</v>
+      </c>
+      <c r="E718" t="n">
+        <v>9</v>
+      </c>
+      <c r="F718" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="719">
+      <c r="A719" t="inlineStr">
+        <is>
+          <t>2026-08-08T17:05:00</t>
+        </is>
+      </c>
+      <c r="B719" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C719" t="inlineStr">
+        <is>
+          <t>TotalPickedParts</t>
+        </is>
+      </c>
+      <c r="D719" t="n">
+        <v>0</v>
+      </c>
+      <c r="E719" t="n">
+        <v>3</v>
+      </c>
+      <c r="F719" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="720">
+      <c r="A720" t="inlineStr">
+        <is>
+          <t>2026-08-08T17:05:00</t>
+        </is>
+      </c>
+      <c r="B720" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C720" t="inlineStr">
+        <is>
+          <t>TotalPickedAcceptParts</t>
+        </is>
+      </c>
+      <c r="D720" t="n">
+        <v>0</v>
+      </c>
+      <c r="E720" t="n">
+        <v>3</v>
+      </c>
+      <c r="F720" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="721">
+      <c r="A721" t="inlineStr">
+        <is>
+          <t>2026-08-08T17:05:00</t>
+        </is>
+      </c>
+      <c r="B721" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C721" t="inlineStr">
+        <is>
+          <t>TotalPickedRejectParts</t>
+        </is>
+      </c>
+      <c r="D721" t="n">
+        <v>0</v>
+      </c>
+      <c r="E721" t="n">
+        <v>3</v>
+      </c>
+      <c r="F721" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="722">
+      <c r="A722" t="inlineStr">
+        <is>
+          <t>2026-08-08T17:05:00</t>
+        </is>
+      </c>
+      <c r="B722" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C722" t="inlineStr">
+        <is>
+          <t>TotalTiePlatesLaid</t>
+        </is>
+      </c>
+      <c r="D722" t="n">
+        <v>0</v>
+      </c>
+      <c r="E722" t="n">
+        <v>3</v>
+      </c>
+      <c r="F722" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="723">
+      <c r="A723" t="inlineStr">
+        <is>
+          <t>2026-08-08T17:05:00</t>
+        </is>
+      </c>
+      <c r="B723" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C723" t="inlineStr">
+        <is>
+          <t>Daily_TotalLaidPlates</t>
+        </is>
+      </c>
+      <c r="D723" t="n">
+        <v>0</v>
+      </c>
+      <c r="E723" t="n">
+        <v>3</v>
+      </c>
+      <c r="F723" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="724">
+      <c r="A724" t="inlineStr">
+        <is>
+          <t>2026-08-08T17:05:00</t>
+        </is>
+      </c>
+      <c r="B724" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C724" t="inlineStr">
+        <is>
+          <t>CountPicked14in</t>
+        </is>
+      </c>
+      <c r="D724" t="n">
+        <v>0</v>
+      </c>
+      <c r="E724" t="n">
+        <v>3</v>
+      </c>
+      <c r="F724" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="725">
+      <c r="A725" t="inlineStr">
+        <is>
+          <t>2026-08-08T17:05:00</t>
+        </is>
+      </c>
+      <c r="B725" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C725" t="inlineStr">
+        <is>
+          <t>CountPicked18in</t>
+        </is>
+      </c>
+      <c r="D725" t="n">
+        <v>0</v>
+      </c>
+      <c r="E725" t="n">
+        <v>3</v>
+      </c>
+      <c r="F725" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="726">
+      <c r="A726" t="inlineStr">
+        <is>
+          <t>2026-08-08T17:05:00</t>
+        </is>
+      </c>
+      <c r="B726" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C726" t="inlineStr">
+        <is>
+          <t>CountPickedPandral</t>
+        </is>
+      </c>
+      <c r="D726" t="n">
+        <v>0</v>
+      </c>
+      <c r="E726" t="n">
+        <v>3</v>
+      </c>
+      <c r="F726" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="727">
+      <c r="A727" t="inlineStr">
+        <is>
+          <t>2026-08-08T17:05:00</t>
+        </is>
+      </c>
+      <c r="B727" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C727" t="inlineStr">
+        <is>
+          <t>CountPickedOTM</t>
+        </is>
+      </c>
+      <c r="D727" t="n">
+        <v>0</v>
+      </c>
+      <c r="E727" t="n">
+        <v>3</v>
+      </c>
+      <c r="F727" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="728">
+      <c r="A728" t="inlineStr">
+        <is>
+          <t>2026-08-08T17:05:00</t>
+        </is>
+      </c>
+      <c r="B728" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C728" t="inlineStr">
+        <is>
+          <t>RoCals</t>
+        </is>
+      </c>
+      <c r="D728" t="n">
+        <v>0</v>
+      </c>
+      <c r="E728" t="n">
+        <v>3</v>
+      </c>
+      <c r="F728" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="729">
+      <c r="A729" t="inlineStr">
+        <is>
+          <t>2026-08-08T17:05:00</t>
+        </is>
+      </c>
+      <c r="B729" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C729" t="inlineStr">
+        <is>
+          <t>TPS_JamsUsr</t>
+        </is>
+      </c>
+      <c r="D729" t="n">
+        <v>0</v>
+      </c>
+      <c r="E729" t="n">
+        <v>3</v>
+      </c>
+      <c r="F729" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="730">
+      <c r="A730" t="inlineStr">
+        <is>
+          <t>2026-08-08T17:05:00</t>
+        </is>
+      </c>
+      <c r="B730" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C730" t="inlineStr">
+        <is>
+          <t>TPS_JamsMASTER</t>
+        </is>
+      </c>
+      <c r="D730" t="n">
+        <v>0</v>
+      </c>
+      <c r="E730" t="n">
+        <v>3</v>
+      </c>
+      <c r="F730" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="731">
+      <c r="A731" t="inlineStr">
+        <is>
+          <t>2026-08-08T17:05:00</t>
+        </is>
+      </c>
+      <c r="B731" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C731" t="inlineStr">
+        <is>
+          <t>ABORT_Master</t>
+        </is>
+      </c>
+      <c r="D731" t="n">
+        <v>0</v>
+      </c>
+      <c r="E731" t="n">
+        <v>3</v>
+      </c>
+      <c r="F731" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="732">
+      <c r="A732" t="inlineStr">
+        <is>
+          <t>2026-08-08T17:05:13</t>
+        </is>
+      </c>
+      <c r="B732" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C732" t="inlineStr">
+        <is>
+          <t>CountLaidButton</t>
+        </is>
+      </c>
+      <c r="D732" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E732" t="inlineStr"/>
+      <c r="F732" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g2</t>
+        </is>
+      </c>
+    </row>
+    <row r="733">
+      <c r="A733" t="inlineStr">
+        <is>
+          <t>2026-08-08T17:05:13</t>
+        </is>
+      </c>
+      <c r="B733" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C733" t="inlineStr">
+        <is>
+          <t>CountLaidDetector</t>
+        </is>
+      </c>
+      <c r="D733" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E733" t="inlineStr"/>
+      <c r="F733" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g3</t>
+        </is>
+      </c>
+    </row>
+    <row r="734">
+      <c r="A734" t="inlineStr">
+        <is>
+          <t>2026-08-08T17:05:13</t>
+        </is>
+      </c>
+      <c r="B734" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C734" t="inlineStr">
+        <is>
+          <t>CountLaidEncoder</t>
+        </is>
+      </c>
+      <c r="D734" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E734" t="inlineStr"/>
+      <c r="F734" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g4</t>
+        </is>
+      </c>
+    </row>
+    <row r="735">
+      <c r="A735" t="inlineStr">
+        <is>
+          <t>2026-08-08T17:05:13</t>
+        </is>
+      </c>
+      <c r="B735" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C735" t="inlineStr">
+        <is>
+          <t>CountLaid14in</t>
+        </is>
+      </c>
+      <c r="D735" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E735" t="inlineStr"/>
+      <c r="F735" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g5</t>
+        </is>
+      </c>
+    </row>
+    <row r="736">
+      <c r="A736" t="inlineStr">
+        <is>
+          <t>2026-08-08T17:05:13</t>
+        </is>
+      </c>
+      <c r="B736" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C736" t="inlineStr">
+        <is>
+          <t>CountLaid18in</t>
+        </is>
+      </c>
+      <c r="D736" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E736" t="inlineStr"/>
+      <c r="F736" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g6</t>
+        </is>
+      </c>
+    </row>
+    <row r="737">
+      <c r="A737" t="inlineStr">
+        <is>
+          <t>2026-08-08T17:05:13</t>
+        </is>
+      </c>
+      <c r="B737" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C737" t="inlineStr">
+        <is>
+          <t>CountLaidPandral</t>
+        </is>
+      </c>
+      <c r="D737" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E737" t="inlineStr"/>
+      <c r="F737" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g7</t>
+        </is>
+      </c>
+    </row>
+    <row r="738">
+      <c r="A738" t="inlineStr">
+        <is>
+          <t>2026-08-08T17:05:13</t>
+        </is>
+      </c>
+      <c r="B738" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C738" t="inlineStr">
+        <is>
+          <t>18in Job</t>
+        </is>
+      </c>
+      <c r="D738" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E738" t="inlineStr"/>
+      <c r="F738" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g13</t>
+        </is>
+      </c>
+    </row>
+    <row r="739">
+      <c r="A739" t="inlineStr">
+        <is>
+          <t>2026-08-08T17:05:13</t>
+        </is>
+      </c>
+      <c r="B739" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C739" t="inlineStr">
+        <is>
+          <t>CountAcceptedTotal</t>
+        </is>
+      </c>
+      <c r="D739" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E739" t="inlineStr"/>
+      <c r="F739" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g15</t>
+        </is>
+      </c>
+    </row>
+    <row r="740">
+      <c r="A740" t="inlineStr">
+        <is>
+          <t>2026-08-08T17:05:13</t>
+        </is>
+      </c>
+      <c r="B740" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C740" t="inlineStr">
+        <is>
+          <t>Servos_Enabled</t>
+        </is>
+      </c>
+      <c r="D740" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E740" t="inlineStr"/>
+      <c r="F740" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g17</t>
+        </is>
+      </c>
+    </row>
+    <row r="741">
+      <c r="A741" t="inlineStr">
+        <is>
+          <t>2026-08-08T17:05:13</t>
+        </is>
+      </c>
+      <c r="B741" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C741" t="inlineStr">
+        <is>
+          <t>TotalPickPartsCount</t>
+        </is>
+      </c>
+      <c r="D741" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E741" t="inlineStr"/>
+      <c r="F741" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g18</t>
+        </is>
+      </c>
+    </row>
+    <row r="742">
+      <c r="A742" t="inlineStr">
+        <is>
+          <t>2026-08-08T17:05:13</t>
+        </is>
+      </c>
+      <c r="B742" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C742" t="inlineStr">
+        <is>
+          <t>AcceptsPartsCount</t>
+        </is>
+      </c>
+      <c r="D742" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E742" t="inlineStr"/>
+      <c r="F742" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g19</t>
+        </is>
+      </c>
+    </row>
+    <row r="743">
+      <c r="A743" t="inlineStr">
+        <is>
+          <t>2026-08-08T17:05:13</t>
+        </is>
+      </c>
+      <c r="B743" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C743" t="inlineStr">
+        <is>
+          <t>day_Servotime Hours10th</t>
+        </is>
+      </c>
+      <c r="D743" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E743" t="inlineStr"/>
+      <c r="F743" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g22</t>
+        </is>
+      </c>
+    </row>
+    <row r="744">
+      <c r="A744" t="inlineStr">
+        <is>
+          <t>2026-08-08T17:05:13</t>
+        </is>
+      </c>
+      <c r="B744" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C744" t="inlineStr">
+        <is>
+          <t>tk_Cycle</t>
+        </is>
+      </c>
+      <c r="D744" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E744" t="inlineStr"/>
+      <c r="F744" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g23</t>
+        </is>
+      </c>
+    </row>
+    <row r="745">
+      <c r="A745" t="inlineStr">
+        <is>
+          <t>2026-08-08T17:05:13</t>
+        </is>
+      </c>
+      <c r="B745" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C745" t="inlineStr">
+        <is>
+          <t>tk_Abort</t>
+        </is>
+      </c>
+      <c r="D745" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E745" t="inlineStr"/>
+      <c r="F745" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g24</t>
+        </is>
+      </c>
+    </row>
+    <row r="746">
+      <c r="A746" t="inlineStr">
+        <is>
+          <t>2026-08-08T17:05:13</t>
+        </is>
+      </c>
+      <c r="B746" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C746" t="inlineStr">
+        <is>
+          <t>tk_ClearPos</t>
+        </is>
+      </c>
+      <c r="D746" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E746" t="inlineStr"/>
+      <c r="F746" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g25</t>
+        </is>
+      </c>
+    </row>
+    <row r="747">
+      <c r="A747" t="inlineStr">
+        <is>
+          <t>2026-08-08T17:05:13</t>
+        </is>
+      </c>
+      <c r="B747" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C747" t="inlineStr">
+        <is>
+          <t>temp_J2motor</t>
+        </is>
+      </c>
+      <c r="D747" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E747" t="inlineStr"/>
+      <c r="F747" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g33</t>
+        </is>
+      </c>
+    </row>
+    <row r="748">
+      <c r="A748" t="inlineStr">
+        <is>
+          <t>2026-08-08T17:05:13</t>
+        </is>
+      </c>
+      <c r="B748" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C748" t="inlineStr">
+        <is>
+          <t>temp_J3motor</t>
+        </is>
+      </c>
+      <c r="D748" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E748" t="inlineStr"/>
+      <c r="F748" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g34</t>
+        </is>
+      </c>
+    </row>
+    <row r="749">
+      <c r="A749" t="inlineStr">
+        <is>
+          <t>2026-08-08T17:05:13</t>
+        </is>
+      </c>
+      <c r="B749" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C749" t="inlineStr">
+        <is>
+          <t>temp_J5motor</t>
+        </is>
+      </c>
+      <c r="D749" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E749" t="inlineStr"/>
+      <c r="F749" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g36</t>
+        </is>
+      </c>
+    </row>
+    <row r="750">
+      <c r="A750" t="inlineStr">
+        <is>
+          <t>2026-08-08T17:05:13</t>
+        </is>
+      </c>
+      <c r="B750" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C750" t="inlineStr">
+        <is>
+          <t>CountPickedReject18in</t>
+        </is>
+      </c>
+      <c r="D750" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E750" t="inlineStr"/>
+      <c r="F750" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g40</t>
+        </is>
+      </c>
+    </row>
+    <row r="751">
+      <c r="A751" t="inlineStr">
+        <is>
+          <t>2026-08-08T17:05:13</t>
+        </is>
+      </c>
+      <c r="B751" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C751" t="inlineStr">
+        <is>
+          <t>TotalTiePlatesLaid</t>
+        </is>
+      </c>
+      <c r="D751" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E751" t="inlineStr"/>
+      <c r="F751" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g1</t>
+        </is>
+      </c>
+    </row>
+    <row r="752">
+      <c r="A752" t="inlineStr">
+        <is>
+          <t>2026-08-08T17:05:13</t>
+        </is>
+      </c>
+      <c r="B752" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C752" t="inlineStr">
+        <is>
+          <t>usr_TPStime Hours10th</t>
+        </is>
+      </c>
+      <c r="D752" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E752" t="inlineStr"/>
+      <c r="F752" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g8</t>
+        </is>
+      </c>
+    </row>
+    <row r="753">
+      <c r="A753" t="inlineStr">
+        <is>
+          <t>2026-08-08T17:05:13</t>
+        </is>
+      </c>
+      <c r="B753" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C753" t="inlineStr">
+        <is>
+          <t>usrTPS_miles xxx</t>
+        </is>
+      </c>
+      <c r="D753" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E753" t="inlineStr"/>
+      <c r="F753" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g9</t>
+        </is>
+      </c>
+    </row>
+    <row r="754">
+      <c r="A754" t="inlineStr">
+        <is>
+          <t>2026-08-08T17:05:13</t>
+        </is>
+      </c>
+      <c r="B754" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C754" t="inlineStr">
+        <is>
+          <t>TPS Connected</t>
+        </is>
+      </c>
+      <c r="D754" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E754" t="inlineStr"/>
+      <c r="F754" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g10</t>
+        </is>
+      </c>
+    </row>
+    <row r="755">
+      <c r="A755" t="inlineStr">
+        <is>
+          <t>2026-08-08T17:05:13</t>
+        </is>
+      </c>
+      <c r="B755" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C755" t="inlineStr">
+        <is>
+          <t>TPS Enabled</t>
+        </is>
+      </c>
+      <c r="D755" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E755" t="inlineStr"/>
+      <c r="F755" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g11</t>
+        </is>
+      </c>
+    </row>
+    <row r="756">
+      <c r="A756" t="inlineStr">
+        <is>
+          <t>2026-08-08T17:05:13</t>
+        </is>
+      </c>
+      <c r="B756" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C756" t="inlineStr">
+        <is>
+          <t>14in Job</t>
+        </is>
+      </c>
+      <c r="D756" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E756" t="inlineStr"/>
+      <c r="F756" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g12</t>
+        </is>
+      </c>
+    </row>
+    <row r="757">
+      <c r="A757" t="inlineStr">
+        <is>
+          <t>2026-08-08T17:05:13</t>
+        </is>
+      </c>
+      <c r="B757" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C757" t="inlineStr">
+        <is>
+          <t>Pandral Job</t>
+        </is>
+      </c>
+      <c r="D757" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E757" t="inlineStr"/>
+      <c r="F757" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g14</t>
+        </is>
+      </c>
+    </row>
+    <row r="758">
+      <c r="A758" t="inlineStr">
+        <is>
+          <t>2026-08-08T17:05:13</t>
+        </is>
+      </c>
+      <c r="B758" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C758" t="inlineStr">
+        <is>
+          <t>CountRejectedTotal</t>
+        </is>
+      </c>
+      <c r="D758" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E758" t="inlineStr"/>
+      <c r="F758" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g16</t>
+        </is>
+      </c>
+    </row>
+    <row r="759">
+      <c r="A759" t="inlineStr">
+        <is>
+          <t>2026-08-08T17:05:13</t>
+        </is>
+      </c>
+      <c r="B759" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C759" t="inlineStr">
+        <is>
+          <t>RejectPartsCount</t>
+        </is>
+      </c>
+      <c r="D759" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E759" t="inlineStr"/>
+      <c r="F759" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g20</t>
+        </is>
+      </c>
+    </row>
+    <row r="760">
+      <c r="A760" t="inlineStr">
+        <is>
+          <t>2026-08-08T17:05:13</t>
+        </is>
+      </c>
+      <c r="B760" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C760" t="inlineStr">
+        <is>
+          <t>tk_Cycle hrs</t>
+        </is>
+      </c>
+      <c r="D760" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E760" t="inlineStr"/>
+      <c r="F760" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g21</t>
+        </is>
+      </c>
+    </row>
+    <row r="761">
+      <c r="A761" t="inlineStr">
+        <is>
+          <t>2026-08-08T17:05:13</t>
+        </is>
+      </c>
+      <c r="B761" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C761" t="inlineStr">
+        <is>
+          <t>tk_Warmup</t>
+        </is>
+      </c>
+      <c r="D761" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E761" t="inlineStr"/>
+      <c r="F761" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g26</t>
+        </is>
+      </c>
+    </row>
+    <row r="762">
+      <c r="A762" t="inlineStr">
+        <is>
+          <t>2026-08-08T17:05:13</t>
+        </is>
+      </c>
+      <c r="B762" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C762" t="inlineStr">
+        <is>
+          <t>FindingParts min</t>
+        </is>
+      </c>
+      <c r="D762" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E762" t="inlineStr"/>
+      <c r="F762" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g27</t>
+        </is>
+      </c>
+    </row>
+    <row r="763">
+      <c r="A763" t="inlineStr">
+        <is>
+          <t>2026-08-08T17:05:13</t>
+        </is>
+      </c>
+      <c r="B763" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C763" t="inlineStr">
+        <is>
+          <t>PickingParts min</t>
+        </is>
+      </c>
+      <c r="D763" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E763" t="inlineStr"/>
+      <c r="F763" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g28</t>
+        </is>
+      </c>
+    </row>
+    <row r="764">
+      <c r="A764" t="inlineStr">
+        <is>
+          <t>2026-08-08T17:05:13</t>
+        </is>
+      </c>
+      <c r="B764" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C764" t="inlineStr">
+        <is>
+          <t>PlacingParts min</t>
+        </is>
+      </c>
+      <c r="D764" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E764" t="inlineStr"/>
+      <c r="F764" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g29</t>
+        </is>
+      </c>
+    </row>
+    <row r="765">
+      <c r="A765" t="inlineStr">
+        <is>
+          <t>2026-08-08T17:05:13</t>
+        </is>
+      </c>
+      <c r="B765" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C765" t="inlineStr">
+        <is>
+          <t>CountPickedReject14in</t>
+        </is>
+      </c>
+      <c r="D765" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E765" t="inlineStr"/>
+      <c r="F765" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g30</t>
+        </is>
+      </c>
+    </row>
+    <row r="766">
+      <c r="A766" t="inlineStr">
+        <is>
+          <t>2026-08-08T17:05:13</t>
+        </is>
+      </c>
+      <c r="B766" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C766" t="inlineStr">
+        <is>
+          <t>temp_dsi</t>
+        </is>
+      </c>
+      <c r="D766" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E766" t="inlineStr"/>
+      <c r="F766" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g31</t>
+        </is>
+      </c>
+    </row>
+    <row r="767">
+      <c r="A767" t="inlineStr">
+        <is>
+          <t>2026-08-08T17:05:13</t>
+        </is>
+      </c>
+      <c r="B767" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C767" t="inlineStr">
+        <is>
+          <t>temp_J1motor</t>
+        </is>
+      </c>
+      <c r="D767" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E767" t="inlineStr"/>
+      <c r="F767" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g32</t>
+        </is>
+      </c>
+    </row>
+    <row r="768">
+      <c r="A768" t="inlineStr">
+        <is>
+          <t>2026-08-08T17:05:13</t>
+        </is>
+      </c>
+      <c r="B768" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C768" t="inlineStr">
+        <is>
+          <t>temp_J4motor</t>
+        </is>
+      </c>
+      <c r="D768" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E768" t="inlineStr"/>
+      <c r="F768" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g35</t>
+        </is>
+      </c>
+    </row>
+    <row r="769">
+      <c r="A769" t="inlineStr">
+        <is>
+          <t>2026-08-08T17:05:13</t>
+        </is>
+      </c>
+      <c r="B769" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C769" t="inlineStr">
+        <is>
+          <t>temp_J6motor</t>
+        </is>
+      </c>
+      <c r="D769" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E769" t="inlineStr"/>
+      <c r="F769" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g37</t>
+        </is>
+      </c>
+    </row>
+    <row r="770">
+      <c r="A770" t="inlineStr">
+        <is>
+          <t>2026-08-08T17:05:13</t>
+        </is>
+      </c>
+      <c r="B770" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C770" t="inlineStr">
+        <is>
+          <t>CountPickedRejectOTM</t>
+        </is>
+      </c>
+      <c r="D770" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E770" t="inlineStr"/>
+      <c r="F770" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g38</t>
+        </is>
+      </c>
+    </row>
+    <row r="771">
+      <c r="A771" t="inlineStr">
+        <is>
+          <t>2026-08-08T17:05:13</t>
+        </is>
+      </c>
+      <c r="B771" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C771" t="inlineStr">
+        <is>
+          <t>CountPickedRejectPandral</t>
+        </is>
+      </c>
+      <c r="D771" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E771" t="inlineStr"/>
+      <c r="F771" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g39</t>
+        </is>
+      </c>
+    </row>
+    <row r="772">
+      <c r="A772" t="inlineStr">
+        <is>
+          <t>2026-08-08T17:06:00</t>
+        </is>
+      </c>
+      <c r="B772" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C772" t="inlineStr">
+        <is>
+          <t>_1st_SCAN</t>
+        </is>
+      </c>
+      <c r="D772" t="b">
+        <v>0</v>
+      </c>
+      <c r="E772" t="n">
+        <v>11</v>
+      </c>
+      <c r="F772" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="773">
+      <c r="A773" t="inlineStr">
+        <is>
+          <t>2026-08-08T17:06:00</t>
+        </is>
+      </c>
+      <c r="B773" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C773" t="inlineStr">
+        <is>
+          <t>TieDetectOffset_B</t>
+        </is>
+      </c>
+      <c r="D773" t="b">
+        <v>0</v>
+      </c>
+      <c r="E773" t="n">
+        <v>11</v>
+      </c>
+      <c r="F773" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="774">
+      <c r="A774" t="inlineStr">
+        <is>
+          <t>2026-08-08T17:06:00</t>
+        </is>
+      </c>
+      <c r="B774" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C774" t="inlineStr">
+        <is>
+          <t>Tie Detector</t>
+        </is>
+      </c>
+      <c r="D774" t="b">
+        <v>0</v>
+      </c>
+      <c r="E774" t="n">
+        <v>11</v>
+      </c>
+      <c r="F774" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="775">
+      <c r="A775" t="inlineStr">
+        <is>
+          <t>2026-08-08T17:06:00</t>
+        </is>
+      </c>
+      <c r="B775" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C775" t="inlineStr">
+        <is>
+          <t>TPS Full</t>
+        </is>
+      </c>
+      <c r="D775" t="b">
+        <v>0</v>
+      </c>
+      <c r="E775" t="n">
+        <v>11</v>
+      </c>
+      <c r="F775" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="776">
+      <c r="A776" t="inlineStr">
+        <is>
+          <t>2026-08-08T17:06:00</t>
+        </is>
+      </c>
+      <c r="B776" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C776" t="inlineStr">
+        <is>
+          <t>TieDetectOffset_A</t>
+        </is>
+      </c>
+      <c r="D776" t="b">
+        <v>0</v>
+      </c>
+      <c r="E776" t="n">
+        <v>11</v>
+      </c>
+      <c r="F776" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="777">
+      <c r="A777" t="inlineStr">
+        <is>
+          <t>2026-08-08T17:06:00</t>
+        </is>
+      </c>
+      <c r="B777" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C777" t="inlineStr">
+        <is>
+          <t>TPS Connected</t>
+        </is>
+      </c>
+      <c r="D777" t="b">
+        <v>0</v>
+      </c>
+      <c r="E777" t="n">
+        <v>11</v>
+      </c>
+      <c r="F777" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="778">
+      <c r="A778" t="inlineStr">
+        <is>
+          <t>2026-08-08T17:06:00</t>
+        </is>
+      </c>
+      <c r="B778" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C778" t="inlineStr">
+        <is>
+          <t>TPS_Enable_ Button</t>
+        </is>
+      </c>
+      <c r="D778" t="b">
+        <v>0</v>
+      </c>
+      <c r="E778" t="n">
+        <v>11</v>
+      </c>
+      <c r="F778" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="779">
+      <c r="A779" t="inlineStr">
+        <is>
+          <t>2026-08-08T17:06:00</t>
+        </is>
+      </c>
+      <c r="B779" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C779" t="inlineStr">
+        <is>
+          <t>AirEagle Eject Plate</t>
+        </is>
+      </c>
+      <c r="D779" t="b">
+        <v>0</v>
+      </c>
+      <c r="E779" t="n">
+        <v>11</v>
+      </c>
+      <c r="F779" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="780">
+      <c r="A780" t="inlineStr">
+        <is>
+          <t>2026-08-08T17:06:00</t>
+        </is>
+      </c>
+      <c r="B780" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C780" t="inlineStr">
+        <is>
+          <t>tk_Cycle</t>
+        </is>
+      </c>
+      <c r="D780" t="b">
+        <v>0</v>
+      </c>
+      <c r="E780" t="n">
+        <v>11</v>
+      </c>
+      <c r="F780" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="781">
+      <c r="A781" t="inlineStr">
+        <is>
+          <t>2026-08-08T17:06:00</t>
+        </is>
+      </c>
+      <c r="B781" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C781" t="inlineStr">
+        <is>
+          <t>Servos_Enabled</t>
+        </is>
+      </c>
+      <c r="D781" t="b">
+        <v>0</v>
+      </c>
+      <c r="E781" t="n">
+        <v>11</v>
+      </c>
+      <c r="F781" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="782">
+      <c r="A782" t="inlineStr">
+        <is>
+          <t>2026-08-08T17:06:00</t>
+        </is>
+      </c>
+      <c r="B782" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C782" t="inlineStr">
+        <is>
+          <t>TPS Enabled</t>
+        </is>
+      </c>
+      <c r="D782" t="b">
+        <v>0</v>
+      </c>
+      <c r="E782" t="n">
+        <v>11</v>
+      </c>
+      <c r="F782" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="783">
+      <c r="A783" t="inlineStr">
+        <is>
+          <t>2026-08-08T17:06:00</t>
+        </is>
+      </c>
+      <c r="B783" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C783" t="inlineStr">
+        <is>
+          <t>tk_Abort</t>
+        </is>
+      </c>
+      <c r="D783" t="b">
+        <v>0</v>
+      </c>
+      <c r="E783" t="n">
+        <v>11</v>
+      </c>
+      <c r="F783" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="784">
+      <c r="A784" t="inlineStr">
+        <is>
+          <t>2026-08-08T17:06:00</t>
+        </is>
+      </c>
+      <c r="B784" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C784" t="inlineStr">
+        <is>
+          <t>Robot_isMoving</t>
+        </is>
+      </c>
+      <c r="D784" t="b">
+        <v>0</v>
+      </c>
+      <c r="E784" t="n">
+        <v>11</v>
+      </c>
+      <c r="F784" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="785">
+      <c r="A785" t="inlineStr">
+        <is>
+          <t>2026-08-08T17:06:00</t>
+        </is>
+      </c>
+      <c r="B785" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C785" t="inlineStr">
+        <is>
+          <t>Eject Tie Plate</t>
+        </is>
+      </c>
+      <c r="D785" t="b">
+        <v>0</v>
+      </c>
+      <c r="E785" t="n">
+        <v>11</v>
+      </c>
+      <c r="F785" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="786">
+      <c r="A786" t="inlineStr">
+        <is>
+          <t>2026-08-08T17:06:00</t>
+        </is>
+      </c>
+      <c r="B786" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C786" t="inlineStr">
+        <is>
+          <t>TPS BACKUP ALARM</t>
+        </is>
+      </c>
+      <c r="D786" t="b">
+        <v>0</v>
+      </c>
+      <c r="E786" t="n">
+        <v>11</v>
+      </c>
+      <c r="F786" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="787">
+      <c r="A787" t="inlineStr">
+        <is>
+          <t>2026-08-08T17:06:00</t>
+        </is>
+      </c>
+      <c r="B787" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C787" t="inlineStr">
+        <is>
+          <t>14in Job</t>
+        </is>
+      </c>
+      <c r="D787" t="b">
+        <v>1</v>
+      </c>
+      <c r="E787" t="n">
+        <v>11</v>
+      </c>
+      <c r="F787" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="788">
+      <c r="A788" t="inlineStr">
+        <is>
+          <t>2026-08-08T17:06:00</t>
+        </is>
+      </c>
+      <c r="B788" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C788" t="inlineStr">
+        <is>
+          <t>18in Job</t>
+        </is>
+      </c>
+      <c r="D788" t="b">
+        <v>0</v>
+      </c>
+      <c r="E788" t="n">
+        <v>11</v>
+      </c>
+      <c r="F788" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="789">
+      <c r="A789" t="inlineStr">
+        <is>
+          <t>2026-08-08T17:06:00</t>
+        </is>
+      </c>
+      <c r="B789" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C789" t="inlineStr">
+        <is>
+          <t>Pandral Job</t>
+        </is>
+      </c>
+      <c r="D789" t="b">
+        <v>0</v>
+      </c>
+      <c r="E789" t="n">
+        <v>11</v>
+      </c>
+      <c r="F789" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="790">
+      <c r="A790" t="inlineStr">
+        <is>
+          <t>2026-08-08T17:06:00</t>
+        </is>
+      </c>
+      <c r="B790" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C790" t="inlineStr">
+        <is>
+          <t>DoubleLay Job</t>
+        </is>
+      </c>
+      <c r="D790" t="b">
+        <v>0</v>
+      </c>
+      <c r="E790" t="n">
+        <v>11</v>
+      </c>
+      <c r="F790" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="791">
+      <c r="A791" t="inlineStr">
+        <is>
+          <t>2026-08-08T17:06:00</t>
+        </is>
+      </c>
+      <c r="B791" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C791" t="inlineStr">
+        <is>
+          <t>TPSjam_FLAG</t>
+        </is>
+      </c>
+      <c r="D791" t="b">
+        <v>0</v>
+      </c>
+      <c r="E791" t="n">
+        <v>11</v>
+      </c>
+      <c r="F791" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="792">
+      <c r="A792" t="inlineStr">
+        <is>
+          <t>2026-08-08T17:06:00</t>
+        </is>
+      </c>
+      <c r="B792" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C792" t="inlineStr">
+        <is>
+          <t>RoCalRequest</t>
+        </is>
+      </c>
+      <c r="D792" t="b">
+        <v>0</v>
+      </c>
+      <c r="E792" t="n">
+        <v>11</v>
+      </c>
+      <c r="F792" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="793">
+      <c r="A793" t="inlineStr">
+        <is>
+          <t>2026-08-08T17:06:00</t>
+        </is>
+      </c>
+      <c r="B793" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C793" t="inlineStr">
+        <is>
+          <t>tkCycle_TotalSeconds</t>
+        </is>
+      </c>
+      <c r="D793" t="n">
+        <v>0</v>
+      </c>
+      <c r="E793" t="n">
+        <v>9</v>
+      </c>
+      <c r="F793" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="794">
+      <c r="A794" t="inlineStr">
+        <is>
+          <t>2026-08-08T17:06:00</t>
+        </is>
+      </c>
+      <c r="B794" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C794" t="inlineStr">
+        <is>
+          <t>tkCycle_NoMoveSec</t>
+        </is>
+      </c>
+      <c r="D794" t="n">
+        <v>0</v>
+      </c>
+      <c r="E794" t="n">
+        <v>9</v>
+      </c>
+      <c r="F794" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="795">
+      <c r="A795" t="inlineStr">
+        <is>
+          <t>2026-08-08T17:06:00</t>
+        </is>
+      </c>
+      <c r="B795" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C795" t="inlineStr">
+        <is>
+          <t>tkCycle_MoveSeconds</t>
+        </is>
+      </c>
+      <c r="D795" t="n">
+        <v>0</v>
+      </c>
+      <c r="E795" t="n">
+        <v>9</v>
+      </c>
+      <c r="F795" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="796">
+      <c r="A796" t="inlineStr">
+        <is>
+          <t>2026-08-08T17:06:00</t>
+        </is>
+      </c>
+      <c r="B796" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C796" t="inlineStr">
+        <is>
+          <t>Percent time moveing</t>
+        </is>
+      </c>
+      <c r="D796" t="n">
+        <v>0</v>
+      </c>
+      <c r="E796" t="n">
+        <v>9</v>
+      </c>
+      <c r="F796" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="797">
+      <c r="A797" t="inlineStr">
+        <is>
+          <t>2026-08-08T17:06:00</t>
+        </is>
+      </c>
+      <c r="B797" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C797" t="inlineStr">
+        <is>
+          <t>Percent time not moving</t>
+        </is>
+      </c>
+      <c r="D797" t="n">
+        <v>0</v>
+      </c>
+      <c r="E797" t="n">
+        <v>9</v>
+      </c>
+      <c r="F797" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="798">
+      <c r="A798" t="inlineStr">
+        <is>
+          <t>2026-08-08T17:06:00</t>
+        </is>
+      </c>
+      <c r="B798" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C798" t="inlineStr">
+        <is>
+          <t>TotalPickPartsCount</t>
+        </is>
+      </c>
+      <c r="D798" t="n">
+        <v>0</v>
+      </c>
+      <c r="E798" t="n">
+        <v>9</v>
+      </c>
+      <c r="F798" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="799">
+      <c r="A799" t="inlineStr">
+        <is>
+          <t>2026-08-08T17:06:00</t>
+        </is>
+      </c>
+      <c r="B799" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C799" t="inlineStr">
+        <is>
+          <t>RejectPartsCount</t>
+        </is>
+      </c>
+      <c r="D799" t="n">
+        <v>0</v>
+      </c>
+      <c r="E799" t="n">
+        <v>9</v>
+      </c>
+      <c r="F799" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="800">
+      <c r="A800" t="inlineStr">
+        <is>
+          <t>2026-08-08T17:06:00</t>
+        </is>
+      </c>
+      <c r="B800" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C800" t="inlineStr">
+        <is>
+          <t>AcceptsPartsCount</t>
+        </is>
+      </c>
+      <c r="D800" t="n">
+        <v>0</v>
+      </c>
+      <c r="E800" t="n">
+        <v>9</v>
+      </c>
+      <c r="F800" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="801">
+      <c r="A801" t="inlineStr">
+        <is>
+          <t>2026-08-08T17:06:00</t>
+        </is>
+      </c>
+      <c r="B801" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C801" t="inlineStr">
+        <is>
+          <t>percentCount_accept</t>
+        </is>
+      </c>
+      <c r="D801" t="n">
+        <v>0</v>
+      </c>
+      <c r="E801" t="n">
+        <v>9</v>
+      </c>
+      <c r="F801" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="802">
+      <c r="A802" t="inlineStr">
+        <is>
+          <t>2026-08-08T17:06:00</t>
+        </is>
+      </c>
+      <c r="B802" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C802" t="inlineStr">
+        <is>
+          <t>percentCount_reject</t>
+        </is>
+      </c>
+      <c r="D802" t="n">
+        <v>0</v>
+      </c>
+      <c r="E802" t="n">
+        <v>9</v>
+      </c>
+      <c r="F802" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="803">
+      <c r="A803" t="inlineStr">
+        <is>
+          <t>2026-08-08T17:06:00</t>
+        </is>
+      </c>
+      <c r="B803" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C803" t="inlineStr">
+        <is>
+          <t>Avg Parts per min_total</t>
+        </is>
+      </c>
+      <c r="D803" t="n">
+        <v>0</v>
+      </c>
+      <c r="E803" t="n">
+        <v>9</v>
+      </c>
+      <c r="F803" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="804">
+      <c r="A804" t="inlineStr">
+        <is>
+          <t>2026-08-08T17:06:00</t>
+        </is>
+      </c>
+      <c r="B804" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C804" t="inlineStr">
+        <is>
+          <t>TotalPickedParts</t>
+        </is>
+      </c>
+      <c r="D804" t="n">
+        <v>0</v>
+      </c>
+      <c r="E804" t="n">
+        <v>3</v>
+      </c>
+      <c r="F804" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="805">
+      <c r="A805" t="inlineStr">
+        <is>
+          <t>2026-08-08T17:06:00</t>
+        </is>
+      </c>
+      <c r="B805" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C805" t="inlineStr">
+        <is>
+          <t>TotalPickedAcceptParts</t>
+        </is>
+      </c>
+      <c r="D805" t="n">
+        <v>0</v>
+      </c>
+      <c r="E805" t="n">
+        <v>3</v>
+      </c>
+      <c r="F805" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="806">
+      <c r="A806" t="inlineStr">
+        <is>
+          <t>2026-08-08T17:06:00</t>
+        </is>
+      </c>
+      <c r="B806" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C806" t="inlineStr">
+        <is>
+          <t>TotalPickedRejectParts</t>
+        </is>
+      </c>
+      <c r="D806" t="n">
+        <v>0</v>
+      </c>
+      <c r="E806" t="n">
+        <v>3</v>
+      </c>
+      <c r="F806" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="807">
+      <c r="A807" t="inlineStr">
+        <is>
+          <t>2026-08-08T17:06:00</t>
+        </is>
+      </c>
+      <c r="B807" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C807" t="inlineStr">
+        <is>
+          <t>TotalTiePlatesLaid</t>
+        </is>
+      </c>
+      <c r="D807" t="n">
+        <v>0</v>
+      </c>
+      <c r="E807" t="n">
+        <v>3</v>
+      </c>
+      <c r="F807" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="808">
+      <c r="A808" t="inlineStr">
+        <is>
+          <t>2026-08-08T17:06:00</t>
+        </is>
+      </c>
+      <c r="B808" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C808" t="inlineStr">
+        <is>
+          <t>Daily_TotalLaidPlates</t>
+        </is>
+      </c>
+      <c r="D808" t="n">
+        <v>0</v>
+      </c>
+      <c r="E808" t="n">
+        <v>3</v>
+      </c>
+      <c r="F808" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="809">
+      <c r="A809" t="inlineStr">
+        <is>
+          <t>2026-08-08T17:06:00</t>
+        </is>
+      </c>
+      <c r="B809" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C809" t="inlineStr">
+        <is>
+          <t>CountPicked14in</t>
+        </is>
+      </c>
+      <c r="D809" t="n">
+        <v>0</v>
+      </c>
+      <c r="E809" t="n">
+        <v>3</v>
+      </c>
+      <c r="F809" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="810">
+      <c r="A810" t="inlineStr">
+        <is>
+          <t>2026-08-08T17:06:00</t>
+        </is>
+      </c>
+      <c r="B810" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C810" t="inlineStr">
+        <is>
+          <t>CountPicked18in</t>
+        </is>
+      </c>
+      <c r="D810" t="n">
+        <v>0</v>
+      </c>
+      <c r="E810" t="n">
+        <v>3</v>
+      </c>
+      <c r="F810" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="811">
+      <c r="A811" t="inlineStr">
+        <is>
+          <t>2026-08-08T17:06:00</t>
+        </is>
+      </c>
+      <c r="B811" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C811" t="inlineStr">
+        <is>
+          <t>CountPickedPandral</t>
+        </is>
+      </c>
+      <c r="D811" t="n">
+        <v>0</v>
+      </c>
+      <c r="E811" t="n">
+        <v>3</v>
+      </c>
+      <c r="F811" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="812">
+      <c r="A812" t="inlineStr">
+        <is>
+          <t>2026-08-08T17:06:00</t>
+        </is>
+      </c>
+      <c r="B812" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C812" t="inlineStr">
+        <is>
+          <t>CountPickedOTM</t>
+        </is>
+      </c>
+      <c r="D812" t="n">
+        <v>0</v>
+      </c>
+      <c r="E812" t="n">
+        <v>3</v>
+      </c>
+      <c r="F812" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="813">
+      <c r="A813" t="inlineStr">
+        <is>
+          <t>2026-08-08T17:06:00</t>
+        </is>
+      </c>
+      <c r="B813" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C813" t="inlineStr">
+        <is>
+          <t>RoCals</t>
+        </is>
+      </c>
+      <c r="D813" t="n">
+        <v>0</v>
+      </c>
+      <c r="E813" t="n">
+        <v>3</v>
+      </c>
+      <c r="F813" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="814">
+      <c r="A814" t="inlineStr">
+        <is>
+          <t>2026-08-08T17:06:00</t>
+        </is>
+      </c>
+      <c r="B814" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C814" t="inlineStr">
+        <is>
+          <t>TPS_JamsUsr</t>
+        </is>
+      </c>
+      <c r="D814" t="n">
+        <v>0</v>
+      </c>
+      <c r="E814" t="n">
+        <v>3</v>
+      </c>
+      <c r="F814" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="815">
+      <c r="A815" t="inlineStr">
+        <is>
+          <t>2026-08-08T17:06:00</t>
+        </is>
+      </c>
+      <c r="B815" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C815" t="inlineStr">
+        <is>
+          <t>TPS_JamsMASTER</t>
+        </is>
+      </c>
+      <c r="D815" t="n">
+        <v>0</v>
+      </c>
+      <c r="E815" t="n">
+        <v>3</v>
+      </c>
+      <c r="F815" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="816">
+      <c r="A816" t="inlineStr">
+        <is>
+          <t>2026-08-08T17:06:00</t>
+        </is>
+      </c>
+      <c r="B816" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C816" t="inlineStr">
+        <is>
+          <t>ABORT_Master</t>
+        </is>
+      </c>
+      <c r="D816" t="n">
+        <v>0</v>
+      </c>
+      <c r="E816" t="n">
+        <v>3</v>
+      </c>
+      <c r="F816" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Log MQTT data 2026-08-08 18:06 UTC
</commit_message>
<xml_diff>
--- a/logs/raiv_tracker_2026-08-08.xlsx
+++ b/logs/raiv_tracker_2026-08-08.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F816"/>
+  <dimension ref="A1:F946"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -20629,7 +20629,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E732" t="inlineStr"/>
       <c r="F732" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g2</t>
@@ -20657,7 +20656,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E733" t="inlineStr"/>
       <c r="F733" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g3</t>
@@ -20685,7 +20683,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E734" t="inlineStr"/>
       <c r="F734" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g4</t>
@@ -20713,7 +20710,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E735" t="inlineStr"/>
       <c r="F735" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g5</t>
@@ -20741,7 +20737,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E736" t="inlineStr"/>
       <c r="F736" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g6</t>
@@ -20769,7 +20764,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E737" t="inlineStr"/>
       <c r="F737" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g7</t>
@@ -20797,7 +20791,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E738" t="inlineStr"/>
       <c r="F738" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g13</t>
@@ -20825,7 +20818,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E739" t="inlineStr"/>
       <c r="F739" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g15</t>
@@ -20853,7 +20845,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E740" t="inlineStr"/>
       <c r="F740" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g17</t>
@@ -20881,7 +20872,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E741" t="inlineStr"/>
       <c r="F741" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g18</t>
@@ -20909,7 +20899,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E742" t="inlineStr"/>
       <c r="F742" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g19</t>
@@ -20937,7 +20926,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E743" t="inlineStr"/>
       <c r="F743" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g22</t>
@@ -20965,7 +20953,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E744" t="inlineStr"/>
       <c r="F744" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g23</t>
@@ -20993,7 +20980,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E745" t="inlineStr"/>
       <c r="F745" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g24</t>
@@ -21021,7 +21007,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E746" t="inlineStr"/>
       <c r="F746" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g25</t>
@@ -21049,7 +21034,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E747" t="inlineStr"/>
       <c r="F747" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g33</t>
@@ -21077,7 +21061,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E748" t="inlineStr"/>
       <c r="F748" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g34</t>
@@ -21105,7 +21088,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E749" t="inlineStr"/>
       <c r="F749" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g36</t>
@@ -21133,7 +21115,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E750" t="inlineStr"/>
       <c r="F750" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g40</t>
@@ -21161,7 +21142,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E751" t="inlineStr"/>
       <c r="F751" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g1</t>
@@ -21189,7 +21169,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E752" t="inlineStr"/>
       <c r="F752" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g8</t>
@@ -21217,7 +21196,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E753" t="inlineStr"/>
       <c r="F753" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g9</t>
@@ -21245,7 +21223,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E754" t="inlineStr"/>
       <c r="F754" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g10</t>
@@ -21273,7 +21250,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E755" t="inlineStr"/>
       <c r="F755" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g11</t>
@@ -21301,7 +21277,6 @@
           <t>1</t>
         </is>
       </c>
-      <c r="E756" t="inlineStr"/>
       <c r="F756" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g12</t>
@@ -21329,7 +21304,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E757" t="inlineStr"/>
       <c r="F757" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g14</t>
@@ -21357,7 +21331,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E758" t="inlineStr"/>
       <c r="F758" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g16</t>
@@ -21385,7 +21358,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E759" t="inlineStr"/>
       <c r="F759" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g20</t>
@@ -21413,7 +21385,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E760" t="inlineStr"/>
       <c r="F760" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g21</t>
@@ -21441,7 +21412,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E761" t="inlineStr"/>
       <c r="F761" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g26</t>
@@ -21469,7 +21439,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E762" t="inlineStr"/>
       <c r="F762" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g27</t>
@@ -21497,7 +21466,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E763" t="inlineStr"/>
       <c r="F763" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g28</t>
@@ -21525,7 +21493,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E764" t="inlineStr"/>
       <c r="F764" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g29</t>
@@ -21553,7 +21520,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E765" t="inlineStr"/>
       <c r="F765" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g30</t>
@@ -21581,7 +21547,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E766" t="inlineStr"/>
       <c r="F766" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g31</t>
@@ -21609,7 +21574,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E767" t="inlineStr"/>
       <c r="F767" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g32</t>
@@ -21637,7 +21601,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E768" t="inlineStr"/>
       <c r="F768" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g35</t>
@@ -21665,7 +21628,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E769" t="inlineStr"/>
       <c r="F769" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g37</t>
@@ -21693,7 +21655,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E770" t="inlineStr"/>
       <c r="F770" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g38</t>
@@ -21721,7 +21682,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E771" t="inlineStr"/>
       <c r="F771" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g39</t>
@@ -22983,6 +22943,3646 @@
         <v>3</v>
       </c>
       <c r="F816" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="817">
+      <c r="A817" t="inlineStr">
+        <is>
+          <t>2026-08-08T18:05:00</t>
+        </is>
+      </c>
+      <c r="B817" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C817" t="inlineStr">
+        <is>
+          <t>_1st_SCAN</t>
+        </is>
+      </c>
+      <c r="D817" t="b">
+        <v>0</v>
+      </c>
+      <c r="E817" t="n">
+        <v>11</v>
+      </c>
+      <c r="F817" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="818">
+      <c r="A818" t="inlineStr">
+        <is>
+          <t>2026-08-08T18:05:00</t>
+        </is>
+      </c>
+      <c r="B818" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C818" t="inlineStr">
+        <is>
+          <t>TieDetectOffset_B</t>
+        </is>
+      </c>
+      <c r="D818" t="b">
+        <v>0</v>
+      </c>
+      <c r="E818" t="n">
+        <v>11</v>
+      </c>
+      <c r="F818" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="819">
+      <c r="A819" t="inlineStr">
+        <is>
+          <t>2026-08-08T18:05:00</t>
+        </is>
+      </c>
+      <c r="B819" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C819" t="inlineStr">
+        <is>
+          <t>Tie Detector</t>
+        </is>
+      </c>
+      <c r="D819" t="b">
+        <v>0</v>
+      </c>
+      <c r="E819" t="n">
+        <v>11</v>
+      </c>
+      <c r="F819" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="820">
+      <c r="A820" t="inlineStr">
+        <is>
+          <t>2026-08-08T18:05:00</t>
+        </is>
+      </c>
+      <c r="B820" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C820" t="inlineStr">
+        <is>
+          <t>TPS Full</t>
+        </is>
+      </c>
+      <c r="D820" t="b">
+        <v>0</v>
+      </c>
+      <c r="E820" t="n">
+        <v>11</v>
+      </c>
+      <c r="F820" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="821">
+      <c r="A821" t="inlineStr">
+        <is>
+          <t>2026-08-08T18:05:00</t>
+        </is>
+      </c>
+      <c r="B821" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C821" t="inlineStr">
+        <is>
+          <t>TieDetectOffset_A</t>
+        </is>
+      </c>
+      <c r="D821" t="b">
+        <v>0</v>
+      </c>
+      <c r="E821" t="n">
+        <v>11</v>
+      </c>
+      <c r="F821" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="822">
+      <c r="A822" t="inlineStr">
+        <is>
+          <t>2026-08-08T18:05:00</t>
+        </is>
+      </c>
+      <c r="B822" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C822" t="inlineStr">
+        <is>
+          <t>TPS Connected</t>
+        </is>
+      </c>
+      <c r="D822" t="b">
+        <v>0</v>
+      </c>
+      <c r="E822" t="n">
+        <v>11</v>
+      </c>
+      <c r="F822" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="823">
+      <c r="A823" t="inlineStr">
+        <is>
+          <t>2026-08-08T18:05:00</t>
+        </is>
+      </c>
+      <c r="B823" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C823" t="inlineStr">
+        <is>
+          <t>TPS_Enable_ Button</t>
+        </is>
+      </c>
+      <c r="D823" t="b">
+        <v>0</v>
+      </c>
+      <c r="E823" t="n">
+        <v>11</v>
+      </c>
+      <c r="F823" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="824">
+      <c r="A824" t="inlineStr">
+        <is>
+          <t>2026-08-08T18:05:00</t>
+        </is>
+      </c>
+      <c r="B824" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C824" t="inlineStr">
+        <is>
+          <t>AirEagle Eject Plate</t>
+        </is>
+      </c>
+      <c r="D824" t="b">
+        <v>0</v>
+      </c>
+      <c r="E824" t="n">
+        <v>11</v>
+      </c>
+      <c r="F824" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="825">
+      <c r="A825" t="inlineStr">
+        <is>
+          <t>2026-08-08T18:05:00</t>
+        </is>
+      </c>
+      <c r="B825" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C825" t="inlineStr">
+        <is>
+          <t>tk_Cycle</t>
+        </is>
+      </c>
+      <c r="D825" t="b">
+        <v>0</v>
+      </c>
+      <c r="E825" t="n">
+        <v>11</v>
+      </c>
+      <c r="F825" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="826">
+      <c r="A826" t="inlineStr">
+        <is>
+          <t>2026-08-08T18:05:00</t>
+        </is>
+      </c>
+      <c r="B826" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C826" t="inlineStr">
+        <is>
+          <t>Servos_Enabled</t>
+        </is>
+      </c>
+      <c r="D826" t="b">
+        <v>0</v>
+      </c>
+      <c r="E826" t="n">
+        <v>11</v>
+      </c>
+      <c r="F826" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="827">
+      <c r="A827" t="inlineStr">
+        <is>
+          <t>2026-08-08T18:05:00</t>
+        </is>
+      </c>
+      <c r="B827" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C827" t="inlineStr">
+        <is>
+          <t>TPS Enabled</t>
+        </is>
+      </c>
+      <c r="D827" t="b">
+        <v>0</v>
+      </c>
+      <c r="E827" t="n">
+        <v>11</v>
+      </c>
+      <c r="F827" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="828">
+      <c r="A828" t="inlineStr">
+        <is>
+          <t>2026-08-08T18:05:00</t>
+        </is>
+      </c>
+      <c r="B828" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C828" t="inlineStr">
+        <is>
+          <t>tk_Abort</t>
+        </is>
+      </c>
+      <c r="D828" t="b">
+        <v>0</v>
+      </c>
+      <c r="E828" t="n">
+        <v>11</v>
+      </c>
+      <c r="F828" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="829">
+      <c r="A829" t="inlineStr">
+        <is>
+          <t>2026-08-08T18:05:00</t>
+        </is>
+      </c>
+      <c r="B829" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C829" t="inlineStr">
+        <is>
+          <t>Robot_isMoving</t>
+        </is>
+      </c>
+      <c r="D829" t="b">
+        <v>0</v>
+      </c>
+      <c r="E829" t="n">
+        <v>11</v>
+      </c>
+      <c r="F829" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="830">
+      <c r="A830" t="inlineStr">
+        <is>
+          <t>2026-08-08T18:05:00</t>
+        </is>
+      </c>
+      <c r="B830" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C830" t="inlineStr">
+        <is>
+          <t>Eject Tie Plate</t>
+        </is>
+      </c>
+      <c r="D830" t="b">
+        <v>0</v>
+      </c>
+      <c r="E830" t="n">
+        <v>11</v>
+      </c>
+      <c r="F830" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="831">
+      <c r="A831" t="inlineStr">
+        <is>
+          <t>2026-08-08T18:05:00</t>
+        </is>
+      </c>
+      <c r="B831" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C831" t="inlineStr">
+        <is>
+          <t>TPS BACKUP ALARM</t>
+        </is>
+      </c>
+      <c r="D831" t="b">
+        <v>0</v>
+      </c>
+      <c r="E831" t="n">
+        <v>11</v>
+      </c>
+      <c r="F831" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="832">
+      <c r="A832" t="inlineStr">
+        <is>
+          <t>2026-08-08T18:05:00</t>
+        </is>
+      </c>
+      <c r="B832" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C832" t="inlineStr">
+        <is>
+          <t>14in Job</t>
+        </is>
+      </c>
+      <c r="D832" t="b">
+        <v>1</v>
+      </c>
+      <c r="E832" t="n">
+        <v>11</v>
+      </c>
+      <c r="F832" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="833">
+      <c r="A833" t="inlineStr">
+        <is>
+          <t>2026-08-08T18:05:00</t>
+        </is>
+      </c>
+      <c r="B833" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C833" t="inlineStr">
+        <is>
+          <t>18in Job</t>
+        </is>
+      </c>
+      <c r="D833" t="b">
+        <v>0</v>
+      </c>
+      <c r="E833" t="n">
+        <v>11</v>
+      </c>
+      <c r="F833" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="834">
+      <c r="A834" t="inlineStr">
+        <is>
+          <t>2026-08-08T18:05:00</t>
+        </is>
+      </c>
+      <c r="B834" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C834" t="inlineStr">
+        <is>
+          <t>Pandral Job</t>
+        </is>
+      </c>
+      <c r="D834" t="b">
+        <v>0</v>
+      </c>
+      <c r="E834" t="n">
+        <v>11</v>
+      </c>
+      <c r="F834" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="835">
+      <c r="A835" t="inlineStr">
+        <is>
+          <t>2026-08-08T18:05:00</t>
+        </is>
+      </c>
+      <c r="B835" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C835" t="inlineStr">
+        <is>
+          <t>DoubleLay Job</t>
+        </is>
+      </c>
+      <c r="D835" t="b">
+        <v>0</v>
+      </c>
+      <c r="E835" t="n">
+        <v>11</v>
+      </c>
+      <c r="F835" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="836">
+      <c r="A836" t="inlineStr">
+        <is>
+          <t>2026-08-08T18:05:00</t>
+        </is>
+      </c>
+      <c r="B836" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C836" t="inlineStr">
+        <is>
+          <t>TPSjam_FLAG</t>
+        </is>
+      </c>
+      <c r="D836" t="b">
+        <v>0</v>
+      </c>
+      <c r="E836" t="n">
+        <v>11</v>
+      </c>
+      <c r="F836" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="837">
+      <c r="A837" t="inlineStr">
+        <is>
+          <t>2026-08-08T18:05:00</t>
+        </is>
+      </c>
+      <c r="B837" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C837" t="inlineStr">
+        <is>
+          <t>RoCalRequest</t>
+        </is>
+      </c>
+      <c r="D837" t="b">
+        <v>0</v>
+      </c>
+      <c r="E837" t="n">
+        <v>11</v>
+      </c>
+      <c r="F837" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="838">
+      <c r="A838" t="inlineStr">
+        <is>
+          <t>2026-08-08T18:05:00</t>
+        </is>
+      </c>
+      <c r="B838" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C838" t="inlineStr">
+        <is>
+          <t>tkCycle_TotalSeconds</t>
+        </is>
+      </c>
+      <c r="D838" t="n">
+        <v>0</v>
+      </c>
+      <c r="E838" t="n">
+        <v>9</v>
+      </c>
+      <c r="F838" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="839">
+      <c r="A839" t="inlineStr">
+        <is>
+          <t>2026-08-08T18:05:00</t>
+        </is>
+      </c>
+      <c r="B839" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C839" t="inlineStr">
+        <is>
+          <t>tkCycle_NoMoveSec</t>
+        </is>
+      </c>
+      <c r="D839" t="n">
+        <v>0</v>
+      </c>
+      <c r="E839" t="n">
+        <v>9</v>
+      </c>
+      <c r="F839" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="840">
+      <c r="A840" t="inlineStr">
+        <is>
+          <t>2026-08-08T18:05:00</t>
+        </is>
+      </c>
+      <c r="B840" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C840" t="inlineStr">
+        <is>
+          <t>tkCycle_MoveSeconds</t>
+        </is>
+      </c>
+      <c r="D840" t="n">
+        <v>0</v>
+      </c>
+      <c r="E840" t="n">
+        <v>9</v>
+      </c>
+      <c r="F840" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="841">
+      <c r="A841" t="inlineStr">
+        <is>
+          <t>2026-08-08T18:05:00</t>
+        </is>
+      </c>
+      <c r="B841" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C841" t="inlineStr">
+        <is>
+          <t>Percent time moveing</t>
+        </is>
+      </c>
+      <c r="D841" t="n">
+        <v>0</v>
+      </c>
+      <c r="E841" t="n">
+        <v>9</v>
+      </c>
+      <c r="F841" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="842">
+      <c r="A842" t="inlineStr">
+        <is>
+          <t>2026-08-08T18:05:00</t>
+        </is>
+      </c>
+      <c r="B842" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C842" t="inlineStr">
+        <is>
+          <t>Percent time not moving</t>
+        </is>
+      </c>
+      <c r="D842" t="n">
+        <v>0</v>
+      </c>
+      <c r="E842" t="n">
+        <v>9</v>
+      </c>
+      <c r="F842" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="843">
+      <c r="A843" t="inlineStr">
+        <is>
+          <t>2026-08-08T18:05:00</t>
+        </is>
+      </c>
+      <c r="B843" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C843" t="inlineStr">
+        <is>
+          <t>TotalPickPartsCount</t>
+        </is>
+      </c>
+      <c r="D843" t="n">
+        <v>0</v>
+      </c>
+      <c r="E843" t="n">
+        <v>9</v>
+      </c>
+      <c r="F843" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="844">
+      <c r="A844" t="inlineStr">
+        <is>
+          <t>2026-08-08T18:05:00</t>
+        </is>
+      </c>
+      <c r="B844" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C844" t="inlineStr">
+        <is>
+          <t>RejectPartsCount</t>
+        </is>
+      </c>
+      <c r="D844" t="n">
+        <v>0</v>
+      </c>
+      <c r="E844" t="n">
+        <v>9</v>
+      </c>
+      <c r="F844" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="845">
+      <c r="A845" t="inlineStr">
+        <is>
+          <t>2026-08-08T18:05:00</t>
+        </is>
+      </c>
+      <c r="B845" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C845" t="inlineStr">
+        <is>
+          <t>AcceptsPartsCount</t>
+        </is>
+      </c>
+      <c r="D845" t="n">
+        <v>0</v>
+      </c>
+      <c r="E845" t="n">
+        <v>9</v>
+      </c>
+      <c r="F845" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="846">
+      <c r="A846" t="inlineStr">
+        <is>
+          <t>2026-08-08T18:05:00</t>
+        </is>
+      </c>
+      <c r="B846" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C846" t="inlineStr">
+        <is>
+          <t>percentCount_accept</t>
+        </is>
+      </c>
+      <c r="D846" t="n">
+        <v>0</v>
+      </c>
+      <c r="E846" t="n">
+        <v>9</v>
+      </c>
+      <c r="F846" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="847">
+      <c r="A847" t="inlineStr">
+        <is>
+          <t>2026-08-08T18:05:00</t>
+        </is>
+      </c>
+      <c r="B847" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C847" t="inlineStr">
+        <is>
+          <t>percentCount_reject</t>
+        </is>
+      </c>
+      <c r="D847" t="n">
+        <v>0</v>
+      </c>
+      <c r="E847" t="n">
+        <v>9</v>
+      </c>
+      <c r="F847" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="848">
+      <c r="A848" t="inlineStr">
+        <is>
+          <t>2026-08-08T18:05:00</t>
+        </is>
+      </c>
+      <c r="B848" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C848" t="inlineStr">
+        <is>
+          <t>Avg Parts per min_total</t>
+        </is>
+      </c>
+      <c r="D848" t="n">
+        <v>0</v>
+      </c>
+      <c r="E848" t="n">
+        <v>9</v>
+      </c>
+      <c r="F848" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="849">
+      <c r="A849" t="inlineStr">
+        <is>
+          <t>2026-08-08T18:05:00</t>
+        </is>
+      </c>
+      <c r="B849" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C849" t="inlineStr">
+        <is>
+          <t>TotalPickedParts</t>
+        </is>
+      </c>
+      <c r="D849" t="n">
+        <v>0</v>
+      </c>
+      <c r="E849" t="n">
+        <v>3</v>
+      </c>
+      <c r="F849" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="850">
+      <c r="A850" t="inlineStr">
+        <is>
+          <t>2026-08-08T18:05:00</t>
+        </is>
+      </c>
+      <c r="B850" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C850" t="inlineStr">
+        <is>
+          <t>TotalPickedAcceptParts</t>
+        </is>
+      </c>
+      <c r="D850" t="n">
+        <v>0</v>
+      </c>
+      <c r="E850" t="n">
+        <v>3</v>
+      </c>
+      <c r="F850" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="851">
+      <c r="A851" t="inlineStr">
+        <is>
+          <t>2026-08-08T18:05:00</t>
+        </is>
+      </c>
+      <c r="B851" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C851" t="inlineStr">
+        <is>
+          <t>TotalPickedRejectParts</t>
+        </is>
+      </c>
+      <c r="D851" t="n">
+        <v>0</v>
+      </c>
+      <c r="E851" t="n">
+        <v>3</v>
+      </c>
+      <c r="F851" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="852">
+      <c r="A852" t="inlineStr">
+        <is>
+          <t>2026-08-08T18:05:00</t>
+        </is>
+      </c>
+      <c r="B852" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C852" t="inlineStr">
+        <is>
+          <t>TotalTiePlatesLaid</t>
+        </is>
+      </c>
+      <c r="D852" t="n">
+        <v>0</v>
+      </c>
+      <c r="E852" t="n">
+        <v>3</v>
+      </c>
+      <c r="F852" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="853">
+      <c r="A853" t="inlineStr">
+        <is>
+          <t>2026-08-08T18:05:00</t>
+        </is>
+      </c>
+      <c r="B853" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C853" t="inlineStr">
+        <is>
+          <t>Daily_TotalLaidPlates</t>
+        </is>
+      </c>
+      <c r="D853" t="n">
+        <v>0</v>
+      </c>
+      <c r="E853" t="n">
+        <v>3</v>
+      </c>
+      <c r="F853" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="854">
+      <c r="A854" t="inlineStr">
+        <is>
+          <t>2026-08-08T18:05:00</t>
+        </is>
+      </c>
+      <c r="B854" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C854" t="inlineStr">
+        <is>
+          <t>CountPicked14in</t>
+        </is>
+      </c>
+      <c r="D854" t="n">
+        <v>0</v>
+      </c>
+      <c r="E854" t="n">
+        <v>3</v>
+      </c>
+      <c r="F854" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="855">
+      <c r="A855" t="inlineStr">
+        <is>
+          <t>2026-08-08T18:05:00</t>
+        </is>
+      </c>
+      <c r="B855" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C855" t="inlineStr">
+        <is>
+          <t>CountPicked18in</t>
+        </is>
+      </c>
+      <c r="D855" t="n">
+        <v>0</v>
+      </c>
+      <c r="E855" t="n">
+        <v>3</v>
+      </c>
+      <c r="F855" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="856">
+      <c r="A856" t="inlineStr">
+        <is>
+          <t>2026-08-08T18:05:00</t>
+        </is>
+      </c>
+      <c r="B856" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C856" t="inlineStr">
+        <is>
+          <t>CountPickedPandral</t>
+        </is>
+      </c>
+      <c r="D856" t="n">
+        <v>0</v>
+      </c>
+      <c r="E856" t="n">
+        <v>3</v>
+      </c>
+      <c r="F856" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="857">
+      <c r="A857" t="inlineStr">
+        <is>
+          <t>2026-08-08T18:05:00</t>
+        </is>
+      </c>
+      <c r="B857" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C857" t="inlineStr">
+        <is>
+          <t>CountPickedOTM</t>
+        </is>
+      </c>
+      <c r="D857" t="n">
+        <v>0</v>
+      </c>
+      <c r="E857" t="n">
+        <v>3</v>
+      </c>
+      <c r="F857" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="858">
+      <c r="A858" t="inlineStr">
+        <is>
+          <t>2026-08-08T18:05:00</t>
+        </is>
+      </c>
+      <c r="B858" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C858" t="inlineStr">
+        <is>
+          <t>RoCals</t>
+        </is>
+      </c>
+      <c r="D858" t="n">
+        <v>0</v>
+      </c>
+      <c r="E858" t="n">
+        <v>3</v>
+      </c>
+      <c r="F858" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="859">
+      <c r="A859" t="inlineStr">
+        <is>
+          <t>2026-08-08T18:05:00</t>
+        </is>
+      </c>
+      <c r="B859" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C859" t="inlineStr">
+        <is>
+          <t>TPS_JamsUsr</t>
+        </is>
+      </c>
+      <c r="D859" t="n">
+        <v>0</v>
+      </c>
+      <c r="E859" t="n">
+        <v>3</v>
+      </c>
+      <c r="F859" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="860">
+      <c r="A860" t="inlineStr">
+        <is>
+          <t>2026-08-08T18:05:00</t>
+        </is>
+      </c>
+      <c r="B860" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C860" t="inlineStr">
+        <is>
+          <t>TPS_JamsMASTER</t>
+        </is>
+      </c>
+      <c r="D860" t="n">
+        <v>0</v>
+      </c>
+      <c r="E860" t="n">
+        <v>3</v>
+      </c>
+      <c r="F860" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="861">
+      <c r="A861" t="inlineStr">
+        <is>
+          <t>2026-08-08T18:05:00</t>
+        </is>
+      </c>
+      <c r="B861" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C861" t="inlineStr">
+        <is>
+          <t>ABORT_Master</t>
+        </is>
+      </c>
+      <c r="D861" t="n">
+        <v>0</v>
+      </c>
+      <c r="E861" t="n">
+        <v>3</v>
+      </c>
+      <c r="F861" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="862">
+      <c r="A862" t="inlineStr">
+        <is>
+          <t>2026-08-08T18:05:13</t>
+        </is>
+      </c>
+      <c r="B862" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C862" t="inlineStr">
+        <is>
+          <t>CountLaidButton</t>
+        </is>
+      </c>
+      <c r="D862" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E862" t="inlineStr"/>
+      <c r="F862" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g2</t>
+        </is>
+      </c>
+    </row>
+    <row r="863">
+      <c r="A863" t="inlineStr">
+        <is>
+          <t>2026-08-08T18:05:13</t>
+        </is>
+      </c>
+      <c r="B863" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C863" t="inlineStr">
+        <is>
+          <t>CountLaidDetector</t>
+        </is>
+      </c>
+      <c r="D863" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E863" t="inlineStr"/>
+      <c r="F863" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g3</t>
+        </is>
+      </c>
+    </row>
+    <row r="864">
+      <c r="A864" t="inlineStr">
+        <is>
+          <t>2026-08-08T18:05:13</t>
+        </is>
+      </c>
+      <c r="B864" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C864" t="inlineStr">
+        <is>
+          <t>CountLaidEncoder</t>
+        </is>
+      </c>
+      <c r="D864" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E864" t="inlineStr"/>
+      <c r="F864" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g4</t>
+        </is>
+      </c>
+    </row>
+    <row r="865">
+      <c r="A865" t="inlineStr">
+        <is>
+          <t>2026-08-08T18:05:13</t>
+        </is>
+      </c>
+      <c r="B865" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C865" t="inlineStr">
+        <is>
+          <t>CountLaid14in</t>
+        </is>
+      </c>
+      <c r="D865" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E865" t="inlineStr"/>
+      <c r="F865" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g5</t>
+        </is>
+      </c>
+    </row>
+    <row r="866">
+      <c r="A866" t="inlineStr">
+        <is>
+          <t>2026-08-08T18:05:13</t>
+        </is>
+      </c>
+      <c r="B866" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C866" t="inlineStr">
+        <is>
+          <t>CountLaid18in</t>
+        </is>
+      </c>
+      <c r="D866" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E866" t="inlineStr"/>
+      <c r="F866" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g6</t>
+        </is>
+      </c>
+    </row>
+    <row r="867">
+      <c r="A867" t="inlineStr">
+        <is>
+          <t>2026-08-08T18:05:13</t>
+        </is>
+      </c>
+      <c r="B867" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C867" t="inlineStr">
+        <is>
+          <t>CountLaidPandral</t>
+        </is>
+      </c>
+      <c r="D867" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E867" t="inlineStr"/>
+      <c r="F867" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g7</t>
+        </is>
+      </c>
+    </row>
+    <row r="868">
+      <c r="A868" t="inlineStr">
+        <is>
+          <t>2026-08-08T18:05:13</t>
+        </is>
+      </c>
+      <c r="B868" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C868" t="inlineStr">
+        <is>
+          <t>18in Job</t>
+        </is>
+      </c>
+      <c r="D868" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E868" t="inlineStr"/>
+      <c r="F868" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g13</t>
+        </is>
+      </c>
+    </row>
+    <row r="869">
+      <c r="A869" t="inlineStr">
+        <is>
+          <t>2026-08-08T18:05:13</t>
+        </is>
+      </c>
+      <c r="B869" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C869" t="inlineStr">
+        <is>
+          <t>CountAcceptedTotal</t>
+        </is>
+      </c>
+      <c r="D869" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E869" t="inlineStr"/>
+      <c r="F869" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g15</t>
+        </is>
+      </c>
+    </row>
+    <row r="870">
+      <c r="A870" t="inlineStr">
+        <is>
+          <t>2026-08-08T18:05:13</t>
+        </is>
+      </c>
+      <c r="B870" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C870" t="inlineStr">
+        <is>
+          <t>Servos_Enabled</t>
+        </is>
+      </c>
+      <c r="D870" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E870" t="inlineStr"/>
+      <c r="F870" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g17</t>
+        </is>
+      </c>
+    </row>
+    <row r="871">
+      <c r="A871" t="inlineStr">
+        <is>
+          <t>2026-08-08T18:05:13</t>
+        </is>
+      </c>
+      <c r="B871" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C871" t="inlineStr">
+        <is>
+          <t>TotalPickPartsCount</t>
+        </is>
+      </c>
+      <c r="D871" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E871" t="inlineStr"/>
+      <c r="F871" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g18</t>
+        </is>
+      </c>
+    </row>
+    <row r="872">
+      <c r="A872" t="inlineStr">
+        <is>
+          <t>2026-08-08T18:05:13</t>
+        </is>
+      </c>
+      <c r="B872" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C872" t="inlineStr">
+        <is>
+          <t>AcceptsPartsCount</t>
+        </is>
+      </c>
+      <c r="D872" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E872" t="inlineStr"/>
+      <c r="F872" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g19</t>
+        </is>
+      </c>
+    </row>
+    <row r="873">
+      <c r="A873" t="inlineStr">
+        <is>
+          <t>2026-08-08T18:05:13</t>
+        </is>
+      </c>
+      <c r="B873" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C873" t="inlineStr">
+        <is>
+          <t>day_Servotime Hours10th</t>
+        </is>
+      </c>
+      <c r="D873" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E873" t="inlineStr"/>
+      <c r="F873" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g22</t>
+        </is>
+      </c>
+    </row>
+    <row r="874">
+      <c r="A874" t="inlineStr">
+        <is>
+          <t>2026-08-08T18:05:13</t>
+        </is>
+      </c>
+      <c r="B874" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C874" t="inlineStr">
+        <is>
+          <t>tk_Cycle</t>
+        </is>
+      </c>
+      <c r="D874" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E874" t="inlineStr"/>
+      <c r="F874" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g23</t>
+        </is>
+      </c>
+    </row>
+    <row r="875">
+      <c r="A875" t="inlineStr">
+        <is>
+          <t>2026-08-08T18:05:13</t>
+        </is>
+      </c>
+      <c r="B875" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C875" t="inlineStr">
+        <is>
+          <t>tk_Abort</t>
+        </is>
+      </c>
+      <c r="D875" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E875" t="inlineStr"/>
+      <c r="F875" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g24</t>
+        </is>
+      </c>
+    </row>
+    <row r="876">
+      <c r="A876" t="inlineStr">
+        <is>
+          <t>2026-08-08T18:05:13</t>
+        </is>
+      </c>
+      <c r="B876" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C876" t="inlineStr">
+        <is>
+          <t>tk_ClearPos</t>
+        </is>
+      </c>
+      <c r="D876" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E876" t="inlineStr"/>
+      <c r="F876" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g25</t>
+        </is>
+      </c>
+    </row>
+    <row r="877">
+      <c r="A877" t="inlineStr">
+        <is>
+          <t>2026-08-08T18:05:13</t>
+        </is>
+      </c>
+      <c r="B877" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C877" t="inlineStr">
+        <is>
+          <t>temp_J2motor</t>
+        </is>
+      </c>
+      <c r="D877" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E877" t="inlineStr"/>
+      <c r="F877" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g33</t>
+        </is>
+      </c>
+    </row>
+    <row r="878">
+      <c r="A878" t="inlineStr">
+        <is>
+          <t>2026-08-08T18:05:13</t>
+        </is>
+      </c>
+      <c r="B878" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C878" t="inlineStr">
+        <is>
+          <t>temp_J3motor</t>
+        </is>
+      </c>
+      <c r="D878" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E878" t="inlineStr"/>
+      <c r="F878" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g34</t>
+        </is>
+      </c>
+    </row>
+    <row r="879">
+      <c r="A879" t="inlineStr">
+        <is>
+          <t>2026-08-08T18:05:13</t>
+        </is>
+      </c>
+      <c r="B879" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C879" t="inlineStr">
+        <is>
+          <t>temp_J5motor</t>
+        </is>
+      </c>
+      <c r="D879" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E879" t="inlineStr"/>
+      <c r="F879" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g36</t>
+        </is>
+      </c>
+    </row>
+    <row r="880">
+      <c r="A880" t="inlineStr">
+        <is>
+          <t>2026-08-08T18:05:13</t>
+        </is>
+      </c>
+      <c r="B880" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C880" t="inlineStr">
+        <is>
+          <t>CountPickedReject18in</t>
+        </is>
+      </c>
+      <c r="D880" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E880" t="inlineStr"/>
+      <c r="F880" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g40</t>
+        </is>
+      </c>
+    </row>
+    <row r="881">
+      <c r="A881" t="inlineStr">
+        <is>
+          <t>2026-08-08T18:05:13</t>
+        </is>
+      </c>
+      <c r="B881" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C881" t="inlineStr">
+        <is>
+          <t>TotalTiePlatesLaid</t>
+        </is>
+      </c>
+      <c r="D881" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E881" t="inlineStr"/>
+      <c r="F881" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g1</t>
+        </is>
+      </c>
+    </row>
+    <row r="882">
+      <c r="A882" t="inlineStr">
+        <is>
+          <t>2026-08-08T18:05:13</t>
+        </is>
+      </c>
+      <c r="B882" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C882" t="inlineStr">
+        <is>
+          <t>usr_TPStime Hours10th</t>
+        </is>
+      </c>
+      <c r="D882" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E882" t="inlineStr"/>
+      <c r="F882" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g8</t>
+        </is>
+      </c>
+    </row>
+    <row r="883">
+      <c r="A883" t="inlineStr">
+        <is>
+          <t>2026-08-08T18:05:13</t>
+        </is>
+      </c>
+      <c r="B883" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C883" t="inlineStr">
+        <is>
+          <t>usrTPS_miles xxx</t>
+        </is>
+      </c>
+      <c r="D883" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E883" t="inlineStr"/>
+      <c r="F883" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g9</t>
+        </is>
+      </c>
+    </row>
+    <row r="884">
+      <c r="A884" t="inlineStr">
+        <is>
+          <t>2026-08-08T18:05:13</t>
+        </is>
+      </c>
+      <c r="B884" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C884" t="inlineStr">
+        <is>
+          <t>TPS Connected</t>
+        </is>
+      </c>
+      <c r="D884" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E884" t="inlineStr"/>
+      <c r="F884" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g10</t>
+        </is>
+      </c>
+    </row>
+    <row r="885">
+      <c r="A885" t="inlineStr">
+        <is>
+          <t>2026-08-08T18:05:13</t>
+        </is>
+      </c>
+      <c r="B885" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C885" t="inlineStr">
+        <is>
+          <t>TPS Enabled</t>
+        </is>
+      </c>
+      <c r="D885" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E885" t="inlineStr"/>
+      <c r="F885" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g11</t>
+        </is>
+      </c>
+    </row>
+    <row r="886">
+      <c r="A886" t="inlineStr">
+        <is>
+          <t>2026-08-08T18:05:13</t>
+        </is>
+      </c>
+      <c r="B886" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C886" t="inlineStr">
+        <is>
+          <t>14in Job</t>
+        </is>
+      </c>
+      <c r="D886" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E886" t="inlineStr"/>
+      <c r="F886" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g12</t>
+        </is>
+      </c>
+    </row>
+    <row r="887">
+      <c r="A887" t="inlineStr">
+        <is>
+          <t>2026-08-08T18:05:13</t>
+        </is>
+      </c>
+      <c r="B887" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C887" t="inlineStr">
+        <is>
+          <t>Pandral Job</t>
+        </is>
+      </c>
+      <c r="D887" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E887" t="inlineStr"/>
+      <c r="F887" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g14</t>
+        </is>
+      </c>
+    </row>
+    <row r="888">
+      <c r="A888" t="inlineStr">
+        <is>
+          <t>2026-08-08T18:05:13</t>
+        </is>
+      </c>
+      <c r="B888" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C888" t="inlineStr">
+        <is>
+          <t>CountRejectedTotal</t>
+        </is>
+      </c>
+      <c r="D888" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E888" t="inlineStr"/>
+      <c r="F888" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g16</t>
+        </is>
+      </c>
+    </row>
+    <row r="889">
+      <c r="A889" t="inlineStr">
+        <is>
+          <t>2026-08-08T18:05:13</t>
+        </is>
+      </c>
+      <c r="B889" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C889" t="inlineStr">
+        <is>
+          <t>RejectPartsCount</t>
+        </is>
+      </c>
+      <c r="D889" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E889" t="inlineStr"/>
+      <c r="F889" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g20</t>
+        </is>
+      </c>
+    </row>
+    <row r="890">
+      <c r="A890" t="inlineStr">
+        <is>
+          <t>2026-08-08T18:05:13</t>
+        </is>
+      </c>
+      <c r="B890" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C890" t="inlineStr">
+        <is>
+          <t>tk_Cycle hrs</t>
+        </is>
+      </c>
+      <c r="D890" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E890" t="inlineStr"/>
+      <c r="F890" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g21</t>
+        </is>
+      </c>
+    </row>
+    <row r="891">
+      <c r="A891" t="inlineStr">
+        <is>
+          <t>2026-08-08T18:05:13</t>
+        </is>
+      </c>
+      <c r="B891" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C891" t="inlineStr">
+        <is>
+          <t>tk_Warmup</t>
+        </is>
+      </c>
+      <c r="D891" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E891" t="inlineStr"/>
+      <c r="F891" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g26</t>
+        </is>
+      </c>
+    </row>
+    <row r="892">
+      <c r="A892" t="inlineStr">
+        <is>
+          <t>2026-08-08T18:05:13</t>
+        </is>
+      </c>
+      <c r="B892" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C892" t="inlineStr">
+        <is>
+          <t>FindingParts min</t>
+        </is>
+      </c>
+      <c r="D892" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E892" t="inlineStr"/>
+      <c r="F892" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g27</t>
+        </is>
+      </c>
+    </row>
+    <row r="893">
+      <c r="A893" t="inlineStr">
+        <is>
+          <t>2026-08-08T18:05:13</t>
+        </is>
+      </c>
+      <c r="B893" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C893" t="inlineStr">
+        <is>
+          <t>PickingParts min</t>
+        </is>
+      </c>
+      <c r="D893" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E893" t="inlineStr"/>
+      <c r="F893" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g28</t>
+        </is>
+      </c>
+    </row>
+    <row r="894">
+      <c r="A894" t="inlineStr">
+        <is>
+          <t>2026-08-08T18:05:13</t>
+        </is>
+      </c>
+      <c r="B894" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C894" t="inlineStr">
+        <is>
+          <t>PlacingParts min</t>
+        </is>
+      </c>
+      <c r="D894" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E894" t="inlineStr"/>
+      <c r="F894" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g29</t>
+        </is>
+      </c>
+    </row>
+    <row r="895">
+      <c r="A895" t="inlineStr">
+        <is>
+          <t>2026-08-08T18:05:13</t>
+        </is>
+      </c>
+      <c r="B895" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C895" t="inlineStr">
+        <is>
+          <t>CountPickedReject14in</t>
+        </is>
+      </c>
+      <c r="D895" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E895" t="inlineStr"/>
+      <c r="F895" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g30</t>
+        </is>
+      </c>
+    </row>
+    <row r="896">
+      <c r="A896" t="inlineStr">
+        <is>
+          <t>2026-08-08T18:05:13</t>
+        </is>
+      </c>
+      <c r="B896" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C896" t="inlineStr">
+        <is>
+          <t>temp_dsi</t>
+        </is>
+      </c>
+      <c r="D896" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E896" t="inlineStr"/>
+      <c r="F896" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g31</t>
+        </is>
+      </c>
+    </row>
+    <row r="897">
+      <c r="A897" t="inlineStr">
+        <is>
+          <t>2026-08-08T18:05:13</t>
+        </is>
+      </c>
+      <c r="B897" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C897" t="inlineStr">
+        <is>
+          <t>temp_J1motor</t>
+        </is>
+      </c>
+      <c r="D897" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E897" t="inlineStr"/>
+      <c r="F897" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g32</t>
+        </is>
+      </c>
+    </row>
+    <row r="898">
+      <c r="A898" t="inlineStr">
+        <is>
+          <t>2026-08-08T18:05:13</t>
+        </is>
+      </c>
+      <c r="B898" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C898" t="inlineStr">
+        <is>
+          <t>temp_J4motor</t>
+        </is>
+      </c>
+      <c r="D898" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E898" t="inlineStr"/>
+      <c r="F898" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g35</t>
+        </is>
+      </c>
+    </row>
+    <row r="899">
+      <c r="A899" t="inlineStr">
+        <is>
+          <t>2026-08-08T18:05:13</t>
+        </is>
+      </c>
+      <c r="B899" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C899" t="inlineStr">
+        <is>
+          <t>temp_J6motor</t>
+        </is>
+      </c>
+      <c r="D899" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E899" t="inlineStr"/>
+      <c r="F899" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g37</t>
+        </is>
+      </c>
+    </row>
+    <row r="900">
+      <c r="A900" t="inlineStr">
+        <is>
+          <t>2026-08-08T18:05:13</t>
+        </is>
+      </c>
+      <c r="B900" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C900" t="inlineStr">
+        <is>
+          <t>CountPickedRejectOTM</t>
+        </is>
+      </c>
+      <c r="D900" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E900" t="inlineStr"/>
+      <c r="F900" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g38</t>
+        </is>
+      </c>
+    </row>
+    <row r="901">
+      <c r="A901" t="inlineStr">
+        <is>
+          <t>2026-08-08T18:05:13</t>
+        </is>
+      </c>
+      <c r="B901" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C901" t="inlineStr">
+        <is>
+          <t>CountPickedRejectPandral</t>
+        </is>
+      </c>
+      <c r="D901" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E901" t="inlineStr"/>
+      <c r="F901" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g39</t>
+        </is>
+      </c>
+    </row>
+    <row r="902">
+      <c r="A902" t="inlineStr">
+        <is>
+          <t>2026-08-08T18:06:00</t>
+        </is>
+      </c>
+      <c r="B902" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C902" t="inlineStr">
+        <is>
+          <t>_1st_SCAN</t>
+        </is>
+      </c>
+      <c r="D902" t="b">
+        <v>0</v>
+      </c>
+      <c r="E902" t="n">
+        <v>11</v>
+      </c>
+      <c r="F902" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="903">
+      <c r="A903" t="inlineStr">
+        <is>
+          <t>2026-08-08T18:06:00</t>
+        </is>
+      </c>
+      <c r="B903" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C903" t="inlineStr">
+        <is>
+          <t>TieDetectOffset_B</t>
+        </is>
+      </c>
+      <c r="D903" t="b">
+        <v>0</v>
+      </c>
+      <c r="E903" t="n">
+        <v>11</v>
+      </c>
+      <c r="F903" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="904">
+      <c r="A904" t="inlineStr">
+        <is>
+          <t>2026-08-08T18:06:00</t>
+        </is>
+      </c>
+      <c r="B904" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C904" t="inlineStr">
+        <is>
+          <t>Tie Detector</t>
+        </is>
+      </c>
+      <c r="D904" t="b">
+        <v>0</v>
+      </c>
+      <c r="E904" t="n">
+        <v>11</v>
+      </c>
+      <c r="F904" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="905">
+      <c r="A905" t="inlineStr">
+        <is>
+          <t>2026-08-08T18:06:00</t>
+        </is>
+      </c>
+      <c r="B905" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C905" t="inlineStr">
+        <is>
+          <t>TPS Full</t>
+        </is>
+      </c>
+      <c r="D905" t="b">
+        <v>0</v>
+      </c>
+      <c r="E905" t="n">
+        <v>11</v>
+      </c>
+      <c r="F905" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="906">
+      <c r="A906" t="inlineStr">
+        <is>
+          <t>2026-08-08T18:06:00</t>
+        </is>
+      </c>
+      <c r="B906" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C906" t="inlineStr">
+        <is>
+          <t>TieDetectOffset_A</t>
+        </is>
+      </c>
+      <c r="D906" t="b">
+        <v>0</v>
+      </c>
+      <c r="E906" t="n">
+        <v>11</v>
+      </c>
+      <c r="F906" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="907">
+      <c r="A907" t="inlineStr">
+        <is>
+          <t>2026-08-08T18:06:00</t>
+        </is>
+      </c>
+      <c r="B907" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C907" t="inlineStr">
+        <is>
+          <t>TPS Connected</t>
+        </is>
+      </c>
+      <c r="D907" t="b">
+        <v>0</v>
+      </c>
+      <c r="E907" t="n">
+        <v>11</v>
+      </c>
+      <c r="F907" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="908">
+      <c r="A908" t="inlineStr">
+        <is>
+          <t>2026-08-08T18:06:00</t>
+        </is>
+      </c>
+      <c r="B908" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C908" t="inlineStr">
+        <is>
+          <t>TPS_Enable_ Button</t>
+        </is>
+      </c>
+      <c r="D908" t="b">
+        <v>0</v>
+      </c>
+      <c r="E908" t="n">
+        <v>11</v>
+      </c>
+      <c r="F908" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="909">
+      <c r="A909" t="inlineStr">
+        <is>
+          <t>2026-08-08T18:06:00</t>
+        </is>
+      </c>
+      <c r="B909" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C909" t="inlineStr">
+        <is>
+          <t>AirEagle Eject Plate</t>
+        </is>
+      </c>
+      <c r="D909" t="b">
+        <v>0</v>
+      </c>
+      <c r="E909" t="n">
+        <v>11</v>
+      </c>
+      <c r="F909" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="910">
+      <c r="A910" t="inlineStr">
+        <is>
+          <t>2026-08-08T18:06:00</t>
+        </is>
+      </c>
+      <c r="B910" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C910" t="inlineStr">
+        <is>
+          <t>tk_Cycle</t>
+        </is>
+      </c>
+      <c r="D910" t="b">
+        <v>0</v>
+      </c>
+      <c r="E910" t="n">
+        <v>11</v>
+      </c>
+      <c r="F910" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="911">
+      <c r="A911" t="inlineStr">
+        <is>
+          <t>2026-08-08T18:06:00</t>
+        </is>
+      </c>
+      <c r="B911" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C911" t="inlineStr">
+        <is>
+          <t>Servos_Enabled</t>
+        </is>
+      </c>
+      <c r="D911" t="b">
+        <v>0</v>
+      </c>
+      <c r="E911" t="n">
+        <v>11</v>
+      </c>
+      <c r="F911" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="912">
+      <c r="A912" t="inlineStr">
+        <is>
+          <t>2026-08-08T18:06:00</t>
+        </is>
+      </c>
+      <c r="B912" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C912" t="inlineStr">
+        <is>
+          <t>TPS Enabled</t>
+        </is>
+      </c>
+      <c r="D912" t="b">
+        <v>0</v>
+      </c>
+      <c r="E912" t="n">
+        <v>11</v>
+      </c>
+      <c r="F912" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="913">
+      <c r="A913" t="inlineStr">
+        <is>
+          <t>2026-08-08T18:06:00</t>
+        </is>
+      </c>
+      <c r="B913" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C913" t="inlineStr">
+        <is>
+          <t>tk_Abort</t>
+        </is>
+      </c>
+      <c r="D913" t="b">
+        <v>0</v>
+      </c>
+      <c r="E913" t="n">
+        <v>11</v>
+      </c>
+      <c r="F913" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="914">
+      <c r="A914" t="inlineStr">
+        <is>
+          <t>2026-08-08T18:06:00</t>
+        </is>
+      </c>
+      <c r="B914" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C914" t="inlineStr">
+        <is>
+          <t>Robot_isMoving</t>
+        </is>
+      </c>
+      <c r="D914" t="b">
+        <v>0</v>
+      </c>
+      <c r="E914" t="n">
+        <v>11</v>
+      </c>
+      <c r="F914" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="915">
+      <c r="A915" t="inlineStr">
+        <is>
+          <t>2026-08-08T18:06:00</t>
+        </is>
+      </c>
+      <c r="B915" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C915" t="inlineStr">
+        <is>
+          <t>Eject Tie Plate</t>
+        </is>
+      </c>
+      <c r="D915" t="b">
+        <v>0</v>
+      </c>
+      <c r="E915" t="n">
+        <v>11</v>
+      </c>
+      <c r="F915" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="916">
+      <c r="A916" t="inlineStr">
+        <is>
+          <t>2026-08-08T18:06:00</t>
+        </is>
+      </c>
+      <c r="B916" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C916" t="inlineStr">
+        <is>
+          <t>TPS BACKUP ALARM</t>
+        </is>
+      </c>
+      <c r="D916" t="b">
+        <v>0</v>
+      </c>
+      <c r="E916" t="n">
+        <v>11</v>
+      </c>
+      <c r="F916" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="917">
+      <c r="A917" t="inlineStr">
+        <is>
+          <t>2026-08-08T18:06:00</t>
+        </is>
+      </c>
+      <c r="B917" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C917" t="inlineStr">
+        <is>
+          <t>14in Job</t>
+        </is>
+      </c>
+      <c r="D917" t="b">
+        <v>1</v>
+      </c>
+      <c r="E917" t="n">
+        <v>11</v>
+      </c>
+      <c r="F917" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="918">
+      <c r="A918" t="inlineStr">
+        <is>
+          <t>2026-08-08T18:06:00</t>
+        </is>
+      </c>
+      <c r="B918" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C918" t="inlineStr">
+        <is>
+          <t>18in Job</t>
+        </is>
+      </c>
+      <c r="D918" t="b">
+        <v>0</v>
+      </c>
+      <c r="E918" t="n">
+        <v>11</v>
+      </c>
+      <c r="F918" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="919">
+      <c r="A919" t="inlineStr">
+        <is>
+          <t>2026-08-08T18:06:00</t>
+        </is>
+      </c>
+      <c r="B919" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C919" t="inlineStr">
+        <is>
+          <t>Pandral Job</t>
+        </is>
+      </c>
+      <c r="D919" t="b">
+        <v>0</v>
+      </c>
+      <c r="E919" t="n">
+        <v>11</v>
+      </c>
+      <c r="F919" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="920">
+      <c r="A920" t="inlineStr">
+        <is>
+          <t>2026-08-08T18:06:00</t>
+        </is>
+      </c>
+      <c r="B920" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C920" t="inlineStr">
+        <is>
+          <t>DoubleLay Job</t>
+        </is>
+      </c>
+      <c r="D920" t="b">
+        <v>0</v>
+      </c>
+      <c r="E920" t="n">
+        <v>11</v>
+      </c>
+      <c r="F920" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="921">
+      <c r="A921" t="inlineStr">
+        <is>
+          <t>2026-08-08T18:06:00</t>
+        </is>
+      </c>
+      <c r="B921" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C921" t="inlineStr">
+        <is>
+          <t>TPSjam_FLAG</t>
+        </is>
+      </c>
+      <c r="D921" t="b">
+        <v>0</v>
+      </c>
+      <c r="E921" t="n">
+        <v>11</v>
+      </c>
+      <c r="F921" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="922">
+      <c r="A922" t="inlineStr">
+        <is>
+          <t>2026-08-08T18:06:00</t>
+        </is>
+      </c>
+      <c r="B922" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C922" t="inlineStr">
+        <is>
+          <t>RoCalRequest</t>
+        </is>
+      </c>
+      <c r="D922" t="b">
+        <v>0</v>
+      </c>
+      <c r="E922" t="n">
+        <v>11</v>
+      </c>
+      <c r="F922" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="923">
+      <c r="A923" t="inlineStr">
+        <is>
+          <t>2026-08-08T18:06:00</t>
+        </is>
+      </c>
+      <c r="B923" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C923" t="inlineStr">
+        <is>
+          <t>tkCycle_TotalSeconds</t>
+        </is>
+      </c>
+      <c r="D923" t="n">
+        <v>0</v>
+      </c>
+      <c r="E923" t="n">
+        <v>9</v>
+      </c>
+      <c r="F923" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="924">
+      <c r="A924" t="inlineStr">
+        <is>
+          <t>2026-08-08T18:06:00</t>
+        </is>
+      </c>
+      <c r="B924" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C924" t="inlineStr">
+        <is>
+          <t>tkCycle_NoMoveSec</t>
+        </is>
+      </c>
+      <c r="D924" t="n">
+        <v>0</v>
+      </c>
+      <c r="E924" t="n">
+        <v>9</v>
+      </c>
+      <c r="F924" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="925">
+      <c r="A925" t="inlineStr">
+        <is>
+          <t>2026-08-08T18:06:00</t>
+        </is>
+      </c>
+      <c r="B925" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C925" t="inlineStr">
+        <is>
+          <t>tkCycle_MoveSeconds</t>
+        </is>
+      </c>
+      <c r="D925" t="n">
+        <v>0</v>
+      </c>
+      <c r="E925" t="n">
+        <v>9</v>
+      </c>
+      <c r="F925" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="926">
+      <c r="A926" t="inlineStr">
+        <is>
+          <t>2026-08-08T18:06:00</t>
+        </is>
+      </c>
+      <c r="B926" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C926" t="inlineStr">
+        <is>
+          <t>Percent time moveing</t>
+        </is>
+      </c>
+      <c r="D926" t="n">
+        <v>0</v>
+      </c>
+      <c r="E926" t="n">
+        <v>9</v>
+      </c>
+      <c r="F926" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="927">
+      <c r="A927" t="inlineStr">
+        <is>
+          <t>2026-08-08T18:06:00</t>
+        </is>
+      </c>
+      <c r="B927" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C927" t="inlineStr">
+        <is>
+          <t>Percent time not moving</t>
+        </is>
+      </c>
+      <c r="D927" t="n">
+        <v>0</v>
+      </c>
+      <c r="E927" t="n">
+        <v>9</v>
+      </c>
+      <c r="F927" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="928">
+      <c r="A928" t="inlineStr">
+        <is>
+          <t>2026-08-08T18:06:00</t>
+        </is>
+      </c>
+      <c r="B928" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C928" t="inlineStr">
+        <is>
+          <t>TotalPickPartsCount</t>
+        </is>
+      </c>
+      <c r="D928" t="n">
+        <v>0</v>
+      </c>
+      <c r="E928" t="n">
+        <v>9</v>
+      </c>
+      <c r="F928" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="929">
+      <c r="A929" t="inlineStr">
+        <is>
+          <t>2026-08-08T18:06:00</t>
+        </is>
+      </c>
+      <c r="B929" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C929" t="inlineStr">
+        <is>
+          <t>RejectPartsCount</t>
+        </is>
+      </c>
+      <c r="D929" t="n">
+        <v>0</v>
+      </c>
+      <c r="E929" t="n">
+        <v>9</v>
+      </c>
+      <c r="F929" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="930">
+      <c r="A930" t="inlineStr">
+        <is>
+          <t>2026-08-08T18:06:00</t>
+        </is>
+      </c>
+      <c r="B930" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C930" t="inlineStr">
+        <is>
+          <t>AcceptsPartsCount</t>
+        </is>
+      </c>
+      <c r="D930" t="n">
+        <v>0</v>
+      </c>
+      <c r="E930" t="n">
+        <v>9</v>
+      </c>
+      <c r="F930" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="931">
+      <c r="A931" t="inlineStr">
+        <is>
+          <t>2026-08-08T18:06:00</t>
+        </is>
+      </c>
+      <c r="B931" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C931" t="inlineStr">
+        <is>
+          <t>percentCount_accept</t>
+        </is>
+      </c>
+      <c r="D931" t="n">
+        <v>0</v>
+      </c>
+      <c r="E931" t="n">
+        <v>9</v>
+      </c>
+      <c r="F931" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="932">
+      <c r="A932" t="inlineStr">
+        <is>
+          <t>2026-08-08T18:06:00</t>
+        </is>
+      </c>
+      <c r="B932" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C932" t="inlineStr">
+        <is>
+          <t>percentCount_reject</t>
+        </is>
+      </c>
+      <c r="D932" t="n">
+        <v>0</v>
+      </c>
+      <c r="E932" t="n">
+        <v>9</v>
+      </c>
+      <c r="F932" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="933">
+      <c r="A933" t="inlineStr">
+        <is>
+          <t>2026-08-08T18:06:00</t>
+        </is>
+      </c>
+      <c r="B933" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C933" t="inlineStr">
+        <is>
+          <t>Avg Parts per min_total</t>
+        </is>
+      </c>
+      <c r="D933" t="n">
+        <v>0</v>
+      </c>
+      <c r="E933" t="n">
+        <v>9</v>
+      </c>
+      <c r="F933" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="934">
+      <c r="A934" t="inlineStr">
+        <is>
+          <t>2026-08-08T18:06:00</t>
+        </is>
+      </c>
+      <c r="B934" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C934" t="inlineStr">
+        <is>
+          <t>TotalPickedParts</t>
+        </is>
+      </c>
+      <c r="D934" t="n">
+        <v>0</v>
+      </c>
+      <c r="E934" t="n">
+        <v>3</v>
+      </c>
+      <c r="F934" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="935">
+      <c r="A935" t="inlineStr">
+        <is>
+          <t>2026-08-08T18:06:00</t>
+        </is>
+      </c>
+      <c r="B935" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C935" t="inlineStr">
+        <is>
+          <t>TotalPickedAcceptParts</t>
+        </is>
+      </c>
+      <c r="D935" t="n">
+        <v>0</v>
+      </c>
+      <c r="E935" t="n">
+        <v>3</v>
+      </c>
+      <c r="F935" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="936">
+      <c r="A936" t="inlineStr">
+        <is>
+          <t>2026-08-08T18:06:00</t>
+        </is>
+      </c>
+      <c r="B936" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C936" t="inlineStr">
+        <is>
+          <t>TotalPickedRejectParts</t>
+        </is>
+      </c>
+      <c r="D936" t="n">
+        <v>0</v>
+      </c>
+      <c r="E936" t="n">
+        <v>3</v>
+      </c>
+      <c r="F936" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="937">
+      <c r="A937" t="inlineStr">
+        <is>
+          <t>2026-08-08T18:06:00</t>
+        </is>
+      </c>
+      <c r="B937" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C937" t="inlineStr">
+        <is>
+          <t>TotalTiePlatesLaid</t>
+        </is>
+      </c>
+      <c r="D937" t="n">
+        <v>0</v>
+      </c>
+      <c r="E937" t="n">
+        <v>3</v>
+      </c>
+      <c r="F937" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="938">
+      <c r="A938" t="inlineStr">
+        <is>
+          <t>2026-08-08T18:06:00</t>
+        </is>
+      </c>
+      <c r="B938" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C938" t="inlineStr">
+        <is>
+          <t>Daily_TotalLaidPlates</t>
+        </is>
+      </c>
+      <c r="D938" t="n">
+        <v>0</v>
+      </c>
+      <c r="E938" t="n">
+        <v>3</v>
+      </c>
+      <c r="F938" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="939">
+      <c r="A939" t="inlineStr">
+        <is>
+          <t>2026-08-08T18:06:00</t>
+        </is>
+      </c>
+      <c r="B939" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C939" t="inlineStr">
+        <is>
+          <t>CountPicked14in</t>
+        </is>
+      </c>
+      <c r="D939" t="n">
+        <v>0</v>
+      </c>
+      <c r="E939" t="n">
+        <v>3</v>
+      </c>
+      <c r="F939" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="940">
+      <c r="A940" t="inlineStr">
+        <is>
+          <t>2026-08-08T18:06:00</t>
+        </is>
+      </c>
+      <c r="B940" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C940" t="inlineStr">
+        <is>
+          <t>CountPicked18in</t>
+        </is>
+      </c>
+      <c r="D940" t="n">
+        <v>0</v>
+      </c>
+      <c r="E940" t="n">
+        <v>3</v>
+      </c>
+      <c r="F940" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="941">
+      <c r="A941" t="inlineStr">
+        <is>
+          <t>2026-08-08T18:06:00</t>
+        </is>
+      </c>
+      <c r="B941" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C941" t="inlineStr">
+        <is>
+          <t>CountPickedPandral</t>
+        </is>
+      </c>
+      <c r="D941" t="n">
+        <v>0</v>
+      </c>
+      <c r="E941" t="n">
+        <v>3</v>
+      </c>
+      <c r="F941" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="942">
+      <c r="A942" t="inlineStr">
+        <is>
+          <t>2026-08-08T18:06:00</t>
+        </is>
+      </c>
+      <c r="B942" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C942" t="inlineStr">
+        <is>
+          <t>CountPickedOTM</t>
+        </is>
+      </c>
+      <c r="D942" t="n">
+        <v>0</v>
+      </c>
+      <c r="E942" t="n">
+        <v>3</v>
+      </c>
+      <c r="F942" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="943">
+      <c r="A943" t="inlineStr">
+        <is>
+          <t>2026-08-08T18:06:00</t>
+        </is>
+      </c>
+      <c r="B943" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C943" t="inlineStr">
+        <is>
+          <t>RoCals</t>
+        </is>
+      </c>
+      <c r="D943" t="n">
+        <v>0</v>
+      </c>
+      <c r="E943" t="n">
+        <v>3</v>
+      </c>
+      <c r="F943" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="944">
+      <c r="A944" t="inlineStr">
+        <is>
+          <t>2026-08-08T18:06:00</t>
+        </is>
+      </c>
+      <c r="B944" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C944" t="inlineStr">
+        <is>
+          <t>TPS_JamsUsr</t>
+        </is>
+      </c>
+      <c r="D944" t="n">
+        <v>0</v>
+      </c>
+      <c r="E944" t="n">
+        <v>3</v>
+      </c>
+      <c r="F944" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="945">
+      <c r="A945" t="inlineStr">
+        <is>
+          <t>2026-08-08T18:06:00</t>
+        </is>
+      </c>
+      <c r="B945" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C945" t="inlineStr">
+        <is>
+          <t>TPS_JamsMASTER</t>
+        </is>
+      </c>
+      <c r="D945" t="n">
+        <v>0</v>
+      </c>
+      <c r="E945" t="n">
+        <v>3</v>
+      </c>
+      <c r="F945" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="946">
+      <c r="A946" t="inlineStr">
+        <is>
+          <t>2026-08-08T18:06:00</t>
+        </is>
+      </c>
+      <c r="B946" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C946" t="inlineStr">
+        <is>
+          <t>ABORT_Master</t>
+        </is>
+      </c>
+      <c r="D946" t="n">
+        <v>0</v>
+      </c>
+      <c r="E946" t="n">
+        <v>3</v>
+      </c>
+      <c r="F946" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/plc</t>
         </is>

</xml_diff>

<commit_message>
Log MQTT data 2026-08-08 19:47 UTC
</commit_message>
<xml_diff>
--- a/logs/raiv_tracker_2026-08-08.xlsx
+++ b/logs/raiv_tracker_2026-08-08.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F946"/>
+  <dimension ref="A1:F1076"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -24229,7 +24229,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E862" t="inlineStr"/>
       <c r="F862" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g2</t>
@@ -24257,7 +24256,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E863" t="inlineStr"/>
       <c r="F863" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g3</t>
@@ -24285,7 +24283,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E864" t="inlineStr"/>
       <c r="F864" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g4</t>
@@ -24313,7 +24310,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E865" t="inlineStr"/>
       <c r="F865" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g5</t>
@@ -24341,7 +24337,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E866" t="inlineStr"/>
       <c r="F866" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g6</t>
@@ -24369,7 +24364,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E867" t="inlineStr"/>
       <c r="F867" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g7</t>
@@ -24397,7 +24391,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E868" t="inlineStr"/>
       <c r="F868" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g13</t>
@@ -24425,7 +24418,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E869" t="inlineStr"/>
       <c r="F869" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g15</t>
@@ -24453,7 +24445,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E870" t="inlineStr"/>
       <c r="F870" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g17</t>
@@ -24481,7 +24472,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E871" t="inlineStr"/>
       <c r="F871" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g18</t>
@@ -24509,7 +24499,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E872" t="inlineStr"/>
       <c r="F872" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g19</t>
@@ -24537,7 +24526,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E873" t="inlineStr"/>
       <c r="F873" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g22</t>
@@ -24565,7 +24553,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E874" t="inlineStr"/>
       <c r="F874" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g23</t>
@@ -24593,7 +24580,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E875" t="inlineStr"/>
       <c r="F875" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g24</t>
@@ -24621,7 +24607,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E876" t="inlineStr"/>
       <c r="F876" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g25</t>
@@ -24649,7 +24634,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E877" t="inlineStr"/>
       <c r="F877" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g33</t>
@@ -24677,7 +24661,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E878" t="inlineStr"/>
       <c r="F878" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g34</t>
@@ -24705,7 +24688,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E879" t="inlineStr"/>
       <c r="F879" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g36</t>
@@ -24733,7 +24715,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E880" t="inlineStr"/>
       <c r="F880" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g40</t>
@@ -24761,7 +24742,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E881" t="inlineStr"/>
       <c r="F881" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g1</t>
@@ -24789,7 +24769,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E882" t="inlineStr"/>
       <c r="F882" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g8</t>
@@ -24817,7 +24796,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E883" t="inlineStr"/>
       <c r="F883" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g9</t>
@@ -24845,7 +24823,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E884" t="inlineStr"/>
       <c r="F884" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g10</t>
@@ -24873,7 +24850,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E885" t="inlineStr"/>
       <c r="F885" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g11</t>
@@ -24901,7 +24877,6 @@
           <t>1</t>
         </is>
       </c>
-      <c r="E886" t="inlineStr"/>
       <c r="F886" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g12</t>
@@ -24929,7 +24904,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E887" t="inlineStr"/>
       <c r="F887" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g14</t>
@@ -24957,7 +24931,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E888" t="inlineStr"/>
       <c r="F888" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g16</t>
@@ -24985,7 +24958,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E889" t="inlineStr"/>
       <c r="F889" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g20</t>
@@ -25013,7 +24985,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E890" t="inlineStr"/>
       <c r="F890" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g21</t>
@@ -25041,7 +25012,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E891" t="inlineStr"/>
       <c r="F891" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g26</t>
@@ -25069,7 +25039,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E892" t="inlineStr"/>
       <c r="F892" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g27</t>
@@ -25097,7 +25066,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E893" t="inlineStr"/>
       <c r="F893" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g28</t>
@@ -25125,7 +25093,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E894" t="inlineStr"/>
       <c r="F894" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g29</t>
@@ -25153,7 +25120,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E895" t="inlineStr"/>
       <c r="F895" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g30</t>
@@ -25181,7 +25147,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E896" t="inlineStr"/>
       <c r="F896" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g31</t>
@@ -25209,7 +25174,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E897" t="inlineStr"/>
       <c r="F897" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g32</t>
@@ -25237,7 +25201,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E898" t="inlineStr"/>
       <c r="F898" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g35</t>
@@ -25265,7 +25228,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E899" t="inlineStr"/>
       <c r="F899" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g37</t>
@@ -25293,7 +25255,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E900" t="inlineStr"/>
       <c r="F900" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g38</t>
@@ -25321,7 +25282,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E901" t="inlineStr"/>
       <c r="F901" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g39</t>
@@ -26583,6 +26543,3646 @@
         <v>3</v>
       </c>
       <c r="F946" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="947">
+      <c r="A947" t="inlineStr">
+        <is>
+          <t>2026-08-08T19:46:00</t>
+        </is>
+      </c>
+      <c r="B947" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C947" t="inlineStr">
+        <is>
+          <t>_1st_SCAN</t>
+        </is>
+      </c>
+      <c r="D947" t="b">
+        <v>0</v>
+      </c>
+      <c r="E947" t="n">
+        <v>11</v>
+      </c>
+      <c r="F947" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="948">
+      <c r="A948" t="inlineStr">
+        <is>
+          <t>2026-08-08T19:46:00</t>
+        </is>
+      </c>
+      <c r="B948" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C948" t="inlineStr">
+        <is>
+          <t>TieDetectOffset_B</t>
+        </is>
+      </c>
+      <c r="D948" t="b">
+        <v>0</v>
+      </c>
+      <c r="E948" t="n">
+        <v>11</v>
+      </c>
+      <c r="F948" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="949">
+      <c r="A949" t="inlineStr">
+        <is>
+          <t>2026-08-08T19:46:00</t>
+        </is>
+      </c>
+      <c r="B949" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C949" t="inlineStr">
+        <is>
+          <t>Tie Detector</t>
+        </is>
+      </c>
+      <c r="D949" t="b">
+        <v>0</v>
+      </c>
+      <c r="E949" t="n">
+        <v>11</v>
+      </c>
+      <c r="F949" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="950">
+      <c r="A950" t="inlineStr">
+        <is>
+          <t>2026-08-08T19:46:00</t>
+        </is>
+      </c>
+      <c r="B950" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C950" t="inlineStr">
+        <is>
+          <t>TPS Full</t>
+        </is>
+      </c>
+      <c r="D950" t="b">
+        <v>0</v>
+      </c>
+      <c r="E950" t="n">
+        <v>11</v>
+      </c>
+      <c r="F950" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="951">
+      <c r="A951" t="inlineStr">
+        <is>
+          <t>2026-08-08T19:46:00</t>
+        </is>
+      </c>
+      <c r="B951" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C951" t="inlineStr">
+        <is>
+          <t>TieDetectOffset_A</t>
+        </is>
+      </c>
+      <c r="D951" t="b">
+        <v>0</v>
+      </c>
+      <c r="E951" t="n">
+        <v>11</v>
+      </c>
+      <c r="F951" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="952">
+      <c r="A952" t="inlineStr">
+        <is>
+          <t>2026-08-08T19:46:00</t>
+        </is>
+      </c>
+      <c r="B952" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C952" t="inlineStr">
+        <is>
+          <t>TPS Connected</t>
+        </is>
+      </c>
+      <c r="D952" t="b">
+        <v>0</v>
+      </c>
+      <c r="E952" t="n">
+        <v>11</v>
+      </c>
+      <c r="F952" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="953">
+      <c r="A953" t="inlineStr">
+        <is>
+          <t>2026-08-08T19:46:00</t>
+        </is>
+      </c>
+      <c r="B953" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C953" t="inlineStr">
+        <is>
+          <t>TPS_Enable_ Button</t>
+        </is>
+      </c>
+      <c r="D953" t="b">
+        <v>0</v>
+      </c>
+      <c r="E953" t="n">
+        <v>11</v>
+      </c>
+      <c r="F953" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="954">
+      <c r="A954" t="inlineStr">
+        <is>
+          <t>2026-08-08T19:46:00</t>
+        </is>
+      </c>
+      <c r="B954" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C954" t="inlineStr">
+        <is>
+          <t>AirEagle Eject Plate</t>
+        </is>
+      </c>
+      <c r="D954" t="b">
+        <v>0</v>
+      </c>
+      <c r="E954" t="n">
+        <v>11</v>
+      </c>
+      <c r="F954" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="955">
+      <c r="A955" t="inlineStr">
+        <is>
+          <t>2026-08-08T19:46:00</t>
+        </is>
+      </c>
+      <c r="B955" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C955" t="inlineStr">
+        <is>
+          <t>tk_Cycle</t>
+        </is>
+      </c>
+      <c r="D955" t="b">
+        <v>0</v>
+      </c>
+      <c r="E955" t="n">
+        <v>11</v>
+      </c>
+      <c r="F955" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="956">
+      <c r="A956" t="inlineStr">
+        <is>
+          <t>2026-08-08T19:46:00</t>
+        </is>
+      </c>
+      <c r="B956" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C956" t="inlineStr">
+        <is>
+          <t>Servos_Enabled</t>
+        </is>
+      </c>
+      <c r="D956" t="b">
+        <v>0</v>
+      </c>
+      <c r="E956" t="n">
+        <v>11</v>
+      </c>
+      <c r="F956" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="957">
+      <c r="A957" t="inlineStr">
+        <is>
+          <t>2026-08-08T19:46:00</t>
+        </is>
+      </c>
+      <c r="B957" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C957" t="inlineStr">
+        <is>
+          <t>TPS Enabled</t>
+        </is>
+      </c>
+      <c r="D957" t="b">
+        <v>0</v>
+      </c>
+      <c r="E957" t="n">
+        <v>11</v>
+      </c>
+      <c r="F957" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="958">
+      <c r="A958" t="inlineStr">
+        <is>
+          <t>2026-08-08T19:46:00</t>
+        </is>
+      </c>
+      <c r="B958" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C958" t="inlineStr">
+        <is>
+          <t>tk_Abort</t>
+        </is>
+      </c>
+      <c r="D958" t="b">
+        <v>0</v>
+      </c>
+      <c r="E958" t="n">
+        <v>11</v>
+      </c>
+      <c r="F958" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="959">
+      <c r="A959" t="inlineStr">
+        <is>
+          <t>2026-08-08T19:46:00</t>
+        </is>
+      </c>
+      <c r="B959" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C959" t="inlineStr">
+        <is>
+          <t>Robot_isMoving</t>
+        </is>
+      </c>
+      <c r="D959" t="b">
+        <v>0</v>
+      </c>
+      <c r="E959" t="n">
+        <v>11</v>
+      </c>
+      <c r="F959" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="960">
+      <c r="A960" t="inlineStr">
+        <is>
+          <t>2026-08-08T19:46:00</t>
+        </is>
+      </c>
+      <c r="B960" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C960" t="inlineStr">
+        <is>
+          <t>Eject Tie Plate</t>
+        </is>
+      </c>
+      <c r="D960" t="b">
+        <v>0</v>
+      </c>
+      <c r="E960" t="n">
+        <v>11</v>
+      </c>
+      <c r="F960" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="961">
+      <c r="A961" t="inlineStr">
+        <is>
+          <t>2026-08-08T19:46:00</t>
+        </is>
+      </c>
+      <c r="B961" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C961" t="inlineStr">
+        <is>
+          <t>TPS BACKUP ALARM</t>
+        </is>
+      </c>
+      <c r="D961" t="b">
+        <v>0</v>
+      </c>
+      <c r="E961" t="n">
+        <v>11</v>
+      </c>
+      <c r="F961" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="962">
+      <c r="A962" t="inlineStr">
+        <is>
+          <t>2026-08-08T19:46:00</t>
+        </is>
+      </c>
+      <c r="B962" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C962" t="inlineStr">
+        <is>
+          <t>14in Job</t>
+        </is>
+      </c>
+      <c r="D962" t="b">
+        <v>1</v>
+      </c>
+      <c r="E962" t="n">
+        <v>11</v>
+      </c>
+      <c r="F962" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="963">
+      <c r="A963" t="inlineStr">
+        <is>
+          <t>2026-08-08T19:46:00</t>
+        </is>
+      </c>
+      <c r="B963" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C963" t="inlineStr">
+        <is>
+          <t>18in Job</t>
+        </is>
+      </c>
+      <c r="D963" t="b">
+        <v>0</v>
+      </c>
+      <c r="E963" t="n">
+        <v>11</v>
+      </c>
+      <c r="F963" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="964">
+      <c r="A964" t="inlineStr">
+        <is>
+          <t>2026-08-08T19:46:00</t>
+        </is>
+      </c>
+      <c r="B964" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C964" t="inlineStr">
+        <is>
+          <t>Pandral Job</t>
+        </is>
+      </c>
+      <c r="D964" t="b">
+        <v>0</v>
+      </c>
+      <c r="E964" t="n">
+        <v>11</v>
+      </c>
+      <c r="F964" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="965">
+      <c r="A965" t="inlineStr">
+        <is>
+          <t>2026-08-08T19:46:00</t>
+        </is>
+      </c>
+      <c r="B965" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C965" t="inlineStr">
+        <is>
+          <t>DoubleLay Job</t>
+        </is>
+      </c>
+      <c r="D965" t="b">
+        <v>0</v>
+      </c>
+      <c r="E965" t="n">
+        <v>11</v>
+      </c>
+      <c r="F965" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="966">
+      <c r="A966" t="inlineStr">
+        <is>
+          <t>2026-08-08T19:46:00</t>
+        </is>
+      </c>
+      <c r="B966" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C966" t="inlineStr">
+        <is>
+          <t>TPSjam_FLAG</t>
+        </is>
+      </c>
+      <c r="D966" t="b">
+        <v>0</v>
+      </c>
+      <c r="E966" t="n">
+        <v>11</v>
+      </c>
+      <c r="F966" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="967">
+      <c r="A967" t="inlineStr">
+        <is>
+          <t>2026-08-08T19:46:00</t>
+        </is>
+      </c>
+      <c r="B967" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C967" t="inlineStr">
+        <is>
+          <t>RoCalRequest</t>
+        </is>
+      </c>
+      <c r="D967" t="b">
+        <v>0</v>
+      </c>
+      <c r="E967" t="n">
+        <v>11</v>
+      </c>
+      <c r="F967" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="968">
+      <c r="A968" t="inlineStr">
+        <is>
+          <t>2026-08-08T19:46:00</t>
+        </is>
+      </c>
+      <c r="B968" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C968" t="inlineStr">
+        <is>
+          <t>tkCycle_TotalSeconds</t>
+        </is>
+      </c>
+      <c r="D968" t="n">
+        <v>0</v>
+      </c>
+      <c r="E968" t="n">
+        <v>9</v>
+      </c>
+      <c r="F968" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="969">
+      <c r="A969" t="inlineStr">
+        <is>
+          <t>2026-08-08T19:46:00</t>
+        </is>
+      </c>
+      <c r="B969" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C969" t="inlineStr">
+        <is>
+          <t>tkCycle_NoMoveSec</t>
+        </is>
+      </c>
+      <c r="D969" t="n">
+        <v>0</v>
+      </c>
+      <c r="E969" t="n">
+        <v>9</v>
+      </c>
+      <c r="F969" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="970">
+      <c r="A970" t="inlineStr">
+        <is>
+          <t>2026-08-08T19:46:00</t>
+        </is>
+      </c>
+      <c r="B970" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C970" t="inlineStr">
+        <is>
+          <t>tkCycle_MoveSeconds</t>
+        </is>
+      </c>
+      <c r="D970" t="n">
+        <v>0</v>
+      </c>
+      <c r="E970" t="n">
+        <v>9</v>
+      </c>
+      <c r="F970" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="971">
+      <c r="A971" t="inlineStr">
+        <is>
+          <t>2026-08-08T19:46:00</t>
+        </is>
+      </c>
+      <c r="B971" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C971" t="inlineStr">
+        <is>
+          <t>Percent time moveing</t>
+        </is>
+      </c>
+      <c r="D971" t="n">
+        <v>0</v>
+      </c>
+      <c r="E971" t="n">
+        <v>9</v>
+      </c>
+      <c r="F971" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="972">
+      <c r="A972" t="inlineStr">
+        <is>
+          <t>2026-08-08T19:46:00</t>
+        </is>
+      </c>
+      <c r="B972" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C972" t="inlineStr">
+        <is>
+          <t>Percent time not moving</t>
+        </is>
+      </c>
+      <c r="D972" t="n">
+        <v>0</v>
+      </c>
+      <c r="E972" t="n">
+        <v>9</v>
+      </c>
+      <c r="F972" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="973">
+      <c r="A973" t="inlineStr">
+        <is>
+          <t>2026-08-08T19:46:00</t>
+        </is>
+      </c>
+      <c r="B973" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C973" t="inlineStr">
+        <is>
+          <t>TotalPickPartsCount</t>
+        </is>
+      </c>
+      <c r="D973" t="n">
+        <v>0</v>
+      </c>
+      <c r="E973" t="n">
+        <v>9</v>
+      </c>
+      <c r="F973" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="974">
+      <c r="A974" t="inlineStr">
+        <is>
+          <t>2026-08-08T19:46:00</t>
+        </is>
+      </c>
+      <c r="B974" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C974" t="inlineStr">
+        <is>
+          <t>RejectPartsCount</t>
+        </is>
+      </c>
+      <c r="D974" t="n">
+        <v>0</v>
+      </c>
+      <c r="E974" t="n">
+        <v>9</v>
+      </c>
+      <c r="F974" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="975">
+      <c r="A975" t="inlineStr">
+        <is>
+          <t>2026-08-08T19:46:00</t>
+        </is>
+      </c>
+      <c r="B975" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C975" t="inlineStr">
+        <is>
+          <t>AcceptsPartsCount</t>
+        </is>
+      </c>
+      <c r="D975" t="n">
+        <v>0</v>
+      </c>
+      <c r="E975" t="n">
+        <v>9</v>
+      </c>
+      <c r="F975" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="976">
+      <c r="A976" t="inlineStr">
+        <is>
+          <t>2026-08-08T19:46:00</t>
+        </is>
+      </c>
+      <c r="B976" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C976" t="inlineStr">
+        <is>
+          <t>percentCount_accept</t>
+        </is>
+      </c>
+      <c r="D976" t="n">
+        <v>0</v>
+      </c>
+      <c r="E976" t="n">
+        <v>9</v>
+      </c>
+      <c r="F976" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="977">
+      <c r="A977" t="inlineStr">
+        <is>
+          <t>2026-08-08T19:46:00</t>
+        </is>
+      </c>
+      <c r="B977" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C977" t="inlineStr">
+        <is>
+          <t>percentCount_reject</t>
+        </is>
+      </c>
+      <c r="D977" t="n">
+        <v>0</v>
+      </c>
+      <c r="E977" t="n">
+        <v>9</v>
+      </c>
+      <c r="F977" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="978">
+      <c r="A978" t="inlineStr">
+        <is>
+          <t>2026-08-08T19:46:00</t>
+        </is>
+      </c>
+      <c r="B978" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C978" t="inlineStr">
+        <is>
+          <t>Avg Parts per min_total</t>
+        </is>
+      </c>
+      <c r="D978" t="n">
+        <v>0</v>
+      </c>
+      <c r="E978" t="n">
+        <v>9</v>
+      </c>
+      <c r="F978" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="979">
+      <c r="A979" t="inlineStr">
+        <is>
+          <t>2026-08-08T19:46:00</t>
+        </is>
+      </c>
+      <c r="B979" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C979" t="inlineStr">
+        <is>
+          <t>TotalPickedParts</t>
+        </is>
+      </c>
+      <c r="D979" t="n">
+        <v>0</v>
+      </c>
+      <c r="E979" t="n">
+        <v>3</v>
+      </c>
+      <c r="F979" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="980">
+      <c r="A980" t="inlineStr">
+        <is>
+          <t>2026-08-08T19:46:00</t>
+        </is>
+      </c>
+      <c r="B980" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C980" t="inlineStr">
+        <is>
+          <t>TotalPickedAcceptParts</t>
+        </is>
+      </c>
+      <c r="D980" t="n">
+        <v>0</v>
+      </c>
+      <c r="E980" t="n">
+        <v>3</v>
+      </c>
+      <c r="F980" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="981">
+      <c r="A981" t="inlineStr">
+        <is>
+          <t>2026-08-08T19:46:00</t>
+        </is>
+      </c>
+      <c r="B981" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C981" t="inlineStr">
+        <is>
+          <t>TotalPickedRejectParts</t>
+        </is>
+      </c>
+      <c r="D981" t="n">
+        <v>0</v>
+      </c>
+      <c r="E981" t="n">
+        <v>3</v>
+      </c>
+      <c r="F981" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="982">
+      <c r="A982" t="inlineStr">
+        <is>
+          <t>2026-08-08T19:46:00</t>
+        </is>
+      </c>
+      <c r="B982" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C982" t="inlineStr">
+        <is>
+          <t>TotalTiePlatesLaid</t>
+        </is>
+      </c>
+      <c r="D982" t="n">
+        <v>0</v>
+      </c>
+      <c r="E982" t="n">
+        <v>3</v>
+      </c>
+      <c r="F982" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="983">
+      <c r="A983" t="inlineStr">
+        <is>
+          <t>2026-08-08T19:46:00</t>
+        </is>
+      </c>
+      <c r="B983" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C983" t="inlineStr">
+        <is>
+          <t>Daily_TotalLaidPlates</t>
+        </is>
+      </c>
+      <c r="D983" t="n">
+        <v>0</v>
+      </c>
+      <c r="E983" t="n">
+        <v>3</v>
+      </c>
+      <c r="F983" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="984">
+      <c r="A984" t="inlineStr">
+        <is>
+          <t>2026-08-08T19:46:00</t>
+        </is>
+      </c>
+      <c r="B984" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C984" t="inlineStr">
+        <is>
+          <t>CountPicked14in</t>
+        </is>
+      </c>
+      <c r="D984" t="n">
+        <v>0</v>
+      </c>
+      <c r="E984" t="n">
+        <v>3</v>
+      </c>
+      <c r="F984" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="985">
+      <c r="A985" t="inlineStr">
+        <is>
+          <t>2026-08-08T19:46:00</t>
+        </is>
+      </c>
+      <c r="B985" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C985" t="inlineStr">
+        <is>
+          <t>CountPicked18in</t>
+        </is>
+      </c>
+      <c r="D985" t="n">
+        <v>0</v>
+      </c>
+      <c r="E985" t="n">
+        <v>3</v>
+      </c>
+      <c r="F985" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="986">
+      <c r="A986" t="inlineStr">
+        <is>
+          <t>2026-08-08T19:46:00</t>
+        </is>
+      </c>
+      <c r="B986" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C986" t="inlineStr">
+        <is>
+          <t>CountPickedPandral</t>
+        </is>
+      </c>
+      <c r="D986" t="n">
+        <v>0</v>
+      </c>
+      <c r="E986" t="n">
+        <v>3</v>
+      </c>
+      <c r="F986" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="987">
+      <c r="A987" t="inlineStr">
+        <is>
+          <t>2026-08-08T19:46:00</t>
+        </is>
+      </c>
+      <c r="B987" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C987" t="inlineStr">
+        <is>
+          <t>CountPickedOTM</t>
+        </is>
+      </c>
+      <c r="D987" t="n">
+        <v>0</v>
+      </c>
+      <c r="E987" t="n">
+        <v>3</v>
+      </c>
+      <c r="F987" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="988">
+      <c r="A988" t="inlineStr">
+        <is>
+          <t>2026-08-08T19:46:00</t>
+        </is>
+      </c>
+      <c r="B988" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C988" t="inlineStr">
+        <is>
+          <t>RoCals</t>
+        </is>
+      </c>
+      <c r="D988" t="n">
+        <v>0</v>
+      </c>
+      <c r="E988" t="n">
+        <v>3</v>
+      </c>
+      <c r="F988" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="989">
+      <c r="A989" t="inlineStr">
+        <is>
+          <t>2026-08-08T19:46:00</t>
+        </is>
+      </c>
+      <c r="B989" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C989" t="inlineStr">
+        <is>
+          <t>TPS_JamsUsr</t>
+        </is>
+      </c>
+      <c r="D989" t="n">
+        <v>0</v>
+      </c>
+      <c r="E989" t="n">
+        <v>3</v>
+      </c>
+      <c r="F989" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="990">
+      <c r="A990" t="inlineStr">
+        <is>
+          <t>2026-08-08T19:46:00</t>
+        </is>
+      </c>
+      <c r="B990" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C990" t="inlineStr">
+        <is>
+          <t>TPS_JamsMASTER</t>
+        </is>
+      </c>
+      <c r="D990" t="n">
+        <v>0</v>
+      </c>
+      <c r="E990" t="n">
+        <v>3</v>
+      </c>
+      <c r="F990" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="991">
+      <c r="A991" t="inlineStr">
+        <is>
+          <t>2026-08-08T19:46:00</t>
+        </is>
+      </c>
+      <c r="B991" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C991" t="inlineStr">
+        <is>
+          <t>ABORT_Master</t>
+        </is>
+      </c>
+      <c r="D991" t="n">
+        <v>0</v>
+      </c>
+      <c r="E991" t="n">
+        <v>3</v>
+      </c>
+      <c r="F991" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="992">
+      <c r="A992" t="inlineStr">
+        <is>
+          <t>2026-08-08T19:46:13</t>
+        </is>
+      </c>
+      <c r="B992" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C992" t="inlineStr">
+        <is>
+          <t>CountLaidButton</t>
+        </is>
+      </c>
+      <c r="D992" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E992" t="inlineStr"/>
+      <c r="F992" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g2</t>
+        </is>
+      </c>
+    </row>
+    <row r="993">
+      <c r="A993" t="inlineStr">
+        <is>
+          <t>2026-08-08T19:46:13</t>
+        </is>
+      </c>
+      <c r="B993" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C993" t="inlineStr">
+        <is>
+          <t>CountLaidDetector</t>
+        </is>
+      </c>
+      <c r="D993" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E993" t="inlineStr"/>
+      <c r="F993" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g3</t>
+        </is>
+      </c>
+    </row>
+    <row r="994">
+      <c r="A994" t="inlineStr">
+        <is>
+          <t>2026-08-08T19:46:13</t>
+        </is>
+      </c>
+      <c r="B994" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C994" t="inlineStr">
+        <is>
+          <t>CountLaidEncoder</t>
+        </is>
+      </c>
+      <c r="D994" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E994" t="inlineStr"/>
+      <c r="F994" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g4</t>
+        </is>
+      </c>
+    </row>
+    <row r="995">
+      <c r="A995" t="inlineStr">
+        <is>
+          <t>2026-08-08T19:46:13</t>
+        </is>
+      </c>
+      <c r="B995" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C995" t="inlineStr">
+        <is>
+          <t>CountLaid14in</t>
+        </is>
+      </c>
+      <c r="D995" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E995" t="inlineStr"/>
+      <c r="F995" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g5</t>
+        </is>
+      </c>
+    </row>
+    <row r="996">
+      <c r="A996" t="inlineStr">
+        <is>
+          <t>2026-08-08T19:46:13</t>
+        </is>
+      </c>
+      <c r="B996" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C996" t="inlineStr">
+        <is>
+          <t>CountLaid18in</t>
+        </is>
+      </c>
+      <c r="D996" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E996" t="inlineStr"/>
+      <c r="F996" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g6</t>
+        </is>
+      </c>
+    </row>
+    <row r="997">
+      <c r="A997" t="inlineStr">
+        <is>
+          <t>2026-08-08T19:46:13</t>
+        </is>
+      </c>
+      <c r="B997" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C997" t="inlineStr">
+        <is>
+          <t>CountLaidPandral</t>
+        </is>
+      </c>
+      <c r="D997" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E997" t="inlineStr"/>
+      <c r="F997" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g7</t>
+        </is>
+      </c>
+    </row>
+    <row r="998">
+      <c r="A998" t="inlineStr">
+        <is>
+          <t>2026-08-08T19:46:13</t>
+        </is>
+      </c>
+      <c r="B998" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C998" t="inlineStr">
+        <is>
+          <t>TotalTiePlatesLaid</t>
+        </is>
+      </c>
+      <c r="D998" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E998" t="inlineStr"/>
+      <c r="F998" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g1</t>
+        </is>
+      </c>
+    </row>
+    <row r="999">
+      <c r="A999" t="inlineStr">
+        <is>
+          <t>2026-08-08T19:46:13</t>
+        </is>
+      </c>
+      <c r="B999" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C999" t="inlineStr">
+        <is>
+          <t>usr_TPStime Hours10th</t>
+        </is>
+      </c>
+      <c r="D999" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E999" t="inlineStr"/>
+      <c r="F999" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g8</t>
+        </is>
+      </c>
+    </row>
+    <row r="1000">
+      <c r="A1000" t="inlineStr">
+        <is>
+          <t>2026-08-08T19:46:13</t>
+        </is>
+      </c>
+      <c r="B1000" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1000" t="inlineStr">
+        <is>
+          <t>usrTPS_miles xxx</t>
+        </is>
+      </c>
+      <c r="D1000" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E1000" t="inlineStr"/>
+      <c r="F1000" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g9</t>
+        </is>
+      </c>
+    </row>
+    <row r="1001">
+      <c r="A1001" t="inlineStr">
+        <is>
+          <t>2026-08-08T19:46:13</t>
+        </is>
+      </c>
+      <c r="B1001" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1001" t="inlineStr">
+        <is>
+          <t>TPS Connected</t>
+        </is>
+      </c>
+      <c r="D1001" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E1001" t="inlineStr"/>
+      <c r="F1001" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g10</t>
+        </is>
+      </c>
+    </row>
+    <row r="1002">
+      <c r="A1002" t="inlineStr">
+        <is>
+          <t>2026-08-08T19:46:13</t>
+        </is>
+      </c>
+      <c r="B1002" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1002" t="inlineStr">
+        <is>
+          <t>TPS Enabled</t>
+        </is>
+      </c>
+      <c r="D1002" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E1002" t="inlineStr"/>
+      <c r="F1002" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g11</t>
+        </is>
+      </c>
+    </row>
+    <row r="1003">
+      <c r="A1003" t="inlineStr">
+        <is>
+          <t>2026-08-08T19:46:13</t>
+        </is>
+      </c>
+      <c r="B1003" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1003" t="inlineStr">
+        <is>
+          <t>18in Job</t>
+        </is>
+      </c>
+      <c r="D1003" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E1003" t="inlineStr"/>
+      <c r="F1003" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g13</t>
+        </is>
+      </c>
+    </row>
+    <row r="1004">
+      <c r="A1004" t="inlineStr">
+        <is>
+          <t>2026-08-08T19:46:13</t>
+        </is>
+      </c>
+      <c r="B1004" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1004" t="inlineStr">
+        <is>
+          <t>CountAcceptedTotal</t>
+        </is>
+      </c>
+      <c r="D1004" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E1004" t="inlineStr"/>
+      <c r="F1004" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g15</t>
+        </is>
+      </c>
+    </row>
+    <row r="1005">
+      <c r="A1005" t="inlineStr">
+        <is>
+          <t>2026-08-08T19:46:13</t>
+        </is>
+      </c>
+      <c r="B1005" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1005" t="inlineStr">
+        <is>
+          <t>Servos_Enabled</t>
+        </is>
+      </c>
+      <c r="D1005" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E1005" t="inlineStr"/>
+      <c r="F1005" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g17</t>
+        </is>
+      </c>
+    </row>
+    <row r="1006">
+      <c r="A1006" t="inlineStr">
+        <is>
+          <t>2026-08-08T19:46:13</t>
+        </is>
+      </c>
+      <c r="B1006" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1006" t="inlineStr">
+        <is>
+          <t>TotalPickPartsCount</t>
+        </is>
+      </c>
+      <c r="D1006" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E1006" t="inlineStr"/>
+      <c r="F1006" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g18</t>
+        </is>
+      </c>
+    </row>
+    <row r="1007">
+      <c r="A1007" t="inlineStr">
+        <is>
+          <t>2026-08-08T19:46:13</t>
+        </is>
+      </c>
+      <c r="B1007" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1007" t="inlineStr">
+        <is>
+          <t>AcceptsPartsCount</t>
+        </is>
+      </c>
+      <c r="D1007" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E1007" t="inlineStr"/>
+      <c r="F1007" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g19</t>
+        </is>
+      </c>
+    </row>
+    <row r="1008">
+      <c r="A1008" t="inlineStr">
+        <is>
+          <t>2026-08-08T19:46:13</t>
+        </is>
+      </c>
+      <c r="B1008" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1008" t="inlineStr">
+        <is>
+          <t>day_Servotime Hours10th</t>
+        </is>
+      </c>
+      <c r="D1008" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E1008" t="inlineStr"/>
+      <c r="F1008" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g22</t>
+        </is>
+      </c>
+    </row>
+    <row r="1009">
+      <c r="A1009" t="inlineStr">
+        <is>
+          <t>2026-08-08T19:46:13</t>
+        </is>
+      </c>
+      <c r="B1009" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1009" t="inlineStr">
+        <is>
+          <t>tk_Cycle</t>
+        </is>
+      </c>
+      <c r="D1009" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E1009" t="inlineStr"/>
+      <c r="F1009" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g23</t>
+        </is>
+      </c>
+    </row>
+    <row r="1010">
+      <c r="A1010" t="inlineStr">
+        <is>
+          <t>2026-08-08T19:46:13</t>
+        </is>
+      </c>
+      <c r="B1010" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1010" t="inlineStr">
+        <is>
+          <t>tk_Abort</t>
+        </is>
+      </c>
+      <c r="D1010" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E1010" t="inlineStr"/>
+      <c r="F1010" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g24</t>
+        </is>
+      </c>
+    </row>
+    <row r="1011">
+      <c r="A1011" t="inlineStr">
+        <is>
+          <t>2026-08-08T19:46:13</t>
+        </is>
+      </c>
+      <c r="B1011" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1011" t="inlineStr">
+        <is>
+          <t>tk_ClearPos</t>
+        </is>
+      </c>
+      <c r="D1011" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E1011" t="inlineStr"/>
+      <c r="F1011" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g25</t>
+        </is>
+      </c>
+    </row>
+    <row r="1012">
+      <c r="A1012" t="inlineStr">
+        <is>
+          <t>2026-08-08T19:46:13</t>
+        </is>
+      </c>
+      <c r="B1012" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1012" t="inlineStr">
+        <is>
+          <t>temp_J2motor</t>
+        </is>
+      </c>
+      <c r="D1012" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E1012" t="inlineStr"/>
+      <c r="F1012" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g33</t>
+        </is>
+      </c>
+    </row>
+    <row r="1013">
+      <c r="A1013" t="inlineStr">
+        <is>
+          <t>2026-08-08T19:46:13</t>
+        </is>
+      </c>
+      <c r="B1013" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1013" t="inlineStr">
+        <is>
+          <t>temp_J3motor</t>
+        </is>
+      </c>
+      <c r="D1013" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E1013" t="inlineStr"/>
+      <c r="F1013" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g34</t>
+        </is>
+      </c>
+    </row>
+    <row r="1014">
+      <c r="A1014" t="inlineStr">
+        <is>
+          <t>2026-08-08T19:46:13</t>
+        </is>
+      </c>
+      <c r="B1014" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1014" t="inlineStr">
+        <is>
+          <t>temp_J5motor</t>
+        </is>
+      </c>
+      <c r="D1014" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E1014" t="inlineStr"/>
+      <c r="F1014" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g36</t>
+        </is>
+      </c>
+    </row>
+    <row r="1015">
+      <c r="A1015" t="inlineStr">
+        <is>
+          <t>2026-08-08T19:46:13</t>
+        </is>
+      </c>
+      <c r="B1015" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1015" t="inlineStr">
+        <is>
+          <t>CountPickedReject18in</t>
+        </is>
+      </c>
+      <c r="D1015" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E1015" t="inlineStr"/>
+      <c r="F1015" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g40</t>
+        </is>
+      </c>
+    </row>
+    <row r="1016">
+      <c r="A1016" t="inlineStr">
+        <is>
+          <t>2026-08-08T19:46:13</t>
+        </is>
+      </c>
+      <c r="B1016" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1016" t="inlineStr">
+        <is>
+          <t>14in Job</t>
+        </is>
+      </c>
+      <c r="D1016" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E1016" t="inlineStr"/>
+      <c r="F1016" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g12</t>
+        </is>
+      </c>
+    </row>
+    <row r="1017">
+      <c r="A1017" t="inlineStr">
+        <is>
+          <t>2026-08-08T19:46:13</t>
+        </is>
+      </c>
+      <c r="B1017" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1017" t="inlineStr">
+        <is>
+          <t>Pandral Job</t>
+        </is>
+      </c>
+      <c r="D1017" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E1017" t="inlineStr"/>
+      <c r="F1017" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g14</t>
+        </is>
+      </c>
+    </row>
+    <row r="1018">
+      <c r="A1018" t="inlineStr">
+        <is>
+          <t>2026-08-08T19:46:13</t>
+        </is>
+      </c>
+      <c r="B1018" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1018" t="inlineStr">
+        <is>
+          <t>CountRejectedTotal</t>
+        </is>
+      </c>
+      <c r="D1018" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E1018" t="inlineStr"/>
+      <c r="F1018" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g16</t>
+        </is>
+      </c>
+    </row>
+    <row r="1019">
+      <c r="A1019" t="inlineStr">
+        <is>
+          <t>2026-08-08T19:46:13</t>
+        </is>
+      </c>
+      <c r="B1019" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1019" t="inlineStr">
+        <is>
+          <t>RejectPartsCount</t>
+        </is>
+      </c>
+      <c r="D1019" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E1019" t="inlineStr"/>
+      <c r="F1019" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g20</t>
+        </is>
+      </c>
+    </row>
+    <row r="1020">
+      <c r="A1020" t="inlineStr">
+        <is>
+          <t>2026-08-08T19:46:13</t>
+        </is>
+      </c>
+      <c r="B1020" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1020" t="inlineStr">
+        <is>
+          <t>tk_Cycle hrs</t>
+        </is>
+      </c>
+      <c r="D1020" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E1020" t="inlineStr"/>
+      <c r="F1020" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g21</t>
+        </is>
+      </c>
+    </row>
+    <row r="1021">
+      <c r="A1021" t="inlineStr">
+        <is>
+          <t>2026-08-08T19:46:13</t>
+        </is>
+      </c>
+      <c r="B1021" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1021" t="inlineStr">
+        <is>
+          <t>tk_Warmup</t>
+        </is>
+      </c>
+      <c r="D1021" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E1021" t="inlineStr"/>
+      <c r="F1021" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g26</t>
+        </is>
+      </c>
+    </row>
+    <row r="1022">
+      <c r="A1022" t="inlineStr">
+        <is>
+          <t>2026-08-08T19:46:13</t>
+        </is>
+      </c>
+      <c r="B1022" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1022" t="inlineStr">
+        <is>
+          <t>FindingParts min</t>
+        </is>
+      </c>
+      <c r="D1022" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E1022" t="inlineStr"/>
+      <c r="F1022" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g27</t>
+        </is>
+      </c>
+    </row>
+    <row r="1023">
+      <c r="A1023" t="inlineStr">
+        <is>
+          <t>2026-08-08T19:46:13</t>
+        </is>
+      </c>
+      <c r="B1023" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1023" t="inlineStr">
+        <is>
+          <t>PickingParts min</t>
+        </is>
+      </c>
+      <c r="D1023" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E1023" t="inlineStr"/>
+      <c r="F1023" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g28</t>
+        </is>
+      </c>
+    </row>
+    <row r="1024">
+      <c r="A1024" t="inlineStr">
+        <is>
+          <t>2026-08-08T19:46:13</t>
+        </is>
+      </c>
+      <c r="B1024" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1024" t="inlineStr">
+        <is>
+          <t>PlacingParts min</t>
+        </is>
+      </c>
+      <c r="D1024" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E1024" t="inlineStr"/>
+      <c r="F1024" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g29</t>
+        </is>
+      </c>
+    </row>
+    <row r="1025">
+      <c r="A1025" t="inlineStr">
+        <is>
+          <t>2026-08-08T19:46:13</t>
+        </is>
+      </c>
+      <c r="B1025" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1025" t="inlineStr">
+        <is>
+          <t>CountPickedReject14in</t>
+        </is>
+      </c>
+      <c r="D1025" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E1025" t="inlineStr"/>
+      <c r="F1025" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g30</t>
+        </is>
+      </c>
+    </row>
+    <row r="1026">
+      <c r="A1026" t="inlineStr">
+        <is>
+          <t>2026-08-08T19:46:13</t>
+        </is>
+      </c>
+      <c r="B1026" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1026" t="inlineStr">
+        <is>
+          <t>temp_dsi</t>
+        </is>
+      </c>
+      <c r="D1026" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E1026" t="inlineStr"/>
+      <c r="F1026" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g31</t>
+        </is>
+      </c>
+    </row>
+    <row r="1027">
+      <c r="A1027" t="inlineStr">
+        <is>
+          <t>2026-08-08T19:46:13</t>
+        </is>
+      </c>
+      <c r="B1027" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1027" t="inlineStr">
+        <is>
+          <t>temp_J1motor</t>
+        </is>
+      </c>
+      <c r="D1027" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E1027" t="inlineStr"/>
+      <c r="F1027" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g32</t>
+        </is>
+      </c>
+    </row>
+    <row r="1028">
+      <c r="A1028" t="inlineStr">
+        <is>
+          <t>2026-08-08T19:46:13</t>
+        </is>
+      </c>
+      <c r="B1028" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1028" t="inlineStr">
+        <is>
+          <t>temp_J4motor</t>
+        </is>
+      </c>
+      <c r="D1028" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E1028" t="inlineStr"/>
+      <c r="F1028" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g35</t>
+        </is>
+      </c>
+    </row>
+    <row r="1029">
+      <c r="A1029" t="inlineStr">
+        <is>
+          <t>2026-08-08T19:46:13</t>
+        </is>
+      </c>
+      <c r="B1029" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1029" t="inlineStr">
+        <is>
+          <t>temp_J6motor</t>
+        </is>
+      </c>
+      <c r="D1029" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E1029" t="inlineStr"/>
+      <c r="F1029" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g37</t>
+        </is>
+      </c>
+    </row>
+    <row r="1030">
+      <c r="A1030" t="inlineStr">
+        <is>
+          <t>2026-08-08T19:46:13</t>
+        </is>
+      </c>
+      <c r="B1030" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1030" t="inlineStr">
+        <is>
+          <t>CountPickedRejectOTM</t>
+        </is>
+      </c>
+      <c r="D1030" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E1030" t="inlineStr"/>
+      <c r="F1030" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g38</t>
+        </is>
+      </c>
+    </row>
+    <row r="1031">
+      <c r="A1031" t="inlineStr">
+        <is>
+          <t>2026-08-08T19:46:13</t>
+        </is>
+      </c>
+      <c r="B1031" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1031" t="inlineStr">
+        <is>
+          <t>CountPickedRejectPandral</t>
+        </is>
+      </c>
+      <c r="D1031" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E1031" t="inlineStr"/>
+      <c r="F1031" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g39</t>
+        </is>
+      </c>
+    </row>
+    <row r="1032">
+      <c r="A1032" t="inlineStr">
+        <is>
+          <t>2026-08-08T19:47:00</t>
+        </is>
+      </c>
+      <c r="B1032" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1032" t="inlineStr">
+        <is>
+          <t>_1st_SCAN</t>
+        </is>
+      </c>
+      <c r="D1032" t="b">
+        <v>0</v>
+      </c>
+      <c r="E1032" t="n">
+        <v>11</v>
+      </c>
+      <c r="F1032" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1033">
+      <c r="A1033" t="inlineStr">
+        <is>
+          <t>2026-08-08T19:47:00</t>
+        </is>
+      </c>
+      <c r="B1033" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1033" t="inlineStr">
+        <is>
+          <t>TieDetectOffset_B</t>
+        </is>
+      </c>
+      <c r="D1033" t="b">
+        <v>0</v>
+      </c>
+      <c r="E1033" t="n">
+        <v>11</v>
+      </c>
+      <c r="F1033" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1034">
+      <c r="A1034" t="inlineStr">
+        <is>
+          <t>2026-08-08T19:47:00</t>
+        </is>
+      </c>
+      <c r="B1034" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1034" t="inlineStr">
+        <is>
+          <t>Tie Detector</t>
+        </is>
+      </c>
+      <c r="D1034" t="b">
+        <v>0</v>
+      </c>
+      <c r="E1034" t="n">
+        <v>11</v>
+      </c>
+      <c r="F1034" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1035">
+      <c r="A1035" t="inlineStr">
+        <is>
+          <t>2026-08-08T19:47:00</t>
+        </is>
+      </c>
+      <c r="B1035" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1035" t="inlineStr">
+        <is>
+          <t>TPS Full</t>
+        </is>
+      </c>
+      <c r="D1035" t="b">
+        <v>0</v>
+      </c>
+      <c r="E1035" t="n">
+        <v>11</v>
+      </c>
+      <c r="F1035" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1036">
+      <c r="A1036" t="inlineStr">
+        <is>
+          <t>2026-08-08T19:47:00</t>
+        </is>
+      </c>
+      <c r="B1036" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1036" t="inlineStr">
+        <is>
+          <t>TieDetectOffset_A</t>
+        </is>
+      </c>
+      <c r="D1036" t="b">
+        <v>0</v>
+      </c>
+      <c r="E1036" t="n">
+        <v>11</v>
+      </c>
+      <c r="F1036" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1037">
+      <c r="A1037" t="inlineStr">
+        <is>
+          <t>2026-08-08T19:47:00</t>
+        </is>
+      </c>
+      <c r="B1037" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1037" t="inlineStr">
+        <is>
+          <t>TPS Connected</t>
+        </is>
+      </c>
+      <c r="D1037" t="b">
+        <v>0</v>
+      </c>
+      <c r="E1037" t="n">
+        <v>11</v>
+      </c>
+      <c r="F1037" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1038">
+      <c r="A1038" t="inlineStr">
+        <is>
+          <t>2026-08-08T19:47:00</t>
+        </is>
+      </c>
+      <c r="B1038" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1038" t="inlineStr">
+        <is>
+          <t>TPS_Enable_ Button</t>
+        </is>
+      </c>
+      <c r="D1038" t="b">
+        <v>0</v>
+      </c>
+      <c r="E1038" t="n">
+        <v>11</v>
+      </c>
+      <c r="F1038" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1039">
+      <c r="A1039" t="inlineStr">
+        <is>
+          <t>2026-08-08T19:47:00</t>
+        </is>
+      </c>
+      <c r="B1039" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1039" t="inlineStr">
+        <is>
+          <t>AirEagle Eject Plate</t>
+        </is>
+      </c>
+      <c r="D1039" t="b">
+        <v>0</v>
+      </c>
+      <c r="E1039" t="n">
+        <v>11</v>
+      </c>
+      <c r="F1039" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1040">
+      <c r="A1040" t="inlineStr">
+        <is>
+          <t>2026-08-08T19:47:00</t>
+        </is>
+      </c>
+      <c r="B1040" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1040" t="inlineStr">
+        <is>
+          <t>tk_Cycle</t>
+        </is>
+      </c>
+      <c r="D1040" t="b">
+        <v>0</v>
+      </c>
+      <c r="E1040" t="n">
+        <v>11</v>
+      </c>
+      <c r="F1040" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1041">
+      <c r="A1041" t="inlineStr">
+        <is>
+          <t>2026-08-08T19:47:00</t>
+        </is>
+      </c>
+      <c r="B1041" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1041" t="inlineStr">
+        <is>
+          <t>Servos_Enabled</t>
+        </is>
+      </c>
+      <c r="D1041" t="b">
+        <v>0</v>
+      </c>
+      <c r="E1041" t="n">
+        <v>11</v>
+      </c>
+      <c r="F1041" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1042">
+      <c r="A1042" t="inlineStr">
+        <is>
+          <t>2026-08-08T19:47:00</t>
+        </is>
+      </c>
+      <c r="B1042" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1042" t="inlineStr">
+        <is>
+          <t>TPS Enabled</t>
+        </is>
+      </c>
+      <c r="D1042" t="b">
+        <v>0</v>
+      </c>
+      <c r="E1042" t="n">
+        <v>11</v>
+      </c>
+      <c r="F1042" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1043">
+      <c r="A1043" t="inlineStr">
+        <is>
+          <t>2026-08-08T19:47:00</t>
+        </is>
+      </c>
+      <c r="B1043" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1043" t="inlineStr">
+        <is>
+          <t>tk_Abort</t>
+        </is>
+      </c>
+      <c r="D1043" t="b">
+        <v>0</v>
+      </c>
+      <c r="E1043" t="n">
+        <v>11</v>
+      </c>
+      <c r="F1043" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1044">
+      <c r="A1044" t="inlineStr">
+        <is>
+          <t>2026-08-08T19:47:00</t>
+        </is>
+      </c>
+      <c r="B1044" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1044" t="inlineStr">
+        <is>
+          <t>Robot_isMoving</t>
+        </is>
+      </c>
+      <c r="D1044" t="b">
+        <v>0</v>
+      </c>
+      <c r="E1044" t="n">
+        <v>11</v>
+      </c>
+      <c r="F1044" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1045">
+      <c r="A1045" t="inlineStr">
+        <is>
+          <t>2026-08-08T19:47:00</t>
+        </is>
+      </c>
+      <c r="B1045" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1045" t="inlineStr">
+        <is>
+          <t>Eject Tie Plate</t>
+        </is>
+      </c>
+      <c r="D1045" t="b">
+        <v>0</v>
+      </c>
+      <c r="E1045" t="n">
+        <v>11</v>
+      </c>
+      <c r="F1045" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1046">
+      <c r="A1046" t="inlineStr">
+        <is>
+          <t>2026-08-08T19:47:00</t>
+        </is>
+      </c>
+      <c r="B1046" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1046" t="inlineStr">
+        <is>
+          <t>TPS BACKUP ALARM</t>
+        </is>
+      </c>
+      <c r="D1046" t="b">
+        <v>0</v>
+      </c>
+      <c r="E1046" t="n">
+        <v>11</v>
+      </c>
+      <c r="F1046" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1047">
+      <c r="A1047" t="inlineStr">
+        <is>
+          <t>2026-08-08T19:47:00</t>
+        </is>
+      </c>
+      <c r="B1047" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1047" t="inlineStr">
+        <is>
+          <t>14in Job</t>
+        </is>
+      </c>
+      <c r="D1047" t="b">
+        <v>1</v>
+      </c>
+      <c r="E1047" t="n">
+        <v>11</v>
+      </c>
+      <c r="F1047" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1048">
+      <c r="A1048" t="inlineStr">
+        <is>
+          <t>2026-08-08T19:47:00</t>
+        </is>
+      </c>
+      <c r="B1048" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1048" t="inlineStr">
+        <is>
+          <t>18in Job</t>
+        </is>
+      </c>
+      <c r="D1048" t="b">
+        <v>0</v>
+      </c>
+      <c r="E1048" t="n">
+        <v>11</v>
+      </c>
+      <c r="F1048" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1049">
+      <c r="A1049" t="inlineStr">
+        <is>
+          <t>2026-08-08T19:47:00</t>
+        </is>
+      </c>
+      <c r="B1049" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1049" t="inlineStr">
+        <is>
+          <t>Pandral Job</t>
+        </is>
+      </c>
+      <c r="D1049" t="b">
+        <v>0</v>
+      </c>
+      <c r="E1049" t="n">
+        <v>11</v>
+      </c>
+      <c r="F1049" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1050">
+      <c r="A1050" t="inlineStr">
+        <is>
+          <t>2026-08-08T19:47:00</t>
+        </is>
+      </c>
+      <c r="B1050" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1050" t="inlineStr">
+        <is>
+          <t>DoubleLay Job</t>
+        </is>
+      </c>
+      <c r="D1050" t="b">
+        <v>0</v>
+      </c>
+      <c r="E1050" t="n">
+        <v>11</v>
+      </c>
+      <c r="F1050" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1051">
+      <c r="A1051" t="inlineStr">
+        <is>
+          <t>2026-08-08T19:47:00</t>
+        </is>
+      </c>
+      <c r="B1051" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1051" t="inlineStr">
+        <is>
+          <t>TPSjam_FLAG</t>
+        </is>
+      </c>
+      <c r="D1051" t="b">
+        <v>0</v>
+      </c>
+      <c r="E1051" t="n">
+        <v>11</v>
+      </c>
+      <c r="F1051" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1052">
+      <c r="A1052" t="inlineStr">
+        <is>
+          <t>2026-08-08T19:47:00</t>
+        </is>
+      </c>
+      <c r="B1052" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1052" t="inlineStr">
+        <is>
+          <t>RoCalRequest</t>
+        </is>
+      </c>
+      <c r="D1052" t="b">
+        <v>0</v>
+      </c>
+      <c r="E1052" t="n">
+        <v>11</v>
+      </c>
+      <c r="F1052" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1053">
+      <c r="A1053" t="inlineStr">
+        <is>
+          <t>2026-08-08T19:47:00</t>
+        </is>
+      </c>
+      <c r="B1053" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1053" t="inlineStr">
+        <is>
+          <t>tkCycle_TotalSeconds</t>
+        </is>
+      </c>
+      <c r="D1053" t="n">
+        <v>0</v>
+      </c>
+      <c r="E1053" t="n">
+        <v>9</v>
+      </c>
+      <c r="F1053" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1054">
+      <c r="A1054" t="inlineStr">
+        <is>
+          <t>2026-08-08T19:47:00</t>
+        </is>
+      </c>
+      <c r="B1054" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1054" t="inlineStr">
+        <is>
+          <t>tkCycle_NoMoveSec</t>
+        </is>
+      </c>
+      <c r="D1054" t="n">
+        <v>0</v>
+      </c>
+      <c r="E1054" t="n">
+        <v>9</v>
+      </c>
+      <c r="F1054" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1055">
+      <c r="A1055" t="inlineStr">
+        <is>
+          <t>2026-08-08T19:47:00</t>
+        </is>
+      </c>
+      <c r="B1055" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1055" t="inlineStr">
+        <is>
+          <t>tkCycle_MoveSeconds</t>
+        </is>
+      </c>
+      <c r="D1055" t="n">
+        <v>0</v>
+      </c>
+      <c r="E1055" t="n">
+        <v>9</v>
+      </c>
+      <c r="F1055" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1056">
+      <c r="A1056" t="inlineStr">
+        <is>
+          <t>2026-08-08T19:47:00</t>
+        </is>
+      </c>
+      <c r="B1056" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1056" t="inlineStr">
+        <is>
+          <t>Percent time moveing</t>
+        </is>
+      </c>
+      <c r="D1056" t="n">
+        <v>0</v>
+      </c>
+      <c r="E1056" t="n">
+        <v>9</v>
+      </c>
+      <c r="F1056" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1057">
+      <c r="A1057" t="inlineStr">
+        <is>
+          <t>2026-08-08T19:47:00</t>
+        </is>
+      </c>
+      <c r="B1057" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1057" t="inlineStr">
+        <is>
+          <t>Percent time not moving</t>
+        </is>
+      </c>
+      <c r="D1057" t="n">
+        <v>0</v>
+      </c>
+      <c r="E1057" t="n">
+        <v>9</v>
+      </c>
+      <c r="F1057" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1058">
+      <c r="A1058" t="inlineStr">
+        <is>
+          <t>2026-08-08T19:47:00</t>
+        </is>
+      </c>
+      <c r="B1058" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1058" t="inlineStr">
+        <is>
+          <t>TotalPickPartsCount</t>
+        </is>
+      </c>
+      <c r="D1058" t="n">
+        <v>0</v>
+      </c>
+      <c r="E1058" t="n">
+        <v>9</v>
+      </c>
+      <c r="F1058" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1059">
+      <c r="A1059" t="inlineStr">
+        <is>
+          <t>2026-08-08T19:47:00</t>
+        </is>
+      </c>
+      <c r="B1059" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1059" t="inlineStr">
+        <is>
+          <t>RejectPartsCount</t>
+        </is>
+      </c>
+      <c r="D1059" t="n">
+        <v>0</v>
+      </c>
+      <c r="E1059" t="n">
+        <v>9</v>
+      </c>
+      <c r="F1059" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1060">
+      <c r="A1060" t="inlineStr">
+        <is>
+          <t>2026-08-08T19:47:00</t>
+        </is>
+      </c>
+      <c r="B1060" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1060" t="inlineStr">
+        <is>
+          <t>AcceptsPartsCount</t>
+        </is>
+      </c>
+      <c r="D1060" t="n">
+        <v>0</v>
+      </c>
+      <c r="E1060" t="n">
+        <v>9</v>
+      </c>
+      <c r="F1060" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1061">
+      <c r="A1061" t="inlineStr">
+        <is>
+          <t>2026-08-08T19:47:00</t>
+        </is>
+      </c>
+      <c r="B1061" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1061" t="inlineStr">
+        <is>
+          <t>percentCount_accept</t>
+        </is>
+      </c>
+      <c r="D1061" t="n">
+        <v>0</v>
+      </c>
+      <c r="E1061" t="n">
+        <v>9</v>
+      </c>
+      <c r="F1061" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1062">
+      <c r="A1062" t="inlineStr">
+        <is>
+          <t>2026-08-08T19:47:00</t>
+        </is>
+      </c>
+      <c r="B1062" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1062" t="inlineStr">
+        <is>
+          <t>percentCount_reject</t>
+        </is>
+      </c>
+      <c r="D1062" t="n">
+        <v>0</v>
+      </c>
+      <c r="E1062" t="n">
+        <v>9</v>
+      </c>
+      <c r="F1062" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1063">
+      <c r="A1063" t="inlineStr">
+        <is>
+          <t>2026-08-08T19:47:00</t>
+        </is>
+      </c>
+      <c r="B1063" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1063" t="inlineStr">
+        <is>
+          <t>Avg Parts per min_total</t>
+        </is>
+      </c>
+      <c r="D1063" t="n">
+        <v>0</v>
+      </c>
+      <c r="E1063" t="n">
+        <v>9</v>
+      </c>
+      <c r="F1063" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1064">
+      <c r="A1064" t="inlineStr">
+        <is>
+          <t>2026-08-08T19:47:00</t>
+        </is>
+      </c>
+      <c r="B1064" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1064" t="inlineStr">
+        <is>
+          <t>TotalPickedParts</t>
+        </is>
+      </c>
+      <c r="D1064" t="n">
+        <v>0</v>
+      </c>
+      <c r="E1064" t="n">
+        <v>3</v>
+      </c>
+      <c r="F1064" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1065">
+      <c r="A1065" t="inlineStr">
+        <is>
+          <t>2026-08-08T19:47:00</t>
+        </is>
+      </c>
+      <c r="B1065" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1065" t="inlineStr">
+        <is>
+          <t>TotalPickedAcceptParts</t>
+        </is>
+      </c>
+      <c r="D1065" t="n">
+        <v>0</v>
+      </c>
+      <c r="E1065" t="n">
+        <v>3</v>
+      </c>
+      <c r="F1065" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1066">
+      <c r="A1066" t="inlineStr">
+        <is>
+          <t>2026-08-08T19:47:00</t>
+        </is>
+      </c>
+      <c r="B1066" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1066" t="inlineStr">
+        <is>
+          <t>TotalPickedRejectParts</t>
+        </is>
+      </c>
+      <c r="D1066" t="n">
+        <v>0</v>
+      </c>
+      <c r="E1066" t="n">
+        <v>3</v>
+      </c>
+      <c r="F1066" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1067">
+      <c r="A1067" t="inlineStr">
+        <is>
+          <t>2026-08-08T19:47:00</t>
+        </is>
+      </c>
+      <c r="B1067" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1067" t="inlineStr">
+        <is>
+          <t>TotalTiePlatesLaid</t>
+        </is>
+      </c>
+      <c r="D1067" t="n">
+        <v>0</v>
+      </c>
+      <c r="E1067" t="n">
+        <v>3</v>
+      </c>
+      <c r="F1067" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1068">
+      <c r="A1068" t="inlineStr">
+        <is>
+          <t>2026-08-08T19:47:00</t>
+        </is>
+      </c>
+      <c r="B1068" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1068" t="inlineStr">
+        <is>
+          <t>Daily_TotalLaidPlates</t>
+        </is>
+      </c>
+      <c r="D1068" t="n">
+        <v>0</v>
+      </c>
+      <c r="E1068" t="n">
+        <v>3</v>
+      </c>
+      <c r="F1068" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1069">
+      <c r="A1069" t="inlineStr">
+        <is>
+          <t>2026-08-08T19:47:00</t>
+        </is>
+      </c>
+      <c r="B1069" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1069" t="inlineStr">
+        <is>
+          <t>CountPicked14in</t>
+        </is>
+      </c>
+      <c r="D1069" t="n">
+        <v>0</v>
+      </c>
+      <c r="E1069" t="n">
+        <v>3</v>
+      </c>
+      <c r="F1069" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1070">
+      <c r="A1070" t="inlineStr">
+        <is>
+          <t>2026-08-08T19:47:00</t>
+        </is>
+      </c>
+      <c r="B1070" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1070" t="inlineStr">
+        <is>
+          <t>CountPicked18in</t>
+        </is>
+      </c>
+      <c r="D1070" t="n">
+        <v>0</v>
+      </c>
+      <c r="E1070" t="n">
+        <v>3</v>
+      </c>
+      <c r="F1070" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1071">
+      <c r="A1071" t="inlineStr">
+        <is>
+          <t>2026-08-08T19:47:00</t>
+        </is>
+      </c>
+      <c r="B1071" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1071" t="inlineStr">
+        <is>
+          <t>CountPickedPandral</t>
+        </is>
+      </c>
+      <c r="D1071" t="n">
+        <v>0</v>
+      </c>
+      <c r="E1071" t="n">
+        <v>3</v>
+      </c>
+      <c r="F1071" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1072">
+      <c r="A1072" t="inlineStr">
+        <is>
+          <t>2026-08-08T19:47:00</t>
+        </is>
+      </c>
+      <c r="B1072" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1072" t="inlineStr">
+        <is>
+          <t>CountPickedOTM</t>
+        </is>
+      </c>
+      <c r="D1072" t="n">
+        <v>0</v>
+      </c>
+      <c r="E1072" t="n">
+        <v>3</v>
+      </c>
+      <c r="F1072" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1073">
+      <c r="A1073" t="inlineStr">
+        <is>
+          <t>2026-08-08T19:47:00</t>
+        </is>
+      </c>
+      <c r="B1073" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1073" t="inlineStr">
+        <is>
+          <t>RoCals</t>
+        </is>
+      </c>
+      <c r="D1073" t="n">
+        <v>0</v>
+      </c>
+      <c r="E1073" t="n">
+        <v>3</v>
+      </c>
+      <c r="F1073" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1074">
+      <c r="A1074" t="inlineStr">
+        <is>
+          <t>2026-08-08T19:47:00</t>
+        </is>
+      </c>
+      <c r="B1074" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1074" t="inlineStr">
+        <is>
+          <t>TPS_JamsUsr</t>
+        </is>
+      </c>
+      <c r="D1074" t="n">
+        <v>0</v>
+      </c>
+      <c r="E1074" t="n">
+        <v>3</v>
+      </c>
+      <c r="F1074" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1075">
+      <c r="A1075" t="inlineStr">
+        <is>
+          <t>2026-08-08T19:47:00</t>
+        </is>
+      </c>
+      <c r="B1075" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1075" t="inlineStr">
+        <is>
+          <t>TPS_JamsMASTER</t>
+        </is>
+      </c>
+      <c r="D1075" t="n">
+        <v>0</v>
+      </c>
+      <c r="E1075" t="n">
+        <v>3</v>
+      </c>
+      <c r="F1075" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1076">
+      <c r="A1076" t="inlineStr">
+        <is>
+          <t>2026-08-08T19:47:00</t>
+        </is>
+      </c>
+      <c r="B1076" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1076" t="inlineStr">
+        <is>
+          <t>ABORT_Master</t>
+        </is>
+      </c>
+      <c r="D1076" t="n">
+        <v>0</v>
+      </c>
+      <c r="E1076" t="n">
+        <v>3</v>
+      </c>
+      <c r="F1076" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/plc</t>
         </is>

</xml_diff>

<commit_message>
Log MQTT data 2026-08-08 21:05 UTC
</commit_message>
<xml_diff>
--- a/logs/raiv_tracker_2026-08-08.xlsx
+++ b/logs/raiv_tracker_2026-08-08.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F1076"/>
+  <dimension ref="A1:F1206"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -27829,7 +27829,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E992" t="inlineStr"/>
       <c r="F992" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g2</t>
@@ -27857,7 +27856,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E993" t="inlineStr"/>
       <c r="F993" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g3</t>
@@ -27885,7 +27883,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E994" t="inlineStr"/>
       <c r="F994" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g4</t>
@@ -27913,7 +27910,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E995" t="inlineStr"/>
       <c r="F995" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g5</t>
@@ -27941,7 +27937,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E996" t="inlineStr"/>
       <c r="F996" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g6</t>
@@ -27969,7 +27964,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E997" t="inlineStr"/>
       <c r="F997" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g7</t>
@@ -27997,7 +27991,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E998" t="inlineStr"/>
       <c r="F998" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g1</t>
@@ -28025,7 +28018,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E999" t="inlineStr"/>
       <c r="F999" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g8</t>
@@ -28053,7 +28045,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E1000" t="inlineStr"/>
       <c r="F1000" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g9</t>
@@ -28081,7 +28072,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E1001" t="inlineStr"/>
       <c r="F1001" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g10</t>
@@ -28109,7 +28099,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E1002" t="inlineStr"/>
       <c r="F1002" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g11</t>
@@ -28137,7 +28126,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E1003" t="inlineStr"/>
       <c r="F1003" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g13</t>
@@ -28165,7 +28153,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E1004" t="inlineStr"/>
       <c r="F1004" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g15</t>
@@ -28193,7 +28180,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E1005" t="inlineStr"/>
       <c r="F1005" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g17</t>
@@ -28221,7 +28207,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E1006" t="inlineStr"/>
       <c r="F1006" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g18</t>
@@ -28249,7 +28234,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E1007" t="inlineStr"/>
       <c r="F1007" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g19</t>
@@ -28277,7 +28261,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E1008" t="inlineStr"/>
       <c r="F1008" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g22</t>
@@ -28305,7 +28288,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E1009" t="inlineStr"/>
       <c r="F1009" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g23</t>
@@ -28333,7 +28315,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E1010" t="inlineStr"/>
       <c r="F1010" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g24</t>
@@ -28361,7 +28342,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E1011" t="inlineStr"/>
       <c r="F1011" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g25</t>
@@ -28389,7 +28369,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E1012" t="inlineStr"/>
       <c r="F1012" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g33</t>
@@ -28417,7 +28396,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E1013" t="inlineStr"/>
       <c r="F1013" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g34</t>
@@ -28445,7 +28423,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E1014" t="inlineStr"/>
       <c r="F1014" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g36</t>
@@ -28473,7 +28450,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E1015" t="inlineStr"/>
       <c r="F1015" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g40</t>
@@ -28501,7 +28477,6 @@
           <t>1</t>
         </is>
       </c>
-      <c r="E1016" t="inlineStr"/>
       <c r="F1016" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g12</t>
@@ -28529,7 +28504,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E1017" t="inlineStr"/>
       <c r="F1017" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g14</t>
@@ -28557,7 +28531,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E1018" t="inlineStr"/>
       <c r="F1018" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g16</t>
@@ -28585,7 +28558,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E1019" t="inlineStr"/>
       <c r="F1019" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g20</t>
@@ -28613,7 +28585,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E1020" t="inlineStr"/>
       <c r="F1020" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g21</t>
@@ -28641,7 +28612,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E1021" t="inlineStr"/>
       <c r="F1021" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g26</t>
@@ -28669,7 +28639,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E1022" t="inlineStr"/>
       <c r="F1022" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g27</t>
@@ -28697,7 +28666,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E1023" t="inlineStr"/>
       <c r="F1023" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g28</t>
@@ -28725,7 +28693,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E1024" t="inlineStr"/>
       <c r="F1024" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g29</t>
@@ -28753,7 +28720,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E1025" t="inlineStr"/>
       <c r="F1025" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g30</t>
@@ -28781,7 +28747,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E1026" t="inlineStr"/>
       <c r="F1026" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g31</t>
@@ -28809,7 +28774,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E1027" t="inlineStr"/>
       <c r="F1027" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g32</t>
@@ -28837,7 +28801,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E1028" t="inlineStr"/>
       <c r="F1028" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g35</t>
@@ -28865,7 +28828,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E1029" t="inlineStr"/>
       <c r="F1029" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g37</t>
@@ -28893,7 +28855,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E1030" t="inlineStr"/>
       <c r="F1030" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g38</t>
@@ -28921,7 +28882,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E1031" t="inlineStr"/>
       <c r="F1031" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g39</t>
@@ -30183,6 +30143,3646 @@
         <v>3</v>
       </c>
       <c r="F1076" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1077">
+      <c r="A1077" t="inlineStr">
+        <is>
+          <t>2026-08-08T21:04:00</t>
+        </is>
+      </c>
+      <c r="B1077" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1077" t="inlineStr">
+        <is>
+          <t>_1st_SCAN</t>
+        </is>
+      </c>
+      <c r="D1077" t="b">
+        <v>0</v>
+      </c>
+      <c r="E1077" t="n">
+        <v>11</v>
+      </c>
+      <c r="F1077" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1078">
+      <c r="A1078" t="inlineStr">
+        <is>
+          <t>2026-08-08T21:04:00</t>
+        </is>
+      </c>
+      <c r="B1078" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1078" t="inlineStr">
+        <is>
+          <t>TieDetectOffset_B</t>
+        </is>
+      </c>
+      <c r="D1078" t="b">
+        <v>0</v>
+      </c>
+      <c r="E1078" t="n">
+        <v>11</v>
+      </c>
+      <c r="F1078" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1079">
+      <c r="A1079" t="inlineStr">
+        <is>
+          <t>2026-08-08T21:04:00</t>
+        </is>
+      </c>
+      <c r="B1079" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1079" t="inlineStr">
+        <is>
+          <t>Tie Detector</t>
+        </is>
+      </c>
+      <c r="D1079" t="b">
+        <v>0</v>
+      </c>
+      <c r="E1079" t="n">
+        <v>11</v>
+      </c>
+      <c r="F1079" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1080">
+      <c r="A1080" t="inlineStr">
+        <is>
+          <t>2026-08-08T21:04:00</t>
+        </is>
+      </c>
+      <c r="B1080" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1080" t="inlineStr">
+        <is>
+          <t>TPS Full</t>
+        </is>
+      </c>
+      <c r="D1080" t="b">
+        <v>0</v>
+      </c>
+      <c r="E1080" t="n">
+        <v>11</v>
+      </c>
+      <c r="F1080" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1081">
+      <c r="A1081" t="inlineStr">
+        <is>
+          <t>2026-08-08T21:04:00</t>
+        </is>
+      </c>
+      <c r="B1081" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1081" t="inlineStr">
+        <is>
+          <t>TieDetectOffset_A</t>
+        </is>
+      </c>
+      <c r="D1081" t="b">
+        <v>0</v>
+      </c>
+      <c r="E1081" t="n">
+        <v>11</v>
+      </c>
+      <c r="F1081" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1082">
+      <c r="A1082" t="inlineStr">
+        <is>
+          <t>2026-08-08T21:04:00</t>
+        </is>
+      </c>
+      <c r="B1082" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1082" t="inlineStr">
+        <is>
+          <t>TPS Connected</t>
+        </is>
+      </c>
+      <c r="D1082" t="b">
+        <v>0</v>
+      </c>
+      <c r="E1082" t="n">
+        <v>11</v>
+      </c>
+      <c r="F1082" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1083">
+      <c r="A1083" t="inlineStr">
+        <is>
+          <t>2026-08-08T21:04:00</t>
+        </is>
+      </c>
+      <c r="B1083" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1083" t="inlineStr">
+        <is>
+          <t>TPS_Enable_ Button</t>
+        </is>
+      </c>
+      <c r="D1083" t="b">
+        <v>0</v>
+      </c>
+      <c r="E1083" t="n">
+        <v>11</v>
+      </c>
+      <c r="F1083" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1084">
+      <c r="A1084" t="inlineStr">
+        <is>
+          <t>2026-08-08T21:04:00</t>
+        </is>
+      </c>
+      <c r="B1084" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1084" t="inlineStr">
+        <is>
+          <t>AirEagle Eject Plate</t>
+        </is>
+      </c>
+      <c r="D1084" t="b">
+        <v>0</v>
+      </c>
+      <c r="E1084" t="n">
+        <v>11</v>
+      </c>
+      <c r="F1084" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1085">
+      <c r="A1085" t="inlineStr">
+        <is>
+          <t>2026-08-08T21:04:00</t>
+        </is>
+      </c>
+      <c r="B1085" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1085" t="inlineStr">
+        <is>
+          <t>tk_Cycle</t>
+        </is>
+      </c>
+      <c r="D1085" t="b">
+        <v>0</v>
+      </c>
+      <c r="E1085" t="n">
+        <v>11</v>
+      </c>
+      <c r="F1085" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1086">
+      <c r="A1086" t="inlineStr">
+        <is>
+          <t>2026-08-08T21:04:00</t>
+        </is>
+      </c>
+      <c r="B1086" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1086" t="inlineStr">
+        <is>
+          <t>Servos_Enabled</t>
+        </is>
+      </c>
+      <c r="D1086" t="b">
+        <v>0</v>
+      </c>
+      <c r="E1086" t="n">
+        <v>11</v>
+      </c>
+      <c r="F1086" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1087">
+      <c r="A1087" t="inlineStr">
+        <is>
+          <t>2026-08-08T21:04:00</t>
+        </is>
+      </c>
+      <c r="B1087" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1087" t="inlineStr">
+        <is>
+          <t>TPS Enabled</t>
+        </is>
+      </c>
+      <c r="D1087" t="b">
+        <v>0</v>
+      </c>
+      <c r="E1087" t="n">
+        <v>11</v>
+      </c>
+      <c r="F1087" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1088">
+      <c r="A1088" t="inlineStr">
+        <is>
+          <t>2026-08-08T21:04:00</t>
+        </is>
+      </c>
+      <c r="B1088" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1088" t="inlineStr">
+        <is>
+          <t>tk_Abort</t>
+        </is>
+      </c>
+      <c r="D1088" t="b">
+        <v>0</v>
+      </c>
+      <c r="E1088" t="n">
+        <v>11</v>
+      </c>
+      <c r="F1088" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1089">
+      <c r="A1089" t="inlineStr">
+        <is>
+          <t>2026-08-08T21:04:00</t>
+        </is>
+      </c>
+      <c r="B1089" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1089" t="inlineStr">
+        <is>
+          <t>Robot_isMoving</t>
+        </is>
+      </c>
+      <c r="D1089" t="b">
+        <v>0</v>
+      </c>
+      <c r="E1089" t="n">
+        <v>11</v>
+      </c>
+      <c r="F1089" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1090">
+      <c r="A1090" t="inlineStr">
+        <is>
+          <t>2026-08-08T21:04:00</t>
+        </is>
+      </c>
+      <c r="B1090" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1090" t="inlineStr">
+        <is>
+          <t>Eject Tie Plate</t>
+        </is>
+      </c>
+      <c r="D1090" t="b">
+        <v>0</v>
+      </c>
+      <c r="E1090" t="n">
+        <v>11</v>
+      </c>
+      <c r="F1090" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1091">
+      <c r="A1091" t="inlineStr">
+        <is>
+          <t>2026-08-08T21:04:00</t>
+        </is>
+      </c>
+      <c r="B1091" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1091" t="inlineStr">
+        <is>
+          <t>TPS BACKUP ALARM</t>
+        </is>
+      </c>
+      <c r="D1091" t="b">
+        <v>0</v>
+      </c>
+      <c r="E1091" t="n">
+        <v>11</v>
+      </c>
+      <c r="F1091" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1092">
+      <c r="A1092" t="inlineStr">
+        <is>
+          <t>2026-08-08T21:04:00</t>
+        </is>
+      </c>
+      <c r="B1092" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1092" t="inlineStr">
+        <is>
+          <t>14in Job</t>
+        </is>
+      </c>
+      <c r="D1092" t="b">
+        <v>1</v>
+      </c>
+      <c r="E1092" t="n">
+        <v>11</v>
+      </c>
+      <c r="F1092" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1093">
+      <c r="A1093" t="inlineStr">
+        <is>
+          <t>2026-08-08T21:04:00</t>
+        </is>
+      </c>
+      <c r="B1093" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1093" t="inlineStr">
+        <is>
+          <t>18in Job</t>
+        </is>
+      </c>
+      <c r="D1093" t="b">
+        <v>0</v>
+      </c>
+      <c r="E1093" t="n">
+        <v>11</v>
+      </c>
+      <c r="F1093" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1094">
+      <c r="A1094" t="inlineStr">
+        <is>
+          <t>2026-08-08T21:04:00</t>
+        </is>
+      </c>
+      <c r="B1094" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1094" t="inlineStr">
+        <is>
+          <t>Pandral Job</t>
+        </is>
+      </c>
+      <c r="D1094" t="b">
+        <v>0</v>
+      </c>
+      <c r="E1094" t="n">
+        <v>11</v>
+      </c>
+      <c r="F1094" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1095">
+      <c r="A1095" t="inlineStr">
+        <is>
+          <t>2026-08-08T21:04:00</t>
+        </is>
+      </c>
+      <c r="B1095" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1095" t="inlineStr">
+        <is>
+          <t>DoubleLay Job</t>
+        </is>
+      </c>
+      <c r="D1095" t="b">
+        <v>0</v>
+      </c>
+      <c r="E1095" t="n">
+        <v>11</v>
+      </c>
+      <c r="F1095" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1096">
+      <c r="A1096" t="inlineStr">
+        <is>
+          <t>2026-08-08T21:04:00</t>
+        </is>
+      </c>
+      <c r="B1096" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1096" t="inlineStr">
+        <is>
+          <t>TPSjam_FLAG</t>
+        </is>
+      </c>
+      <c r="D1096" t="b">
+        <v>0</v>
+      </c>
+      <c r="E1096" t="n">
+        <v>11</v>
+      </c>
+      <c r="F1096" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1097">
+      <c r="A1097" t="inlineStr">
+        <is>
+          <t>2026-08-08T21:04:00</t>
+        </is>
+      </c>
+      <c r="B1097" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1097" t="inlineStr">
+        <is>
+          <t>RoCalRequest</t>
+        </is>
+      </c>
+      <c r="D1097" t="b">
+        <v>0</v>
+      </c>
+      <c r="E1097" t="n">
+        <v>11</v>
+      </c>
+      <c r="F1097" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1098">
+      <c r="A1098" t="inlineStr">
+        <is>
+          <t>2026-08-08T21:04:00</t>
+        </is>
+      </c>
+      <c r="B1098" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1098" t="inlineStr">
+        <is>
+          <t>tkCycle_TotalSeconds</t>
+        </is>
+      </c>
+      <c r="D1098" t="n">
+        <v>0</v>
+      </c>
+      <c r="E1098" t="n">
+        <v>9</v>
+      </c>
+      <c r="F1098" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1099">
+      <c r="A1099" t="inlineStr">
+        <is>
+          <t>2026-08-08T21:04:00</t>
+        </is>
+      </c>
+      <c r="B1099" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1099" t="inlineStr">
+        <is>
+          <t>tkCycle_NoMoveSec</t>
+        </is>
+      </c>
+      <c r="D1099" t="n">
+        <v>0</v>
+      </c>
+      <c r="E1099" t="n">
+        <v>9</v>
+      </c>
+      <c r="F1099" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1100">
+      <c r="A1100" t="inlineStr">
+        <is>
+          <t>2026-08-08T21:04:00</t>
+        </is>
+      </c>
+      <c r="B1100" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1100" t="inlineStr">
+        <is>
+          <t>tkCycle_MoveSeconds</t>
+        </is>
+      </c>
+      <c r="D1100" t="n">
+        <v>0</v>
+      </c>
+      <c r="E1100" t="n">
+        <v>9</v>
+      </c>
+      <c r="F1100" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1101">
+      <c r="A1101" t="inlineStr">
+        <is>
+          <t>2026-08-08T21:04:00</t>
+        </is>
+      </c>
+      <c r="B1101" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1101" t="inlineStr">
+        <is>
+          <t>Percent time moveing</t>
+        </is>
+      </c>
+      <c r="D1101" t="n">
+        <v>0</v>
+      </c>
+      <c r="E1101" t="n">
+        <v>9</v>
+      </c>
+      <c r="F1101" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1102">
+      <c r="A1102" t="inlineStr">
+        <is>
+          <t>2026-08-08T21:04:00</t>
+        </is>
+      </c>
+      <c r="B1102" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1102" t="inlineStr">
+        <is>
+          <t>Percent time not moving</t>
+        </is>
+      </c>
+      <c r="D1102" t="n">
+        <v>0</v>
+      </c>
+      <c r="E1102" t="n">
+        <v>9</v>
+      </c>
+      <c r="F1102" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1103">
+      <c r="A1103" t="inlineStr">
+        <is>
+          <t>2026-08-08T21:04:00</t>
+        </is>
+      </c>
+      <c r="B1103" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1103" t="inlineStr">
+        <is>
+          <t>TotalPickPartsCount</t>
+        </is>
+      </c>
+      <c r="D1103" t="n">
+        <v>0</v>
+      </c>
+      <c r="E1103" t="n">
+        <v>9</v>
+      </c>
+      <c r="F1103" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1104">
+      <c r="A1104" t="inlineStr">
+        <is>
+          <t>2026-08-08T21:04:00</t>
+        </is>
+      </c>
+      <c r="B1104" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1104" t="inlineStr">
+        <is>
+          <t>RejectPartsCount</t>
+        </is>
+      </c>
+      <c r="D1104" t="n">
+        <v>0</v>
+      </c>
+      <c r="E1104" t="n">
+        <v>9</v>
+      </c>
+      <c r="F1104" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1105">
+      <c r="A1105" t="inlineStr">
+        <is>
+          <t>2026-08-08T21:04:00</t>
+        </is>
+      </c>
+      <c r="B1105" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1105" t="inlineStr">
+        <is>
+          <t>AcceptsPartsCount</t>
+        </is>
+      </c>
+      <c r="D1105" t="n">
+        <v>0</v>
+      </c>
+      <c r="E1105" t="n">
+        <v>9</v>
+      </c>
+      <c r="F1105" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1106">
+      <c r="A1106" t="inlineStr">
+        <is>
+          <t>2026-08-08T21:04:00</t>
+        </is>
+      </c>
+      <c r="B1106" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1106" t="inlineStr">
+        <is>
+          <t>percentCount_accept</t>
+        </is>
+      </c>
+      <c r="D1106" t="n">
+        <v>0</v>
+      </c>
+      <c r="E1106" t="n">
+        <v>9</v>
+      </c>
+      <c r="F1106" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1107">
+      <c r="A1107" t="inlineStr">
+        <is>
+          <t>2026-08-08T21:04:00</t>
+        </is>
+      </c>
+      <c r="B1107" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1107" t="inlineStr">
+        <is>
+          <t>percentCount_reject</t>
+        </is>
+      </c>
+      <c r="D1107" t="n">
+        <v>0</v>
+      </c>
+      <c r="E1107" t="n">
+        <v>9</v>
+      </c>
+      <c r="F1107" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1108">
+      <c r="A1108" t="inlineStr">
+        <is>
+          <t>2026-08-08T21:04:00</t>
+        </is>
+      </c>
+      <c r="B1108" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1108" t="inlineStr">
+        <is>
+          <t>Avg Parts per min_total</t>
+        </is>
+      </c>
+      <c r="D1108" t="n">
+        <v>0</v>
+      </c>
+      <c r="E1108" t="n">
+        <v>9</v>
+      </c>
+      <c r="F1108" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1109">
+      <c r="A1109" t="inlineStr">
+        <is>
+          <t>2026-08-08T21:04:00</t>
+        </is>
+      </c>
+      <c r="B1109" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1109" t="inlineStr">
+        <is>
+          <t>TotalPickedParts</t>
+        </is>
+      </c>
+      <c r="D1109" t="n">
+        <v>0</v>
+      </c>
+      <c r="E1109" t="n">
+        <v>3</v>
+      </c>
+      <c r="F1109" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1110">
+      <c r="A1110" t="inlineStr">
+        <is>
+          <t>2026-08-08T21:04:00</t>
+        </is>
+      </c>
+      <c r="B1110" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1110" t="inlineStr">
+        <is>
+          <t>TotalPickedAcceptParts</t>
+        </is>
+      </c>
+      <c r="D1110" t="n">
+        <v>0</v>
+      </c>
+      <c r="E1110" t="n">
+        <v>3</v>
+      </c>
+      <c r="F1110" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1111">
+      <c r="A1111" t="inlineStr">
+        <is>
+          <t>2026-08-08T21:04:00</t>
+        </is>
+      </c>
+      <c r="B1111" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1111" t="inlineStr">
+        <is>
+          <t>TotalPickedRejectParts</t>
+        </is>
+      </c>
+      <c r="D1111" t="n">
+        <v>0</v>
+      </c>
+      <c r="E1111" t="n">
+        <v>3</v>
+      </c>
+      <c r="F1111" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1112">
+      <c r="A1112" t="inlineStr">
+        <is>
+          <t>2026-08-08T21:04:00</t>
+        </is>
+      </c>
+      <c r="B1112" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1112" t="inlineStr">
+        <is>
+          <t>TotalTiePlatesLaid</t>
+        </is>
+      </c>
+      <c r="D1112" t="n">
+        <v>0</v>
+      </c>
+      <c r="E1112" t="n">
+        <v>3</v>
+      </c>
+      <c r="F1112" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1113">
+      <c r="A1113" t="inlineStr">
+        <is>
+          <t>2026-08-08T21:04:00</t>
+        </is>
+      </c>
+      <c r="B1113" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1113" t="inlineStr">
+        <is>
+          <t>Daily_TotalLaidPlates</t>
+        </is>
+      </c>
+      <c r="D1113" t="n">
+        <v>0</v>
+      </c>
+      <c r="E1113" t="n">
+        <v>3</v>
+      </c>
+      <c r="F1113" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1114">
+      <c r="A1114" t="inlineStr">
+        <is>
+          <t>2026-08-08T21:04:00</t>
+        </is>
+      </c>
+      <c r="B1114" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1114" t="inlineStr">
+        <is>
+          <t>CountPicked14in</t>
+        </is>
+      </c>
+      <c r="D1114" t="n">
+        <v>0</v>
+      </c>
+      <c r="E1114" t="n">
+        <v>3</v>
+      </c>
+      <c r="F1114" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1115">
+      <c r="A1115" t="inlineStr">
+        <is>
+          <t>2026-08-08T21:04:00</t>
+        </is>
+      </c>
+      <c r="B1115" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1115" t="inlineStr">
+        <is>
+          <t>CountPicked18in</t>
+        </is>
+      </c>
+      <c r="D1115" t="n">
+        <v>0</v>
+      </c>
+      <c r="E1115" t="n">
+        <v>3</v>
+      </c>
+      <c r="F1115" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1116">
+      <c r="A1116" t="inlineStr">
+        <is>
+          <t>2026-08-08T21:04:00</t>
+        </is>
+      </c>
+      <c r="B1116" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1116" t="inlineStr">
+        <is>
+          <t>CountPickedPandral</t>
+        </is>
+      </c>
+      <c r="D1116" t="n">
+        <v>0</v>
+      </c>
+      <c r="E1116" t="n">
+        <v>3</v>
+      </c>
+      <c r="F1116" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1117">
+      <c r="A1117" t="inlineStr">
+        <is>
+          <t>2026-08-08T21:04:00</t>
+        </is>
+      </c>
+      <c r="B1117" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1117" t="inlineStr">
+        <is>
+          <t>CountPickedOTM</t>
+        </is>
+      </c>
+      <c r="D1117" t="n">
+        <v>0</v>
+      </c>
+      <c r="E1117" t="n">
+        <v>3</v>
+      </c>
+      <c r="F1117" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1118">
+      <c r="A1118" t="inlineStr">
+        <is>
+          <t>2026-08-08T21:04:00</t>
+        </is>
+      </c>
+      <c r="B1118" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1118" t="inlineStr">
+        <is>
+          <t>RoCals</t>
+        </is>
+      </c>
+      <c r="D1118" t="n">
+        <v>0</v>
+      </c>
+      <c r="E1118" t="n">
+        <v>3</v>
+      </c>
+      <c r="F1118" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1119">
+      <c r="A1119" t="inlineStr">
+        <is>
+          <t>2026-08-08T21:04:00</t>
+        </is>
+      </c>
+      <c r="B1119" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1119" t="inlineStr">
+        <is>
+          <t>TPS_JamsUsr</t>
+        </is>
+      </c>
+      <c r="D1119" t="n">
+        <v>0</v>
+      </c>
+      <c r="E1119" t="n">
+        <v>3</v>
+      </c>
+      <c r="F1119" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1120">
+      <c r="A1120" t="inlineStr">
+        <is>
+          <t>2026-08-08T21:04:00</t>
+        </is>
+      </c>
+      <c r="B1120" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1120" t="inlineStr">
+        <is>
+          <t>TPS_JamsMASTER</t>
+        </is>
+      </c>
+      <c r="D1120" t="n">
+        <v>0</v>
+      </c>
+      <c r="E1120" t="n">
+        <v>3</v>
+      </c>
+      <c r="F1120" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1121">
+      <c r="A1121" t="inlineStr">
+        <is>
+          <t>2026-08-08T21:04:00</t>
+        </is>
+      </c>
+      <c r="B1121" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1121" t="inlineStr">
+        <is>
+          <t>ABORT_Master</t>
+        </is>
+      </c>
+      <c r="D1121" t="n">
+        <v>0</v>
+      </c>
+      <c r="E1121" t="n">
+        <v>3</v>
+      </c>
+      <c r="F1121" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1122">
+      <c r="A1122" t="inlineStr">
+        <is>
+          <t>2026-08-08T21:04:13</t>
+        </is>
+      </c>
+      <c r="B1122" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1122" t="inlineStr">
+        <is>
+          <t>CountLaidButton</t>
+        </is>
+      </c>
+      <c r="D1122" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E1122" t="inlineStr"/>
+      <c r="F1122" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g2</t>
+        </is>
+      </c>
+    </row>
+    <row r="1123">
+      <c r="A1123" t="inlineStr">
+        <is>
+          <t>2026-08-08T21:04:13</t>
+        </is>
+      </c>
+      <c r="B1123" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1123" t="inlineStr">
+        <is>
+          <t>CountLaidDetector</t>
+        </is>
+      </c>
+      <c r="D1123" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E1123" t="inlineStr"/>
+      <c r="F1123" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g3</t>
+        </is>
+      </c>
+    </row>
+    <row r="1124">
+      <c r="A1124" t="inlineStr">
+        <is>
+          <t>2026-08-08T21:04:13</t>
+        </is>
+      </c>
+      <c r="B1124" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1124" t="inlineStr">
+        <is>
+          <t>CountLaidEncoder</t>
+        </is>
+      </c>
+      <c r="D1124" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E1124" t="inlineStr"/>
+      <c r="F1124" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g4</t>
+        </is>
+      </c>
+    </row>
+    <row r="1125">
+      <c r="A1125" t="inlineStr">
+        <is>
+          <t>2026-08-08T21:04:13</t>
+        </is>
+      </c>
+      <c r="B1125" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1125" t="inlineStr">
+        <is>
+          <t>CountLaid14in</t>
+        </is>
+      </c>
+      <c r="D1125" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E1125" t="inlineStr"/>
+      <c r="F1125" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g5</t>
+        </is>
+      </c>
+    </row>
+    <row r="1126">
+      <c r="A1126" t="inlineStr">
+        <is>
+          <t>2026-08-08T21:04:13</t>
+        </is>
+      </c>
+      <c r="B1126" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1126" t="inlineStr">
+        <is>
+          <t>CountLaid18in</t>
+        </is>
+      </c>
+      <c r="D1126" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E1126" t="inlineStr"/>
+      <c r="F1126" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g6</t>
+        </is>
+      </c>
+    </row>
+    <row r="1127">
+      <c r="A1127" t="inlineStr">
+        <is>
+          <t>2026-08-08T21:04:13</t>
+        </is>
+      </c>
+      <c r="B1127" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1127" t="inlineStr">
+        <is>
+          <t>CountLaidPandral</t>
+        </is>
+      </c>
+      <c r="D1127" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E1127" t="inlineStr"/>
+      <c r="F1127" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g7</t>
+        </is>
+      </c>
+    </row>
+    <row r="1128">
+      <c r="A1128" t="inlineStr">
+        <is>
+          <t>2026-08-08T21:04:13</t>
+        </is>
+      </c>
+      <c r="B1128" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1128" t="inlineStr">
+        <is>
+          <t>TotalTiePlatesLaid</t>
+        </is>
+      </c>
+      <c r="D1128" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E1128" t="inlineStr"/>
+      <c r="F1128" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g1</t>
+        </is>
+      </c>
+    </row>
+    <row r="1129">
+      <c r="A1129" t="inlineStr">
+        <is>
+          <t>2026-08-08T21:04:13</t>
+        </is>
+      </c>
+      <c r="B1129" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1129" t="inlineStr">
+        <is>
+          <t>usr_TPStime Hours10th</t>
+        </is>
+      </c>
+      <c r="D1129" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E1129" t="inlineStr"/>
+      <c r="F1129" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g8</t>
+        </is>
+      </c>
+    </row>
+    <row r="1130">
+      <c r="A1130" t="inlineStr">
+        <is>
+          <t>2026-08-08T21:04:13</t>
+        </is>
+      </c>
+      <c r="B1130" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1130" t="inlineStr">
+        <is>
+          <t>usrTPS_miles xxx</t>
+        </is>
+      </c>
+      <c r="D1130" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E1130" t="inlineStr"/>
+      <c r="F1130" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g9</t>
+        </is>
+      </c>
+    </row>
+    <row r="1131">
+      <c r="A1131" t="inlineStr">
+        <is>
+          <t>2026-08-08T21:04:13</t>
+        </is>
+      </c>
+      <c r="B1131" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1131" t="inlineStr">
+        <is>
+          <t>TPS Connected</t>
+        </is>
+      </c>
+      <c r="D1131" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E1131" t="inlineStr"/>
+      <c r="F1131" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g10</t>
+        </is>
+      </c>
+    </row>
+    <row r="1132">
+      <c r="A1132" t="inlineStr">
+        <is>
+          <t>2026-08-08T21:04:13</t>
+        </is>
+      </c>
+      <c r="B1132" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1132" t="inlineStr">
+        <is>
+          <t>TPS Enabled</t>
+        </is>
+      </c>
+      <c r="D1132" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E1132" t="inlineStr"/>
+      <c r="F1132" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g11</t>
+        </is>
+      </c>
+    </row>
+    <row r="1133">
+      <c r="A1133" t="inlineStr">
+        <is>
+          <t>2026-08-08T21:04:13</t>
+        </is>
+      </c>
+      <c r="B1133" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1133" t="inlineStr">
+        <is>
+          <t>18in Job</t>
+        </is>
+      </c>
+      <c r="D1133" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E1133" t="inlineStr"/>
+      <c r="F1133" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g13</t>
+        </is>
+      </c>
+    </row>
+    <row r="1134">
+      <c r="A1134" t="inlineStr">
+        <is>
+          <t>2026-08-08T21:04:13</t>
+        </is>
+      </c>
+      <c r="B1134" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1134" t="inlineStr">
+        <is>
+          <t>CountAcceptedTotal</t>
+        </is>
+      </c>
+      <c r="D1134" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E1134" t="inlineStr"/>
+      <c r="F1134" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g15</t>
+        </is>
+      </c>
+    </row>
+    <row r="1135">
+      <c r="A1135" t="inlineStr">
+        <is>
+          <t>2026-08-08T21:04:13</t>
+        </is>
+      </c>
+      <c r="B1135" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1135" t="inlineStr">
+        <is>
+          <t>Servos_Enabled</t>
+        </is>
+      </c>
+      <c r="D1135" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E1135" t="inlineStr"/>
+      <c r="F1135" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g17</t>
+        </is>
+      </c>
+    </row>
+    <row r="1136">
+      <c r="A1136" t="inlineStr">
+        <is>
+          <t>2026-08-08T21:04:13</t>
+        </is>
+      </c>
+      <c r="B1136" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1136" t="inlineStr">
+        <is>
+          <t>TotalPickPartsCount</t>
+        </is>
+      </c>
+      <c r="D1136" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E1136" t="inlineStr"/>
+      <c r="F1136" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g18</t>
+        </is>
+      </c>
+    </row>
+    <row r="1137">
+      <c r="A1137" t="inlineStr">
+        <is>
+          <t>2026-08-08T21:04:13</t>
+        </is>
+      </c>
+      <c r="B1137" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1137" t="inlineStr">
+        <is>
+          <t>AcceptsPartsCount</t>
+        </is>
+      </c>
+      <c r="D1137" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E1137" t="inlineStr"/>
+      <c r="F1137" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g19</t>
+        </is>
+      </c>
+    </row>
+    <row r="1138">
+      <c r="A1138" t="inlineStr">
+        <is>
+          <t>2026-08-08T21:04:13</t>
+        </is>
+      </c>
+      <c r="B1138" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1138" t="inlineStr">
+        <is>
+          <t>day_Servotime Hours10th</t>
+        </is>
+      </c>
+      <c r="D1138" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E1138" t="inlineStr"/>
+      <c r="F1138" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g22</t>
+        </is>
+      </c>
+    </row>
+    <row r="1139">
+      <c r="A1139" t="inlineStr">
+        <is>
+          <t>2026-08-08T21:04:13</t>
+        </is>
+      </c>
+      <c r="B1139" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1139" t="inlineStr">
+        <is>
+          <t>tk_Cycle</t>
+        </is>
+      </c>
+      <c r="D1139" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E1139" t="inlineStr"/>
+      <c r="F1139" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g23</t>
+        </is>
+      </c>
+    </row>
+    <row r="1140">
+      <c r="A1140" t="inlineStr">
+        <is>
+          <t>2026-08-08T21:04:13</t>
+        </is>
+      </c>
+      <c r="B1140" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1140" t="inlineStr">
+        <is>
+          <t>tk_Abort</t>
+        </is>
+      </c>
+      <c r="D1140" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E1140" t="inlineStr"/>
+      <c r="F1140" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g24</t>
+        </is>
+      </c>
+    </row>
+    <row r="1141">
+      <c r="A1141" t="inlineStr">
+        <is>
+          <t>2026-08-08T21:04:13</t>
+        </is>
+      </c>
+      <c r="B1141" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1141" t="inlineStr">
+        <is>
+          <t>tk_ClearPos</t>
+        </is>
+      </c>
+      <c r="D1141" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E1141" t="inlineStr"/>
+      <c r="F1141" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g25</t>
+        </is>
+      </c>
+    </row>
+    <row r="1142">
+      <c r="A1142" t="inlineStr">
+        <is>
+          <t>2026-08-08T21:04:13</t>
+        </is>
+      </c>
+      <c r="B1142" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1142" t="inlineStr">
+        <is>
+          <t>temp_J2motor</t>
+        </is>
+      </c>
+      <c r="D1142" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E1142" t="inlineStr"/>
+      <c r="F1142" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g33</t>
+        </is>
+      </c>
+    </row>
+    <row r="1143">
+      <c r="A1143" t="inlineStr">
+        <is>
+          <t>2026-08-08T21:04:13</t>
+        </is>
+      </c>
+      <c r="B1143" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1143" t="inlineStr">
+        <is>
+          <t>temp_J3motor</t>
+        </is>
+      </c>
+      <c r="D1143" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E1143" t="inlineStr"/>
+      <c r="F1143" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g34</t>
+        </is>
+      </c>
+    </row>
+    <row r="1144">
+      <c r="A1144" t="inlineStr">
+        <is>
+          <t>2026-08-08T21:04:13</t>
+        </is>
+      </c>
+      <c r="B1144" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1144" t="inlineStr">
+        <is>
+          <t>temp_J5motor</t>
+        </is>
+      </c>
+      <c r="D1144" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E1144" t="inlineStr"/>
+      <c r="F1144" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g36</t>
+        </is>
+      </c>
+    </row>
+    <row r="1145">
+      <c r="A1145" t="inlineStr">
+        <is>
+          <t>2026-08-08T21:04:13</t>
+        </is>
+      </c>
+      <c r="B1145" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1145" t="inlineStr">
+        <is>
+          <t>14in Job</t>
+        </is>
+      </c>
+      <c r="D1145" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E1145" t="inlineStr"/>
+      <c r="F1145" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g12</t>
+        </is>
+      </c>
+    </row>
+    <row r="1146">
+      <c r="A1146" t="inlineStr">
+        <is>
+          <t>2026-08-08T21:04:13</t>
+        </is>
+      </c>
+      <c r="B1146" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1146" t="inlineStr">
+        <is>
+          <t>Pandral Job</t>
+        </is>
+      </c>
+      <c r="D1146" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E1146" t="inlineStr"/>
+      <c r="F1146" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g14</t>
+        </is>
+      </c>
+    </row>
+    <row r="1147">
+      <c r="A1147" t="inlineStr">
+        <is>
+          <t>2026-08-08T21:04:13</t>
+        </is>
+      </c>
+      <c r="B1147" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1147" t="inlineStr">
+        <is>
+          <t>CountRejectedTotal</t>
+        </is>
+      </c>
+      <c r="D1147" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E1147" t="inlineStr"/>
+      <c r="F1147" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g16</t>
+        </is>
+      </c>
+    </row>
+    <row r="1148">
+      <c r="A1148" t="inlineStr">
+        <is>
+          <t>2026-08-08T21:04:13</t>
+        </is>
+      </c>
+      <c r="B1148" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1148" t="inlineStr">
+        <is>
+          <t>RejectPartsCount</t>
+        </is>
+      </c>
+      <c r="D1148" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E1148" t="inlineStr"/>
+      <c r="F1148" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g20</t>
+        </is>
+      </c>
+    </row>
+    <row r="1149">
+      <c r="A1149" t="inlineStr">
+        <is>
+          <t>2026-08-08T21:04:13</t>
+        </is>
+      </c>
+      <c r="B1149" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1149" t="inlineStr">
+        <is>
+          <t>tk_Cycle hrs</t>
+        </is>
+      </c>
+      <c r="D1149" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E1149" t="inlineStr"/>
+      <c r="F1149" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g21</t>
+        </is>
+      </c>
+    </row>
+    <row r="1150">
+      <c r="A1150" t="inlineStr">
+        <is>
+          <t>2026-08-08T21:04:13</t>
+        </is>
+      </c>
+      <c r="B1150" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1150" t="inlineStr">
+        <is>
+          <t>tk_Warmup</t>
+        </is>
+      </c>
+      <c r="D1150" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E1150" t="inlineStr"/>
+      <c r="F1150" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g26</t>
+        </is>
+      </c>
+    </row>
+    <row r="1151">
+      <c r="A1151" t="inlineStr">
+        <is>
+          <t>2026-08-08T21:04:13</t>
+        </is>
+      </c>
+      <c r="B1151" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1151" t="inlineStr">
+        <is>
+          <t>FindingParts min</t>
+        </is>
+      </c>
+      <c r="D1151" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E1151" t="inlineStr"/>
+      <c r="F1151" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g27</t>
+        </is>
+      </c>
+    </row>
+    <row r="1152">
+      <c r="A1152" t="inlineStr">
+        <is>
+          <t>2026-08-08T21:04:13</t>
+        </is>
+      </c>
+      <c r="B1152" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1152" t="inlineStr">
+        <is>
+          <t>PickingParts min</t>
+        </is>
+      </c>
+      <c r="D1152" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E1152" t="inlineStr"/>
+      <c r="F1152" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g28</t>
+        </is>
+      </c>
+    </row>
+    <row r="1153">
+      <c r="A1153" t="inlineStr">
+        <is>
+          <t>2026-08-08T21:04:13</t>
+        </is>
+      </c>
+      <c r="B1153" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1153" t="inlineStr">
+        <is>
+          <t>PlacingParts min</t>
+        </is>
+      </c>
+      <c r="D1153" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E1153" t="inlineStr"/>
+      <c r="F1153" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g29</t>
+        </is>
+      </c>
+    </row>
+    <row r="1154">
+      <c r="A1154" t="inlineStr">
+        <is>
+          <t>2026-08-08T21:04:13</t>
+        </is>
+      </c>
+      <c r="B1154" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1154" t="inlineStr">
+        <is>
+          <t>CountPickedReject14in</t>
+        </is>
+      </c>
+      <c r="D1154" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E1154" t="inlineStr"/>
+      <c r="F1154" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g30</t>
+        </is>
+      </c>
+    </row>
+    <row r="1155">
+      <c r="A1155" t="inlineStr">
+        <is>
+          <t>2026-08-08T21:04:13</t>
+        </is>
+      </c>
+      <c r="B1155" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1155" t="inlineStr">
+        <is>
+          <t>temp_dsi</t>
+        </is>
+      </c>
+      <c r="D1155" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E1155" t="inlineStr"/>
+      <c r="F1155" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g31</t>
+        </is>
+      </c>
+    </row>
+    <row r="1156">
+      <c r="A1156" t="inlineStr">
+        <is>
+          <t>2026-08-08T21:04:13</t>
+        </is>
+      </c>
+      <c r="B1156" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1156" t="inlineStr">
+        <is>
+          <t>temp_J1motor</t>
+        </is>
+      </c>
+      <c r="D1156" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E1156" t="inlineStr"/>
+      <c r="F1156" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g32</t>
+        </is>
+      </c>
+    </row>
+    <row r="1157">
+      <c r="A1157" t="inlineStr">
+        <is>
+          <t>2026-08-08T21:04:13</t>
+        </is>
+      </c>
+      <c r="B1157" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1157" t="inlineStr">
+        <is>
+          <t>temp_J4motor</t>
+        </is>
+      </c>
+      <c r="D1157" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E1157" t="inlineStr"/>
+      <c r="F1157" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g35</t>
+        </is>
+      </c>
+    </row>
+    <row r="1158">
+      <c r="A1158" t="inlineStr">
+        <is>
+          <t>2026-08-08T21:04:13</t>
+        </is>
+      </c>
+      <c r="B1158" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1158" t="inlineStr">
+        <is>
+          <t>temp_J6motor</t>
+        </is>
+      </c>
+      <c r="D1158" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E1158" t="inlineStr"/>
+      <c r="F1158" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g37</t>
+        </is>
+      </c>
+    </row>
+    <row r="1159">
+      <c r="A1159" t="inlineStr">
+        <is>
+          <t>2026-08-08T21:04:13</t>
+        </is>
+      </c>
+      <c r="B1159" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1159" t="inlineStr">
+        <is>
+          <t>CountPickedRejectOTM</t>
+        </is>
+      </c>
+      <c r="D1159" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E1159" t="inlineStr"/>
+      <c r="F1159" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g38</t>
+        </is>
+      </c>
+    </row>
+    <row r="1160">
+      <c r="A1160" t="inlineStr">
+        <is>
+          <t>2026-08-08T21:04:13</t>
+        </is>
+      </c>
+      <c r="B1160" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1160" t="inlineStr">
+        <is>
+          <t>CountPickedRejectPandral</t>
+        </is>
+      </c>
+      <c r="D1160" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E1160" t="inlineStr"/>
+      <c r="F1160" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g39</t>
+        </is>
+      </c>
+    </row>
+    <row r="1161">
+      <c r="A1161" t="inlineStr">
+        <is>
+          <t>2026-08-08T21:04:13</t>
+        </is>
+      </c>
+      <c r="B1161" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1161" t="inlineStr">
+        <is>
+          <t>CountPickedReject18in</t>
+        </is>
+      </c>
+      <c r="D1161" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E1161" t="inlineStr"/>
+      <c r="F1161" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g40</t>
+        </is>
+      </c>
+    </row>
+    <row r="1162">
+      <c r="A1162" t="inlineStr">
+        <is>
+          <t>2026-08-08T21:05:00</t>
+        </is>
+      </c>
+      <c r="B1162" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1162" t="inlineStr">
+        <is>
+          <t>_1st_SCAN</t>
+        </is>
+      </c>
+      <c r="D1162" t="b">
+        <v>0</v>
+      </c>
+      <c r="E1162" t="n">
+        <v>11</v>
+      </c>
+      <c r="F1162" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1163">
+      <c r="A1163" t="inlineStr">
+        <is>
+          <t>2026-08-08T21:05:00</t>
+        </is>
+      </c>
+      <c r="B1163" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1163" t="inlineStr">
+        <is>
+          <t>TieDetectOffset_B</t>
+        </is>
+      </c>
+      <c r="D1163" t="b">
+        <v>0</v>
+      </c>
+      <c r="E1163" t="n">
+        <v>11</v>
+      </c>
+      <c r="F1163" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1164">
+      <c r="A1164" t="inlineStr">
+        <is>
+          <t>2026-08-08T21:05:00</t>
+        </is>
+      </c>
+      <c r="B1164" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1164" t="inlineStr">
+        <is>
+          <t>Tie Detector</t>
+        </is>
+      </c>
+      <c r="D1164" t="b">
+        <v>0</v>
+      </c>
+      <c r="E1164" t="n">
+        <v>11</v>
+      </c>
+      <c r="F1164" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1165">
+      <c r="A1165" t="inlineStr">
+        <is>
+          <t>2026-08-08T21:05:00</t>
+        </is>
+      </c>
+      <c r="B1165" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1165" t="inlineStr">
+        <is>
+          <t>TPS Full</t>
+        </is>
+      </c>
+      <c r="D1165" t="b">
+        <v>0</v>
+      </c>
+      <c r="E1165" t="n">
+        <v>11</v>
+      </c>
+      <c r="F1165" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1166">
+      <c r="A1166" t="inlineStr">
+        <is>
+          <t>2026-08-08T21:05:00</t>
+        </is>
+      </c>
+      <c r="B1166" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1166" t="inlineStr">
+        <is>
+          <t>TieDetectOffset_A</t>
+        </is>
+      </c>
+      <c r="D1166" t="b">
+        <v>0</v>
+      </c>
+      <c r="E1166" t="n">
+        <v>11</v>
+      </c>
+      <c r="F1166" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1167">
+      <c r="A1167" t="inlineStr">
+        <is>
+          <t>2026-08-08T21:05:00</t>
+        </is>
+      </c>
+      <c r="B1167" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1167" t="inlineStr">
+        <is>
+          <t>TPS Connected</t>
+        </is>
+      </c>
+      <c r="D1167" t="b">
+        <v>0</v>
+      </c>
+      <c r="E1167" t="n">
+        <v>11</v>
+      </c>
+      <c r="F1167" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1168">
+      <c r="A1168" t="inlineStr">
+        <is>
+          <t>2026-08-08T21:05:00</t>
+        </is>
+      </c>
+      <c r="B1168" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1168" t="inlineStr">
+        <is>
+          <t>TPS_Enable_ Button</t>
+        </is>
+      </c>
+      <c r="D1168" t="b">
+        <v>0</v>
+      </c>
+      <c r="E1168" t="n">
+        <v>11</v>
+      </c>
+      <c r="F1168" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1169">
+      <c r="A1169" t="inlineStr">
+        <is>
+          <t>2026-08-08T21:05:00</t>
+        </is>
+      </c>
+      <c r="B1169" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1169" t="inlineStr">
+        <is>
+          <t>AirEagle Eject Plate</t>
+        </is>
+      </c>
+      <c r="D1169" t="b">
+        <v>0</v>
+      </c>
+      <c r="E1169" t="n">
+        <v>11</v>
+      </c>
+      <c r="F1169" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1170">
+      <c r="A1170" t="inlineStr">
+        <is>
+          <t>2026-08-08T21:05:00</t>
+        </is>
+      </c>
+      <c r="B1170" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1170" t="inlineStr">
+        <is>
+          <t>tk_Cycle</t>
+        </is>
+      </c>
+      <c r="D1170" t="b">
+        <v>0</v>
+      </c>
+      <c r="E1170" t="n">
+        <v>11</v>
+      </c>
+      <c r="F1170" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1171">
+      <c r="A1171" t="inlineStr">
+        <is>
+          <t>2026-08-08T21:05:00</t>
+        </is>
+      </c>
+      <c r="B1171" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1171" t="inlineStr">
+        <is>
+          <t>Servos_Enabled</t>
+        </is>
+      </c>
+      <c r="D1171" t="b">
+        <v>0</v>
+      </c>
+      <c r="E1171" t="n">
+        <v>11</v>
+      </c>
+      <c r="F1171" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1172">
+      <c r="A1172" t="inlineStr">
+        <is>
+          <t>2026-08-08T21:05:00</t>
+        </is>
+      </c>
+      <c r="B1172" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1172" t="inlineStr">
+        <is>
+          <t>TPS Enabled</t>
+        </is>
+      </c>
+      <c r="D1172" t="b">
+        <v>0</v>
+      </c>
+      <c r="E1172" t="n">
+        <v>11</v>
+      </c>
+      <c r="F1172" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1173">
+      <c r="A1173" t="inlineStr">
+        <is>
+          <t>2026-08-08T21:05:00</t>
+        </is>
+      </c>
+      <c r="B1173" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1173" t="inlineStr">
+        <is>
+          <t>tk_Abort</t>
+        </is>
+      </c>
+      <c r="D1173" t="b">
+        <v>0</v>
+      </c>
+      <c r="E1173" t="n">
+        <v>11</v>
+      </c>
+      <c r="F1173" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1174">
+      <c r="A1174" t="inlineStr">
+        <is>
+          <t>2026-08-08T21:05:00</t>
+        </is>
+      </c>
+      <c r="B1174" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1174" t="inlineStr">
+        <is>
+          <t>Robot_isMoving</t>
+        </is>
+      </c>
+      <c r="D1174" t="b">
+        <v>0</v>
+      </c>
+      <c r="E1174" t="n">
+        <v>11</v>
+      </c>
+      <c r="F1174" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1175">
+      <c r="A1175" t="inlineStr">
+        <is>
+          <t>2026-08-08T21:05:00</t>
+        </is>
+      </c>
+      <c r="B1175" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1175" t="inlineStr">
+        <is>
+          <t>Eject Tie Plate</t>
+        </is>
+      </c>
+      <c r="D1175" t="b">
+        <v>0</v>
+      </c>
+      <c r="E1175" t="n">
+        <v>11</v>
+      </c>
+      <c r="F1175" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1176">
+      <c r="A1176" t="inlineStr">
+        <is>
+          <t>2026-08-08T21:05:00</t>
+        </is>
+      </c>
+      <c r="B1176" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1176" t="inlineStr">
+        <is>
+          <t>TPS BACKUP ALARM</t>
+        </is>
+      </c>
+      <c r="D1176" t="b">
+        <v>0</v>
+      </c>
+      <c r="E1176" t="n">
+        <v>11</v>
+      </c>
+      <c r="F1176" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1177">
+      <c r="A1177" t="inlineStr">
+        <is>
+          <t>2026-08-08T21:05:00</t>
+        </is>
+      </c>
+      <c r="B1177" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1177" t="inlineStr">
+        <is>
+          <t>14in Job</t>
+        </is>
+      </c>
+      <c r="D1177" t="b">
+        <v>1</v>
+      </c>
+      <c r="E1177" t="n">
+        <v>11</v>
+      </c>
+      <c r="F1177" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1178">
+      <c r="A1178" t="inlineStr">
+        <is>
+          <t>2026-08-08T21:05:00</t>
+        </is>
+      </c>
+      <c r="B1178" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1178" t="inlineStr">
+        <is>
+          <t>18in Job</t>
+        </is>
+      </c>
+      <c r="D1178" t="b">
+        <v>0</v>
+      </c>
+      <c r="E1178" t="n">
+        <v>11</v>
+      </c>
+      <c r="F1178" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1179">
+      <c r="A1179" t="inlineStr">
+        <is>
+          <t>2026-08-08T21:05:00</t>
+        </is>
+      </c>
+      <c r="B1179" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1179" t="inlineStr">
+        <is>
+          <t>Pandral Job</t>
+        </is>
+      </c>
+      <c r="D1179" t="b">
+        <v>0</v>
+      </c>
+      <c r="E1179" t="n">
+        <v>11</v>
+      </c>
+      <c r="F1179" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1180">
+      <c r="A1180" t="inlineStr">
+        <is>
+          <t>2026-08-08T21:05:00</t>
+        </is>
+      </c>
+      <c r="B1180" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1180" t="inlineStr">
+        <is>
+          <t>DoubleLay Job</t>
+        </is>
+      </c>
+      <c r="D1180" t="b">
+        <v>0</v>
+      </c>
+      <c r="E1180" t="n">
+        <v>11</v>
+      </c>
+      <c r="F1180" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1181">
+      <c r="A1181" t="inlineStr">
+        <is>
+          <t>2026-08-08T21:05:00</t>
+        </is>
+      </c>
+      <c r="B1181" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1181" t="inlineStr">
+        <is>
+          <t>TPSjam_FLAG</t>
+        </is>
+      </c>
+      <c r="D1181" t="b">
+        <v>0</v>
+      </c>
+      <c r="E1181" t="n">
+        <v>11</v>
+      </c>
+      <c r="F1181" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1182">
+      <c r="A1182" t="inlineStr">
+        <is>
+          <t>2026-08-08T21:05:00</t>
+        </is>
+      </c>
+      <c r="B1182" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1182" t="inlineStr">
+        <is>
+          <t>RoCalRequest</t>
+        </is>
+      </c>
+      <c r="D1182" t="b">
+        <v>0</v>
+      </c>
+      <c r="E1182" t="n">
+        <v>11</v>
+      </c>
+      <c r="F1182" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1183">
+      <c r="A1183" t="inlineStr">
+        <is>
+          <t>2026-08-08T21:05:00</t>
+        </is>
+      </c>
+      <c r="B1183" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1183" t="inlineStr">
+        <is>
+          <t>tkCycle_TotalSeconds</t>
+        </is>
+      </c>
+      <c r="D1183" t="n">
+        <v>0</v>
+      </c>
+      <c r="E1183" t="n">
+        <v>9</v>
+      </c>
+      <c r="F1183" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1184">
+      <c r="A1184" t="inlineStr">
+        <is>
+          <t>2026-08-08T21:05:00</t>
+        </is>
+      </c>
+      <c r="B1184" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1184" t="inlineStr">
+        <is>
+          <t>tkCycle_NoMoveSec</t>
+        </is>
+      </c>
+      <c r="D1184" t="n">
+        <v>0</v>
+      </c>
+      <c r="E1184" t="n">
+        <v>9</v>
+      </c>
+      <c r="F1184" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1185">
+      <c r="A1185" t="inlineStr">
+        <is>
+          <t>2026-08-08T21:05:00</t>
+        </is>
+      </c>
+      <c r="B1185" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1185" t="inlineStr">
+        <is>
+          <t>tkCycle_MoveSeconds</t>
+        </is>
+      </c>
+      <c r="D1185" t="n">
+        <v>0</v>
+      </c>
+      <c r="E1185" t="n">
+        <v>9</v>
+      </c>
+      <c r="F1185" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1186">
+      <c r="A1186" t="inlineStr">
+        <is>
+          <t>2026-08-08T21:05:00</t>
+        </is>
+      </c>
+      <c r="B1186" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1186" t="inlineStr">
+        <is>
+          <t>Percent time moveing</t>
+        </is>
+      </c>
+      <c r="D1186" t="n">
+        <v>0</v>
+      </c>
+      <c r="E1186" t="n">
+        <v>9</v>
+      </c>
+      <c r="F1186" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1187">
+      <c r="A1187" t="inlineStr">
+        <is>
+          <t>2026-08-08T21:05:00</t>
+        </is>
+      </c>
+      <c r="B1187" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1187" t="inlineStr">
+        <is>
+          <t>Percent time not moving</t>
+        </is>
+      </c>
+      <c r="D1187" t="n">
+        <v>0</v>
+      </c>
+      <c r="E1187" t="n">
+        <v>9</v>
+      </c>
+      <c r="F1187" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1188">
+      <c r="A1188" t="inlineStr">
+        <is>
+          <t>2026-08-08T21:05:00</t>
+        </is>
+      </c>
+      <c r="B1188" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1188" t="inlineStr">
+        <is>
+          <t>TotalPickPartsCount</t>
+        </is>
+      </c>
+      <c r="D1188" t="n">
+        <v>0</v>
+      </c>
+      <c r="E1188" t="n">
+        <v>9</v>
+      </c>
+      <c r="F1188" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1189">
+      <c r="A1189" t="inlineStr">
+        <is>
+          <t>2026-08-08T21:05:00</t>
+        </is>
+      </c>
+      <c r="B1189" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1189" t="inlineStr">
+        <is>
+          <t>RejectPartsCount</t>
+        </is>
+      </c>
+      <c r="D1189" t="n">
+        <v>0</v>
+      </c>
+      <c r="E1189" t="n">
+        <v>9</v>
+      </c>
+      <c r="F1189" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1190">
+      <c r="A1190" t="inlineStr">
+        <is>
+          <t>2026-08-08T21:05:00</t>
+        </is>
+      </c>
+      <c r="B1190" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1190" t="inlineStr">
+        <is>
+          <t>AcceptsPartsCount</t>
+        </is>
+      </c>
+      <c r="D1190" t="n">
+        <v>0</v>
+      </c>
+      <c r="E1190" t="n">
+        <v>9</v>
+      </c>
+      <c r="F1190" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1191">
+      <c r="A1191" t="inlineStr">
+        <is>
+          <t>2026-08-08T21:05:00</t>
+        </is>
+      </c>
+      <c r="B1191" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1191" t="inlineStr">
+        <is>
+          <t>percentCount_accept</t>
+        </is>
+      </c>
+      <c r="D1191" t="n">
+        <v>0</v>
+      </c>
+      <c r="E1191" t="n">
+        <v>9</v>
+      </c>
+      <c r="F1191" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1192">
+      <c r="A1192" t="inlineStr">
+        <is>
+          <t>2026-08-08T21:05:00</t>
+        </is>
+      </c>
+      <c r="B1192" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1192" t="inlineStr">
+        <is>
+          <t>percentCount_reject</t>
+        </is>
+      </c>
+      <c r="D1192" t="n">
+        <v>0</v>
+      </c>
+      <c r="E1192" t="n">
+        <v>9</v>
+      </c>
+      <c r="F1192" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1193">
+      <c r="A1193" t="inlineStr">
+        <is>
+          <t>2026-08-08T21:05:00</t>
+        </is>
+      </c>
+      <c r="B1193" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1193" t="inlineStr">
+        <is>
+          <t>Avg Parts per min_total</t>
+        </is>
+      </c>
+      <c r="D1193" t="n">
+        <v>0</v>
+      </c>
+      <c r="E1193" t="n">
+        <v>9</v>
+      </c>
+      <c r="F1193" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1194">
+      <c r="A1194" t="inlineStr">
+        <is>
+          <t>2026-08-08T21:05:00</t>
+        </is>
+      </c>
+      <c r="B1194" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1194" t="inlineStr">
+        <is>
+          <t>TotalPickedParts</t>
+        </is>
+      </c>
+      <c r="D1194" t="n">
+        <v>0</v>
+      </c>
+      <c r="E1194" t="n">
+        <v>3</v>
+      </c>
+      <c r="F1194" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1195">
+      <c r="A1195" t="inlineStr">
+        <is>
+          <t>2026-08-08T21:05:00</t>
+        </is>
+      </c>
+      <c r="B1195" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1195" t="inlineStr">
+        <is>
+          <t>TotalPickedAcceptParts</t>
+        </is>
+      </c>
+      <c r="D1195" t="n">
+        <v>0</v>
+      </c>
+      <c r="E1195" t="n">
+        <v>3</v>
+      </c>
+      <c r="F1195" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1196">
+      <c r="A1196" t="inlineStr">
+        <is>
+          <t>2026-08-08T21:05:00</t>
+        </is>
+      </c>
+      <c r="B1196" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1196" t="inlineStr">
+        <is>
+          <t>TotalPickedRejectParts</t>
+        </is>
+      </c>
+      <c r="D1196" t="n">
+        <v>0</v>
+      </c>
+      <c r="E1196" t="n">
+        <v>3</v>
+      </c>
+      <c r="F1196" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1197">
+      <c r="A1197" t="inlineStr">
+        <is>
+          <t>2026-08-08T21:05:00</t>
+        </is>
+      </c>
+      <c r="B1197" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1197" t="inlineStr">
+        <is>
+          <t>TotalTiePlatesLaid</t>
+        </is>
+      </c>
+      <c r="D1197" t="n">
+        <v>0</v>
+      </c>
+      <c r="E1197" t="n">
+        <v>3</v>
+      </c>
+      <c r="F1197" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1198">
+      <c r="A1198" t="inlineStr">
+        <is>
+          <t>2026-08-08T21:05:00</t>
+        </is>
+      </c>
+      <c r="B1198" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1198" t="inlineStr">
+        <is>
+          <t>Daily_TotalLaidPlates</t>
+        </is>
+      </c>
+      <c r="D1198" t="n">
+        <v>0</v>
+      </c>
+      <c r="E1198" t="n">
+        <v>3</v>
+      </c>
+      <c r="F1198" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1199">
+      <c r="A1199" t="inlineStr">
+        <is>
+          <t>2026-08-08T21:05:00</t>
+        </is>
+      </c>
+      <c r="B1199" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1199" t="inlineStr">
+        <is>
+          <t>CountPicked14in</t>
+        </is>
+      </c>
+      <c r="D1199" t="n">
+        <v>0</v>
+      </c>
+      <c r="E1199" t="n">
+        <v>3</v>
+      </c>
+      <c r="F1199" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1200">
+      <c r="A1200" t="inlineStr">
+        <is>
+          <t>2026-08-08T21:05:00</t>
+        </is>
+      </c>
+      <c r="B1200" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1200" t="inlineStr">
+        <is>
+          <t>CountPicked18in</t>
+        </is>
+      </c>
+      <c r="D1200" t="n">
+        <v>0</v>
+      </c>
+      <c r="E1200" t="n">
+        <v>3</v>
+      </c>
+      <c r="F1200" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1201">
+      <c r="A1201" t="inlineStr">
+        <is>
+          <t>2026-08-08T21:05:00</t>
+        </is>
+      </c>
+      <c r="B1201" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1201" t="inlineStr">
+        <is>
+          <t>CountPickedPandral</t>
+        </is>
+      </c>
+      <c r="D1201" t="n">
+        <v>0</v>
+      </c>
+      <c r="E1201" t="n">
+        <v>3</v>
+      </c>
+      <c r="F1201" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1202">
+      <c r="A1202" t="inlineStr">
+        <is>
+          <t>2026-08-08T21:05:00</t>
+        </is>
+      </c>
+      <c r="B1202" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1202" t="inlineStr">
+        <is>
+          <t>CountPickedOTM</t>
+        </is>
+      </c>
+      <c r="D1202" t="n">
+        <v>0</v>
+      </c>
+      <c r="E1202" t="n">
+        <v>3</v>
+      </c>
+      <c r="F1202" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1203">
+      <c r="A1203" t="inlineStr">
+        <is>
+          <t>2026-08-08T21:05:00</t>
+        </is>
+      </c>
+      <c r="B1203" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1203" t="inlineStr">
+        <is>
+          <t>RoCals</t>
+        </is>
+      </c>
+      <c r="D1203" t="n">
+        <v>0</v>
+      </c>
+      <c r="E1203" t="n">
+        <v>3</v>
+      </c>
+      <c r="F1203" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1204">
+      <c r="A1204" t="inlineStr">
+        <is>
+          <t>2026-08-08T21:05:00</t>
+        </is>
+      </c>
+      <c r="B1204" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1204" t="inlineStr">
+        <is>
+          <t>TPS_JamsUsr</t>
+        </is>
+      </c>
+      <c r="D1204" t="n">
+        <v>0</v>
+      </c>
+      <c r="E1204" t="n">
+        <v>3</v>
+      </c>
+      <c r="F1204" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1205">
+      <c r="A1205" t="inlineStr">
+        <is>
+          <t>2026-08-08T21:05:00</t>
+        </is>
+      </c>
+      <c r="B1205" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1205" t="inlineStr">
+        <is>
+          <t>TPS_JamsMASTER</t>
+        </is>
+      </c>
+      <c r="D1205" t="n">
+        <v>0</v>
+      </c>
+      <c r="E1205" t="n">
+        <v>3</v>
+      </c>
+      <c r="F1205" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1206">
+      <c r="A1206" t="inlineStr">
+        <is>
+          <t>2026-08-08T21:05:00</t>
+        </is>
+      </c>
+      <c r="B1206" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1206" t="inlineStr">
+        <is>
+          <t>ABORT_Master</t>
+        </is>
+      </c>
+      <c r="D1206" t="n">
+        <v>0</v>
+      </c>
+      <c r="E1206" t="n">
+        <v>3</v>
+      </c>
+      <c r="F1206" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/plc</t>
         </is>

</xml_diff>

<commit_message>
Log MQTT data 2026-08-08 22:04 UTC
</commit_message>
<xml_diff>
--- a/logs/raiv_tracker_2026-08-08.xlsx
+++ b/logs/raiv_tracker_2026-08-08.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F1206"/>
+  <dimension ref="A1:F1336"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -31429,7 +31429,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E1122" t="inlineStr"/>
       <c r="F1122" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g2</t>
@@ -31457,7 +31456,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E1123" t="inlineStr"/>
       <c r="F1123" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g3</t>
@@ -31485,7 +31483,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E1124" t="inlineStr"/>
       <c r="F1124" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g4</t>
@@ -31513,7 +31510,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E1125" t="inlineStr"/>
       <c r="F1125" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g5</t>
@@ -31541,7 +31537,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E1126" t="inlineStr"/>
       <c r="F1126" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g6</t>
@@ -31569,7 +31564,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E1127" t="inlineStr"/>
       <c r="F1127" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g7</t>
@@ -31597,7 +31591,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E1128" t="inlineStr"/>
       <c r="F1128" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g1</t>
@@ -31625,7 +31618,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E1129" t="inlineStr"/>
       <c r="F1129" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g8</t>
@@ -31653,7 +31645,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E1130" t="inlineStr"/>
       <c r="F1130" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g9</t>
@@ -31681,7 +31672,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E1131" t="inlineStr"/>
       <c r="F1131" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g10</t>
@@ -31709,7 +31699,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E1132" t="inlineStr"/>
       <c r="F1132" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g11</t>
@@ -31737,7 +31726,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E1133" t="inlineStr"/>
       <c r="F1133" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g13</t>
@@ -31765,7 +31753,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E1134" t="inlineStr"/>
       <c r="F1134" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g15</t>
@@ -31793,7 +31780,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E1135" t="inlineStr"/>
       <c r="F1135" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g17</t>
@@ -31821,7 +31807,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E1136" t="inlineStr"/>
       <c r="F1136" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g18</t>
@@ -31849,7 +31834,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E1137" t="inlineStr"/>
       <c r="F1137" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g19</t>
@@ -31877,7 +31861,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E1138" t="inlineStr"/>
       <c r="F1138" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g22</t>
@@ -31905,7 +31888,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E1139" t="inlineStr"/>
       <c r="F1139" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g23</t>
@@ -31933,7 +31915,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E1140" t="inlineStr"/>
       <c r="F1140" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g24</t>
@@ -31961,7 +31942,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E1141" t="inlineStr"/>
       <c r="F1141" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g25</t>
@@ -31989,7 +31969,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E1142" t="inlineStr"/>
       <c r="F1142" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g33</t>
@@ -32017,7 +31996,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E1143" t="inlineStr"/>
       <c r="F1143" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g34</t>
@@ -32045,7 +32023,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E1144" t="inlineStr"/>
       <c r="F1144" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g36</t>
@@ -32073,7 +32050,6 @@
           <t>1</t>
         </is>
       </c>
-      <c r="E1145" t="inlineStr"/>
       <c r="F1145" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g12</t>
@@ -32101,7 +32077,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E1146" t="inlineStr"/>
       <c r="F1146" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g14</t>
@@ -32129,7 +32104,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E1147" t="inlineStr"/>
       <c r="F1147" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g16</t>
@@ -32157,7 +32131,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E1148" t="inlineStr"/>
       <c r="F1148" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g20</t>
@@ -32185,7 +32158,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E1149" t="inlineStr"/>
       <c r="F1149" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g21</t>
@@ -32213,7 +32185,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E1150" t="inlineStr"/>
       <c r="F1150" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g26</t>
@@ -32241,7 +32212,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E1151" t="inlineStr"/>
       <c r="F1151" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g27</t>
@@ -32269,7 +32239,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E1152" t="inlineStr"/>
       <c r="F1152" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g28</t>
@@ -32297,7 +32266,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E1153" t="inlineStr"/>
       <c r="F1153" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g29</t>
@@ -32325,7 +32293,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E1154" t="inlineStr"/>
       <c r="F1154" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g30</t>
@@ -32353,7 +32320,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E1155" t="inlineStr"/>
       <c r="F1155" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g31</t>
@@ -32381,7 +32347,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E1156" t="inlineStr"/>
       <c r="F1156" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g32</t>
@@ -32409,7 +32374,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E1157" t="inlineStr"/>
       <c r="F1157" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g35</t>
@@ -32437,7 +32401,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E1158" t="inlineStr"/>
       <c r="F1158" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g37</t>
@@ -32465,7 +32428,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E1159" t="inlineStr"/>
       <c r="F1159" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g38</t>
@@ -32493,7 +32455,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E1160" t="inlineStr"/>
       <c r="F1160" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g39</t>
@@ -32521,7 +32482,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E1161" t="inlineStr"/>
       <c r="F1161" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g40</t>
@@ -33783,6 +33743,3646 @@
         <v>3</v>
       </c>
       <c r="F1206" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1207">
+      <c r="A1207" t="inlineStr">
+        <is>
+          <t>2026-08-08T22:03:00</t>
+        </is>
+      </c>
+      <c r="B1207" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1207" t="inlineStr">
+        <is>
+          <t>_1st_SCAN</t>
+        </is>
+      </c>
+      <c r="D1207" t="b">
+        <v>0</v>
+      </c>
+      <c r="E1207" t="n">
+        <v>11</v>
+      </c>
+      <c r="F1207" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1208">
+      <c r="A1208" t="inlineStr">
+        <is>
+          <t>2026-08-08T22:03:00</t>
+        </is>
+      </c>
+      <c r="B1208" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1208" t="inlineStr">
+        <is>
+          <t>TieDetectOffset_B</t>
+        </is>
+      </c>
+      <c r="D1208" t="b">
+        <v>0</v>
+      </c>
+      <c r="E1208" t="n">
+        <v>11</v>
+      </c>
+      <c r="F1208" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1209">
+      <c r="A1209" t="inlineStr">
+        <is>
+          <t>2026-08-08T22:03:00</t>
+        </is>
+      </c>
+      <c r="B1209" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1209" t="inlineStr">
+        <is>
+          <t>Tie Detector</t>
+        </is>
+      </c>
+      <c r="D1209" t="b">
+        <v>0</v>
+      </c>
+      <c r="E1209" t="n">
+        <v>11</v>
+      </c>
+      <c r="F1209" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1210">
+      <c r="A1210" t="inlineStr">
+        <is>
+          <t>2026-08-08T22:03:00</t>
+        </is>
+      </c>
+      <c r="B1210" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1210" t="inlineStr">
+        <is>
+          <t>TPS Full</t>
+        </is>
+      </c>
+      <c r="D1210" t="b">
+        <v>0</v>
+      </c>
+      <c r="E1210" t="n">
+        <v>11</v>
+      </c>
+      <c r="F1210" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1211">
+      <c r="A1211" t="inlineStr">
+        <is>
+          <t>2026-08-08T22:03:00</t>
+        </is>
+      </c>
+      <c r="B1211" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1211" t="inlineStr">
+        <is>
+          <t>TieDetectOffset_A</t>
+        </is>
+      </c>
+      <c r="D1211" t="b">
+        <v>0</v>
+      </c>
+      <c r="E1211" t="n">
+        <v>11</v>
+      </c>
+      <c r="F1211" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1212">
+      <c r="A1212" t="inlineStr">
+        <is>
+          <t>2026-08-08T22:03:00</t>
+        </is>
+      </c>
+      <c r="B1212" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1212" t="inlineStr">
+        <is>
+          <t>TPS Connected</t>
+        </is>
+      </c>
+      <c r="D1212" t="b">
+        <v>0</v>
+      </c>
+      <c r="E1212" t="n">
+        <v>11</v>
+      </c>
+      <c r="F1212" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1213">
+      <c r="A1213" t="inlineStr">
+        <is>
+          <t>2026-08-08T22:03:00</t>
+        </is>
+      </c>
+      <c r="B1213" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1213" t="inlineStr">
+        <is>
+          <t>TPS_Enable_ Button</t>
+        </is>
+      </c>
+      <c r="D1213" t="b">
+        <v>0</v>
+      </c>
+      <c r="E1213" t="n">
+        <v>11</v>
+      </c>
+      <c r="F1213" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1214">
+      <c r="A1214" t="inlineStr">
+        <is>
+          <t>2026-08-08T22:03:00</t>
+        </is>
+      </c>
+      <c r="B1214" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1214" t="inlineStr">
+        <is>
+          <t>AirEagle Eject Plate</t>
+        </is>
+      </c>
+      <c r="D1214" t="b">
+        <v>0</v>
+      </c>
+      <c r="E1214" t="n">
+        <v>11</v>
+      </c>
+      <c r="F1214" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1215">
+      <c r="A1215" t="inlineStr">
+        <is>
+          <t>2026-08-08T22:03:00</t>
+        </is>
+      </c>
+      <c r="B1215" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1215" t="inlineStr">
+        <is>
+          <t>tk_Cycle</t>
+        </is>
+      </c>
+      <c r="D1215" t="b">
+        <v>0</v>
+      </c>
+      <c r="E1215" t="n">
+        <v>11</v>
+      </c>
+      <c r="F1215" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1216">
+      <c r="A1216" t="inlineStr">
+        <is>
+          <t>2026-08-08T22:03:00</t>
+        </is>
+      </c>
+      <c r="B1216" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1216" t="inlineStr">
+        <is>
+          <t>Servos_Enabled</t>
+        </is>
+      </c>
+      <c r="D1216" t="b">
+        <v>0</v>
+      </c>
+      <c r="E1216" t="n">
+        <v>11</v>
+      </c>
+      <c r="F1216" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1217">
+      <c r="A1217" t="inlineStr">
+        <is>
+          <t>2026-08-08T22:03:00</t>
+        </is>
+      </c>
+      <c r="B1217" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1217" t="inlineStr">
+        <is>
+          <t>TPS Enabled</t>
+        </is>
+      </c>
+      <c r="D1217" t="b">
+        <v>0</v>
+      </c>
+      <c r="E1217" t="n">
+        <v>11</v>
+      </c>
+      <c r="F1217" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1218">
+      <c r="A1218" t="inlineStr">
+        <is>
+          <t>2026-08-08T22:03:00</t>
+        </is>
+      </c>
+      <c r="B1218" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1218" t="inlineStr">
+        <is>
+          <t>tk_Abort</t>
+        </is>
+      </c>
+      <c r="D1218" t="b">
+        <v>0</v>
+      </c>
+      <c r="E1218" t="n">
+        <v>11</v>
+      </c>
+      <c r="F1218" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1219">
+      <c r="A1219" t="inlineStr">
+        <is>
+          <t>2026-08-08T22:03:00</t>
+        </is>
+      </c>
+      <c r="B1219" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1219" t="inlineStr">
+        <is>
+          <t>Robot_isMoving</t>
+        </is>
+      </c>
+      <c r="D1219" t="b">
+        <v>0</v>
+      </c>
+      <c r="E1219" t="n">
+        <v>11</v>
+      </c>
+      <c r="F1219" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1220">
+      <c r="A1220" t="inlineStr">
+        <is>
+          <t>2026-08-08T22:03:00</t>
+        </is>
+      </c>
+      <c r="B1220" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1220" t="inlineStr">
+        <is>
+          <t>Eject Tie Plate</t>
+        </is>
+      </c>
+      <c r="D1220" t="b">
+        <v>0</v>
+      </c>
+      <c r="E1220" t="n">
+        <v>11</v>
+      </c>
+      <c r="F1220" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1221">
+      <c r="A1221" t="inlineStr">
+        <is>
+          <t>2026-08-08T22:03:00</t>
+        </is>
+      </c>
+      <c r="B1221" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1221" t="inlineStr">
+        <is>
+          <t>TPS BACKUP ALARM</t>
+        </is>
+      </c>
+      <c r="D1221" t="b">
+        <v>0</v>
+      </c>
+      <c r="E1221" t="n">
+        <v>11</v>
+      </c>
+      <c r="F1221" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1222">
+      <c r="A1222" t="inlineStr">
+        <is>
+          <t>2026-08-08T22:03:00</t>
+        </is>
+      </c>
+      <c r="B1222" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1222" t="inlineStr">
+        <is>
+          <t>14in Job</t>
+        </is>
+      </c>
+      <c r="D1222" t="b">
+        <v>1</v>
+      </c>
+      <c r="E1222" t="n">
+        <v>11</v>
+      </c>
+      <c r="F1222" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1223">
+      <c r="A1223" t="inlineStr">
+        <is>
+          <t>2026-08-08T22:03:00</t>
+        </is>
+      </c>
+      <c r="B1223" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1223" t="inlineStr">
+        <is>
+          <t>18in Job</t>
+        </is>
+      </c>
+      <c r="D1223" t="b">
+        <v>0</v>
+      </c>
+      <c r="E1223" t="n">
+        <v>11</v>
+      </c>
+      <c r="F1223" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1224">
+      <c r="A1224" t="inlineStr">
+        <is>
+          <t>2026-08-08T22:03:00</t>
+        </is>
+      </c>
+      <c r="B1224" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1224" t="inlineStr">
+        <is>
+          <t>Pandral Job</t>
+        </is>
+      </c>
+      <c r="D1224" t="b">
+        <v>0</v>
+      </c>
+      <c r="E1224" t="n">
+        <v>11</v>
+      </c>
+      <c r="F1224" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1225">
+      <c r="A1225" t="inlineStr">
+        <is>
+          <t>2026-08-08T22:03:00</t>
+        </is>
+      </c>
+      <c r="B1225" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1225" t="inlineStr">
+        <is>
+          <t>DoubleLay Job</t>
+        </is>
+      </c>
+      <c r="D1225" t="b">
+        <v>0</v>
+      </c>
+      <c r="E1225" t="n">
+        <v>11</v>
+      </c>
+      <c r="F1225" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1226">
+      <c r="A1226" t="inlineStr">
+        <is>
+          <t>2026-08-08T22:03:00</t>
+        </is>
+      </c>
+      <c r="B1226" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1226" t="inlineStr">
+        <is>
+          <t>TPSjam_FLAG</t>
+        </is>
+      </c>
+      <c r="D1226" t="b">
+        <v>0</v>
+      </c>
+      <c r="E1226" t="n">
+        <v>11</v>
+      </c>
+      <c r="F1226" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1227">
+      <c r="A1227" t="inlineStr">
+        <is>
+          <t>2026-08-08T22:03:00</t>
+        </is>
+      </c>
+      <c r="B1227" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1227" t="inlineStr">
+        <is>
+          <t>RoCalRequest</t>
+        </is>
+      </c>
+      <c r="D1227" t="b">
+        <v>0</v>
+      </c>
+      <c r="E1227" t="n">
+        <v>11</v>
+      </c>
+      <c r="F1227" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1228">
+      <c r="A1228" t="inlineStr">
+        <is>
+          <t>2026-08-08T22:03:00</t>
+        </is>
+      </c>
+      <c r="B1228" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1228" t="inlineStr">
+        <is>
+          <t>tkCycle_TotalSeconds</t>
+        </is>
+      </c>
+      <c r="D1228" t="n">
+        <v>0</v>
+      </c>
+      <c r="E1228" t="n">
+        <v>9</v>
+      </c>
+      <c r="F1228" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1229">
+      <c r="A1229" t="inlineStr">
+        <is>
+          <t>2026-08-08T22:03:00</t>
+        </is>
+      </c>
+      <c r="B1229" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1229" t="inlineStr">
+        <is>
+          <t>tkCycle_NoMoveSec</t>
+        </is>
+      </c>
+      <c r="D1229" t="n">
+        <v>0</v>
+      </c>
+      <c r="E1229" t="n">
+        <v>9</v>
+      </c>
+      <c r="F1229" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1230">
+      <c r="A1230" t="inlineStr">
+        <is>
+          <t>2026-08-08T22:03:00</t>
+        </is>
+      </c>
+      <c r="B1230" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1230" t="inlineStr">
+        <is>
+          <t>tkCycle_MoveSeconds</t>
+        </is>
+      </c>
+      <c r="D1230" t="n">
+        <v>0</v>
+      </c>
+      <c r="E1230" t="n">
+        <v>9</v>
+      </c>
+      <c r="F1230" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1231">
+      <c r="A1231" t="inlineStr">
+        <is>
+          <t>2026-08-08T22:03:00</t>
+        </is>
+      </c>
+      <c r="B1231" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1231" t="inlineStr">
+        <is>
+          <t>Percent time moveing</t>
+        </is>
+      </c>
+      <c r="D1231" t="n">
+        <v>0</v>
+      </c>
+      <c r="E1231" t="n">
+        <v>9</v>
+      </c>
+      <c r="F1231" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1232">
+      <c r="A1232" t="inlineStr">
+        <is>
+          <t>2026-08-08T22:03:00</t>
+        </is>
+      </c>
+      <c r="B1232" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1232" t="inlineStr">
+        <is>
+          <t>Percent time not moving</t>
+        </is>
+      </c>
+      <c r="D1232" t="n">
+        <v>0</v>
+      </c>
+      <c r="E1232" t="n">
+        <v>9</v>
+      </c>
+      <c r="F1232" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1233">
+      <c r="A1233" t="inlineStr">
+        <is>
+          <t>2026-08-08T22:03:00</t>
+        </is>
+      </c>
+      <c r="B1233" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1233" t="inlineStr">
+        <is>
+          <t>TotalPickPartsCount</t>
+        </is>
+      </c>
+      <c r="D1233" t="n">
+        <v>0</v>
+      </c>
+      <c r="E1233" t="n">
+        <v>9</v>
+      </c>
+      <c r="F1233" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1234">
+      <c r="A1234" t="inlineStr">
+        <is>
+          <t>2026-08-08T22:03:00</t>
+        </is>
+      </c>
+      <c r="B1234" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1234" t="inlineStr">
+        <is>
+          <t>RejectPartsCount</t>
+        </is>
+      </c>
+      <c r="D1234" t="n">
+        <v>0</v>
+      </c>
+      <c r="E1234" t="n">
+        <v>9</v>
+      </c>
+      <c r="F1234" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1235">
+      <c r="A1235" t="inlineStr">
+        <is>
+          <t>2026-08-08T22:03:00</t>
+        </is>
+      </c>
+      <c r="B1235" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1235" t="inlineStr">
+        <is>
+          <t>AcceptsPartsCount</t>
+        </is>
+      </c>
+      <c r="D1235" t="n">
+        <v>0</v>
+      </c>
+      <c r="E1235" t="n">
+        <v>9</v>
+      </c>
+      <c r="F1235" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1236">
+      <c r="A1236" t="inlineStr">
+        <is>
+          <t>2026-08-08T22:03:00</t>
+        </is>
+      </c>
+      <c r="B1236" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1236" t="inlineStr">
+        <is>
+          <t>percentCount_accept</t>
+        </is>
+      </c>
+      <c r="D1236" t="n">
+        <v>0</v>
+      </c>
+      <c r="E1236" t="n">
+        <v>9</v>
+      </c>
+      <c r="F1236" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1237">
+      <c r="A1237" t="inlineStr">
+        <is>
+          <t>2026-08-08T22:03:00</t>
+        </is>
+      </c>
+      <c r="B1237" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1237" t="inlineStr">
+        <is>
+          <t>percentCount_reject</t>
+        </is>
+      </c>
+      <c r="D1237" t="n">
+        <v>0</v>
+      </c>
+      <c r="E1237" t="n">
+        <v>9</v>
+      </c>
+      <c r="F1237" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1238">
+      <c r="A1238" t="inlineStr">
+        <is>
+          <t>2026-08-08T22:03:00</t>
+        </is>
+      </c>
+      <c r="B1238" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1238" t="inlineStr">
+        <is>
+          <t>Avg Parts per min_total</t>
+        </is>
+      </c>
+      <c r="D1238" t="n">
+        <v>0</v>
+      </c>
+      <c r="E1238" t="n">
+        <v>9</v>
+      </c>
+      <c r="F1238" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1239">
+      <c r="A1239" t="inlineStr">
+        <is>
+          <t>2026-08-08T22:03:00</t>
+        </is>
+      </c>
+      <c r="B1239" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1239" t="inlineStr">
+        <is>
+          <t>TotalPickedParts</t>
+        </is>
+      </c>
+      <c r="D1239" t="n">
+        <v>0</v>
+      </c>
+      <c r="E1239" t="n">
+        <v>3</v>
+      </c>
+      <c r="F1239" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1240">
+      <c r="A1240" t="inlineStr">
+        <is>
+          <t>2026-08-08T22:03:00</t>
+        </is>
+      </c>
+      <c r="B1240" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1240" t="inlineStr">
+        <is>
+          <t>TotalPickedAcceptParts</t>
+        </is>
+      </c>
+      <c r="D1240" t="n">
+        <v>0</v>
+      </c>
+      <c r="E1240" t="n">
+        <v>3</v>
+      </c>
+      <c r="F1240" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1241">
+      <c r="A1241" t="inlineStr">
+        <is>
+          <t>2026-08-08T22:03:00</t>
+        </is>
+      </c>
+      <c r="B1241" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1241" t="inlineStr">
+        <is>
+          <t>TotalPickedRejectParts</t>
+        </is>
+      </c>
+      <c r="D1241" t="n">
+        <v>0</v>
+      </c>
+      <c r="E1241" t="n">
+        <v>3</v>
+      </c>
+      <c r="F1241" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1242">
+      <c r="A1242" t="inlineStr">
+        <is>
+          <t>2026-08-08T22:03:00</t>
+        </is>
+      </c>
+      <c r="B1242" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1242" t="inlineStr">
+        <is>
+          <t>TotalTiePlatesLaid</t>
+        </is>
+      </c>
+      <c r="D1242" t="n">
+        <v>0</v>
+      </c>
+      <c r="E1242" t="n">
+        <v>3</v>
+      </c>
+      <c r="F1242" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1243">
+      <c r="A1243" t="inlineStr">
+        <is>
+          <t>2026-08-08T22:03:00</t>
+        </is>
+      </c>
+      <c r="B1243" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1243" t="inlineStr">
+        <is>
+          <t>Daily_TotalLaidPlates</t>
+        </is>
+      </c>
+      <c r="D1243" t="n">
+        <v>0</v>
+      </c>
+      <c r="E1243" t="n">
+        <v>3</v>
+      </c>
+      <c r="F1243" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1244">
+      <c r="A1244" t="inlineStr">
+        <is>
+          <t>2026-08-08T22:03:00</t>
+        </is>
+      </c>
+      <c r="B1244" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1244" t="inlineStr">
+        <is>
+          <t>CountPicked14in</t>
+        </is>
+      </c>
+      <c r="D1244" t="n">
+        <v>0</v>
+      </c>
+      <c r="E1244" t="n">
+        <v>3</v>
+      </c>
+      <c r="F1244" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1245">
+      <c r="A1245" t="inlineStr">
+        <is>
+          <t>2026-08-08T22:03:00</t>
+        </is>
+      </c>
+      <c r="B1245" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1245" t="inlineStr">
+        <is>
+          <t>CountPicked18in</t>
+        </is>
+      </c>
+      <c r="D1245" t="n">
+        <v>0</v>
+      </c>
+      <c r="E1245" t="n">
+        <v>3</v>
+      </c>
+      <c r="F1245" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1246">
+      <c r="A1246" t="inlineStr">
+        <is>
+          <t>2026-08-08T22:03:00</t>
+        </is>
+      </c>
+      <c r="B1246" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1246" t="inlineStr">
+        <is>
+          <t>CountPickedPandral</t>
+        </is>
+      </c>
+      <c r="D1246" t="n">
+        <v>0</v>
+      </c>
+      <c r="E1246" t="n">
+        <v>3</v>
+      </c>
+      <c r="F1246" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1247">
+      <c r="A1247" t="inlineStr">
+        <is>
+          <t>2026-08-08T22:03:00</t>
+        </is>
+      </c>
+      <c r="B1247" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1247" t="inlineStr">
+        <is>
+          <t>CountPickedOTM</t>
+        </is>
+      </c>
+      <c r="D1247" t="n">
+        <v>0</v>
+      </c>
+      <c r="E1247" t="n">
+        <v>3</v>
+      </c>
+      <c r="F1247" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1248">
+      <c r="A1248" t="inlineStr">
+        <is>
+          <t>2026-08-08T22:03:00</t>
+        </is>
+      </c>
+      <c r="B1248" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1248" t="inlineStr">
+        <is>
+          <t>RoCals</t>
+        </is>
+      </c>
+      <c r="D1248" t="n">
+        <v>0</v>
+      </c>
+      <c r="E1248" t="n">
+        <v>3</v>
+      </c>
+      <c r="F1248" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1249">
+      <c r="A1249" t="inlineStr">
+        <is>
+          <t>2026-08-08T22:03:00</t>
+        </is>
+      </c>
+      <c r="B1249" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1249" t="inlineStr">
+        <is>
+          <t>TPS_JamsUsr</t>
+        </is>
+      </c>
+      <c r="D1249" t="n">
+        <v>0</v>
+      </c>
+      <c r="E1249" t="n">
+        <v>3</v>
+      </c>
+      <c r="F1249" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1250">
+      <c r="A1250" t="inlineStr">
+        <is>
+          <t>2026-08-08T22:03:00</t>
+        </is>
+      </c>
+      <c r="B1250" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1250" t="inlineStr">
+        <is>
+          <t>TPS_JamsMASTER</t>
+        </is>
+      </c>
+      <c r="D1250" t="n">
+        <v>0</v>
+      </c>
+      <c r="E1250" t="n">
+        <v>3</v>
+      </c>
+      <c r="F1250" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1251">
+      <c r="A1251" t="inlineStr">
+        <is>
+          <t>2026-08-08T22:03:00</t>
+        </is>
+      </c>
+      <c r="B1251" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1251" t="inlineStr">
+        <is>
+          <t>ABORT_Master</t>
+        </is>
+      </c>
+      <c r="D1251" t="n">
+        <v>0</v>
+      </c>
+      <c r="E1251" t="n">
+        <v>3</v>
+      </c>
+      <c r="F1251" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1252">
+      <c r="A1252" t="inlineStr">
+        <is>
+          <t>2026-08-08T22:03:13</t>
+        </is>
+      </c>
+      <c r="B1252" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1252" t="inlineStr">
+        <is>
+          <t>TotalTiePlatesLaid</t>
+        </is>
+      </c>
+      <c r="D1252" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E1252" t="inlineStr"/>
+      <c r="F1252" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g1</t>
+        </is>
+      </c>
+    </row>
+    <row r="1253">
+      <c r="A1253" t="inlineStr">
+        <is>
+          <t>2026-08-08T22:03:13</t>
+        </is>
+      </c>
+      <c r="B1253" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1253" t="inlineStr">
+        <is>
+          <t>usr_TPStime Hours10th</t>
+        </is>
+      </c>
+      <c r="D1253" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E1253" t="inlineStr"/>
+      <c r="F1253" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g8</t>
+        </is>
+      </c>
+    </row>
+    <row r="1254">
+      <c r="A1254" t="inlineStr">
+        <is>
+          <t>2026-08-08T22:03:13</t>
+        </is>
+      </c>
+      <c r="B1254" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1254" t="inlineStr">
+        <is>
+          <t>usrTPS_miles xxx</t>
+        </is>
+      </c>
+      <c r="D1254" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E1254" t="inlineStr"/>
+      <c r="F1254" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g9</t>
+        </is>
+      </c>
+    </row>
+    <row r="1255">
+      <c r="A1255" t="inlineStr">
+        <is>
+          <t>2026-08-08T22:03:13</t>
+        </is>
+      </c>
+      <c r="B1255" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1255" t="inlineStr">
+        <is>
+          <t>TPS Connected</t>
+        </is>
+      </c>
+      <c r="D1255" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E1255" t="inlineStr"/>
+      <c r="F1255" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g10</t>
+        </is>
+      </c>
+    </row>
+    <row r="1256">
+      <c r="A1256" t="inlineStr">
+        <is>
+          <t>2026-08-08T22:03:13</t>
+        </is>
+      </c>
+      <c r="B1256" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1256" t="inlineStr">
+        <is>
+          <t>TPS Enabled</t>
+        </is>
+      </c>
+      <c r="D1256" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E1256" t="inlineStr"/>
+      <c r="F1256" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g11</t>
+        </is>
+      </c>
+    </row>
+    <row r="1257">
+      <c r="A1257" t="inlineStr">
+        <is>
+          <t>2026-08-08T22:03:13</t>
+        </is>
+      </c>
+      <c r="B1257" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1257" t="inlineStr">
+        <is>
+          <t>14in Job</t>
+        </is>
+      </c>
+      <c r="D1257" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E1257" t="inlineStr"/>
+      <c r="F1257" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g12</t>
+        </is>
+      </c>
+    </row>
+    <row r="1258">
+      <c r="A1258" t="inlineStr">
+        <is>
+          <t>2026-08-08T22:03:13</t>
+        </is>
+      </c>
+      <c r="B1258" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1258" t="inlineStr">
+        <is>
+          <t>Pandral Job</t>
+        </is>
+      </c>
+      <c r="D1258" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E1258" t="inlineStr"/>
+      <c r="F1258" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g14</t>
+        </is>
+      </c>
+    </row>
+    <row r="1259">
+      <c r="A1259" t="inlineStr">
+        <is>
+          <t>2026-08-08T22:03:13</t>
+        </is>
+      </c>
+      <c r="B1259" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1259" t="inlineStr">
+        <is>
+          <t>CountRejectedTotal</t>
+        </is>
+      </c>
+      <c r="D1259" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E1259" t="inlineStr"/>
+      <c r="F1259" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g16</t>
+        </is>
+      </c>
+    </row>
+    <row r="1260">
+      <c r="A1260" t="inlineStr">
+        <is>
+          <t>2026-08-08T22:03:13</t>
+        </is>
+      </c>
+      <c r="B1260" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1260" t="inlineStr">
+        <is>
+          <t>RejectPartsCount</t>
+        </is>
+      </c>
+      <c r="D1260" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E1260" t="inlineStr"/>
+      <c r="F1260" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g20</t>
+        </is>
+      </c>
+    </row>
+    <row r="1261">
+      <c r="A1261" t="inlineStr">
+        <is>
+          <t>2026-08-08T22:03:13</t>
+        </is>
+      </c>
+      <c r="B1261" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1261" t="inlineStr">
+        <is>
+          <t>tk_Cycle hrs</t>
+        </is>
+      </c>
+      <c r="D1261" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E1261" t="inlineStr"/>
+      <c r="F1261" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g21</t>
+        </is>
+      </c>
+    </row>
+    <row r="1262">
+      <c r="A1262" t="inlineStr">
+        <is>
+          <t>2026-08-08T22:03:13</t>
+        </is>
+      </c>
+      <c r="B1262" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1262" t="inlineStr">
+        <is>
+          <t>tk_Warmup</t>
+        </is>
+      </c>
+      <c r="D1262" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E1262" t="inlineStr"/>
+      <c r="F1262" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g26</t>
+        </is>
+      </c>
+    </row>
+    <row r="1263">
+      <c r="A1263" t="inlineStr">
+        <is>
+          <t>2026-08-08T22:03:13</t>
+        </is>
+      </c>
+      <c r="B1263" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1263" t="inlineStr">
+        <is>
+          <t>FindingParts min</t>
+        </is>
+      </c>
+      <c r="D1263" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E1263" t="inlineStr"/>
+      <c r="F1263" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g27</t>
+        </is>
+      </c>
+    </row>
+    <row r="1264">
+      <c r="A1264" t="inlineStr">
+        <is>
+          <t>2026-08-08T22:03:13</t>
+        </is>
+      </c>
+      <c r="B1264" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1264" t="inlineStr">
+        <is>
+          <t>PickingParts min</t>
+        </is>
+      </c>
+      <c r="D1264" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E1264" t="inlineStr"/>
+      <c r="F1264" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g28</t>
+        </is>
+      </c>
+    </row>
+    <row r="1265">
+      <c r="A1265" t="inlineStr">
+        <is>
+          <t>2026-08-08T22:03:13</t>
+        </is>
+      </c>
+      <c r="B1265" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1265" t="inlineStr">
+        <is>
+          <t>PlacingParts min</t>
+        </is>
+      </c>
+      <c r="D1265" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E1265" t="inlineStr"/>
+      <c r="F1265" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g29</t>
+        </is>
+      </c>
+    </row>
+    <row r="1266">
+      <c r="A1266" t="inlineStr">
+        <is>
+          <t>2026-08-08T22:03:13</t>
+        </is>
+      </c>
+      <c r="B1266" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1266" t="inlineStr">
+        <is>
+          <t>CountPickedReject14in</t>
+        </is>
+      </c>
+      <c r="D1266" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E1266" t="inlineStr"/>
+      <c r="F1266" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g30</t>
+        </is>
+      </c>
+    </row>
+    <row r="1267">
+      <c r="A1267" t="inlineStr">
+        <is>
+          <t>2026-08-08T22:03:13</t>
+        </is>
+      </c>
+      <c r="B1267" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1267" t="inlineStr">
+        <is>
+          <t>temp_dsi</t>
+        </is>
+      </c>
+      <c r="D1267" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E1267" t="inlineStr"/>
+      <c r="F1267" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g31</t>
+        </is>
+      </c>
+    </row>
+    <row r="1268">
+      <c r="A1268" t="inlineStr">
+        <is>
+          <t>2026-08-08T22:03:13</t>
+        </is>
+      </c>
+      <c r="B1268" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1268" t="inlineStr">
+        <is>
+          <t>temp_J1motor</t>
+        </is>
+      </c>
+      <c r="D1268" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E1268" t="inlineStr"/>
+      <c r="F1268" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g32</t>
+        </is>
+      </c>
+    </row>
+    <row r="1269">
+      <c r="A1269" t="inlineStr">
+        <is>
+          <t>2026-08-08T22:03:13</t>
+        </is>
+      </c>
+      <c r="B1269" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1269" t="inlineStr">
+        <is>
+          <t>temp_J4motor</t>
+        </is>
+      </c>
+      <c r="D1269" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E1269" t="inlineStr"/>
+      <c r="F1269" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g35</t>
+        </is>
+      </c>
+    </row>
+    <row r="1270">
+      <c r="A1270" t="inlineStr">
+        <is>
+          <t>2026-08-08T22:03:13</t>
+        </is>
+      </c>
+      <c r="B1270" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1270" t="inlineStr">
+        <is>
+          <t>temp_J6motor</t>
+        </is>
+      </c>
+      <c r="D1270" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E1270" t="inlineStr"/>
+      <c r="F1270" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g37</t>
+        </is>
+      </c>
+    </row>
+    <row r="1271">
+      <c r="A1271" t="inlineStr">
+        <is>
+          <t>2026-08-08T22:03:13</t>
+        </is>
+      </c>
+      <c r="B1271" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1271" t="inlineStr">
+        <is>
+          <t>CountPickedRejectOTM</t>
+        </is>
+      </c>
+      <c r="D1271" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E1271" t="inlineStr"/>
+      <c r="F1271" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g38</t>
+        </is>
+      </c>
+    </row>
+    <row r="1272">
+      <c r="A1272" t="inlineStr">
+        <is>
+          <t>2026-08-08T22:03:13</t>
+        </is>
+      </c>
+      <c r="B1272" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1272" t="inlineStr">
+        <is>
+          <t>CountPickedRejectPandral</t>
+        </is>
+      </c>
+      <c r="D1272" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E1272" t="inlineStr"/>
+      <c r="F1272" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g39</t>
+        </is>
+      </c>
+    </row>
+    <row r="1273">
+      <c r="A1273" t="inlineStr">
+        <is>
+          <t>2026-08-08T22:03:13</t>
+        </is>
+      </c>
+      <c r="B1273" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1273" t="inlineStr">
+        <is>
+          <t>CountLaidButton</t>
+        </is>
+      </c>
+      <c r="D1273" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E1273" t="inlineStr"/>
+      <c r="F1273" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g2</t>
+        </is>
+      </c>
+    </row>
+    <row r="1274">
+      <c r="A1274" t="inlineStr">
+        <is>
+          <t>2026-08-08T22:03:13</t>
+        </is>
+      </c>
+      <c r="B1274" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1274" t="inlineStr">
+        <is>
+          <t>CountLaidDetector</t>
+        </is>
+      </c>
+      <c r="D1274" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E1274" t="inlineStr"/>
+      <c r="F1274" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g3</t>
+        </is>
+      </c>
+    </row>
+    <row r="1275">
+      <c r="A1275" t="inlineStr">
+        <is>
+          <t>2026-08-08T22:03:13</t>
+        </is>
+      </c>
+      <c r="B1275" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1275" t="inlineStr">
+        <is>
+          <t>CountLaidEncoder</t>
+        </is>
+      </c>
+      <c r="D1275" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E1275" t="inlineStr"/>
+      <c r="F1275" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g4</t>
+        </is>
+      </c>
+    </row>
+    <row r="1276">
+      <c r="A1276" t="inlineStr">
+        <is>
+          <t>2026-08-08T22:03:13</t>
+        </is>
+      </c>
+      <c r="B1276" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1276" t="inlineStr">
+        <is>
+          <t>CountLaid14in</t>
+        </is>
+      </c>
+      <c r="D1276" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E1276" t="inlineStr"/>
+      <c r="F1276" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g5</t>
+        </is>
+      </c>
+    </row>
+    <row r="1277">
+      <c r="A1277" t="inlineStr">
+        <is>
+          <t>2026-08-08T22:03:13</t>
+        </is>
+      </c>
+      <c r="B1277" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1277" t="inlineStr">
+        <is>
+          <t>CountLaid18in</t>
+        </is>
+      </c>
+      <c r="D1277" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E1277" t="inlineStr"/>
+      <c r="F1277" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g6</t>
+        </is>
+      </c>
+    </row>
+    <row r="1278">
+      <c r="A1278" t="inlineStr">
+        <is>
+          <t>2026-08-08T22:03:13</t>
+        </is>
+      </c>
+      <c r="B1278" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1278" t="inlineStr">
+        <is>
+          <t>CountLaidPandral</t>
+        </is>
+      </c>
+      <c r="D1278" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E1278" t="inlineStr"/>
+      <c r="F1278" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g7</t>
+        </is>
+      </c>
+    </row>
+    <row r="1279">
+      <c r="A1279" t="inlineStr">
+        <is>
+          <t>2026-08-08T22:03:13</t>
+        </is>
+      </c>
+      <c r="B1279" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1279" t="inlineStr">
+        <is>
+          <t>18in Job</t>
+        </is>
+      </c>
+      <c r="D1279" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E1279" t="inlineStr"/>
+      <c r="F1279" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g13</t>
+        </is>
+      </c>
+    </row>
+    <row r="1280">
+      <c r="A1280" t="inlineStr">
+        <is>
+          <t>2026-08-08T22:03:13</t>
+        </is>
+      </c>
+      <c r="B1280" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1280" t="inlineStr">
+        <is>
+          <t>CountAcceptedTotal</t>
+        </is>
+      </c>
+      <c r="D1280" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E1280" t="inlineStr"/>
+      <c r="F1280" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g15</t>
+        </is>
+      </c>
+    </row>
+    <row r="1281">
+      <c r="A1281" t="inlineStr">
+        <is>
+          <t>2026-08-08T22:03:13</t>
+        </is>
+      </c>
+      <c r="B1281" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1281" t="inlineStr">
+        <is>
+          <t>Servos_Enabled</t>
+        </is>
+      </c>
+      <c r="D1281" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E1281" t="inlineStr"/>
+      <c r="F1281" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g17</t>
+        </is>
+      </c>
+    </row>
+    <row r="1282">
+      <c r="A1282" t="inlineStr">
+        <is>
+          <t>2026-08-08T22:03:13</t>
+        </is>
+      </c>
+      <c r="B1282" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1282" t="inlineStr">
+        <is>
+          <t>TotalPickPartsCount</t>
+        </is>
+      </c>
+      <c r="D1282" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E1282" t="inlineStr"/>
+      <c r="F1282" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g18</t>
+        </is>
+      </c>
+    </row>
+    <row r="1283">
+      <c r="A1283" t="inlineStr">
+        <is>
+          <t>2026-08-08T22:03:13</t>
+        </is>
+      </c>
+      <c r="B1283" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1283" t="inlineStr">
+        <is>
+          <t>AcceptsPartsCount</t>
+        </is>
+      </c>
+      <c r="D1283" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E1283" t="inlineStr"/>
+      <c r="F1283" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g19</t>
+        </is>
+      </c>
+    </row>
+    <row r="1284">
+      <c r="A1284" t="inlineStr">
+        <is>
+          <t>2026-08-08T22:03:13</t>
+        </is>
+      </c>
+      <c r="B1284" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1284" t="inlineStr">
+        <is>
+          <t>day_Servotime Hours10th</t>
+        </is>
+      </c>
+      <c r="D1284" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E1284" t="inlineStr"/>
+      <c r="F1284" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g22</t>
+        </is>
+      </c>
+    </row>
+    <row r="1285">
+      <c r="A1285" t="inlineStr">
+        <is>
+          <t>2026-08-08T22:03:13</t>
+        </is>
+      </c>
+      <c r="B1285" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1285" t="inlineStr">
+        <is>
+          <t>tk_Cycle</t>
+        </is>
+      </c>
+      <c r="D1285" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E1285" t="inlineStr"/>
+      <c r="F1285" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g23</t>
+        </is>
+      </c>
+    </row>
+    <row r="1286">
+      <c r="A1286" t="inlineStr">
+        <is>
+          <t>2026-08-08T22:03:13</t>
+        </is>
+      </c>
+      <c r="B1286" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1286" t="inlineStr">
+        <is>
+          <t>tk_Abort</t>
+        </is>
+      </c>
+      <c r="D1286" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E1286" t="inlineStr"/>
+      <c r="F1286" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g24</t>
+        </is>
+      </c>
+    </row>
+    <row r="1287">
+      <c r="A1287" t="inlineStr">
+        <is>
+          <t>2026-08-08T22:03:13</t>
+        </is>
+      </c>
+      <c r="B1287" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1287" t="inlineStr">
+        <is>
+          <t>tk_ClearPos</t>
+        </is>
+      </c>
+      <c r="D1287" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E1287" t="inlineStr"/>
+      <c r="F1287" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g25</t>
+        </is>
+      </c>
+    </row>
+    <row r="1288">
+      <c r="A1288" t="inlineStr">
+        <is>
+          <t>2026-08-08T22:03:13</t>
+        </is>
+      </c>
+      <c r="B1288" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1288" t="inlineStr">
+        <is>
+          <t>temp_J2motor</t>
+        </is>
+      </c>
+      <c r="D1288" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E1288" t="inlineStr"/>
+      <c r="F1288" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g33</t>
+        </is>
+      </c>
+    </row>
+    <row r="1289">
+      <c r="A1289" t="inlineStr">
+        <is>
+          <t>2026-08-08T22:03:13</t>
+        </is>
+      </c>
+      <c r="B1289" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1289" t="inlineStr">
+        <is>
+          <t>temp_J3motor</t>
+        </is>
+      </c>
+      <c r="D1289" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E1289" t="inlineStr"/>
+      <c r="F1289" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g34</t>
+        </is>
+      </c>
+    </row>
+    <row r="1290">
+      <c r="A1290" t="inlineStr">
+        <is>
+          <t>2026-08-08T22:03:13</t>
+        </is>
+      </c>
+      <c r="B1290" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1290" t="inlineStr">
+        <is>
+          <t>temp_J5motor</t>
+        </is>
+      </c>
+      <c r="D1290" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E1290" t="inlineStr"/>
+      <c r="F1290" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g36</t>
+        </is>
+      </c>
+    </row>
+    <row r="1291">
+      <c r="A1291" t="inlineStr">
+        <is>
+          <t>2026-08-08T22:03:13</t>
+        </is>
+      </c>
+      <c r="B1291" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1291" t="inlineStr">
+        <is>
+          <t>CountPickedReject18in</t>
+        </is>
+      </c>
+      <c r="D1291" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E1291" t="inlineStr"/>
+      <c r="F1291" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g40</t>
+        </is>
+      </c>
+    </row>
+    <row r="1292">
+      <c r="A1292" t="inlineStr">
+        <is>
+          <t>2026-08-08T22:04:00</t>
+        </is>
+      </c>
+      <c r="B1292" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1292" t="inlineStr">
+        <is>
+          <t>_1st_SCAN</t>
+        </is>
+      </c>
+      <c r="D1292" t="b">
+        <v>0</v>
+      </c>
+      <c r="E1292" t="n">
+        <v>11</v>
+      </c>
+      <c r="F1292" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1293">
+      <c r="A1293" t="inlineStr">
+        <is>
+          <t>2026-08-08T22:04:00</t>
+        </is>
+      </c>
+      <c r="B1293" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1293" t="inlineStr">
+        <is>
+          <t>TieDetectOffset_B</t>
+        </is>
+      </c>
+      <c r="D1293" t="b">
+        <v>0</v>
+      </c>
+      <c r="E1293" t="n">
+        <v>11</v>
+      </c>
+      <c r="F1293" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1294">
+      <c r="A1294" t="inlineStr">
+        <is>
+          <t>2026-08-08T22:04:00</t>
+        </is>
+      </c>
+      <c r="B1294" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1294" t="inlineStr">
+        <is>
+          <t>Tie Detector</t>
+        </is>
+      </c>
+      <c r="D1294" t="b">
+        <v>0</v>
+      </c>
+      <c r="E1294" t="n">
+        <v>11</v>
+      </c>
+      <c r="F1294" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1295">
+      <c r="A1295" t="inlineStr">
+        <is>
+          <t>2026-08-08T22:04:00</t>
+        </is>
+      </c>
+      <c r="B1295" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1295" t="inlineStr">
+        <is>
+          <t>TPS Full</t>
+        </is>
+      </c>
+      <c r="D1295" t="b">
+        <v>0</v>
+      </c>
+      <c r="E1295" t="n">
+        <v>11</v>
+      </c>
+      <c r="F1295" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1296">
+      <c r="A1296" t="inlineStr">
+        <is>
+          <t>2026-08-08T22:04:00</t>
+        </is>
+      </c>
+      <c r="B1296" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1296" t="inlineStr">
+        <is>
+          <t>TieDetectOffset_A</t>
+        </is>
+      </c>
+      <c r="D1296" t="b">
+        <v>0</v>
+      </c>
+      <c r="E1296" t="n">
+        <v>11</v>
+      </c>
+      <c r="F1296" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1297">
+      <c r="A1297" t="inlineStr">
+        <is>
+          <t>2026-08-08T22:04:00</t>
+        </is>
+      </c>
+      <c r="B1297" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1297" t="inlineStr">
+        <is>
+          <t>TPS Connected</t>
+        </is>
+      </c>
+      <c r="D1297" t="b">
+        <v>0</v>
+      </c>
+      <c r="E1297" t="n">
+        <v>11</v>
+      </c>
+      <c r="F1297" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1298">
+      <c r="A1298" t="inlineStr">
+        <is>
+          <t>2026-08-08T22:04:00</t>
+        </is>
+      </c>
+      <c r="B1298" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1298" t="inlineStr">
+        <is>
+          <t>TPS_Enable_ Button</t>
+        </is>
+      </c>
+      <c r="D1298" t="b">
+        <v>0</v>
+      </c>
+      <c r="E1298" t="n">
+        <v>11</v>
+      </c>
+      <c r="F1298" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1299">
+      <c r="A1299" t="inlineStr">
+        <is>
+          <t>2026-08-08T22:04:00</t>
+        </is>
+      </c>
+      <c r="B1299" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1299" t="inlineStr">
+        <is>
+          <t>AirEagle Eject Plate</t>
+        </is>
+      </c>
+      <c r="D1299" t="b">
+        <v>0</v>
+      </c>
+      <c r="E1299" t="n">
+        <v>11</v>
+      </c>
+      <c r="F1299" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1300">
+      <c r="A1300" t="inlineStr">
+        <is>
+          <t>2026-08-08T22:04:00</t>
+        </is>
+      </c>
+      <c r="B1300" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1300" t="inlineStr">
+        <is>
+          <t>tk_Cycle</t>
+        </is>
+      </c>
+      <c r="D1300" t="b">
+        <v>0</v>
+      </c>
+      <c r="E1300" t="n">
+        <v>11</v>
+      </c>
+      <c r="F1300" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1301">
+      <c r="A1301" t="inlineStr">
+        <is>
+          <t>2026-08-08T22:04:00</t>
+        </is>
+      </c>
+      <c r="B1301" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1301" t="inlineStr">
+        <is>
+          <t>Servos_Enabled</t>
+        </is>
+      </c>
+      <c r="D1301" t="b">
+        <v>0</v>
+      </c>
+      <c r="E1301" t="n">
+        <v>11</v>
+      </c>
+      <c r="F1301" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1302">
+      <c r="A1302" t="inlineStr">
+        <is>
+          <t>2026-08-08T22:04:00</t>
+        </is>
+      </c>
+      <c r="B1302" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1302" t="inlineStr">
+        <is>
+          <t>TPS Enabled</t>
+        </is>
+      </c>
+      <c r="D1302" t="b">
+        <v>0</v>
+      </c>
+      <c r="E1302" t="n">
+        <v>11</v>
+      </c>
+      <c r="F1302" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1303">
+      <c r="A1303" t="inlineStr">
+        <is>
+          <t>2026-08-08T22:04:00</t>
+        </is>
+      </c>
+      <c r="B1303" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1303" t="inlineStr">
+        <is>
+          <t>tk_Abort</t>
+        </is>
+      </c>
+      <c r="D1303" t="b">
+        <v>0</v>
+      </c>
+      <c r="E1303" t="n">
+        <v>11</v>
+      </c>
+      <c r="F1303" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1304">
+      <c r="A1304" t="inlineStr">
+        <is>
+          <t>2026-08-08T22:04:00</t>
+        </is>
+      </c>
+      <c r="B1304" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1304" t="inlineStr">
+        <is>
+          <t>Robot_isMoving</t>
+        </is>
+      </c>
+      <c r="D1304" t="b">
+        <v>0</v>
+      </c>
+      <c r="E1304" t="n">
+        <v>11</v>
+      </c>
+      <c r="F1304" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1305">
+      <c r="A1305" t="inlineStr">
+        <is>
+          <t>2026-08-08T22:04:00</t>
+        </is>
+      </c>
+      <c r="B1305" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1305" t="inlineStr">
+        <is>
+          <t>Eject Tie Plate</t>
+        </is>
+      </c>
+      <c r="D1305" t="b">
+        <v>0</v>
+      </c>
+      <c r="E1305" t="n">
+        <v>11</v>
+      </c>
+      <c r="F1305" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1306">
+      <c r="A1306" t="inlineStr">
+        <is>
+          <t>2026-08-08T22:04:00</t>
+        </is>
+      </c>
+      <c r="B1306" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1306" t="inlineStr">
+        <is>
+          <t>TPS BACKUP ALARM</t>
+        </is>
+      </c>
+      <c r="D1306" t="b">
+        <v>0</v>
+      </c>
+      <c r="E1306" t="n">
+        <v>11</v>
+      </c>
+      <c r="F1306" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1307">
+      <c r="A1307" t="inlineStr">
+        <is>
+          <t>2026-08-08T22:04:00</t>
+        </is>
+      </c>
+      <c r="B1307" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1307" t="inlineStr">
+        <is>
+          <t>14in Job</t>
+        </is>
+      </c>
+      <c r="D1307" t="b">
+        <v>1</v>
+      </c>
+      <c r="E1307" t="n">
+        <v>11</v>
+      </c>
+      <c r="F1307" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1308">
+      <c r="A1308" t="inlineStr">
+        <is>
+          <t>2026-08-08T22:04:00</t>
+        </is>
+      </c>
+      <c r="B1308" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1308" t="inlineStr">
+        <is>
+          <t>18in Job</t>
+        </is>
+      </c>
+      <c r="D1308" t="b">
+        <v>0</v>
+      </c>
+      <c r="E1308" t="n">
+        <v>11</v>
+      </c>
+      <c r="F1308" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1309">
+      <c r="A1309" t="inlineStr">
+        <is>
+          <t>2026-08-08T22:04:00</t>
+        </is>
+      </c>
+      <c r="B1309" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1309" t="inlineStr">
+        <is>
+          <t>Pandral Job</t>
+        </is>
+      </c>
+      <c r="D1309" t="b">
+        <v>0</v>
+      </c>
+      <c r="E1309" t="n">
+        <v>11</v>
+      </c>
+      <c r="F1309" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1310">
+      <c r="A1310" t="inlineStr">
+        <is>
+          <t>2026-08-08T22:04:00</t>
+        </is>
+      </c>
+      <c r="B1310" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1310" t="inlineStr">
+        <is>
+          <t>DoubleLay Job</t>
+        </is>
+      </c>
+      <c r="D1310" t="b">
+        <v>0</v>
+      </c>
+      <c r="E1310" t="n">
+        <v>11</v>
+      </c>
+      <c r="F1310" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1311">
+      <c r="A1311" t="inlineStr">
+        <is>
+          <t>2026-08-08T22:04:00</t>
+        </is>
+      </c>
+      <c r="B1311" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1311" t="inlineStr">
+        <is>
+          <t>TPSjam_FLAG</t>
+        </is>
+      </c>
+      <c r="D1311" t="b">
+        <v>0</v>
+      </c>
+      <c r="E1311" t="n">
+        <v>11</v>
+      </c>
+      <c r="F1311" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1312">
+      <c r="A1312" t="inlineStr">
+        <is>
+          <t>2026-08-08T22:04:00</t>
+        </is>
+      </c>
+      <c r="B1312" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1312" t="inlineStr">
+        <is>
+          <t>RoCalRequest</t>
+        </is>
+      </c>
+      <c r="D1312" t="b">
+        <v>0</v>
+      </c>
+      <c r="E1312" t="n">
+        <v>11</v>
+      </c>
+      <c r="F1312" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1313">
+      <c r="A1313" t="inlineStr">
+        <is>
+          <t>2026-08-08T22:04:00</t>
+        </is>
+      </c>
+      <c r="B1313" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1313" t="inlineStr">
+        <is>
+          <t>tkCycle_TotalSeconds</t>
+        </is>
+      </c>
+      <c r="D1313" t="n">
+        <v>0</v>
+      </c>
+      <c r="E1313" t="n">
+        <v>9</v>
+      </c>
+      <c r="F1313" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1314">
+      <c r="A1314" t="inlineStr">
+        <is>
+          <t>2026-08-08T22:04:00</t>
+        </is>
+      </c>
+      <c r="B1314" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1314" t="inlineStr">
+        <is>
+          <t>tkCycle_NoMoveSec</t>
+        </is>
+      </c>
+      <c r="D1314" t="n">
+        <v>0</v>
+      </c>
+      <c r="E1314" t="n">
+        <v>9</v>
+      </c>
+      <c r="F1314" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1315">
+      <c r="A1315" t="inlineStr">
+        <is>
+          <t>2026-08-08T22:04:00</t>
+        </is>
+      </c>
+      <c r="B1315" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1315" t="inlineStr">
+        <is>
+          <t>tkCycle_MoveSeconds</t>
+        </is>
+      </c>
+      <c r="D1315" t="n">
+        <v>0</v>
+      </c>
+      <c r="E1315" t="n">
+        <v>9</v>
+      </c>
+      <c r="F1315" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1316">
+      <c r="A1316" t="inlineStr">
+        <is>
+          <t>2026-08-08T22:04:00</t>
+        </is>
+      </c>
+      <c r="B1316" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1316" t="inlineStr">
+        <is>
+          <t>Percent time moveing</t>
+        </is>
+      </c>
+      <c r="D1316" t="n">
+        <v>0</v>
+      </c>
+      <c r="E1316" t="n">
+        <v>9</v>
+      </c>
+      <c r="F1316" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1317">
+      <c r="A1317" t="inlineStr">
+        <is>
+          <t>2026-08-08T22:04:00</t>
+        </is>
+      </c>
+      <c r="B1317" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1317" t="inlineStr">
+        <is>
+          <t>Percent time not moving</t>
+        </is>
+      </c>
+      <c r="D1317" t="n">
+        <v>0</v>
+      </c>
+      <c r="E1317" t="n">
+        <v>9</v>
+      </c>
+      <c r="F1317" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1318">
+      <c r="A1318" t="inlineStr">
+        <is>
+          <t>2026-08-08T22:04:00</t>
+        </is>
+      </c>
+      <c r="B1318" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1318" t="inlineStr">
+        <is>
+          <t>TotalPickPartsCount</t>
+        </is>
+      </c>
+      <c r="D1318" t="n">
+        <v>0</v>
+      </c>
+      <c r="E1318" t="n">
+        <v>9</v>
+      </c>
+      <c r="F1318" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1319">
+      <c r="A1319" t="inlineStr">
+        <is>
+          <t>2026-08-08T22:04:00</t>
+        </is>
+      </c>
+      <c r="B1319" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1319" t="inlineStr">
+        <is>
+          <t>RejectPartsCount</t>
+        </is>
+      </c>
+      <c r="D1319" t="n">
+        <v>0</v>
+      </c>
+      <c r="E1319" t="n">
+        <v>9</v>
+      </c>
+      <c r="F1319" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1320">
+      <c r="A1320" t="inlineStr">
+        <is>
+          <t>2026-08-08T22:04:00</t>
+        </is>
+      </c>
+      <c r="B1320" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1320" t="inlineStr">
+        <is>
+          <t>AcceptsPartsCount</t>
+        </is>
+      </c>
+      <c r="D1320" t="n">
+        <v>0</v>
+      </c>
+      <c r="E1320" t="n">
+        <v>9</v>
+      </c>
+      <c r="F1320" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1321">
+      <c r="A1321" t="inlineStr">
+        <is>
+          <t>2026-08-08T22:04:00</t>
+        </is>
+      </c>
+      <c r="B1321" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1321" t="inlineStr">
+        <is>
+          <t>percentCount_accept</t>
+        </is>
+      </c>
+      <c r="D1321" t="n">
+        <v>0</v>
+      </c>
+      <c r="E1321" t="n">
+        <v>9</v>
+      </c>
+      <c r="F1321" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1322">
+      <c r="A1322" t="inlineStr">
+        <is>
+          <t>2026-08-08T22:04:00</t>
+        </is>
+      </c>
+      <c r="B1322" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1322" t="inlineStr">
+        <is>
+          <t>percentCount_reject</t>
+        </is>
+      </c>
+      <c r="D1322" t="n">
+        <v>0</v>
+      </c>
+      <c r="E1322" t="n">
+        <v>9</v>
+      </c>
+      <c r="F1322" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1323">
+      <c r="A1323" t="inlineStr">
+        <is>
+          <t>2026-08-08T22:04:00</t>
+        </is>
+      </c>
+      <c r="B1323" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1323" t="inlineStr">
+        <is>
+          <t>Avg Parts per min_total</t>
+        </is>
+      </c>
+      <c r="D1323" t="n">
+        <v>0</v>
+      </c>
+      <c r="E1323" t="n">
+        <v>9</v>
+      </c>
+      <c r="F1323" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1324">
+      <c r="A1324" t="inlineStr">
+        <is>
+          <t>2026-08-08T22:04:00</t>
+        </is>
+      </c>
+      <c r="B1324" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1324" t="inlineStr">
+        <is>
+          <t>TotalPickedParts</t>
+        </is>
+      </c>
+      <c r="D1324" t="n">
+        <v>0</v>
+      </c>
+      <c r="E1324" t="n">
+        <v>3</v>
+      </c>
+      <c r="F1324" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1325">
+      <c r="A1325" t="inlineStr">
+        <is>
+          <t>2026-08-08T22:04:00</t>
+        </is>
+      </c>
+      <c r="B1325" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1325" t="inlineStr">
+        <is>
+          <t>TotalPickedAcceptParts</t>
+        </is>
+      </c>
+      <c r="D1325" t="n">
+        <v>0</v>
+      </c>
+      <c r="E1325" t="n">
+        <v>3</v>
+      </c>
+      <c r="F1325" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1326">
+      <c r="A1326" t="inlineStr">
+        <is>
+          <t>2026-08-08T22:04:00</t>
+        </is>
+      </c>
+      <c r="B1326" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1326" t="inlineStr">
+        <is>
+          <t>TotalPickedRejectParts</t>
+        </is>
+      </c>
+      <c r="D1326" t="n">
+        <v>0</v>
+      </c>
+      <c r="E1326" t="n">
+        <v>3</v>
+      </c>
+      <c r="F1326" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1327">
+      <c r="A1327" t="inlineStr">
+        <is>
+          <t>2026-08-08T22:04:00</t>
+        </is>
+      </c>
+      <c r="B1327" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1327" t="inlineStr">
+        <is>
+          <t>TotalTiePlatesLaid</t>
+        </is>
+      </c>
+      <c r="D1327" t="n">
+        <v>0</v>
+      </c>
+      <c r="E1327" t="n">
+        <v>3</v>
+      </c>
+      <c r="F1327" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1328">
+      <c r="A1328" t="inlineStr">
+        <is>
+          <t>2026-08-08T22:04:00</t>
+        </is>
+      </c>
+      <c r="B1328" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1328" t="inlineStr">
+        <is>
+          <t>Daily_TotalLaidPlates</t>
+        </is>
+      </c>
+      <c r="D1328" t="n">
+        <v>0</v>
+      </c>
+      <c r="E1328" t="n">
+        <v>3</v>
+      </c>
+      <c r="F1328" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1329">
+      <c r="A1329" t="inlineStr">
+        <is>
+          <t>2026-08-08T22:04:00</t>
+        </is>
+      </c>
+      <c r="B1329" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1329" t="inlineStr">
+        <is>
+          <t>CountPicked14in</t>
+        </is>
+      </c>
+      <c r="D1329" t="n">
+        <v>0</v>
+      </c>
+      <c r="E1329" t="n">
+        <v>3</v>
+      </c>
+      <c r="F1329" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1330">
+      <c r="A1330" t="inlineStr">
+        <is>
+          <t>2026-08-08T22:04:00</t>
+        </is>
+      </c>
+      <c r="B1330" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1330" t="inlineStr">
+        <is>
+          <t>CountPicked18in</t>
+        </is>
+      </c>
+      <c r="D1330" t="n">
+        <v>0</v>
+      </c>
+      <c r="E1330" t="n">
+        <v>3</v>
+      </c>
+      <c r="F1330" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1331">
+      <c r="A1331" t="inlineStr">
+        <is>
+          <t>2026-08-08T22:04:00</t>
+        </is>
+      </c>
+      <c r="B1331" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1331" t="inlineStr">
+        <is>
+          <t>CountPickedPandral</t>
+        </is>
+      </c>
+      <c r="D1331" t="n">
+        <v>0</v>
+      </c>
+      <c r="E1331" t="n">
+        <v>3</v>
+      </c>
+      <c r="F1331" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1332">
+      <c r="A1332" t="inlineStr">
+        <is>
+          <t>2026-08-08T22:04:00</t>
+        </is>
+      </c>
+      <c r="B1332" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1332" t="inlineStr">
+        <is>
+          <t>CountPickedOTM</t>
+        </is>
+      </c>
+      <c r="D1332" t="n">
+        <v>0</v>
+      </c>
+      <c r="E1332" t="n">
+        <v>3</v>
+      </c>
+      <c r="F1332" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1333">
+      <c r="A1333" t="inlineStr">
+        <is>
+          <t>2026-08-08T22:04:00</t>
+        </is>
+      </c>
+      <c r="B1333" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1333" t="inlineStr">
+        <is>
+          <t>RoCals</t>
+        </is>
+      </c>
+      <c r="D1333" t="n">
+        <v>0</v>
+      </c>
+      <c r="E1333" t="n">
+        <v>3</v>
+      </c>
+      <c r="F1333" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1334">
+      <c r="A1334" t="inlineStr">
+        <is>
+          <t>2026-08-08T22:04:00</t>
+        </is>
+      </c>
+      <c r="B1334" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1334" t="inlineStr">
+        <is>
+          <t>TPS_JamsUsr</t>
+        </is>
+      </c>
+      <c r="D1334" t="n">
+        <v>0</v>
+      </c>
+      <c r="E1334" t="n">
+        <v>3</v>
+      </c>
+      <c r="F1334" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1335">
+      <c r="A1335" t="inlineStr">
+        <is>
+          <t>2026-08-08T22:04:00</t>
+        </is>
+      </c>
+      <c r="B1335" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1335" t="inlineStr">
+        <is>
+          <t>TPS_JamsMASTER</t>
+        </is>
+      </c>
+      <c r="D1335" t="n">
+        <v>0</v>
+      </c>
+      <c r="E1335" t="n">
+        <v>3</v>
+      </c>
+      <c r="F1335" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1336">
+      <c r="A1336" t="inlineStr">
+        <is>
+          <t>2026-08-08T22:04:00</t>
+        </is>
+      </c>
+      <c r="B1336" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1336" t="inlineStr">
+        <is>
+          <t>ABORT_Master</t>
+        </is>
+      </c>
+      <c r="D1336" t="n">
+        <v>0</v>
+      </c>
+      <c r="E1336" t="n">
+        <v>3</v>
+      </c>
+      <c r="F1336" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/plc</t>
         </is>

</xml_diff>

<commit_message>
Log MQTT data 2026-08-08 23:15 UTC
</commit_message>
<xml_diff>
--- a/logs/raiv_tracker_2026-08-08.xlsx
+++ b/logs/raiv_tracker_2026-08-08.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F1336"/>
+  <dimension ref="A1:F1421"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -35029,7 +35029,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E1252" t="inlineStr"/>
       <c r="F1252" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g1</t>
@@ -35057,7 +35056,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E1253" t="inlineStr"/>
       <c r="F1253" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g8</t>
@@ -35085,7 +35083,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E1254" t="inlineStr"/>
       <c r="F1254" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g9</t>
@@ -35113,7 +35110,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E1255" t="inlineStr"/>
       <c r="F1255" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g10</t>
@@ -35141,7 +35137,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E1256" t="inlineStr"/>
       <c r="F1256" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g11</t>
@@ -35169,7 +35164,6 @@
           <t>1</t>
         </is>
       </c>
-      <c r="E1257" t="inlineStr"/>
       <c r="F1257" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g12</t>
@@ -35197,7 +35191,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E1258" t="inlineStr"/>
       <c r="F1258" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g14</t>
@@ -35225,7 +35218,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E1259" t="inlineStr"/>
       <c r="F1259" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g16</t>
@@ -35253,7 +35245,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E1260" t="inlineStr"/>
       <c r="F1260" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g20</t>
@@ -35281,7 +35272,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E1261" t="inlineStr"/>
       <c r="F1261" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g21</t>
@@ -35309,7 +35299,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E1262" t="inlineStr"/>
       <c r="F1262" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g26</t>
@@ -35337,7 +35326,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E1263" t="inlineStr"/>
       <c r="F1263" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g27</t>
@@ -35365,7 +35353,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E1264" t="inlineStr"/>
       <c r="F1264" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g28</t>
@@ -35393,7 +35380,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E1265" t="inlineStr"/>
       <c r="F1265" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g29</t>
@@ -35421,7 +35407,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E1266" t="inlineStr"/>
       <c r="F1266" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g30</t>
@@ -35449,7 +35434,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E1267" t="inlineStr"/>
       <c r="F1267" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g31</t>
@@ -35477,7 +35461,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E1268" t="inlineStr"/>
       <c r="F1268" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g32</t>
@@ -35505,7 +35488,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E1269" t="inlineStr"/>
       <c r="F1269" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g35</t>
@@ -35533,7 +35515,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E1270" t="inlineStr"/>
       <c r="F1270" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g37</t>
@@ -35561,7 +35542,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E1271" t="inlineStr"/>
       <c r="F1271" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g38</t>
@@ -35589,7 +35569,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E1272" t="inlineStr"/>
       <c r="F1272" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g39</t>
@@ -35617,7 +35596,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E1273" t="inlineStr"/>
       <c r="F1273" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g2</t>
@@ -35645,7 +35623,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E1274" t="inlineStr"/>
       <c r="F1274" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g3</t>
@@ -35673,7 +35650,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E1275" t="inlineStr"/>
       <c r="F1275" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g4</t>
@@ -35701,7 +35677,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E1276" t="inlineStr"/>
       <c r="F1276" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g5</t>
@@ -35729,7 +35704,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E1277" t="inlineStr"/>
       <c r="F1277" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g6</t>
@@ -35757,7 +35731,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E1278" t="inlineStr"/>
       <c r="F1278" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g7</t>
@@ -35785,7 +35758,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E1279" t="inlineStr"/>
       <c r="F1279" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g13</t>
@@ -35813,7 +35785,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E1280" t="inlineStr"/>
       <c r="F1280" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g15</t>
@@ -35841,7 +35812,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E1281" t="inlineStr"/>
       <c r="F1281" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g17</t>
@@ -35869,7 +35839,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E1282" t="inlineStr"/>
       <c r="F1282" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g18</t>
@@ -35897,7 +35866,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E1283" t="inlineStr"/>
       <c r="F1283" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g19</t>
@@ -35925,7 +35893,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E1284" t="inlineStr"/>
       <c r="F1284" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g22</t>
@@ -35953,7 +35920,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E1285" t="inlineStr"/>
       <c r="F1285" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g23</t>
@@ -35981,7 +35947,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E1286" t="inlineStr"/>
       <c r="F1286" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g24</t>
@@ -36009,7 +35974,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E1287" t="inlineStr"/>
       <c r="F1287" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g25</t>
@@ -36037,7 +36001,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E1288" t="inlineStr"/>
       <c r="F1288" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g33</t>
@@ -36065,7 +36028,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E1289" t="inlineStr"/>
       <c r="F1289" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g34</t>
@@ -36093,7 +36055,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E1290" t="inlineStr"/>
       <c r="F1290" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g36</t>
@@ -36121,7 +36082,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E1291" t="inlineStr"/>
       <c r="F1291" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/hmi/g40</t>
@@ -37383,6 +37343,2386 @@
         <v>3</v>
       </c>
       <c r="F1336" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1337">
+      <c r="A1337" t="inlineStr">
+        <is>
+          <t>2026-08-08T23:14:13</t>
+        </is>
+      </c>
+      <c r="B1337" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1337" t="inlineStr">
+        <is>
+          <t>TotalTiePlatesLaid</t>
+        </is>
+      </c>
+      <c r="D1337" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E1337" t="inlineStr"/>
+      <c r="F1337" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g1</t>
+        </is>
+      </c>
+    </row>
+    <row r="1338">
+      <c r="A1338" t="inlineStr">
+        <is>
+          <t>2026-08-08T23:14:13</t>
+        </is>
+      </c>
+      <c r="B1338" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1338" t="inlineStr">
+        <is>
+          <t>usr_TPStime Hours10th</t>
+        </is>
+      </c>
+      <c r="D1338" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E1338" t="inlineStr"/>
+      <c r="F1338" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g8</t>
+        </is>
+      </c>
+    </row>
+    <row r="1339">
+      <c r="A1339" t="inlineStr">
+        <is>
+          <t>2026-08-08T23:14:13</t>
+        </is>
+      </c>
+      <c r="B1339" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1339" t="inlineStr">
+        <is>
+          <t>usrTPS_miles xxx</t>
+        </is>
+      </c>
+      <c r="D1339" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E1339" t="inlineStr"/>
+      <c r="F1339" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g9</t>
+        </is>
+      </c>
+    </row>
+    <row r="1340">
+      <c r="A1340" t="inlineStr">
+        <is>
+          <t>2026-08-08T23:14:13</t>
+        </is>
+      </c>
+      <c r="B1340" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1340" t="inlineStr">
+        <is>
+          <t>TPS Connected</t>
+        </is>
+      </c>
+      <c r="D1340" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E1340" t="inlineStr"/>
+      <c r="F1340" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g10</t>
+        </is>
+      </c>
+    </row>
+    <row r="1341">
+      <c r="A1341" t="inlineStr">
+        <is>
+          <t>2026-08-08T23:14:13</t>
+        </is>
+      </c>
+      <c r="B1341" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1341" t="inlineStr">
+        <is>
+          <t>TPS Enabled</t>
+        </is>
+      </c>
+      <c r="D1341" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E1341" t="inlineStr"/>
+      <c r="F1341" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g11</t>
+        </is>
+      </c>
+    </row>
+    <row r="1342">
+      <c r="A1342" t="inlineStr">
+        <is>
+          <t>2026-08-08T23:14:13</t>
+        </is>
+      </c>
+      <c r="B1342" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1342" t="inlineStr">
+        <is>
+          <t>14in Job</t>
+        </is>
+      </c>
+      <c r="D1342" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E1342" t="inlineStr"/>
+      <c r="F1342" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g12</t>
+        </is>
+      </c>
+    </row>
+    <row r="1343">
+      <c r="A1343" t="inlineStr">
+        <is>
+          <t>2026-08-08T23:14:13</t>
+        </is>
+      </c>
+      <c r="B1343" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1343" t="inlineStr">
+        <is>
+          <t>Pandral Job</t>
+        </is>
+      </c>
+      <c r="D1343" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E1343" t="inlineStr"/>
+      <c r="F1343" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g14</t>
+        </is>
+      </c>
+    </row>
+    <row r="1344">
+      <c r="A1344" t="inlineStr">
+        <is>
+          <t>2026-08-08T23:14:13</t>
+        </is>
+      </c>
+      <c r="B1344" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1344" t="inlineStr">
+        <is>
+          <t>CountRejectedTotal</t>
+        </is>
+      </c>
+      <c r="D1344" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E1344" t="inlineStr"/>
+      <c r="F1344" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g16</t>
+        </is>
+      </c>
+    </row>
+    <row r="1345">
+      <c r="A1345" t="inlineStr">
+        <is>
+          <t>2026-08-08T23:14:13</t>
+        </is>
+      </c>
+      <c r="B1345" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1345" t="inlineStr">
+        <is>
+          <t>RejectPartsCount</t>
+        </is>
+      </c>
+      <c r="D1345" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E1345" t="inlineStr"/>
+      <c r="F1345" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g20</t>
+        </is>
+      </c>
+    </row>
+    <row r="1346">
+      <c r="A1346" t="inlineStr">
+        <is>
+          <t>2026-08-08T23:14:13</t>
+        </is>
+      </c>
+      <c r="B1346" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1346" t="inlineStr">
+        <is>
+          <t>tk_Cycle hrs</t>
+        </is>
+      </c>
+      <c r="D1346" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E1346" t="inlineStr"/>
+      <c r="F1346" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g21</t>
+        </is>
+      </c>
+    </row>
+    <row r="1347">
+      <c r="A1347" t="inlineStr">
+        <is>
+          <t>2026-08-08T23:14:13</t>
+        </is>
+      </c>
+      <c r="B1347" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1347" t="inlineStr">
+        <is>
+          <t>tk_Warmup</t>
+        </is>
+      </c>
+      <c r="D1347" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E1347" t="inlineStr"/>
+      <c r="F1347" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g26</t>
+        </is>
+      </c>
+    </row>
+    <row r="1348">
+      <c r="A1348" t="inlineStr">
+        <is>
+          <t>2026-08-08T23:14:13</t>
+        </is>
+      </c>
+      <c r="B1348" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1348" t="inlineStr">
+        <is>
+          <t>FindingParts min</t>
+        </is>
+      </c>
+      <c r="D1348" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E1348" t="inlineStr"/>
+      <c r="F1348" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g27</t>
+        </is>
+      </c>
+    </row>
+    <row r="1349">
+      <c r="A1349" t="inlineStr">
+        <is>
+          <t>2026-08-08T23:14:13</t>
+        </is>
+      </c>
+      <c r="B1349" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1349" t="inlineStr">
+        <is>
+          <t>PickingParts min</t>
+        </is>
+      </c>
+      <c r="D1349" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E1349" t="inlineStr"/>
+      <c r="F1349" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g28</t>
+        </is>
+      </c>
+    </row>
+    <row r="1350">
+      <c r="A1350" t="inlineStr">
+        <is>
+          <t>2026-08-08T23:14:13</t>
+        </is>
+      </c>
+      <c r="B1350" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1350" t="inlineStr">
+        <is>
+          <t>PlacingParts min</t>
+        </is>
+      </c>
+      <c r="D1350" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E1350" t="inlineStr"/>
+      <c r="F1350" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g29</t>
+        </is>
+      </c>
+    </row>
+    <row r="1351">
+      <c r="A1351" t="inlineStr">
+        <is>
+          <t>2026-08-08T23:14:13</t>
+        </is>
+      </c>
+      <c r="B1351" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1351" t="inlineStr">
+        <is>
+          <t>CountPickedReject14in</t>
+        </is>
+      </c>
+      <c r="D1351" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E1351" t="inlineStr"/>
+      <c r="F1351" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g30</t>
+        </is>
+      </c>
+    </row>
+    <row r="1352">
+      <c r="A1352" t="inlineStr">
+        <is>
+          <t>2026-08-08T23:14:13</t>
+        </is>
+      </c>
+      <c r="B1352" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1352" t="inlineStr">
+        <is>
+          <t>temp_dsi</t>
+        </is>
+      </c>
+      <c r="D1352" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E1352" t="inlineStr"/>
+      <c r="F1352" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g31</t>
+        </is>
+      </c>
+    </row>
+    <row r="1353">
+      <c r="A1353" t="inlineStr">
+        <is>
+          <t>2026-08-08T23:14:13</t>
+        </is>
+      </c>
+      <c r="B1353" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1353" t="inlineStr">
+        <is>
+          <t>temp_J1motor</t>
+        </is>
+      </c>
+      <c r="D1353" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E1353" t="inlineStr"/>
+      <c r="F1353" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g32</t>
+        </is>
+      </c>
+    </row>
+    <row r="1354">
+      <c r="A1354" t="inlineStr">
+        <is>
+          <t>2026-08-08T23:14:13</t>
+        </is>
+      </c>
+      <c r="B1354" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1354" t="inlineStr">
+        <is>
+          <t>temp_J4motor</t>
+        </is>
+      </c>
+      <c r="D1354" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E1354" t="inlineStr"/>
+      <c r="F1354" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g35</t>
+        </is>
+      </c>
+    </row>
+    <row r="1355">
+      <c r="A1355" t="inlineStr">
+        <is>
+          <t>2026-08-08T23:14:13</t>
+        </is>
+      </c>
+      <c r="B1355" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1355" t="inlineStr">
+        <is>
+          <t>temp_J6motor</t>
+        </is>
+      </c>
+      <c r="D1355" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E1355" t="inlineStr"/>
+      <c r="F1355" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g37</t>
+        </is>
+      </c>
+    </row>
+    <row r="1356">
+      <c r="A1356" t="inlineStr">
+        <is>
+          <t>2026-08-08T23:14:13</t>
+        </is>
+      </c>
+      <c r="B1356" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1356" t="inlineStr">
+        <is>
+          <t>CountPickedRejectOTM</t>
+        </is>
+      </c>
+      <c r="D1356" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E1356" t="inlineStr"/>
+      <c r="F1356" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g38</t>
+        </is>
+      </c>
+    </row>
+    <row r="1357">
+      <c r="A1357" t="inlineStr">
+        <is>
+          <t>2026-08-08T23:14:13</t>
+        </is>
+      </c>
+      <c r="B1357" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1357" t="inlineStr">
+        <is>
+          <t>CountPickedRejectPandral</t>
+        </is>
+      </c>
+      <c r="D1357" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E1357" t="inlineStr"/>
+      <c r="F1357" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g39</t>
+        </is>
+      </c>
+    </row>
+    <row r="1358">
+      <c r="A1358" t="inlineStr">
+        <is>
+          <t>2026-08-08T23:14:13</t>
+        </is>
+      </c>
+      <c r="B1358" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1358" t="inlineStr">
+        <is>
+          <t>CountLaidButton</t>
+        </is>
+      </c>
+      <c r="D1358" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E1358" t="inlineStr"/>
+      <c r="F1358" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g2</t>
+        </is>
+      </c>
+    </row>
+    <row r="1359">
+      <c r="A1359" t="inlineStr">
+        <is>
+          <t>2026-08-08T23:14:13</t>
+        </is>
+      </c>
+      <c r="B1359" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1359" t="inlineStr">
+        <is>
+          <t>CountLaidDetector</t>
+        </is>
+      </c>
+      <c r="D1359" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E1359" t="inlineStr"/>
+      <c r="F1359" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g3</t>
+        </is>
+      </c>
+    </row>
+    <row r="1360">
+      <c r="A1360" t="inlineStr">
+        <is>
+          <t>2026-08-08T23:14:13</t>
+        </is>
+      </c>
+      <c r="B1360" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1360" t="inlineStr">
+        <is>
+          <t>CountLaidEncoder</t>
+        </is>
+      </c>
+      <c r="D1360" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E1360" t="inlineStr"/>
+      <c r="F1360" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g4</t>
+        </is>
+      </c>
+    </row>
+    <row r="1361">
+      <c r="A1361" t="inlineStr">
+        <is>
+          <t>2026-08-08T23:14:13</t>
+        </is>
+      </c>
+      <c r="B1361" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1361" t="inlineStr">
+        <is>
+          <t>CountLaid14in</t>
+        </is>
+      </c>
+      <c r="D1361" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E1361" t="inlineStr"/>
+      <c r="F1361" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g5</t>
+        </is>
+      </c>
+    </row>
+    <row r="1362">
+      <c r="A1362" t="inlineStr">
+        <is>
+          <t>2026-08-08T23:14:13</t>
+        </is>
+      </c>
+      <c r="B1362" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1362" t="inlineStr">
+        <is>
+          <t>CountLaid18in</t>
+        </is>
+      </c>
+      <c r="D1362" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E1362" t="inlineStr"/>
+      <c r="F1362" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g6</t>
+        </is>
+      </c>
+    </row>
+    <row r="1363">
+      <c r="A1363" t="inlineStr">
+        <is>
+          <t>2026-08-08T23:14:13</t>
+        </is>
+      </c>
+      <c r="B1363" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1363" t="inlineStr">
+        <is>
+          <t>CountLaidPandral</t>
+        </is>
+      </c>
+      <c r="D1363" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E1363" t="inlineStr"/>
+      <c r="F1363" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g7</t>
+        </is>
+      </c>
+    </row>
+    <row r="1364">
+      <c r="A1364" t="inlineStr">
+        <is>
+          <t>2026-08-08T23:14:13</t>
+        </is>
+      </c>
+      <c r="B1364" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1364" t="inlineStr">
+        <is>
+          <t>18in Job</t>
+        </is>
+      </c>
+      <c r="D1364" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E1364" t="inlineStr"/>
+      <c r="F1364" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g13</t>
+        </is>
+      </c>
+    </row>
+    <row r="1365">
+      <c r="A1365" t="inlineStr">
+        <is>
+          <t>2026-08-08T23:14:13</t>
+        </is>
+      </c>
+      <c r="B1365" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1365" t="inlineStr">
+        <is>
+          <t>CountAcceptedTotal</t>
+        </is>
+      </c>
+      <c r="D1365" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E1365" t="inlineStr"/>
+      <c r="F1365" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g15</t>
+        </is>
+      </c>
+    </row>
+    <row r="1366">
+      <c r="A1366" t="inlineStr">
+        <is>
+          <t>2026-08-08T23:14:13</t>
+        </is>
+      </c>
+      <c r="B1366" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1366" t="inlineStr">
+        <is>
+          <t>Servos_Enabled</t>
+        </is>
+      </c>
+      <c r="D1366" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E1366" t="inlineStr"/>
+      <c r="F1366" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g17</t>
+        </is>
+      </c>
+    </row>
+    <row r="1367">
+      <c r="A1367" t="inlineStr">
+        <is>
+          <t>2026-08-08T23:14:13</t>
+        </is>
+      </c>
+      <c r="B1367" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1367" t="inlineStr">
+        <is>
+          <t>TotalPickPartsCount</t>
+        </is>
+      </c>
+      <c r="D1367" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E1367" t="inlineStr"/>
+      <c r="F1367" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g18</t>
+        </is>
+      </c>
+    </row>
+    <row r="1368">
+      <c r="A1368" t="inlineStr">
+        <is>
+          <t>2026-08-08T23:14:13</t>
+        </is>
+      </c>
+      <c r="B1368" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1368" t="inlineStr">
+        <is>
+          <t>AcceptsPartsCount</t>
+        </is>
+      </c>
+      <c r="D1368" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E1368" t="inlineStr"/>
+      <c r="F1368" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g19</t>
+        </is>
+      </c>
+    </row>
+    <row r="1369">
+      <c r="A1369" t="inlineStr">
+        <is>
+          <t>2026-08-08T23:14:13</t>
+        </is>
+      </c>
+      <c r="B1369" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1369" t="inlineStr">
+        <is>
+          <t>day_Servotime Hours10th</t>
+        </is>
+      </c>
+      <c r="D1369" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E1369" t="inlineStr"/>
+      <c r="F1369" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g22</t>
+        </is>
+      </c>
+    </row>
+    <row r="1370">
+      <c r="A1370" t="inlineStr">
+        <is>
+          <t>2026-08-08T23:14:13</t>
+        </is>
+      </c>
+      <c r="B1370" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1370" t="inlineStr">
+        <is>
+          <t>tk_Cycle</t>
+        </is>
+      </c>
+      <c r="D1370" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E1370" t="inlineStr"/>
+      <c r="F1370" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g23</t>
+        </is>
+      </c>
+    </row>
+    <row r="1371">
+      <c r="A1371" t="inlineStr">
+        <is>
+          <t>2026-08-08T23:14:13</t>
+        </is>
+      </c>
+      <c r="B1371" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1371" t="inlineStr">
+        <is>
+          <t>tk_Abort</t>
+        </is>
+      </c>
+      <c r="D1371" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E1371" t="inlineStr"/>
+      <c r="F1371" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g24</t>
+        </is>
+      </c>
+    </row>
+    <row r="1372">
+      <c r="A1372" t="inlineStr">
+        <is>
+          <t>2026-08-08T23:14:13</t>
+        </is>
+      </c>
+      <c r="B1372" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1372" t="inlineStr">
+        <is>
+          <t>tk_ClearPos</t>
+        </is>
+      </c>
+      <c r="D1372" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E1372" t="inlineStr"/>
+      <c r="F1372" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g25</t>
+        </is>
+      </c>
+    </row>
+    <row r="1373">
+      <c r="A1373" t="inlineStr">
+        <is>
+          <t>2026-08-08T23:14:13</t>
+        </is>
+      </c>
+      <c r="B1373" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1373" t="inlineStr">
+        <is>
+          <t>temp_J2motor</t>
+        </is>
+      </c>
+      <c r="D1373" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E1373" t="inlineStr"/>
+      <c r="F1373" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g33</t>
+        </is>
+      </c>
+    </row>
+    <row r="1374">
+      <c r="A1374" t="inlineStr">
+        <is>
+          <t>2026-08-08T23:14:13</t>
+        </is>
+      </c>
+      <c r="B1374" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1374" t="inlineStr">
+        <is>
+          <t>temp_J3motor</t>
+        </is>
+      </c>
+      <c r="D1374" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E1374" t="inlineStr"/>
+      <c r="F1374" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g34</t>
+        </is>
+      </c>
+    </row>
+    <row r="1375">
+      <c r="A1375" t="inlineStr">
+        <is>
+          <t>2026-08-08T23:14:13</t>
+        </is>
+      </c>
+      <c r="B1375" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1375" t="inlineStr">
+        <is>
+          <t>temp_J5motor</t>
+        </is>
+      </c>
+      <c r="D1375" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E1375" t="inlineStr"/>
+      <c r="F1375" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g36</t>
+        </is>
+      </c>
+    </row>
+    <row r="1376">
+      <c r="A1376" t="inlineStr">
+        <is>
+          <t>2026-08-08T23:14:13</t>
+        </is>
+      </c>
+      <c r="B1376" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1376" t="inlineStr">
+        <is>
+          <t>CountPickedReject18in</t>
+        </is>
+      </c>
+      <c r="D1376" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E1376" t="inlineStr"/>
+      <c r="F1376" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/hmi/g40</t>
+        </is>
+      </c>
+    </row>
+    <row r="1377">
+      <c r="A1377" t="inlineStr">
+        <is>
+          <t>2026-08-08T23:15:00</t>
+        </is>
+      </c>
+      <c r="B1377" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1377" t="inlineStr">
+        <is>
+          <t>_1st_SCAN</t>
+        </is>
+      </c>
+      <c r="D1377" t="b">
+        <v>0</v>
+      </c>
+      <c r="E1377" t="n">
+        <v>11</v>
+      </c>
+      <c r="F1377" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1378">
+      <c r="A1378" t="inlineStr">
+        <is>
+          <t>2026-08-08T23:15:00</t>
+        </is>
+      </c>
+      <c r="B1378" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1378" t="inlineStr">
+        <is>
+          <t>TieDetectOffset_B</t>
+        </is>
+      </c>
+      <c r="D1378" t="b">
+        <v>0</v>
+      </c>
+      <c r="E1378" t="n">
+        <v>11</v>
+      </c>
+      <c r="F1378" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1379">
+      <c r="A1379" t="inlineStr">
+        <is>
+          <t>2026-08-08T23:15:00</t>
+        </is>
+      </c>
+      <c r="B1379" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1379" t="inlineStr">
+        <is>
+          <t>Tie Detector</t>
+        </is>
+      </c>
+      <c r="D1379" t="b">
+        <v>0</v>
+      </c>
+      <c r="E1379" t="n">
+        <v>11</v>
+      </c>
+      <c r="F1379" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1380">
+      <c r="A1380" t="inlineStr">
+        <is>
+          <t>2026-08-08T23:15:00</t>
+        </is>
+      </c>
+      <c r="B1380" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1380" t="inlineStr">
+        <is>
+          <t>TPS Full</t>
+        </is>
+      </c>
+      <c r="D1380" t="b">
+        <v>0</v>
+      </c>
+      <c r="E1380" t="n">
+        <v>11</v>
+      </c>
+      <c r="F1380" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1381">
+      <c r="A1381" t="inlineStr">
+        <is>
+          <t>2026-08-08T23:15:00</t>
+        </is>
+      </c>
+      <c r="B1381" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1381" t="inlineStr">
+        <is>
+          <t>TieDetectOffset_A</t>
+        </is>
+      </c>
+      <c r="D1381" t="b">
+        <v>0</v>
+      </c>
+      <c r="E1381" t="n">
+        <v>11</v>
+      </c>
+      <c r="F1381" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1382">
+      <c r="A1382" t="inlineStr">
+        <is>
+          <t>2026-08-08T23:15:00</t>
+        </is>
+      </c>
+      <c r="B1382" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1382" t="inlineStr">
+        <is>
+          <t>TPS Connected</t>
+        </is>
+      </c>
+      <c r="D1382" t="b">
+        <v>0</v>
+      </c>
+      <c r="E1382" t="n">
+        <v>11</v>
+      </c>
+      <c r="F1382" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1383">
+      <c r="A1383" t="inlineStr">
+        <is>
+          <t>2026-08-08T23:15:00</t>
+        </is>
+      </c>
+      <c r="B1383" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1383" t="inlineStr">
+        <is>
+          <t>TPS_Enable_ Button</t>
+        </is>
+      </c>
+      <c r="D1383" t="b">
+        <v>0</v>
+      </c>
+      <c r="E1383" t="n">
+        <v>11</v>
+      </c>
+      <c r="F1383" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1384">
+      <c r="A1384" t="inlineStr">
+        <is>
+          <t>2026-08-08T23:15:00</t>
+        </is>
+      </c>
+      <c r="B1384" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1384" t="inlineStr">
+        <is>
+          <t>AirEagle Eject Plate</t>
+        </is>
+      </c>
+      <c r="D1384" t="b">
+        <v>0</v>
+      </c>
+      <c r="E1384" t="n">
+        <v>11</v>
+      </c>
+      <c r="F1384" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1385">
+      <c r="A1385" t="inlineStr">
+        <is>
+          <t>2026-08-08T23:15:00</t>
+        </is>
+      </c>
+      <c r="B1385" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1385" t="inlineStr">
+        <is>
+          <t>tk_Cycle</t>
+        </is>
+      </c>
+      <c r="D1385" t="b">
+        <v>0</v>
+      </c>
+      <c r="E1385" t="n">
+        <v>11</v>
+      </c>
+      <c r="F1385" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1386">
+      <c r="A1386" t="inlineStr">
+        <is>
+          <t>2026-08-08T23:15:00</t>
+        </is>
+      </c>
+      <c r="B1386" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1386" t="inlineStr">
+        <is>
+          <t>Servos_Enabled</t>
+        </is>
+      </c>
+      <c r="D1386" t="b">
+        <v>0</v>
+      </c>
+      <c r="E1386" t="n">
+        <v>11</v>
+      </c>
+      <c r="F1386" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1387">
+      <c r="A1387" t="inlineStr">
+        <is>
+          <t>2026-08-08T23:15:00</t>
+        </is>
+      </c>
+      <c r="B1387" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1387" t="inlineStr">
+        <is>
+          <t>TPS Enabled</t>
+        </is>
+      </c>
+      <c r="D1387" t="b">
+        <v>0</v>
+      </c>
+      <c r="E1387" t="n">
+        <v>11</v>
+      </c>
+      <c r="F1387" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1388">
+      <c r="A1388" t="inlineStr">
+        <is>
+          <t>2026-08-08T23:15:00</t>
+        </is>
+      </c>
+      <c r="B1388" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1388" t="inlineStr">
+        <is>
+          <t>tk_Abort</t>
+        </is>
+      </c>
+      <c r="D1388" t="b">
+        <v>0</v>
+      </c>
+      <c r="E1388" t="n">
+        <v>11</v>
+      </c>
+      <c r="F1388" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1389">
+      <c r="A1389" t="inlineStr">
+        <is>
+          <t>2026-08-08T23:15:00</t>
+        </is>
+      </c>
+      <c r="B1389" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1389" t="inlineStr">
+        <is>
+          <t>Robot_isMoving</t>
+        </is>
+      </c>
+      <c r="D1389" t="b">
+        <v>0</v>
+      </c>
+      <c r="E1389" t="n">
+        <v>11</v>
+      </c>
+      <c r="F1389" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1390">
+      <c r="A1390" t="inlineStr">
+        <is>
+          <t>2026-08-08T23:15:00</t>
+        </is>
+      </c>
+      <c r="B1390" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1390" t="inlineStr">
+        <is>
+          <t>Eject Tie Plate</t>
+        </is>
+      </c>
+      <c r="D1390" t="b">
+        <v>0</v>
+      </c>
+      <c r="E1390" t="n">
+        <v>11</v>
+      </c>
+      <c r="F1390" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1391">
+      <c r="A1391" t="inlineStr">
+        <is>
+          <t>2026-08-08T23:15:00</t>
+        </is>
+      </c>
+      <c r="B1391" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1391" t="inlineStr">
+        <is>
+          <t>TPS BACKUP ALARM</t>
+        </is>
+      </c>
+      <c r="D1391" t="b">
+        <v>0</v>
+      </c>
+      <c r="E1391" t="n">
+        <v>11</v>
+      </c>
+      <c r="F1391" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1392">
+      <c r="A1392" t="inlineStr">
+        <is>
+          <t>2026-08-08T23:15:00</t>
+        </is>
+      </c>
+      <c r="B1392" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1392" t="inlineStr">
+        <is>
+          <t>14in Job</t>
+        </is>
+      </c>
+      <c r="D1392" t="b">
+        <v>1</v>
+      </c>
+      <c r="E1392" t="n">
+        <v>11</v>
+      </c>
+      <c r="F1392" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1393">
+      <c r="A1393" t="inlineStr">
+        <is>
+          <t>2026-08-08T23:15:00</t>
+        </is>
+      </c>
+      <c r="B1393" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1393" t="inlineStr">
+        <is>
+          <t>18in Job</t>
+        </is>
+      </c>
+      <c r="D1393" t="b">
+        <v>0</v>
+      </c>
+      <c r="E1393" t="n">
+        <v>11</v>
+      </c>
+      <c r="F1393" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1394">
+      <c r="A1394" t="inlineStr">
+        <is>
+          <t>2026-08-08T23:15:00</t>
+        </is>
+      </c>
+      <c r="B1394" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1394" t="inlineStr">
+        <is>
+          <t>Pandral Job</t>
+        </is>
+      </c>
+      <c r="D1394" t="b">
+        <v>0</v>
+      </c>
+      <c r="E1394" t="n">
+        <v>11</v>
+      </c>
+      <c r="F1394" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1395">
+      <c r="A1395" t="inlineStr">
+        <is>
+          <t>2026-08-08T23:15:00</t>
+        </is>
+      </c>
+      <c r="B1395" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1395" t="inlineStr">
+        <is>
+          <t>DoubleLay Job</t>
+        </is>
+      </c>
+      <c r="D1395" t="b">
+        <v>0</v>
+      </c>
+      <c r="E1395" t="n">
+        <v>11</v>
+      </c>
+      <c r="F1395" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1396">
+      <c r="A1396" t="inlineStr">
+        <is>
+          <t>2026-08-08T23:15:00</t>
+        </is>
+      </c>
+      <c r="B1396" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1396" t="inlineStr">
+        <is>
+          <t>TPSjam_FLAG</t>
+        </is>
+      </c>
+      <c r="D1396" t="b">
+        <v>0</v>
+      </c>
+      <c r="E1396" t="n">
+        <v>11</v>
+      </c>
+      <c r="F1396" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1397">
+      <c r="A1397" t="inlineStr">
+        <is>
+          <t>2026-08-08T23:15:00</t>
+        </is>
+      </c>
+      <c r="B1397" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1397" t="inlineStr">
+        <is>
+          <t>RoCalRequest</t>
+        </is>
+      </c>
+      <c r="D1397" t="b">
+        <v>0</v>
+      </c>
+      <c r="E1397" t="n">
+        <v>11</v>
+      </c>
+      <c r="F1397" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1398">
+      <c r="A1398" t="inlineStr">
+        <is>
+          <t>2026-08-08T23:15:00</t>
+        </is>
+      </c>
+      <c r="B1398" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1398" t="inlineStr">
+        <is>
+          <t>tkCycle_TotalSeconds</t>
+        </is>
+      </c>
+      <c r="D1398" t="n">
+        <v>0</v>
+      </c>
+      <c r="E1398" t="n">
+        <v>9</v>
+      </c>
+      <c r="F1398" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1399">
+      <c r="A1399" t="inlineStr">
+        <is>
+          <t>2026-08-08T23:15:00</t>
+        </is>
+      </c>
+      <c r="B1399" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1399" t="inlineStr">
+        <is>
+          <t>tkCycle_NoMoveSec</t>
+        </is>
+      </c>
+      <c r="D1399" t="n">
+        <v>0</v>
+      </c>
+      <c r="E1399" t="n">
+        <v>9</v>
+      </c>
+      <c r="F1399" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1400">
+      <c r="A1400" t="inlineStr">
+        <is>
+          <t>2026-08-08T23:15:00</t>
+        </is>
+      </c>
+      <c r="B1400" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1400" t="inlineStr">
+        <is>
+          <t>tkCycle_MoveSeconds</t>
+        </is>
+      </c>
+      <c r="D1400" t="n">
+        <v>0</v>
+      </c>
+      <c r="E1400" t="n">
+        <v>9</v>
+      </c>
+      <c r="F1400" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1401">
+      <c r="A1401" t="inlineStr">
+        <is>
+          <t>2026-08-08T23:15:00</t>
+        </is>
+      </c>
+      <c r="B1401" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1401" t="inlineStr">
+        <is>
+          <t>Percent time moveing</t>
+        </is>
+      </c>
+      <c r="D1401" t="n">
+        <v>0</v>
+      </c>
+      <c r="E1401" t="n">
+        <v>9</v>
+      </c>
+      <c r="F1401" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1402">
+      <c r="A1402" t="inlineStr">
+        <is>
+          <t>2026-08-08T23:15:00</t>
+        </is>
+      </c>
+      <c r="B1402" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1402" t="inlineStr">
+        <is>
+          <t>Percent time not moving</t>
+        </is>
+      </c>
+      <c r="D1402" t="n">
+        <v>0</v>
+      </c>
+      <c r="E1402" t="n">
+        <v>9</v>
+      </c>
+      <c r="F1402" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1403">
+      <c r="A1403" t="inlineStr">
+        <is>
+          <t>2026-08-08T23:15:00</t>
+        </is>
+      </c>
+      <c r="B1403" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1403" t="inlineStr">
+        <is>
+          <t>TotalPickPartsCount</t>
+        </is>
+      </c>
+      <c r="D1403" t="n">
+        <v>0</v>
+      </c>
+      <c r="E1403" t="n">
+        <v>9</v>
+      </c>
+      <c r="F1403" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1404">
+      <c r="A1404" t="inlineStr">
+        <is>
+          <t>2026-08-08T23:15:00</t>
+        </is>
+      </c>
+      <c r="B1404" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1404" t="inlineStr">
+        <is>
+          <t>RejectPartsCount</t>
+        </is>
+      </c>
+      <c r="D1404" t="n">
+        <v>0</v>
+      </c>
+      <c r="E1404" t="n">
+        <v>9</v>
+      </c>
+      <c r="F1404" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1405">
+      <c r="A1405" t="inlineStr">
+        <is>
+          <t>2026-08-08T23:15:00</t>
+        </is>
+      </c>
+      <c r="B1405" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1405" t="inlineStr">
+        <is>
+          <t>AcceptsPartsCount</t>
+        </is>
+      </c>
+      <c r="D1405" t="n">
+        <v>0</v>
+      </c>
+      <c r="E1405" t="n">
+        <v>9</v>
+      </c>
+      <c r="F1405" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1406">
+      <c r="A1406" t="inlineStr">
+        <is>
+          <t>2026-08-08T23:15:00</t>
+        </is>
+      </c>
+      <c r="B1406" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1406" t="inlineStr">
+        <is>
+          <t>percentCount_accept</t>
+        </is>
+      </c>
+      <c r="D1406" t="n">
+        <v>0</v>
+      </c>
+      <c r="E1406" t="n">
+        <v>9</v>
+      </c>
+      <c r="F1406" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1407">
+      <c r="A1407" t="inlineStr">
+        <is>
+          <t>2026-08-08T23:15:00</t>
+        </is>
+      </c>
+      <c r="B1407" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1407" t="inlineStr">
+        <is>
+          <t>percentCount_reject</t>
+        </is>
+      </c>
+      <c r="D1407" t="n">
+        <v>0</v>
+      </c>
+      <c r="E1407" t="n">
+        <v>9</v>
+      </c>
+      <c r="F1407" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1408">
+      <c r="A1408" t="inlineStr">
+        <is>
+          <t>2026-08-08T23:15:00</t>
+        </is>
+      </c>
+      <c r="B1408" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1408" t="inlineStr">
+        <is>
+          <t>Avg Parts per min_total</t>
+        </is>
+      </c>
+      <c r="D1408" t="n">
+        <v>0</v>
+      </c>
+      <c r="E1408" t="n">
+        <v>9</v>
+      </c>
+      <c r="F1408" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1409">
+      <c r="A1409" t="inlineStr">
+        <is>
+          <t>2026-08-08T23:15:00</t>
+        </is>
+      </c>
+      <c r="B1409" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1409" t="inlineStr">
+        <is>
+          <t>TotalPickedParts</t>
+        </is>
+      </c>
+      <c r="D1409" t="n">
+        <v>0</v>
+      </c>
+      <c r="E1409" t="n">
+        <v>3</v>
+      </c>
+      <c r="F1409" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1410">
+      <c r="A1410" t="inlineStr">
+        <is>
+          <t>2026-08-08T23:15:00</t>
+        </is>
+      </c>
+      <c r="B1410" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1410" t="inlineStr">
+        <is>
+          <t>TotalPickedAcceptParts</t>
+        </is>
+      </c>
+      <c r="D1410" t="n">
+        <v>0</v>
+      </c>
+      <c r="E1410" t="n">
+        <v>3</v>
+      </c>
+      <c r="F1410" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1411">
+      <c r="A1411" t="inlineStr">
+        <is>
+          <t>2026-08-08T23:15:00</t>
+        </is>
+      </c>
+      <c r="B1411" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1411" t="inlineStr">
+        <is>
+          <t>TotalPickedRejectParts</t>
+        </is>
+      </c>
+      <c r="D1411" t="n">
+        <v>0</v>
+      </c>
+      <c r="E1411" t="n">
+        <v>3</v>
+      </c>
+      <c r="F1411" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1412">
+      <c r="A1412" t="inlineStr">
+        <is>
+          <t>2026-08-08T23:15:00</t>
+        </is>
+      </c>
+      <c r="B1412" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1412" t="inlineStr">
+        <is>
+          <t>TotalTiePlatesLaid</t>
+        </is>
+      </c>
+      <c r="D1412" t="n">
+        <v>0</v>
+      </c>
+      <c r="E1412" t="n">
+        <v>3</v>
+      </c>
+      <c r="F1412" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1413">
+      <c r="A1413" t="inlineStr">
+        <is>
+          <t>2026-08-08T23:15:00</t>
+        </is>
+      </c>
+      <c r="B1413" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1413" t="inlineStr">
+        <is>
+          <t>Daily_TotalLaidPlates</t>
+        </is>
+      </c>
+      <c r="D1413" t="n">
+        <v>0</v>
+      </c>
+      <c r="E1413" t="n">
+        <v>3</v>
+      </c>
+      <c r="F1413" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1414">
+      <c r="A1414" t="inlineStr">
+        <is>
+          <t>2026-08-08T23:15:00</t>
+        </is>
+      </c>
+      <c r="B1414" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1414" t="inlineStr">
+        <is>
+          <t>CountPicked14in</t>
+        </is>
+      </c>
+      <c r="D1414" t="n">
+        <v>0</v>
+      </c>
+      <c r="E1414" t="n">
+        <v>3</v>
+      </c>
+      <c r="F1414" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1415">
+      <c r="A1415" t="inlineStr">
+        <is>
+          <t>2026-08-08T23:15:00</t>
+        </is>
+      </c>
+      <c r="B1415" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1415" t="inlineStr">
+        <is>
+          <t>CountPicked18in</t>
+        </is>
+      </c>
+      <c r="D1415" t="n">
+        <v>0</v>
+      </c>
+      <c r="E1415" t="n">
+        <v>3</v>
+      </c>
+      <c r="F1415" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1416">
+      <c r="A1416" t="inlineStr">
+        <is>
+          <t>2026-08-08T23:15:00</t>
+        </is>
+      </c>
+      <c r="B1416" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1416" t="inlineStr">
+        <is>
+          <t>CountPickedPandral</t>
+        </is>
+      </c>
+      <c r="D1416" t="n">
+        <v>0</v>
+      </c>
+      <c r="E1416" t="n">
+        <v>3</v>
+      </c>
+      <c r="F1416" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1417">
+      <c r="A1417" t="inlineStr">
+        <is>
+          <t>2026-08-08T23:15:00</t>
+        </is>
+      </c>
+      <c r="B1417" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1417" t="inlineStr">
+        <is>
+          <t>CountPickedOTM</t>
+        </is>
+      </c>
+      <c r="D1417" t="n">
+        <v>0</v>
+      </c>
+      <c r="E1417" t="n">
+        <v>3</v>
+      </c>
+      <c r="F1417" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1418">
+      <c r="A1418" t="inlineStr">
+        <is>
+          <t>2026-08-08T23:15:00</t>
+        </is>
+      </c>
+      <c r="B1418" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1418" t="inlineStr">
+        <is>
+          <t>RoCals</t>
+        </is>
+      </c>
+      <c r="D1418" t="n">
+        <v>0</v>
+      </c>
+      <c r="E1418" t="n">
+        <v>3</v>
+      </c>
+      <c r="F1418" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1419">
+      <c r="A1419" t="inlineStr">
+        <is>
+          <t>2026-08-08T23:15:00</t>
+        </is>
+      </c>
+      <c r="B1419" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1419" t="inlineStr">
+        <is>
+          <t>TPS_JamsUsr</t>
+        </is>
+      </c>
+      <c r="D1419" t="n">
+        <v>0</v>
+      </c>
+      <c r="E1419" t="n">
+        <v>3</v>
+      </c>
+      <c r="F1419" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1420">
+      <c r="A1420" t="inlineStr">
+        <is>
+          <t>2026-08-08T23:15:00</t>
+        </is>
+      </c>
+      <c r="B1420" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1420" t="inlineStr">
+        <is>
+          <t>TPS_JamsMASTER</t>
+        </is>
+      </c>
+      <c r="D1420" t="n">
+        <v>0</v>
+      </c>
+      <c r="E1420" t="n">
+        <v>3</v>
+      </c>
+      <c r="F1420" t="inlineStr">
+        <is>
+          <t>raiv-tracker/lab/plc</t>
+        </is>
+      </c>
+    </row>
+    <row r="1421">
+      <c r="A1421" t="inlineStr">
+        <is>
+          <t>2026-08-08T23:15:00</t>
+        </is>
+      </c>
+      <c r="B1421" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C1421" t="inlineStr">
+        <is>
+          <t>ABORT_Master</t>
+        </is>
+      </c>
+      <c r="D1421" t="n">
+        <v>0</v>
+      </c>
+      <c r="E1421" t="n">
+        <v>3</v>
+      </c>
+      <c r="F1421" t="inlineStr">
         <is>
           <t>raiv-tracker/lab/plc</t>
         </is>

</xml_diff>